<commit_message>
fix: ajustar perfil estrictamente a nivel Tecnico en Sistemas (excluir cargos de ingenieria/profesional universitario) y filtrar 79 vacantes remotas de soporte y TI
</commit_message>
<xml_diff>
--- a/output/profile_5_tecnico_sistemas_tracker.xlsx
+++ b/output/profile_5_tecnico_sistemas_tracker.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K88"/>
+  <dimension ref="A1:K113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2231,7 +2231,7 @@
       <c r="H37" s="6" t="inlineStr"/>
       <c r="I37" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 73/100 - Alta Afinidad] Alta coincidencia técnica en Programación, Scripts, SQL y Automatización. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 73/100 - Alta Afinidad] Alta coincidencia técnica en Programación Básica, Scripts, SQL y Automatización. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
@@ -2277,7 +2277,7 @@
       <c r="H38" s="6" t="inlineStr"/>
       <c r="I38" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 73/100 - Alta Afinidad] Alta coincidencia técnica en Programación, Scripts, SQL y Automatización. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 73/100 - Alta Afinidad] Alta coincidencia técnica en Programación Básica, Scripts, SQL y Automatización. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
@@ -3398,26 +3398,26 @@
     <row r="63" ht="22" customHeight="1">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>9d88982013279bd8</t>
+          <t>67d48e405d92af2d</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 15:23</t>
+          <t>2026-09-24 15:37</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>Ingeniero/a de agentes de IA y automatización Multiagente – Senior</t>
+          <t>Coordinado de mesa de ayuda con itil practice manager</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>OC People and services</t>
-        </is>
-      </c>
-      <c r="E63" s="7" t="n">
-        <v>0.68</v>
+          <t>Sinergy &amp; Lowells</t>
+        </is>
+      </c>
+      <c r="E63" s="4" t="n">
+        <v>0.73</v>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
@@ -3425,17 +3425,13 @@
         </is>
       </c>
       <c r="G63" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ingenieroa-de-agentes-de-ia-y-automatizacion-multiagente-senior-en-bogota-dc-D1A0C70BCC17904061373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H63" s="6" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/coordinado-de-mesa-de-ayuda-con-itil-practice-manager-1886758471", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H63" s="6" t="inlineStr"/>
       <c r="I63" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 68/100 - Afinidad Moderada] Alta coincidencia técnica en Programación, Scripts, SQL y Automatización. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 73/100 - Alta Afinidad] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J63" s="2" t="inlineStr">
@@ -3448,26 +3444,26 @@
     <row r="64" ht="22" customHeight="1">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>3fa5f6b47656bee5</t>
+          <t>afee514d25ff4533</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 15:23</t>
+          <t>2026-09-24 15:37</t>
         </is>
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>Analista de Automatización</t>
+          <t>Vacante de inclusión laboral - auxiliar de sistemas / mesa de ayuda</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t>CARVAJAL TECNOLOGIA Y SERVICIOS S.A.S</t>
-        </is>
-      </c>
-      <c r="E64" s="7" t="n">
-        <v>0.68</v>
+          <t>Confidencial</t>
+        </is>
+      </c>
+      <c r="E64" s="4" t="n">
+        <v>0.73</v>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
@@ -3475,17 +3471,13 @@
         </is>
       </c>
       <c r="G64" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-analista-de-automatizacion-marketing-en-bogota-dc-8E8A462321A7AD2261373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H64" s="6" t="inlineStr">
-        <is>
-          <t>$ 3.600.000,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/vacante-de-inclusion-laboral-auxiliar-de-sistemas-mesa-de-ayuda-1886764066", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H64" s="6" t="inlineStr"/>
       <c r="I64" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 68/100 - Afinidad Moderada] Alta coincidencia técnica en Programación, Scripts, SQL y Automatización. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 73/100 - Alta Afinidad] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr">
@@ -3498,26 +3490,26 @@
     <row r="65" ht="22" customHeight="1">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>7df56f2b5c6b6dcf</t>
+          <t>bf46f38ff92f8468</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 15:23</t>
+          <t>2026-09-24 15:37</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>Analista de Datos y Automatización</t>
+          <t>Operador de soporte técnico nivel 1</t>
         </is>
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>Tiempos SAS</t>
-        </is>
-      </c>
-      <c r="E65" s="7" t="n">
-        <v>0.68</v>
+          <t>Cinte Colombia SAS</t>
+        </is>
+      </c>
+      <c r="E65" s="4" t="n">
+        <v>0.73</v>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
@@ -3525,17 +3517,13 @@
         </is>
       </c>
       <c r="G65" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-analista-de-datos-y-automatizacion-teletrabajo-en-bogota-dc-E3868169DA8AE7FC61373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H65" s="6" t="inlineStr">
-        <is>
-          <t>$ 4.570.618,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/operador-de-soporte-tecnico-nivel-1-1886759478", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H65" s="6" t="inlineStr"/>
       <c r="I65" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 68/100 - Afinidad Moderada] Alta coincidencia técnica en Programación, Scripts, SQL y Automatización. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 73/100 - Alta Afinidad] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J65" s="2" t="inlineStr">
@@ -3548,26 +3536,26 @@
     <row r="66" ht="22" customHeight="1">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>e03faa9fc91e4b71</t>
+          <t>69c4d327f77f46d2</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 15:23</t>
+          <t>2026-09-24 15:37</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>Ingeniero Senior de Redes 54223</t>
+          <t>Auxiliar de sistemas e infraestructura para trabajar en cota</t>
         </is>
       </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
-          <t>PeakU</t>
-        </is>
-      </c>
-      <c r="E66" s="7" t="n">
-        <v>0.68</v>
+          <t>ATIEMPO S.A.S</t>
+        </is>
+      </c>
+      <c r="E66" s="4" t="n">
+        <v>0.73</v>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
@@ -3575,17 +3563,13 @@
         </is>
       </c>
       <c r="G66" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ingeniero-senior-de-redes-54223-remoto-en-medellin-823C3FC83EA55A7D61373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H66" s="6" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-e-infraestructura-para-trabajar-en-cota-1886766898", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H66" s="6" t="inlineStr"/>
       <c r="I66" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 68/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 73/100 - Alta Afinidad] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J66" s="2" t="inlineStr">
@@ -3598,26 +3582,26 @@
     <row r="67" ht="22" customHeight="1">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>d3844d860d4f45c1</t>
+          <t>8ea6294af7e133d9</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 15:23</t>
+          <t>2026-09-24 15:37</t>
         </is>
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>Especialista en redes sd-wan / networking</t>
+          <t>Técnico o tecnólogo en sistemas | auxiliar de sistemas e infraestructura - cota</t>
         </is>
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>ATCG DE COLOMBIA S.A.S</t>
-        </is>
-      </c>
-      <c r="E67" s="7" t="n">
-        <v>0.68</v>
+          <t>ATIEMPO S.A.S</t>
+        </is>
+      </c>
+      <c r="E67" s="4" t="n">
+        <v>0.73</v>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
@@ -3625,13 +3609,13 @@
         </is>
       </c>
       <c r="G67" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/especialista-en-redes-sdwan-networking-1886771188", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-o-tecnologo-en-sistemas-auxiliar-de-sistemas-e-infraestructura-cota-1886766903", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H67" s="6" t="inlineStr"/>
       <c r="I67" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 68/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 73/100 - Alta Afinidad] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J67" s="2" t="inlineStr">
@@ -3644,26 +3628,26 @@
     <row r="68" ht="22" customHeight="1">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>910a620a68b48ba5</t>
+          <t>0c0fd09d671f3d44</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 15:23</t>
+          <t>2026-09-24 15:37</t>
         </is>
       </c>
       <c r="C68" s="3" t="inlineStr">
         <is>
-          <t>Ingeniero de redes cisco</t>
+          <t>Agente mesa de ayuda con experiencia</t>
         </is>
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
-          <t>ATCG DE COLOMBIA S.A.S</t>
-        </is>
-      </c>
-      <c r="E68" s="7" t="n">
-        <v>0.68</v>
+          <t>SONDA</t>
+        </is>
+      </c>
+      <c r="E68" s="4" t="n">
+        <v>0.73</v>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
@@ -3671,13 +3655,13 @@
         </is>
       </c>
       <c r="G68" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/ingeniero-de-redes-cisco-1886760088", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-mesa-de-ayuda-con-experiencia-1886769727", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H68" s="6" t="inlineStr"/>
       <c r="I68" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 68/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 73/100 - Alta Afinidad] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J68" s="2" t="inlineStr">
@@ -3690,26 +3674,26 @@
     <row r="69" ht="22" customHeight="1">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>ae736277661dc78b</t>
+          <t>7abab155924d34a2</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 15:23</t>
+          <t>2026-09-24 15:37</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>Analista de redes cisco</t>
+          <t>Agente mesa de ayuda</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>ATCG DE COLOMBIA S.A.S</t>
-        </is>
-      </c>
-      <c r="E69" s="7" t="n">
-        <v>0.68</v>
+          <t>Confidencial</t>
+        </is>
+      </c>
+      <c r="E69" s="4" t="n">
+        <v>0.73</v>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
@@ -3717,13 +3701,13 @@
         </is>
       </c>
       <c r="G69" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-cisco-1886760389", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-mesa-de-ayuda-1886771838", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H69" s="6" t="inlineStr"/>
       <c r="I69" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 68/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 73/100 - Alta Afinidad] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J69" s="2" t="inlineStr">
@@ -3736,26 +3720,26 @@
     <row r="70" ht="22" customHeight="1">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>e29676fac3409ad6</t>
+          <t>1c748c123f2775f8</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 15:23</t>
+          <t>2026-09-24 15:37</t>
         </is>
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>Analista de redes y telecomunicaciones - nivel 1</t>
+          <t>Agente de mesa de ayuda</t>
         </is>
       </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
-          <t>MANPOWER</t>
-        </is>
-      </c>
-      <c r="E70" s="7" t="n">
-        <v>0.68</v>
+          <t>SELCOMP INGENIERÍA SAS</t>
+        </is>
+      </c>
+      <c r="E70" s="4" t="n">
+        <v>0.73</v>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
@@ -3763,13 +3747,13 @@
         </is>
       </c>
       <c r="G70" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-y-telecomunicaciones-nivel-1-1886760565", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-de-mesa-de-ayuda-1886764458", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H70" s="6" t="inlineStr"/>
       <c r="I70" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 68/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 73/100 - Alta Afinidad] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J70" s="2" t="inlineStr">
@@ -3782,26 +3766,26 @@
     <row r="71" ht="22" customHeight="1">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>216a52b7ac10333a</t>
+          <t>c2932440f3be50ff</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 15:23</t>
+          <t>2026-09-24 15:37</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de sistemas mesa de ayuda- bogota norte calle 185 presencial</t>
+          <t>Analista mesa de ayuda para tunja</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
-        </is>
-      </c>
-      <c r="E71" s="7" t="n">
-        <v>0.58</v>
+          <t>Gestión de Seguridad Electrónica</t>
+        </is>
+      </c>
+      <c r="E71" s="4" t="n">
+        <v>0.73</v>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
@@ -3809,13 +3793,13 @@
         </is>
       </c>
       <c r="G71" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-sistemas-mesa-de-ayuda-bogota-norte-calle-185-presencial-1886759808", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-para-tunja-1886699884", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H71" s="6" t="inlineStr"/>
       <c r="I71" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Soporte TI Remoto). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 73/100 - Alta Afinidad] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J71" s="2" t="inlineStr">
@@ -3828,26 +3812,26 @@
     <row r="72" ht="22" customHeight="1">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>c20db52fe65351ad</t>
+          <t>0b7f91df03d9708e</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 15:23</t>
+          <t>2026-09-24 15:37</t>
         </is>
       </c>
       <c r="C72" s="3" t="inlineStr">
         <is>
-          <t>Analista de soporte it. presencial, bogotá</t>
+          <t>Analista mesa de ayuda</t>
         </is>
       </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
-          <t>Cinte Colombia SAS</t>
-        </is>
-      </c>
-      <c r="E72" s="7" t="n">
-        <v>0.58</v>
+          <t>Confidencial</t>
+        </is>
+      </c>
+      <c r="E72" s="4" t="n">
+        <v>0.73</v>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
@@ -3855,13 +3839,13 @@
         </is>
       </c>
       <c r="G72" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-soporte-it-presencial-bogota-1886755633", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-1886754619", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H72" s="6" t="inlineStr"/>
       <c r="I72" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Soporte TI Remoto). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 73/100 - Alta Afinidad] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J72" s="2" t="inlineStr">
@@ -3874,26 +3858,26 @@
     <row r="73" ht="22" customHeight="1">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>155fc78897867636</t>
+          <t>6245a0a87c307de3</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 15:23</t>
+          <t>2026-09-24 15:37</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>Help desk analyst n1 - presencial bogotá - horario diurno rotativo</t>
+          <t>Supervisor mesa de ayuda - bogotá- temporal</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>STEFANINI INFORMATICA &amp; TECNOLOGIA S.A.</t>
-        </is>
-      </c>
-      <c r="E73" s="7" t="n">
-        <v>0.58</v>
+          <t>TIVIT COLOMBIA SAS</t>
+        </is>
+      </c>
+      <c r="E73" s="4" t="n">
+        <v>0.73</v>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
@@ -3901,13 +3885,13 @@
         </is>
       </c>
       <c r="G73" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/help-desk-analyst-n1-presencial-bogota-horario-diurno-rotativo-1886765180", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/supervisor-mesa-de-ayuda-bogota-temporal-1886756748", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H73" s="6" t="inlineStr"/>
       <c r="I73" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Soporte TI Remoto). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 73/100 - Alta Afinidad] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J73" s="2" t="inlineStr">
@@ -3920,26 +3904,26 @@
     <row r="74" ht="22" customHeight="1">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>6d55f3dd43e45493</t>
+          <t>03f363ab408877a2</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 15:23</t>
+          <t>2026-09-24 15:37</t>
         </is>
       </c>
       <c r="C74" s="3" t="inlineStr">
         <is>
-          <t>Help desk analyst n1 - presencial bogotá - término fijo 06 meses</t>
+          <t>Coordinador mesa de ayuda</t>
         </is>
       </c>
       <c r="D74" s="3" t="inlineStr">
         <is>
-          <t>STEFANINI INFORMATICA &amp; TECNOLOGIA S.A.</t>
-        </is>
-      </c>
-      <c r="E74" s="7" t="n">
-        <v>0.58</v>
+          <t>Confidencial</t>
+        </is>
+      </c>
+      <c r="E74" s="4" t="n">
+        <v>0.73</v>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
@@ -3947,13 +3931,13 @@
         </is>
       </c>
       <c r="G74" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/help-desk-analyst-n1-presencial-bogota-termino-fijo-06-meses-1886765188", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/coordinador-mesa-de-ayuda-1886753194", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H74" s="6" t="inlineStr"/>
       <c r="I74" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Soporte TI Remoto). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 73/100 - Alta Afinidad] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J74" s="2" t="inlineStr">
@@ -3966,26 +3950,26 @@
     <row r="75" ht="22" customHeight="1">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>456f34fe64104d96</t>
+          <t>42a7050c3f06b2ae</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 15:23</t>
+          <t>2026-09-24 15:37</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>Ingeniero de datos financieros (python/power bi/sql) - hibrido en bogotá</t>
+          <t>Técnico de mesa de ayuda</t>
         </is>
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>Cinte Colombia SAS</t>
-        </is>
-      </c>
-      <c r="E75" s="7" t="n">
-        <v>0.58</v>
+          <t>Colsof S.A.S</t>
+        </is>
+      </c>
+      <c r="E75" s="4" t="n">
+        <v>0.73</v>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
@@ -3993,13 +3977,13 @@
         </is>
       </c>
       <c r="G75" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/ingeniero-de-datos-financieros-python-power-bi-sql-hibrido-en-bogota-1886770211", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-mesa-de-ayuda-1886731992", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H75" s="6" t="inlineStr"/>
       <c r="I75" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Alta coincidencia técnica en Programación, Scripts, SQL y Automatización. Modalidad: Modalidad híbrida / parcial. Alerta: Modalidad híbrida puede requerir presencia ocasional.</t>
+          <t>[Afinidad: 73/100 - Alta Afinidad] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J75" s="2" t="inlineStr">
@@ -4012,26 +3996,26 @@
     <row r="76" ht="22" customHeight="1">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>ccaf9f8780b44030</t>
+          <t>e5d77b0fc7770ea2</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 15:23</t>
+          <t>2026-09-24 15:37</t>
         </is>
       </c>
       <c r="C76" s="3" t="inlineStr">
         <is>
-          <t>Analista de datos (power bi/etl/excel/sql) - híbrido en bogotá</t>
+          <t>Agente de mesa de ayuda</t>
         </is>
       </c>
       <c r="D76" s="3" t="inlineStr">
         <is>
-          <t>Cinte Colombia SAS</t>
-        </is>
-      </c>
-      <c r="E76" s="7" t="n">
-        <v>0.58</v>
+          <t>SONDA</t>
+        </is>
+      </c>
+      <c r="E76" s="4" t="n">
+        <v>0.73</v>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
@@ -4039,13 +4023,13 @@
         </is>
       </c>
       <c r="G76" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-datos-power-bi-etl-excel-sql-hibrido-en-bogota-1886758056", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-de-mesa-de-ayuda-1886748231", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H76" s="6" t="inlineStr"/>
       <c r="I76" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Alta coincidencia técnica en Programación, Scripts, SQL y Automatización. Modalidad: Modalidad híbrida / parcial. Alerta: Modalidad híbrida puede requerir presencia ocasional.</t>
+          <t>[Afinidad: 73/100 - Alta Afinidad] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J76" s="2" t="inlineStr">
@@ -4058,26 +4042,26 @@
     <row r="77" ht="22" customHeight="1">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>75eff91cd86e2d25</t>
+          <t>8bb787ccf4370a8e</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 15:23</t>
+          <t>2026-09-24 15:37</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
         <is>
-          <t>Analista de soporte cisco aci y redes lan - bogotá presencial 100%</t>
+          <t>Mesa de ayuda / bogotá</t>
         </is>
       </c>
       <c r="D77" s="3" t="inlineStr">
         <is>
-          <t>TALYCAP GLOBAL SAS</t>
-        </is>
-      </c>
-      <c r="E77" s="7" t="n">
-        <v>0.58</v>
+          <t>Colsof S.A.S</t>
+        </is>
+      </c>
+      <c r="E77" s="4" t="n">
+        <v>0.73</v>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
@@ -4085,13 +4069,13 @@
         </is>
       </c>
       <c r="G77" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-soporte-cisco-aci-y-redes-lan-bogota-presencial-100-1886751212", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/mesa-de-ayuda-bogota-1886752825", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H77" s="6" t="inlineStr"/>
       <c r="I77" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Soporte TI Remoto). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 73/100 - Alta Afinidad] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J77" s="2" t="inlineStr">
@@ -4104,26 +4088,26 @@
     <row r="78" ht="22" customHeight="1">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>ea62374731b3e510</t>
+          <t>2c0788a7a3b3417d</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 15:23</t>
+          <t>2026-09-24 15:37</t>
         </is>
       </c>
       <c r="C78" s="3" t="inlineStr">
         <is>
-          <t>Frontend Web Application Developer</t>
+          <t>Analista mesa de ayuda nivel 1 / técnico o tecnólogo en sistemas / cota</t>
         </is>
       </c>
       <c r="D78" s="3" t="inlineStr">
         <is>
-          <t>KoboToolbox</t>
-        </is>
-      </c>
-      <c r="E78" s="7" t="n">
-        <v>0.58</v>
+          <t>IMPRESISTEM S.A.</t>
+        </is>
+      </c>
+      <c r="E78" s="4" t="n">
+        <v>0.73</v>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
@@ -4131,17 +4115,13 @@
         </is>
       </c>
       <c r="G78" s="5">
-        <f>HYPERLINK("https://remotive.com/remote-jobs/design/frontend-web-application-developer-2091141", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H78" s="6" t="inlineStr">
-        <is>
-          <t>$90k - $105k</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-nivel-1-tecnico-o-tecnologo-en-sistemas-cota-1886757061", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H78" s="6" t="inlineStr"/>
       <c r="I78" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Alta coincidencia técnica en Programación, Scripts, SQL y Automatización. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 73/100 - Alta Afinidad] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J78" s="2" t="inlineStr">
@@ -4154,26 +4134,26 @@
     <row r="79" ht="22" customHeight="1">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>e8e8c41d26fee7e8</t>
+          <t>97a1b3f2527f8ce8</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 15:23</t>
+          <t>2026-09-24 15:37</t>
         </is>
       </c>
       <c r="C79" s="3" t="inlineStr">
         <is>
-          <t>Senior Shopify Developer</t>
+          <t>Analista de mesa de ayuda l1 - medellín</t>
         </is>
       </c>
       <c r="D79" s="3" t="inlineStr">
         <is>
-          <t>Sanctuary Computer Inc</t>
-        </is>
-      </c>
-      <c r="E79" s="7" t="n">
-        <v>0.58</v>
+          <t>Confidencial</t>
+        </is>
+      </c>
+      <c r="E79" s="4" t="n">
+        <v>0.73</v>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
@@ -4181,17 +4161,13 @@
         </is>
       </c>
       <c r="G79" s="5">
-        <f>HYPERLINK("https://remotive.com/remote-jobs/software-development/senior-shopify-developer-2091140", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H79" s="6" t="inlineStr">
-        <is>
-          <t>$80k - $150k</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-mesa-de-ayuda-l1-medellin-1886747056", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H79" s="6" t="inlineStr"/>
       <c r="I79" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Alta coincidencia técnica en Programación, Scripts, SQL y Automatización. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 73/100 - Alta Afinidad] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J79" s="2" t="inlineStr">
@@ -4204,26 +4180,26 @@
     <row r="80" ht="22" customHeight="1">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>6f9a298b38d7d57b</t>
+          <t>a0df8e7687e7665c</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 15:23</t>
+          <t>2026-09-24 15:37</t>
         </is>
       </c>
       <c r="C80" s="3" t="inlineStr">
         <is>
-          <t>Senior AI Engineer</t>
+          <t>Agente mesa de ayuda</t>
         </is>
       </c>
       <c r="D80" s="3" t="inlineStr">
         <is>
-          <t>Lemon.io</t>
-        </is>
-      </c>
-      <c r="E80" s="7" t="n">
-        <v>0.58</v>
+          <t>Confidencial</t>
+        </is>
+      </c>
+      <c r="E80" s="4" t="n">
+        <v>0.73</v>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
@@ -4231,13 +4207,13 @@
         </is>
       </c>
       <c r="G80" s="5">
-        <f>HYPERLINK("https://remotive.com/remote-jobs/artificial-intelligence/senior-ai-engineer-2091131", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-mesa-de-ayuda-tecnologo-o-minimo-6-semestre-de-ingenieria-1886743820", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H80" s="6" t="inlineStr"/>
       <c r="I80" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Alta coincidencia técnica en Programación, Scripts, SQL y Automatización. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 73/100 - Alta Afinidad] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J80" s="2" t="inlineStr">
@@ -4250,26 +4226,26 @@
     <row r="81" ht="22" customHeight="1">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>4dd048896d0f6d65</t>
+          <t>12aafa5353e0252c</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 15:23</t>
+          <t>2026-09-24 15:37</t>
         </is>
       </c>
       <c r="C81" s="3" t="inlineStr">
         <is>
-          <t>Senior .NET Full-stack Developer</t>
+          <t>Técnico de soporte nivel 1 con itil</t>
         </is>
       </c>
       <c r="D81" s="3" t="inlineStr">
         <is>
-          <t>Lemon.io</t>
-        </is>
-      </c>
-      <c r="E81" s="7" t="n">
-        <v>0.58</v>
+          <t>Confidencial</t>
+        </is>
+      </c>
+      <c r="E81" s="4" t="n">
+        <v>0.73</v>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
@@ -4277,13 +4253,13 @@
         </is>
       </c>
       <c r="G81" s="5">
-        <f>HYPERLINK("https://remotive.com/remote-jobs/software-development/senior-net-full-stack-developer-2091130", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-nivel-1-con-itil-1886769153", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H81" s="6" t="inlineStr"/>
       <c r="I81" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Alta coincidencia técnica en Programación, Scripts, SQL y Automatización. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 73/100 - Alta Afinidad] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J81" s="2" t="inlineStr">
@@ -4296,26 +4272,26 @@
     <row r="82" ht="22" customHeight="1">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>a9d8e6e11954b4ed</t>
+          <t>33bef2c4222966bf</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 15:23</t>
+          <t>2026-09-24 15:37</t>
         </is>
       </c>
       <c r="C82" s="3" t="inlineStr">
         <is>
-          <t>Senior Data Scientist</t>
+          <t>Gestor técnico nivel 1</t>
         </is>
       </c>
       <c r="D82" s="3" t="inlineStr">
         <is>
-          <t>Lemon.io</t>
-        </is>
-      </c>
-      <c r="E82" s="7" t="n">
-        <v>0.58</v>
+          <t>Gestión de Seguridad Electrónica</t>
+        </is>
+      </c>
+      <c r="E82" s="4" t="n">
+        <v>0.73</v>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
@@ -4323,13 +4299,13 @@
         </is>
       </c>
       <c r="G82" s="5">
-        <f>HYPERLINK("https://remotive.com/remote-jobs/data/senior-data-scientist-2091129", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/gestor-tecnico-nivel-1-soporte-ti-tunja-1886700537", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H82" s="6" t="inlineStr"/>
       <c r="I82" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Alta coincidencia técnica en Programación, Scripts, SQL y Automatización. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 73/100 - Alta Afinidad] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J82" s="2" t="inlineStr">
@@ -4342,26 +4318,26 @@
     <row r="83" ht="22" customHeight="1">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>a18589077c92ad8c</t>
+          <t>759c05a3a2a45bb7</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 15:23</t>
+          <t>2026-09-24 15:37</t>
         </is>
       </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t>Senior React Full-stack Developer</t>
+          <t>Técnico de soporte de redes y datacenter - bogotá</t>
         </is>
       </c>
       <c r="D83" s="3" t="inlineStr">
         <is>
-          <t>Lemon.io</t>
-        </is>
-      </c>
-      <c r="E83" s="7" t="n">
-        <v>0.58</v>
+          <t>TALYCAP GLOBAL SAS</t>
+        </is>
+      </c>
+      <c r="E83" s="4" t="n">
+        <v>0.73</v>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
@@ -4369,13 +4345,13 @@
         </is>
       </c>
       <c r="G83" s="5">
-        <f>HYPERLINK("https://remotive.com/remote-jobs/software-development/senior-react-full-stack-developer-2091101", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-de-redes-y-datacenter-bogota-1886765274", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H83" s="6" t="inlineStr"/>
       <c r="I83" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Alta coincidencia técnica en Programación, Scripts, SQL y Automatización. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 73/100 - Alta Afinidad] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J83" s="2" t="inlineStr">
@@ -4388,26 +4364,26 @@
     <row r="84" ht="22" customHeight="1">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>6db39c2f55a85146</t>
+          <t>5d9bd5e6584b63b9</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 15:23</t>
+          <t>2026-09-24 15:37</t>
         </is>
       </c>
       <c r="C84" s="3" t="inlineStr">
         <is>
-          <t>Senior QA Engineer</t>
+          <t>Technical Support Help Desk</t>
         </is>
       </c>
       <c r="D84" s="3" t="inlineStr">
         <is>
-          <t>Lemon.io</t>
-        </is>
-      </c>
-      <c r="E84" s="7" t="n">
-        <v>0.58</v>
+          <t>Sutherland</t>
+        </is>
+      </c>
+      <c r="E84" s="4" t="n">
+        <v>0.73</v>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
@@ -4415,13 +4391,13 @@
         </is>
       </c>
       <c r="G84" s="5">
-        <f>HYPERLINK("https://remotive.com/remote-jobs/qa/senior-qa-engineer-2091100", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/technical-support-help-desk-at-sutherland-4466891252", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H84" s="6" t="inlineStr"/>
       <c r="I84" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Alta coincidencia técnica en Programación, Scripts, SQL y Automatización. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 73/100 - Alta Afinidad] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J84" s="2" t="inlineStr">
@@ -4434,26 +4410,26 @@
     <row r="85" ht="22" customHeight="1">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>5828ee7cdbb35c70</t>
+          <t>7652a72b60c5253a</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 15:23</t>
+          <t>2026-09-24 15:37</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>Senior DevOps Engineer</t>
+          <t>Helpdesk &amp; Customer Suceess Operation Agent</t>
         </is>
       </c>
       <c r="D85" s="3" t="inlineStr">
         <is>
-          <t>Lemon.io</t>
-        </is>
-      </c>
-      <c r="E85" s="7" t="n">
-        <v>0.58</v>
+          <t>Regnology</t>
+        </is>
+      </c>
+      <c r="E85" s="4" t="n">
+        <v>0.73</v>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
@@ -4461,13 +4437,13 @@
         </is>
       </c>
       <c r="G85" s="5">
-        <f>HYPERLINK("https://remotive.com/remote-jobs/devops/senior-devops-engineer-2091099", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/helpdesk-customer-suceess-operation-agent-at-regnology-4463373207", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H85" s="6" t="inlineStr"/>
       <c r="I85" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Alta coincidencia técnica en Programación, Scripts, SQL y Automatización. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 73/100 - Alta Afinidad] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J85" s="2" t="inlineStr">
@@ -4480,7 +4456,7 @@
     <row r="86" ht="22" customHeight="1">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>552066cc9c949c2c</t>
+          <t>9d88982013279bd8</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
@@ -4490,16 +4466,16 @@
       </c>
       <c r="C86" s="3" t="inlineStr">
         <is>
-          <t>Tier III Service Desk Engineer</t>
+          <t>Ingeniero/a de agentes de IA y automatización Multiagente – Senior</t>
         </is>
       </c>
       <c r="D86" s="3" t="inlineStr">
         <is>
-          <t>Unio Digital</t>
+          <t>OC People and services</t>
         </is>
       </c>
       <c r="E86" s="7" t="n">
-        <v>0.58</v>
+        <v>0.68</v>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
@@ -4507,13 +4483,17 @@
         </is>
       </c>
       <c r="G86" s="5">
-        <f>HYPERLINK("https://remotive.com/remote-jobs/information-technology/tier-iii-service-desk-engineer-2091045", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H86" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ingenieroa-de-agentes-de-ia-y-automatizacion-multiagente-senior-en-bogota-dc-D1A0C70BCC17904061373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H86" s="6" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
       <c r="I86" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 68/100 - Afinidad Moderada] Alta coincidencia técnica en Programación, Scripts, SQL y Automatización. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J86" s="2" t="inlineStr">
@@ -4526,7 +4506,7 @@
     <row r="87" ht="22" customHeight="1">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>541d99c3c6e9a353</t>
+          <t>3fa5f6b47656bee5</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
@@ -4536,16 +4516,16 @@
       </c>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>Analista de infraestructura i (redes/firewall) - presencial en bogotá</t>
+          <t>Analista de Automatización</t>
         </is>
       </c>
       <c r="D87" s="3" t="inlineStr">
         <is>
-          <t>Cinte Colombia SAS</t>
+          <t>CARVAJAL TECNOLOGIA Y SERVICIOS S.A.S</t>
         </is>
       </c>
       <c r="E87" s="7" t="n">
-        <v>0.53</v>
+        <v>0.68</v>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
@@ -4553,13 +4533,17 @@
         </is>
       </c>
       <c r="G87" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-infraestructura-i-redes-firewall-presencial-en-bogota-1886756899", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H87" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-analista-de-automatizacion-marketing-en-bogota-dc-8E8A462321A7AD2261373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H87" s="6" t="inlineStr">
+        <is>
+          <t>$ 3.600.000,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I87" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Soporte TI Remoto). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 68/100 - Afinidad Moderada] Alta coincidencia técnica en Programación Básica, Scripts, SQL y Automatización. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J87" s="2" t="inlineStr">
@@ -4572,48 +4556,1214 @@
     <row r="88" ht="22" customHeight="1">
       <c r="A88" s="2" t="inlineStr">
         <is>
+          <t>7df56f2b5c6b6dcf</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24 15:23</t>
+        </is>
+      </c>
+      <c r="C88" s="3" t="inlineStr">
+        <is>
+          <t>Analista de Datos y Automatización</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="inlineStr">
+        <is>
+          <t>Tiempos SAS</t>
+        </is>
+      </c>
+      <c r="E88" s="7" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G88" s="5">
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-analista-de-datos-y-automatizacion-teletrabajo-en-bogota-dc-E3868169DA8AE7FC61373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H88" s="6" t="inlineStr">
+        <is>
+          <t>$ 4.570.618,00 (Mensual)</t>
+        </is>
+      </c>
+      <c r="I88" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 68/100 - Afinidad Moderada] Alta coincidencia técnica en Programación Básica, Scripts, SQL y Automatización. Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J88" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K88" s="3" t="inlineStr"/>
+    </row>
+    <row r="89" ht="22" customHeight="1">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>e03faa9fc91e4b71</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24 15:23</t>
+        </is>
+      </c>
+      <c r="C89" s="3" t="inlineStr">
+        <is>
+          <t>Ingeniero Senior de Redes 54223</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="inlineStr">
+        <is>
+          <t>PeakU</t>
+        </is>
+      </c>
+      <c r="E89" s="7" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="F89" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G89" s="5">
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ingeniero-senior-de-redes-54223-remoto-en-medellin-823C3FC83EA55A7D61373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H89" s="6" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="I89" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 68/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J89" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K89" s="3" t="inlineStr"/>
+    </row>
+    <row r="90" ht="22" customHeight="1">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>d3844d860d4f45c1</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24 15:23</t>
+        </is>
+      </c>
+      <c r="C90" s="3" t="inlineStr">
+        <is>
+          <t>Especialista en redes sd-wan / networking</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="inlineStr">
+        <is>
+          <t>ATCG DE COLOMBIA S.A.S</t>
+        </is>
+      </c>
+      <c r="E90" s="7" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G90" s="5">
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/especialista-en-redes-sdwan-networking-1886771188", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H90" s="6" t="inlineStr"/>
+      <c r="I90" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 68/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J90" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K90" s="3" t="inlineStr"/>
+    </row>
+    <row r="91" ht="22" customHeight="1">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>910a620a68b48ba5</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24 15:23</t>
+        </is>
+      </c>
+      <c r="C91" s="3" t="inlineStr">
+        <is>
+          <t>Ingeniero de redes cisco</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="inlineStr">
+        <is>
+          <t>ATCG DE COLOMBIA S.A.S</t>
+        </is>
+      </c>
+      <c r="E91" s="7" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="F91" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G91" s="5">
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/ingeniero-de-redes-cisco-1886760088", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H91" s="6" t="inlineStr"/>
+      <c r="I91" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 68/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J91" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K91" s="3" t="inlineStr"/>
+    </row>
+    <row r="92" ht="22" customHeight="1">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>ae736277661dc78b</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24 15:23</t>
+        </is>
+      </c>
+      <c r="C92" s="3" t="inlineStr">
+        <is>
+          <t>Analista de redes cisco</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="inlineStr">
+        <is>
+          <t>ATCG DE COLOMBIA S.A.S</t>
+        </is>
+      </c>
+      <c r="E92" s="7" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G92" s="5">
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-cisco-1886760389", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H92" s="6" t="inlineStr"/>
+      <c r="I92" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 68/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J92" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K92" s="3" t="inlineStr"/>
+    </row>
+    <row r="93" ht="22" customHeight="1">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>e29676fac3409ad6</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24 15:23</t>
+        </is>
+      </c>
+      <c r="C93" s="3" t="inlineStr">
+        <is>
+          <t>Analista de redes y telecomunicaciones - nivel 1</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="inlineStr">
+        <is>
+          <t>MANPOWER</t>
+        </is>
+      </c>
+      <c r="E93" s="7" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="F93" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G93" s="5">
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-y-telecomunicaciones-nivel-1-1886760565", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H93" s="6" t="inlineStr"/>
+      <c r="I93" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 68/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J93" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K93" s="3" t="inlineStr"/>
+    </row>
+    <row r="94" ht="22" customHeight="1">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>216a52b7ac10333a</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24 15:23</t>
+        </is>
+      </c>
+      <c r="C94" s="3" t="inlineStr">
+        <is>
+          <t>Tecnico de sistemas mesa de ayuda- bogota norte calle 185 presencial</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="inlineStr">
+        <is>
+          <t>Confidencial</t>
+        </is>
+      </c>
+      <c r="E94" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G94" s="5">
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-sistemas-mesa-de-ayuda-bogota-norte-calle-185-presencial-1886759808", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H94" s="6" t="inlineStr"/>
+      <c r="I94" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Soporte TI Remoto). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J94" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K94" s="3" t="inlineStr"/>
+    </row>
+    <row r="95" ht="22" customHeight="1">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>c20db52fe65351ad</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24 15:23</t>
+        </is>
+      </c>
+      <c r="C95" s="3" t="inlineStr">
+        <is>
+          <t>Analista de soporte it. presencial, bogotá</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="inlineStr">
+        <is>
+          <t>Cinte Colombia SAS</t>
+        </is>
+      </c>
+      <c r="E95" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G95" s="5">
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-soporte-it-presencial-bogota-1886755633", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H95" s="6" t="inlineStr"/>
+      <c r="I95" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Soporte TI Remoto). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J95" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K95" s="3" t="inlineStr"/>
+    </row>
+    <row r="96" ht="22" customHeight="1">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>155fc78897867636</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24 15:23</t>
+        </is>
+      </c>
+      <c r="C96" s="3" t="inlineStr">
+        <is>
+          <t>Help desk analyst n1 - presencial bogotá - horario diurno rotativo</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="inlineStr">
+        <is>
+          <t>STEFANINI INFORMATICA &amp; TECNOLOGIA S.A.</t>
+        </is>
+      </c>
+      <c r="E96" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G96" s="5">
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/help-desk-analyst-n1-presencial-bogota-horario-diurno-rotativo-1886765180", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H96" s="6" t="inlineStr"/>
+      <c r="I96" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Soporte TI Remoto). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J96" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K96" s="3" t="inlineStr"/>
+    </row>
+    <row r="97" ht="22" customHeight="1">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>6d55f3dd43e45493</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24 15:23</t>
+        </is>
+      </c>
+      <c r="C97" s="3" t="inlineStr">
+        <is>
+          <t>Help desk analyst n1 - presencial bogotá - término fijo 06 meses</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="inlineStr">
+        <is>
+          <t>STEFANINI INFORMATICA &amp; TECNOLOGIA S.A.</t>
+        </is>
+      </c>
+      <c r="E97" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F97" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G97" s="5">
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/help-desk-analyst-n1-presencial-bogota-termino-fijo-06-meses-1886765188", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H97" s="6" t="inlineStr"/>
+      <c r="I97" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Soporte TI Remoto). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J97" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K97" s="3" t="inlineStr"/>
+    </row>
+    <row r="98" ht="22" customHeight="1">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>456f34fe64104d96</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24 15:23</t>
+        </is>
+      </c>
+      <c r="C98" s="3" t="inlineStr">
+        <is>
+          <t>Ingeniero de datos financieros (python/power bi/sql) - hibrido en bogotá</t>
+        </is>
+      </c>
+      <c r="D98" s="3" t="inlineStr">
+        <is>
+          <t>Cinte Colombia SAS</t>
+        </is>
+      </c>
+      <c r="E98" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F98" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G98" s="5">
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/ingeniero-de-datos-financieros-python-power-bi-sql-hibrido-en-bogota-1886770211", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H98" s="6" t="inlineStr"/>
+      <c r="I98" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Alta coincidencia técnica en Programación, Scripts, SQL y Automatización. Modalidad: Modalidad híbrida / parcial. Alerta: Modalidad híbrida puede requerir presencia ocasional.</t>
+        </is>
+      </c>
+      <c r="J98" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K98" s="3" t="inlineStr"/>
+    </row>
+    <row r="99" ht="22" customHeight="1">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>ccaf9f8780b44030</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24 15:23</t>
+        </is>
+      </c>
+      <c r="C99" s="3" t="inlineStr">
+        <is>
+          <t>Analista de datos (power bi/etl/excel/sql) - híbrido en bogotá</t>
+        </is>
+      </c>
+      <c r="D99" s="3" t="inlineStr">
+        <is>
+          <t>Cinte Colombia SAS</t>
+        </is>
+      </c>
+      <c r="E99" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F99" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G99" s="5">
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-datos-power-bi-etl-excel-sql-hibrido-en-bogota-1886758056", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H99" s="6" t="inlineStr"/>
+      <c r="I99" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Alta coincidencia técnica en Programación Básica, Scripts, SQL y Automatización. Modalidad: Modalidad híbrida / parcial. Alerta: Modalidad híbrida puede requerir presencia ocasional.</t>
+        </is>
+      </c>
+      <c r="J99" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K99" s="3" t="inlineStr"/>
+    </row>
+    <row r="100" ht="22" customHeight="1">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>75eff91cd86e2d25</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24 15:23</t>
+        </is>
+      </c>
+      <c r="C100" s="3" t="inlineStr">
+        <is>
+          <t>Analista de soporte cisco aci y redes lan - bogotá presencial 100%</t>
+        </is>
+      </c>
+      <c r="D100" s="3" t="inlineStr">
+        <is>
+          <t>TALYCAP GLOBAL SAS</t>
+        </is>
+      </c>
+      <c r="E100" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F100" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G100" s="5">
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-soporte-cisco-aci-y-redes-lan-bogota-presencial-100-1886751212", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H100" s="6" t="inlineStr"/>
+      <c r="I100" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Soporte TI Remoto). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J100" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K100" s="3" t="inlineStr"/>
+    </row>
+    <row r="101" ht="22" customHeight="1">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>ea62374731b3e510</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24 15:23</t>
+        </is>
+      </c>
+      <c r="C101" s="3" t="inlineStr">
+        <is>
+          <t>Frontend Web Application Developer</t>
+        </is>
+      </c>
+      <c r="D101" s="3" t="inlineStr">
+        <is>
+          <t>KoboToolbox</t>
+        </is>
+      </c>
+      <c r="E101" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F101" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G101" s="5">
+        <f>HYPERLINK("https://remotive.com/remote-jobs/design/frontend-web-application-developer-2091141", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H101" s="6" t="inlineStr">
+        <is>
+          <t>$90k - $105k</t>
+        </is>
+      </c>
+      <c r="I101" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Alta coincidencia técnica en Programación Básica, Scripts, SQL y Automatización. Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J101" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K101" s="3" t="inlineStr"/>
+    </row>
+    <row r="102" ht="22" customHeight="1">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>e8e8c41d26fee7e8</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24 15:23</t>
+        </is>
+      </c>
+      <c r="C102" s="3" t="inlineStr">
+        <is>
+          <t>Senior Shopify Developer</t>
+        </is>
+      </c>
+      <c r="D102" s="3" t="inlineStr">
+        <is>
+          <t>Sanctuary Computer Inc</t>
+        </is>
+      </c>
+      <c r="E102" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F102" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G102" s="5">
+        <f>HYPERLINK("https://remotive.com/remote-jobs/software-development/senior-shopify-developer-2091140", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H102" s="6" t="inlineStr">
+        <is>
+          <t>$80k - $150k</t>
+        </is>
+      </c>
+      <c r="I102" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Alta coincidencia técnica en Programación, Scripts, SQL y Automatización. Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J102" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K102" s="3" t="inlineStr"/>
+    </row>
+    <row r="103" ht="22" customHeight="1">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>6f9a298b38d7d57b</t>
+        </is>
+      </c>
+      <c r="B103" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24 15:23</t>
+        </is>
+      </c>
+      <c r="C103" s="3" t="inlineStr">
+        <is>
+          <t>Senior AI Engineer</t>
+        </is>
+      </c>
+      <c r="D103" s="3" t="inlineStr">
+        <is>
+          <t>Lemon.io</t>
+        </is>
+      </c>
+      <c r="E103" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F103" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G103" s="5">
+        <f>HYPERLINK("https://remotive.com/remote-jobs/artificial-intelligence/senior-ai-engineer-2091131", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H103" s="6" t="inlineStr"/>
+      <c r="I103" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Alta coincidencia técnica en Programación, Scripts, SQL y Automatización. Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J103" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K103" s="3" t="inlineStr"/>
+    </row>
+    <row r="104" ht="22" customHeight="1">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>4dd048896d0f6d65</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24 15:23</t>
+        </is>
+      </c>
+      <c r="C104" s="3" t="inlineStr">
+        <is>
+          <t>Senior .NET Full-stack Developer</t>
+        </is>
+      </c>
+      <c r="D104" s="3" t="inlineStr">
+        <is>
+          <t>Lemon.io</t>
+        </is>
+      </c>
+      <c r="E104" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F104" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G104" s="5">
+        <f>HYPERLINK("https://remotive.com/remote-jobs/software-development/senior-net-full-stack-developer-2091130", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H104" s="6" t="inlineStr"/>
+      <c r="I104" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Alta coincidencia técnica en Programación, Scripts, SQL y Automatización. Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J104" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K104" s="3" t="inlineStr"/>
+    </row>
+    <row r="105" ht="22" customHeight="1">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>a9d8e6e11954b4ed</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24 15:23</t>
+        </is>
+      </c>
+      <c r="C105" s="3" t="inlineStr">
+        <is>
+          <t>Senior Data Scientist</t>
+        </is>
+      </c>
+      <c r="D105" s="3" t="inlineStr">
+        <is>
+          <t>Lemon.io</t>
+        </is>
+      </c>
+      <c r="E105" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F105" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G105" s="5">
+        <f>HYPERLINK("https://remotive.com/remote-jobs/data/senior-data-scientist-2091129", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H105" s="6" t="inlineStr"/>
+      <c r="I105" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Alta coincidencia técnica en Programación, Scripts, SQL y Automatización. Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J105" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K105" s="3" t="inlineStr"/>
+    </row>
+    <row r="106" ht="22" customHeight="1">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>a18589077c92ad8c</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24 15:23</t>
+        </is>
+      </c>
+      <c r="C106" s="3" t="inlineStr">
+        <is>
+          <t>Senior React Full-stack Developer</t>
+        </is>
+      </c>
+      <c r="D106" s="3" t="inlineStr">
+        <is>
+          <t>Lemon.io</t>
+        </is>
+      </c>
+      <c r="E106" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F106" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G106" s="5">
+        <f>HYPERLINK("https://remotive.com/remote-jobs/software-development/senior-react-full-stack-developer-2091101", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H106" s="6" t="inlineStr"/>
+      <c r="I106" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Alta coincidencia técnica en Programación, Scripts, SQL y Automatización. Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J106" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K106" s="3" t="inlineStr"/>
+    </row>
+    <row r="107" ht="22" customHeight="1">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>6db39c2f55a85146</t>
+        </is>
+      </c>
+      <c r="B107" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24 15:23</t>
+        </is>
+      </c>
+      <c r="C107" s="3" t="inlineStr">
+        <is>
+          <t>Senior QA Engineer</t>
+        </is>
+      </c>
+      <c r="D107" s="3" t="inlineStr">
+        <is>
+          <t>Lemon.io</t>
+        </is>
+      </c>
+      <c r="E107" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F107" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G107" s="5">
+        <f>HYPERLINK("https://remotive.com/remote-jobs/qa/senior-qa-engineer-2091100", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H107" s="6" t="inlineStr"/>
+      <c r="I107" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Alta coincidencia técnica en Programación, Scripts, SQL y Automatización. Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J107" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K107" s="3" t="inlineStr"/>
+    </row>
+    <row r="108" ht="22" customHeight="1">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>5828ee7cdbb35c70</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24 15:23</t>
+        </is>
+      </c>
+      <c r="C108" s="3" t="inlineStr">
+        <is>
+          <t>Senior DevOps Engineer</t>
+        </is>
+      </c>
+      <c r="D108" s="3" t="inlineStr">
+        <is>
+          <t>Lemon.io</t>
+        </is>
+      </c>
+      <c r="E108" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F108" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G108" s="5">
+        <f>HYPERLINK("https://remotive.com/remote-jobs/devops/senior-devops-engineer-2091099", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H108" s="6" t="inlineStr"/>
+      <c r="I108" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Alta coincidencia técnica en Programación, Scripts, SQL y Automatización. Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J108" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K108" s="3" t="inlineStr"/>
+    </row>
+    <row r="109" ht="22" customHeight="1">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>552066cc9c949c2c</t>
+        </is>
+      </c>
+      <c r="B109" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24 15:23</t>
+        </is>
+      </c>
+      <c r="C109" s="3" t="inlineStr">
+        <is>
+          <t>Tier III Service Desk Engineer</t>
+        </is>
+      </c>
+      <c r="D109" s="3" t="inlineStr">
+        <is>
+          <t>Unio Digital</t>
+        </is>
+      </c>
+      <c r="E109" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F109" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G109" s="5">
+        <f>HYPERLINK("https://remotive.com/remote-jobs/information-technology/tier-iii-service-desk-engineer-2091045", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H109" s="6" t="inlineStr"/>
+      <c r="I109" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J109" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K109" s="3" t="inlineStr"/>
+    </row>
+    <row r="110" ht="22" customHeight="1">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>55fdaa0983ef9124</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24 15:37</t>
+        </is>
+      </c>
+      <c r="C110" s="3" t="inlineStr">
+        <is>
+          <t>Lider técnico con itil practice manager</t>
+        </is>
+      </c>
+      <c r="D110" s="3" t="inlineStr">
+        <is>
+          <t>Sinergy &amp; Lowells</t>
+        </is>
+      </c>
+      <c r="E110" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F110" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G110" s="5">
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/lider-tecnico-con-itil-practice-manager-1886753953", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H110" s="6" t="inlineStr"/>
+      <c r="I110" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J110" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K110" s="3" t="inlineStr"/>
+    </row>
+    <row r="111" ht="22" customHeight="1">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>9c65f710f43158b7</t>
+        </is>
+      </c>
+      <c r="B111" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24 15:37</t>
+        </is>
+      </c>
+      <c r="C111" s="3" t="inlineStr">
+        <is>
+          <t>Tecnico de instalaciones cableado de redes - licencia conte</t>
+        </is>
+      </c>
+      <c r="D111" s="3" t="inlineStr">
+        <is>
+          <t>Confidencial</t>
+        </is>
+      </c>
+      <c r="E111" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F111" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G111" s="5">
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-1886749397", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H111" s="6" t="inlineStr"/>
+      <c r="I111" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J111" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K111" s="3" t="inlineStr"/>
+    </row>
+    <row r="112" ht="22" customHeight="1">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>541d99c3c6e9a353</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24 15:23</t>
+        </is>
+      </c>
+      <c r="C112" s="3" t="inlineStr">
+        <is>
+          <t>Analista de infraestructura i (redes/firewall) - presencial en bogotá</t>
+        </is>
+      </c>
+      <c r="D112" s="3" t="inlineStr">
+        <is>
+          <t>Cinte Colombia SAS</t>
+        </is>
+      </c>
+      <c r="E112" s="7" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="F112" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G112" s="5">
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-infraestructura-i-redes-firewall-presencial-en-bogota-1886756899", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H112" s="6" t="inlineStr"/>
+      <c r="I112" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Soporte TI Remoto). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J112" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K112" s="3" t="inlineStr"/>
+    </row>
+    <row r="113" ht="22" customHeight="1">
+      <c r="A113" s="2" t="inlineStr">
+        <is>
           <t>386eb46216f50233</t>
         </is>
       </c>
-      <c r="B88" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-24 15:23</t>
-        </is>
-      </c>
-      <c r="C88" s="3" t="inlineStr">
+      <c r="B113" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24 15:23</t>
+        </is>
+      </c>
+      <c r="C113" s="3" t="inlineStr">
         <is>
           <t>Profesional junior soporte bases datos - presencial - bogota 114149</t>
         </is>
       </c>
-      <c r="D88" s="3" t="inlineStr">
+      <c r="D113" s="3" t="inlineStr">
         <is>
           <t>NUEVA EPS S.A</t>
         </is>
       </c>
-      <c r="E88" s="7" t="n">
+      <c r="E113" s="7" t="n">
         <v>0.5</v>
       </c>
-      <c r="F88" s="2" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
-      <c r="G88" s="5">
+      <c r="F113" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G113" s="5">
         <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/profesional-junior-soporte-bases-datos-presencial-bogota-114149-1886765098", "Ver Vacante")</f>
         <v/>
       </c>
-      <c r="H88" s="6" t="inlineStr"/>
-      <c r="I88" s="3" t="inlineStr">
+      <c r="H113" s="6" t="inlineStr"/>
+      <c r="I113" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Soporte TI Remoto). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
-      <c r="J88" s="2" t="inlineStr">
-        <is>
-          <t>Nueva</t>
-        </is>
-      </c>
-      <c r="K88" s="3" t="inlineStr"/>
+      <c r="J113" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K113" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
chore(tracker): actualizacion diaria de vacantes 2026-09-25
</commit_message>
<xml_diff>
--- a/output/profile_5_tecnico_sistemas_tracker.xlsx
+++ b/output/profile_5_tecnico_sistemas_tracker.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K52"/>
+  <dimension ref="A1:K63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2931,6 +2931,516 @@
       </c>
       <c r="K52" s="3" t="inlineStr"/>
     </row>
+    <row r="53" ht="22" customHeight="1">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>8d7f304ffb8625b5</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25 15:54</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>Auxiliar de sistemas</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>Confidencial</t>
+        </is>
+      </c>
+      <c r="E53" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G53" s="5">
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886751888", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H53" s="6" t="inlineStr"/>
+      <c r="I53" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J53" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K53" s="3" t="inlineStr"/>
+    </row>
+    <row r="54" ht="22" customHeight="1">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>3b5b26f92a305c0c</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25 15:54</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>Auxiliar de sistemas</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>Confidencial</t>
+        </is>
+      </c>
+      <c r="E54" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G54" s="5">
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886749497", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H54" s="6" t="inlineStr"/>
+      <c r="I54" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K54" s="3" t="inlineStr"/>
+    </row>
+    <row r="55" ht="22" customHeight="1">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>e760bcd88d90fbbe</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25 15:54</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>Agente de mesa de ayuda</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>SELCOMP INGENIERÍA SAS</t>
+        </is>
+      </c>
+      <c r="E55" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G55" s="5">
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-de-mesa-de-ayuda-1886758623", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H55" s="6" t="inlineStr"/>
+      <c r="I55" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J55" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K55" s="3" t="inlineStr"/>
+    </row>
+    <row r="56" ht="22" customHeight="1">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>86dcab5c5d802693</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25 15:54</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>Analista mesa de ayuda para tunja</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>Gestión de Seguridad Electrónica</t>
+        </is>
+      </c>
+      <c r="E56" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G56" s="5">
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-para-tunja-1886766955", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H56" s="6" t="inlineStr"/>
+      <c r="I56" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J56" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K56" s="3" t="inlineStr"/>
+    </row>
+    <row r="57" ht="22" customHeight="1">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>55fdaa0983ef9124</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25 15:54</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>Lider técnico con itil practice manager</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>Sinergy &amp; Lowells</t>
+        </is>
+      </c>
+      <c r="E57" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G57" s="5">
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/lider-tecnico-con-itil-practice-manager-1886753953", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H57" s="6" t="inlineStr"/>
+      <c r="I57" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J57" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K57" s="3" t="inlineStr"/>
+    </row>
+    <row r="58" ht="22" customHeight="1">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>a1ca7bc58cd48fad</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25 15:54</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>Tecnico de mesa de ayuda/mujeres contratacion inmediata</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>Confidencial</t>
+        </is>
+      </c>
+      <c r="E58" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G58" s="5">
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-mesa-de-ayuda-mujeres-contratacion-inmediata-1886770931", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H58" s="6" t="inlineStr"/>
+      <c r="I58" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J58" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K58" s="3" t="inlineStr"/>
+    </row>
+    <row r="59" ht="22" customHeight="1">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>e28aba5df8a2d3ae</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25 15:54</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>Tecnico de mesa de ayuda/mujeres contratacion inmediata</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>Confidencial</t>
+        </is>
+      </c>
+      <c r="E59" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G59" s="5">
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-mesa-de-ayuda-mujeres-contratacion-inmediata-1886769701", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H59" s="6" t="inlineStr"/>
+      <c r="I59" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J59" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K59" s="3" t="inlineStr"/>
+    </row>
+    <row r="60" ht="22" customHeight="1">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>9326784c1a2726fb</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25 15:54</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>Técnico de soporte y mesa de ayuda / medellín</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>Colsof S.A.S</t>
+        </is>
+      </c>
+      <c r="E60" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G60" s="5">
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-y-mesa-de-ayuda-medellin-1886738118", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H60" s="6" t="inlineStr"/>
+      <c r="I60" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J60" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K60" s="3" t="inlineStr"/>
+    </row>
+    <row r="61" ht="22" customHeight="1">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>b67dc9a9be4a1a6f</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25 15:54</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>Service desk agent</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>Confidencial</t>
+        </is>
+      </c>
+      <c r="E61" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G61" s="5">
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/service-desk-agent-soporte-tecnico-nivel-1-1886755112", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H61" s="6" t="inlineStr"/>
+      <c r="I61" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J61" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K61" s="3" t="inlineStr"/>
+    </row>
+    <row r="62" ht="22" customHeight="1">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>9c65f710f43158b7</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25 15:54</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>Tecnico de instalaciones cableado de redes - licencia conte</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>Confidencial</t>
+        </is>
+      </c>
+      <c r="E62" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G62" s="5">
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-1886749397", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H62" s="6" t="inlineStr"/>
+      <c r="I62" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J62" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K62" s="3" t="inlineStr"/>
+    </row>
+    <row r="63" ht="22" customHeight="1">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>0b0ae49f910109bb</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25 15:54</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>Ejecutivo Técnico Arancel Junior</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="inlineStr">
+        <is>
+          <t>Importante Empresa de Logística y Comercio</t>
+        </is>
+      </c>
+      <c r="E63" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G63" s="5">
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-547866639B487E0161373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H63" s="6" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="I63" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J63" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K63" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="J2:J500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">

</xml_diff>

<commit_message>
chore(tracker): actualizacion diaria de vacantes 2026-09-26
</commit_message>
<xml_diff>
--- a/output/profile_5_tecnico_sistemas_tracker.xlsx
+++ b/output/profile_5_tecnico_sistemas_tracker.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K63"/>
+  <dimension ref="A1:K65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2842,26 +2842,26 @@
     <row r="51" ht="22" customHeight="1">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>ae736277661dc78b</t>
+          <t>205fbfca7a1a7d27</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 15:23</t>
+          <t>2026-09-26 15:03</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>Analista de redes cisco</t>
+          <t>Urg instrumentador quirúrgico - soporte técnico - bogotá</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>ATCG DE COLOMBIA S.A.S</t>
-        </is>
-      </c>
-      <c r="E51" s="7" t="n">
-        <v>0.68</v>
+          <t>MEDIREX BIC SAS</t>
+        </is>
+      </c>
+      <c r="E51" s="4" t="n">
+        <v>0.73</v>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
@@ -2869,13 +2869,13 @@
         </is>
       </c>
       <c r="G51" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-cisco-1886760389", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/urg-instrumentador-quirurgico-soporte-tecnico-bogota-1886772422", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H51" s="6" t="inlineStr"/>
       <c r="I51" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 68/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 73/100 - Alta Afinidad] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J51" s="2" t="inlineStr">
@@ -2888,17 +2888,17 @@
     <row r="52" ht="22" customHeight="1">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>e29676fac3409ad6</t>
+          <t>eea27bb5aa0bd8c4</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 15:23</t>
+          <t>2026-09-26 15:03</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>Analista de redes y telecomunicaciones - nivel 1</t>
+          <t>Soporte técnico nivel 1 ccna vigente medellín</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
@@ -2906,8 +2906,8 @@
           <t>MANPOWER</t>
         </is>
       </c>
-      <c r="E52" s="7" t="n">
-        <v>0.68</v>
+      <c r="E52" s="4" t="n">
+        <v>0.73</v>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
@@ -2915,13 +2915,13 @@
         </is>
       </c>
       <c r="G52" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-y-telecomunicaciones-nivel-1-1886760565", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/soporte-tecnico-nivel-1-ccna-vigente-medellin-1886755519", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H52" s="6" t="inlineStr"/>
       <c r="I52" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 68/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 73/100 - Alta Afinidad] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J52" s="2" t="inlineStr">
@@ -2934,26 +2934,26 @@
     <row r="53" ht="22" customHeight="1">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>8d7f304ffb8625b5</t>
+          <t>ae736277661dc78b</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 15:54</t>
+          <t>2026-09-24 15:23</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar de sistemas</t>
+          <t>Analista de redes cisco</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>ATCG DE COLOMBIA S.A.S</t>
         </is>
       </c>
       <c r="E53" s="7" t="n">
-        <v>0.58</v>
+        <v>0.68</v>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
@@ -2961,13 +2961,13 @@
         </is>
       </c>
       <c r="G53" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886751888", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-cisco-1886760389", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H53" s="6" t="inlineStr"/>
       <c r="I53" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 68/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J53" s="2" t="inlineStr">
@@ -2980,26 +2980,26 @@
     <row r="54" ht="22" customHeight="1">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>3b5b26f92a305c0c</t>
+          <t>e29676fac3409ad6</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 15:54</t>
+          <t>2026-09-24 15:23</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar de sistemas</t>
+          <t>Analista de redes y telecomunicaciones - nivel 1</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>MANPOWER</t>
         </is>
       </c>
       <c r="E54" s="7" t="n">
-        <v>0.58</v>
+        <v>0.68</v>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
@@ -3007,13 +3007,13 @@
         </is>
       </c>
       <c r="G54" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886749497", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-y-telecomunicaciones-nivel-1-1886760565", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H54" s="6" t="inlineStr"/>
       <c r="I54" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 68/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J54" s="2" t="inlineStr">
@@ -3026,7 +3026,7 @@
     <row r="55" ht="22" customHeight="1">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>e760bcd88d90fbbe</t>
+          <t>8d7f304ffb8625b5</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
@@ -3036,12 +3036,12 @@
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>Agente de mesa de ayuda</t>
+          <t>Auxiliar de sistemas</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>SELCOMP INGENIERÍA SAS</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E55" s="7" t="n">
@@ -3053,7 +3053,7 @@
         </is>
       </c>
       <c r="G55" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-de-mesa-de-ayuda-1886758623", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886751888", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H55" s="6" t="inlineStr"/>
@@ -3072,7 +3072,7 @@
     <row r="56" ht="22" customHeight="1">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>86dcab5c5d802693</t>
+          <t>3b5b26f92a305c0c</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
@@ -3082,12 +3082,12 @@
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>Analista mesa de ayuda para tunja</t>
+          <t>Auxiliar de sistemas</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>Gestión de Seguridad Electrónica</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E56" s="7" t="n">
@@ -3099,7 +3099,7 @@
         </is>
       </c>
       <c r="G56" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-para-tunja-1886766955", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886749497", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H56" s="6" t="inlineStr"/>
@@ -3118,7 +3118,7 @@
     <row r="57" ht="22" customHeight="1">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>55fdaa0983ef9124</t>
+          <t>e760bcd88d90fbbe</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
@@ -3128,12 +3128,12 @@
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>Lider técnico con itil practice manager</t>
+          <t>Agente de mesa de ayuda</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>Sinergy &amp; Lowells</t>
+          <t>SELCOMP INGENIERÍA SAS</t>
         </is>
       </c>
       <c r="E57" s="7" t="n">
@@ -3145,7 +3145,7 @@
         </is>
       </c>
       <c r="G57" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/lider-tecnico-con-itil-practice-manager-1886753953", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-de-mesa-de-ayuda-1886758623", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H57" s="6" t="inlineStr"/>
@@ -3164,7 +3164,7 @@
     <row r="58" ht="22" customHeight="1">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>a1ca7bc58cd48fad</t>
+          <t>86dcab5c5d802693</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -3174,12 +3174,12 @@
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de mesa de ayuda/mujeres contratacion inmediata</t>
+          <t>Analista mesa de ayuda para tunja</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Gestión de Seguridad Electrónica</t>
         </is>
       </c>
       <c r="E58" s="7" t="n">
@@ -3191,7 +3191,7 @@
         </is>
       </c>
       <c r="G58" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-mesa-de-ayuda-mujeres-contratacion-inmediata-1886770931", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-para-tunja-1886766955", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H58" s="6" t="inlineStr"/>
@@ -3210,7 +3210,7 @@
     <row r="59" ht="22" customHeight="1">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>e28aba5df8a2d3ae</t>
+          <t>55fdaa0983ef9124</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
@@ -3220,12 +3220,12 @@
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de mesa de ayuda/mujeres contratacion inmediata</t>
+          <t>Lider técnico con itil practice manager</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Sinergy &amp; Lowells</t>
         </is>
       </c>
       <c r="E59" s="7" t="n">
@@ -3237,7 +3237,7 @@
         </is>
       </c>
       <c r="G59" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-mesa-de-ayuda-mujeres-contratacion-inmediata-1886769701", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/lider-tecnico-con-itil-practice-manager-1886753953", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H59" s="6" t="inlineStr"/>
@@ -3256,7 +3256,7 @@
     <row r="60" ht="22" customHeight="1">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>9326784c1a2726fb</t>
+          <t>a1ca7bc58cd48fad</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -3266,12 +3266,12 @@
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>Técnico de soporte y mesa de ayuda / medellín</t>
+          <t>Tecnico de mesa de ayuda/mujeres contratacion inmediata</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>Colsof S.A.S</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E60" s="7" t="n">
@@ -3283,7 +3283,7 @@
         </is>
       </c>
       <c r="G60" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-y-mesa-de-ayuda-medellin-1886738118", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-mesa-de-ayuda-mujeres-contratacion-inmediata-1886770931", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H60" s="6" t="inlineStr"/>
@@ -3302,7 +3302,7 @@
     <row r="61" ht="22" customHeight="1">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>b67dc9a9be4a1a6f</t>
+          <t>e28aba5df8a2d3ae</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
@@ -3312,7 +3312,7 @@
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>Service desk agent</t>
+          <t>Tecnico de mesa de ayuda/mujeres contratacion inmediata</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
@@ -3329,13 +3329,13 @@
         </is>
       </c>
       <c r="G61" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/service-desk-agent-soporte-tecnico-nivel-1-1886755112", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-mesa-de-ayuda-mujeres-contratacion-inmediata-1886769701", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H61" s="6" t="inlineStr"/>
       <c r="I61" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J61" s="2" t="inlineStr">
@@ -3348,7 +3348,7 @@
     <row r="62" ht="22" customHeight="1">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>9c65f710f43158b7</t>
+          <t>9326784c1a2726fb</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -3358,12 +3358,12 @@
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de instalaciones cableado de redes - licencia conte</t>
+          <t>Técnico de soporte y mesa de ayuda / medellín</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Colsof S.A.S</t>
         </is>
       </c>
       <c r="E62" s="7" t="n">
@@ -3375,7 +3375,7 @@
         </is>
       </c>
       <c r="G62" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-1886749397", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-y-mesa-de-ayuda-medellin-1886738118", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H62" s="6" t="inlineStr"/>
@@ -3394,52 +3394,144 @@
     <row r="63" ht="22" customHeight="1">
       <c r="A63" s="2" t="inlineStr">
         <is>
+          <t>b67dc9a9be4a1a6f</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25 15:54</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>Service desk agent</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="inlineStr">
+        <is>
+          <t>Confidencial</t>
+        </is>
+      </c>
+      <c r="E63" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G63" s="5">
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/service-desk-agent-soporte-tecnico-nivel-1-1886755112", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H63" s="6" t="inlineStr"/>
+      <c r="I63" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J63" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K63" s="3" t="inlineStr"/>
+    </row>
+    <row r="64" ht="22" customHeight="1">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>9c65f710f43158b7</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25 15:54</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>Tecnico de instalaciones cableado de redes - licencia conte</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="inlineStr">
+        <is>
+          <t>Confidencial</t>
+        </is>
+      </c>
+      <c r="E64" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G64" s="5">
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-1886749397", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H64" s="6" t="inlineStr"/>
+      <c r="I64" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J64" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K64" s="3" t="inlineStr"/>
+    </row>
+    <row r="65" ht="22" customHeight="1">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
           <t>0b0ae49f910109bb</t>
         </is>
       </c>
-      <c r="B63" s="2" t="inlineStr">
+      <c r="B65" s="2" t="inlineStr">
         <is>
           <t>2026-09-25 15:54</t>
         </is>
       </c>
-      <c r="C63" s="3" t="inlineStr">
+      <c r="C65" s="3" t="inlineStr">
         <is>
           <t>Ejecutivo Técnico Arancel Junior</t>
         </is>
       </c>
-      <c r="D63" s="3" t="inlineStr">
+      <c r="D65" s="3" t="inlineStr">
         <is>
           <t>Importante Empresa de Logística y Comercio</t>
         </is>
       </c>
-      <c r="E63" s="7" t="n">
+      <c r="E65" s="7" t="n">
         <v>0.5</v>
       </c>
-      <c r="F63" s="2" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
-      <c r="G63" s="5">
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G65" s="5">
         <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-547866639B487E0161373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
-      <c r="H63" s="6" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
-      <c r="I63" s="3" t="inlineStr">
+      <c r="H65" s="6" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="I65" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
-      <c r="J63" s="2" t="inlineStr">
-        <is>
-          <t>Nueva</t>
-        </is>
-      </c>
-      <c r="K63" s="3" t="inlineStr"/>
+      <c r="J65" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K65" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
chore(tracker): actualizacion diaria de vacantes 2026-09-27
</commit_message>
<xml_diff>
--- a/output/profile_5_tecnico_sistemas_tracker.xlsx
+++ b/output/profile_5_tecnico_sistemas_tracker.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K65"/>
+  <dimension ref="A1:K76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2934,26 +2934,26 @@
     <row r="53" ht="22" customHeight="1">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>ae736277661dc78b</t>
+          <t>da3496c7c6f99d83</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 15:23</t>
+          <t>2026-09-27 15:41</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>Analista de redes cisco</t>
+          <t>Aprendiz de Soporte Técnico TI – Medellín</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>ATCG DE COLOMBIA S.A.S</t>
-        </is>
-      </c>
-      <c r="E53" s="7" t="n">
-        <v>0.68</v>
+          <t>Agencia de Empleo de Comfenalco Antioquia</t>
+        </is>
+      </c>
+      <c r="E53" s="4" t="n">
+        <v>0.73</v>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
@@ -2961,13 +2961,17 @@
         </is>
       </c>
       <c r="G53" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-cisco-1886760389", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H53" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-aprendiz-de-soporte-tecnico-ti-medellin-en-medellin-1A050E5D73BED18C61373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H53" s="6" t="inlineStr">
+        <is>
+          <t>$ 2.000.000,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I53" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 68/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 73/100 - Alta Afinidad] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J53" s="2" t="inlineStr">
@@ -2980,26 +2984,26 @@
     <row r="54" ht="22" customHeight="1">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>e29676fac3409ad6</t>
+          <t>0088d835c7532e43</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 15:23</t>
+          <t>2026-09-27 15:41</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>Analista de redes y telecomunicaciones - nivel 1</t>
+          <t>Analista de Soporte Técnico y Mesa de Ayuda TI</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>MANPOWER</t>
-        </is>
-      </c>
-      <c r="E54" s="7" t="n">
-        <v>0.68</v>
+          <t>E-GLOBAL S.A.</t>
+        </is>
+      </c>
+      <c r="E54" s="4" t="n">
+        <v>0.73</v>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
@@ -3007,13 +3011,17 @@
         </is>
       </c>
       <c r="G54" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-y-telecomunicaciones-nivel-1-1886760565", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H54" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-analista-de-soporte-tecnico-y-mesa-de-ayuda-ti-en-medellin-3C800868C0F5959B61373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H54" s="6" t="inlineStr">
+        <is>
+          <t>$ 2.000.000,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I54" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 68/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 73/100 - Alta Afinidad] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J54" s="2" t="inlineStr">
@@ -3026,26 +3034,26 @@
     <row r="55" ht="22" customHeight="1">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>8d7f304ffb8625b5</t>
+          <t>0084204adfde29e6</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 15:54</t>
+          <t>2026-09-27 15:41</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar de sistemas</t>
+          <t>Analista de Soporte Técnico Español y Portugués</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
-        </is>
-      </c>
-      <c r="E55" s="7" t="n">
-        <v>0.58</v>
+          <t>Importante empresa del sector</t>
+        </is>
+      </c>
+      <c r="E55" s="4" t="n">
+        <v>0.73</v>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
@@ -3053,13 +3061,17 @@
         </is>
       </c>
       <c r="G55" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886751888", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H55" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-analista-de-soporte-tecnico-espanol-y-portugues-en-bogota-dc-0849D1C40E1F247D61373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H55" s="6" t="inlineStr">
+        <is>
+          <t>Presencial y remoto</t>
+        </is>
+      </c>
       <c r="I55" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 73/100 - Alta Afinidad] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J55" s="2" t="inlineStr">
@@ -3072,26 +3084,26 @@
     <row r="56" ht="22" customHeight="1">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>3b5b26f92a305c0c</t>
+          <t>6b4799591cfb3cf7</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 15:54</t>
+          <t>2026-09-27 15:41</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar de sistemas</t>
+          <t>Soporte Tecnico</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
-        </is>
-      </c>
-      <c r="E56" s="7" t="n">
-        <v>0.58</v>
+          <t>INNOVASER SOLUCIONES SAS</t>
+        </is>
+      </c>
+      <c r="E56" s="4" t="n">
+        <v>0.73</v>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
@@ -3099,13 +3111,17 @@
         </is>
       </c>
       <c r="G56" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886749497", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H56" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-soporte-tecnico-en-tocancipa-239FC7D9D20BBA5E61373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H56" s="6" t="inlineStr">
+        <is>
+          <t>$ 1.750.905,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I56" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 73/100 - Alta Afinidad] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J56" s="2" t="inlineStr">
@@ -3118,26 +3134,26 @@
     <row r="57" ht="22" customHeight="1">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>e760bcd88d90fbbe</t>
+          <t>ae736277661dc78b</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 15:54</t>
+          <t>2026-09-24 15:23</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>Agente de mesa de ayuda</t>
+          <t>Analista de redes cisco</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>SELCOMP INGENIERÍA SAS</t>
+          <t>ATCG DE COLOMBIA S.A.S</t>
         </is>
       </c>
       <c r="E57" s="7" t="n">
-        <v>0.58</v>
+        <v>0.68</v>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
@@ -3145,13 +3161,13 @@
         </is>
       </c>
       <c r="G57" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-de-mesa-de-ayuda-1886758623", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-cisco-1886760389", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H57" s="6" t="inlineStr"/>
       <c r="I57" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 68/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J57" s="2" t="inlineStr">
@@ -3164,26 +3180,26 @@
     <row r="58" ht="22" customHeight="1">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>86dcab5c5d802693</t>
+          <t>e29676fac3409ad6</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 15:54</t>
+          <t>2026-09-24 15:23</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>Analista mesa de ayuda para tunja</t>
+          <t>Analista de redes y telecomunicaciones - nivel 1</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>Gestión de Seguridad Electrónica</t>
+          <t>MANPOWER</t>
         </is>
       </c>
       <c r="E58" s="7" t="n">
-        <v>0.58</v>
+        <v>0.68</v>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
@@ -3191,13 +3207,13 @@
         </is>
       </c>
       <c r="G58" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-para-tunja-1886766955", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-y-telecomunicaciones-nivel-1-1886760565", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H58" s="6" t="inlineStr"/>
       <c r="I58" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 68/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J58" s="2" t="inlineStr">
@@ -3210,7 +3226,7 @@
     <row r="59" ht="22" customHeight="1">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>55fdaa0983ef9124</t>
+          <t>8d7f304ffb8625b5</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
@@ -3220,12 +3236,12 @@
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>Lider técnico con itil practice manager</t>
+          <t>Auxiliar de sistemas</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>Sinergy &amp; Lowells</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E59" s="7" t="n">
@@ -3237,7 +3253,7 @@
         </is>
       </c>
       <c r="G59" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/lider-tecnico-con-itil-practice-manager-1886753953", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886751888", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H59" s="6" t="inlineStr"/>
@@ -3256,7 +3272,7 @@
     <row r="60" ht="22" customHeight="1">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>a1ca7bc58cd48fad</t>
+          <t>3b5b26f92a305c0c</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -3266,7 +3282,7 @@
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de mesa de ayuda/mujeres contratacion inmediata</t>
+          <t>Auxiliar de sistemas</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
@@ -3283,7 +3299,7 @@
         </is>
       </c>
       <c r="G60" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-mesa-de-ayuda-mujeres-contratacion-inmediata-1886770931", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886749497", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H60" s="6" t="inlineStr"/>
@@ -3302,7 +3318,7 @@
     <row r="61" ht="22" customHeight="1">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>e28aba5df8a2d3ae</t>
+          <t>e760bcd88d90fbbe</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
@@ -3312,12 +3328,12 @@
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de mesa de ayuda/mujeres contratacion inmediata</t>
+          <t>Agente de mesa de ayuda</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>SELCOMP INGENIERÍA SAS</t>
         </is>
       </c>
       <c r="E61" s="7" t="n">
@@ -3329,7 +3345,7 @@
         </is>
       </c>
       <c r="G61" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-mesa-de-ayuda-mujeres-contratacion-inmediata-1886769701", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-de-mesa-de-ayuda-1886758623", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H61" s="6" t="inlineStr"/>
@@ -3348,7 +3364,7 @@
     <row r="62" ht="22" customHeight="1">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>9326784c1a2726fb</t>
+          <t>86dcab5c5d802693</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -3358,12 +3374,12 @@
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>Técnico de soporte y mesa de ayuda / medellín</t>
+          <t>Analista mesa de ayuda para tunja</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>Colsof S.A.S</t>
+          <t>Gestión de Seguridad Electrónica</t>
         </is>
       </c>
       <c r="E62" s="7" t="n">
@@ -3375,7 +3391,7 @@
         </is>
       </c>
       <c r="G62" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-y-mesa-de-ayuda-medellin-1886738118", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-para-tunja-1886766955", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H62" s="6" t="inlineStr"/>
@@ -3394,7 +3410,7 @@
     <row r="63" ht="22" customHeight="1">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>b67dc9a9be4a1a6f</t>
+          <t>55fdaa0983ef9124</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
@@ -3404,12 +3420,12 @@
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>Service desk agent</t>
+          <t>Lider técnico con itil practice manager</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Sinergy &amp; Lowells</t>
         </is>
       </c>
       <c r="E63" s="7" t="n">
@@ -3421,13 +3437,13 @@
         </is>
       </c>
       <c r="G63" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/service-desk-agent-soporte-tecnico-nivel-1-1886755112", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/lider-tecnico-con-itil-practice-manager-1886753953", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H63" s="6" t="inlineStr"/>
       <c r="I63" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J63" s="2" t="inlineStr">
@@ -3440,7 +3456,7 @@
     <row r="64" ht="22" customHeight="1">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>9c65f710f43158b7</t>
+          <t>a1ca7bc58cd48fad</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -3450,7 +3466,7 @@
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de instalaciones cableado de redes - licencia conte</t>
+          <t>Tecnico de mesa de ayuda/mujeres contratacion inmediata</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
@@ -3467,7 +3483,7 @@
         </is>
       </c>
       <c r="G64" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-1886749397", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-mesa-de-ayuda-mujeres-contratacion-inmediata-1886770931", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H64" s="6" t="inlineStr"/>
@@ -3486,52 +3502,578 @@
     <row r="65" ht="22" customHeight="1">
       <c r="A65" s="2" t="inlineStr">
         <is>
+          <t>e28aba5df8a2d3ae</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25 15:54</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>Tecnico de mesa de ayuda/mujeres contratacion inmediata</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>Confidencial</t>
+        </is>
+      </c>
+      <c r="E65" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G65" s="5">
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-mesa-de-ayuda-mujeres-contratacion-inmediata-1886769701", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H65" s="6" t="inlineStr"/>
+      <c r="I65" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J65" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K65" s="3" t="inlineStr"/>
+    </row>
+    <row r="66" ht="22" customHeight="1">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>9326784c1a2726fb</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25 15:54</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>Técnico de soporte y mesa de ayuda / medellín</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="inlineStr">
+        <is>
+          <t>Colsof S.A.S</t>
+        </is>
+      </c>
+      <c r="E66" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G66" s="5">
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-y-mesa-de-ayuda-medellin-1886738118", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H66" s="6" t="inlineStr"/>
+      <c r="I66" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J66" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K66" s="3" t="inlineStr"/>
+    </row>
+    <row r="67" ht="22" customHeight="1">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>b67dc9a9be4a1a6f</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25 15:54</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>Service desk agent</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>Confidencial</t>
+        </is>
+      </c>
+      <c r="E67" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G67" s="5">
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/service-desk-agent-soporte-tecnico-nivel-1-1886755112", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H67" s="6" t="inlineStr"/>
+      <c r="I67" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J67" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K67" s="3" t="inlineStr"/>
+    </row>
+    <row r="68" ht="22" customHeight="1">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>9c65f710f43158b7</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25 15:54</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>Tecnico de instalaciones cableado de redes - licencia conte</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>Confidencial</t>
+        </is>
+      </c>
+      <c r="E68" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G68" s="5">
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-1886749397", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H68" s="6" t="inlineStr"/>
+      <c r="I68" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J68" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K68" s="3" t="inlineStr"/>
+    </row>
+    <row r="69" ht="22" customHeight="1">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>a95003a0b1fc3d77</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27 15:41</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>Técnico Soporte Nivel 1 Con ITIL</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="inlineStr">
+        <is>
+          <t>Importante empresa del sector de tecnología</t>
+        </is>
+      </c>
+      <c r="E69" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G69" s="5">
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-soporte-nivel-1-con-itil-en-bogota-dc-59E13FA64EF5843C61373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H69" s="6" t="inlineStr">
+        <is>
+          <t>$ 1.750.905,00 (Mensual)</t>
+        </is>
+      </c>
+      <c r="I69" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J69" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K69" s="3" t="inlineStr"/>
+    </row>
+    <row r="70" ht="22" customHeight="1">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>96391fd564d83616</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27 15:41</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>Tecnico de soporte IT con Moto</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="inlineStr">
+        <is>
+          <t>Los Hornitos</t>
+        </is>
+      </c>
+      <c r="E70" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G70" s="5">
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-it-con-moto-empresa-de-alimentos-en-bogota-dc-599938D46A6F4A8F61373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H70" s="6" t="inlineStr">
+        <is>
+          <t>$ 2.125.947,00 (Mensual)</t>
+        </is>
+      </c>
+      <c r="I70" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J70" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K70" s="3" t="inlineStr"/>
+    </row>
+    <row r="71" ht="22" customHeight="1">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>b4f0b8c16fe5543e</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27 15:41</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>Auxiliar de Sistemas</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="inlineStr">
+        <is>
+          <t>ELIS COLOMBIA SAS</t>
+        </is>
+      </c>
+      <c r="E71" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G71" s="5">
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-en-bogota-dc-48C2A0A3B050945661373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H71" s="6" t="inlineStr">
+        <is>
+          <t>$ 2.000.000,00 (Mensual)</t>
+        </is>
+      </c>
+      <c r="I71" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J71" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K71" s="3" t="inlineStr"/>
+    </row>
+    <row r="72" ht="22" customHeight="1">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>7e4b4e4f136a5e31</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27 15:41</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>Agente Mesa de Ayuda</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="inlineStr">
+        <is>
+          <t>Importante empresa del sector</t>
+        </is>
+      </c>
+      <c r="E72" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G72" s="5">
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-agente-mesa-de-ayuda-en-bogota-dc-E39FE355E02E578761373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H72" s="6" t="inlineStr">
+        <is>
+          <t>$ 2.000.000,00 (Mensual)</t>
+        </is>
+      </c>
+      <c r="I72" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J72" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K72" s="3" t="inlineStr"/>
+    </row>
+    <row r="73" ht="22" customHeight="1">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>0ef2cd7667600919</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27 15:41</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>Técnico de Soporte TI Regional</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="inlineStr">
+        <is>
+          <t>POLICOMP COLOMBIA SAS</t>
+        </is>
+      </c>
+      <c r="E73" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G73" s="5">
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-ti-regional-en-bogota-dc-ACF045C94E41CCDE61373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H73" s="6" t="inlineStr"/>
+      <c r="I73" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J73" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K73" s="3" t="inlineStr"/>
+    </row>
+    <row r="74" ht="22" customHeight="1">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>7784997bda962255</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27 15:41</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>Técnico de Soporte TI On Demand/ por horas</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="inlineStr">
+        <is>
+          <t>POLICOMP COLOMBIA SAS</t>
+        </is>
+      </c>
+      <c r="E74" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G74" s="5">
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-ti-on-demand-por-horas-en-bogota-dc-C2338FA0172D59A561373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H74" s="6" t="inlineStr"/>
+      <c r="I74" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J74" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K74" s="3" t="inlineStr"/>
+    </row>
+    <row r="75" ht="22" customHeight="1">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>29d0fe2e42e678f7</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27 15:41</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>Técnico mantenimiento correctivo impresoras</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="inlineStr">
+        <is>
+          <t>Multinacional de Impresión</t>
+        </is>
+      </c>
+      <c r="E75" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G75" s="5">
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-mantenimiento-correctivo-impresoras-en-guarne-BC0E775C0F25B27D61373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H75" s="6" t="inlineStr">
+        <is>
+          <t>$ 1.800.000,00 (Mensual)</t>
+        </is>
+      </c>
+      <c r="I75" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J75" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K75" s="3" t="inlineStr"/>
+    </row>
+    <row r="76" ht="22" customHeight="1">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
           <t>0b0ae49f910109bb</t>
         </is>
       </c>
-      <c r="B65" s="2" t="inlineStr">
+      <c r="B76" s="2" t="inlineStr">
         <is>
           <t>2026-09-25 15:54</t>
         </is>
       </c>
-      <c r="C65" s="3" t="inlineStr">
+      <c r="C76" s="3" t="inlineStr">
         <is>
           <t>Ejecutivo Técnico Arancel Junior</t>
         </is>
       </c>
-      <c r="D65" s="3" t="inlineStr">
+      <c r="D76" s="3" t="inlineStr">
         <is>
           <t>Importante Empresa de Logística y Comercio</t>
         </is>
       </c>
-      <c r="E65" s="7" t="n">
+      <c r="E76" s="7" t="n">
         <v>0.5</v>
       </c>
-      <c r="F65" s="2" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
-      <c r="G65" s="5">
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G76" s="5">
         <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-547866639B487E0161373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
-      <c r="H65" s="6" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
-      <c r="I65" s="3" t="inlineStr">
+      <c r="H76" s="6" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="I76" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
-      <c r="J65" s="2" t="inlineStr">
-        <is>
-          <t>Nueva</t>
-        </is>
-      </c>
-      <c r="K65" s="3" t="inlineStr"/>
+      <c r="J76" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K76" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
chore(tracker): actualizacion diaria de vacantes 2026-09-28
</commit_message>
<xml_diff>
--- a/output/profile_5_tecnico_sistemas_tracker.xlsx
+++ b/output/profile_5_tecnico_sistemas_tracker.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K76"/>
+  <dimension ref="A1:K79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -4028,52 +4028,198 @@
     <row r="76" ht="22" customHeight="1">
       <c r="A76" s="2" t="inlineStr">
         <is>
+          <t>98c9ab11f5b1eace</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28 18:36</t>
+        </is>
+      </c>
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t>Auxiliar de sistemas</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="inlineStr">
+        <is>
+          <t>Importante empresa del sector</t>
+        </is>
+      </c>
+      <c r="E76" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G76" s="5">
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-persona-con-discapacidad-remota-en-bogota-dc-5F2A812D014E159B61373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H76" s="6" t="inlineStr">
+        <is>
+          <t>$ 1.750.905,00 (Mensual)</t>
+        </is>
+      </c>
+      <c r="I76" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J76" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K76" s="3" t="inlineStr"/>
+    </row>
+    <row r="77" ht="22" customHeight="1">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>58133ddc4da9c68e</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28 18:36</t>
+        </is>
+      </c>
+      <c r="C77" s="3" t="inlineStr">
+        <is>
+          <t>Auxiliar de sistemas</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="inlineStr">
+        <is>
+          <t>Importante empresa del sector</t>
+        </is>
+      </c>
+      <c r="E77" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G77" s="5">
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-persona-con-discapacidad-remota-en-bogota-dc-A00C07C9CC9A494B61373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H77" s="6" t="inlineStr">
+        <is>
+          <t>$ 1.750.905,00 (Mensual)</t>
+        </is>
+      </c>
+      <c r="I77" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J77" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K77" s="3" t="inlineStr"/>
+    </row>
+    <row r="78" ht="22" customHeight="1">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>aed3420a4cfdc248</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28 18:36</t>
+        </is>
+      </c>
+      <c r="C78" s="3" t="inlineStr">
+        <is>
+          <t>Consultor de servicios/ mesa de ayuda nómina y erp software</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="inlineStr">
+        <is>
+          <t>Confidencial</t>
+        </is>
+      </c>
+      <c r="E78" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G78" s="5">
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/consultor-de-servicios-mesa-de-ayuda-nomina-y-erp-software-inclusivo-1886716126", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H78" s="6" t="inlineStr"/>
+      <c r="I78" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J78" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K78" s="3" t="inlineStr"/>
+    </row>
+    <row r="79" ht="22" customHeight="1">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
           <t>0b0ae49f910109bb</t>
         </is>
       </c>
-      <c r="B76" s="2" t="inlineStr">
+      <c r="B79" s="2" t="inlineStr">
         <is>
           <t>2026-09-25 15:54</t>
         </is>
       </c>
-      <c r="C76" s="3" t="inlineStr">
+      <c r="C79" s="3" t="inlineStr">
         <is>
           <t>Ejecutivo Técnico Arancel Junior</t>
         </is>
       </c>
-      <c r="D76" s="3" t="inlineStr">
+      <c r="D79" s="3" t="inlineStr">
         <is>
           <t>Importante Empresa de Logística y Comercio</t>
         </is>
       </c>
-      <c r="E76" s="7" t="n">
+      <c r="E79" s="7" t="n">
         <v>0.5</v>
       </c>
-      <c r="F76" s="2" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
-      <c r="G76" s="5">
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G79" s="5">
         <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-547866639B487E0161373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
-      <c r="H76" s="6" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
-      <c r="I76" s="3" t="inlineStr">
+      <c r="H79" s="6" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="I79" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
-      <c r="J76" s="2" t="inlineStr">
-        <is>
-          <t>Nueva</t>
-        </is>
-      </c>
-      <c r="K76" s="3" t="inlineStr"/>
+      <c r="J79" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K79" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
chore(tracker): actualizacion diaria de vacantes 2026-09-29
</commit_message>
<xml_diff>
--- a/output/profile_5_tecnico_sistemas_tracker.xlsx
+++ b/output/profile_5_tecnico_sistemas_tracker.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K79"/>
+  <dimension ref="A1:K82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -4174,52 +4174,190 @@
     <row r="79" ht="22" customHeight="1">
       <c r="A79" s="2" t="inlineStr">
         <is>
+          <t>2b8357189ff315da</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 17:00</t>
+        </is>
+      </c>
+      <c r="C79" s="3" t="inlineStr">
+        <is>
+          <t>Auxiliar de sistemas</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="inlineStr">
+        <is>
+          <t>DAVITA SAS</t>
+        </is>
+      </c>
+      <c r="E79" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G79" s="5">
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886758163", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H79" s="6" t="inlineStr"/>
+      <c r="I79" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J79" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K79" s="3" t="inlineStr"/>
+    </row>
+    <row r="80" ht="22" customHeight="1">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>a87934e7643b2c1c</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 17:00</t>
+        </is>
+      </c>
+      <c r="C80" s="3" t="inlineStr">
+        <is>
+          <t>Tecnico de instalaciones cableado de redes - licencia conte cali</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="inlineStr">
+        <is>
+          <t>Confidencial</t>
+        </is>
+      </c>
+      <c r="E80" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G80" s="5">
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-cali-1886759847", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H80" s="6" t="inlineStr"/>
+      <c r="I80" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J80" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K80" s="3" t="inlineStr"/>
+    </row>
+    <row r="81" ht="22" customHeight="1">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>10b4265e3ad11d81</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 17:00</t>
+        </is>
+      </c>
+      <c r="C81" s="3" t="inlineStr">
+        <is>
+          <t>Information Technology Help Desk Support</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="inlineStr">
+        <is>
+          <t>Booth</t>
+        </is>
+      </c>
+      <c r="E81" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G81" s="5">
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/information-technology-help-desk-support-at-booth-4471203962", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H81" s="6" t="inlineStr"/>
+      <c r="I81" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J81" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K81" s="3" t="inlineStr"/>
+    </row>
+    <row r="82" ht="22" customHeight="1">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
           <t>0b0ae49f910109bb</t>
         </is>
       </c>
-      <c r="B79" s="2" t="inlineStr">
+      <c r="B82" s="2" t="inlineStr">
         <is>
           <t>2026-09-25 15:54</t>
         </is>
       </c>
-      <c r="C79" s="3" t="inlineStr">
+      <c r="C82" s="3" t="inlineStr">
         <is>
           <t>Ejecutivo Técnico Arancel Junior</t>
         </is>
       </c>
-      <c r="D79" s="3" t="inlineStr">
+      <c r="D82" s="3" t="inlineStr">
         <is>
           <t>Importante Empresa de Logística y Comercio</t>
         </is>
       </c>
-      <c r="E79" s="7" t="n">
+      <c r="E82" s="7" t="n">
         <v>0.5</v>
       </c>
-      <c r="F79" s="2" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
-      <c r="G79" s="5">
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G82" s="5">
         <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-547866639B487E0161373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
-      <c r="H79" s="6" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
-      <c r="I79" s="3" t="inlineStr">
+      <c r="H82" s="6" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="I82" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
-      <c r="J79" s="2" t="inlineStr">
-        <is>
-          <t>Nueva</t>
-        </is>
-      </c>
-      <c r="K79" s="3" t="inlineStr"/>
+      <c r="J82" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K82" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
chore(tracker): actualizacion diaria de vacantes 2026-09-30
</commit_message>
<xml_diff>
--- a/output/profile_5_tecnico_sistemas_tracker.xlsx
+++ b/output/profile_5_tecnico_sistemas_tracker.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K82"/>
+  <dimension ref="A1:K86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3134,26 +3134,26 @@
     <row r="57" ht="22" customHeight="1">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>ae736277661dc78b</t>
+          <t>150b576d34126c5c</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 15:23</t>
+          <t>2026-09-30 16:49</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>Analista de redes cisco</t>
+          <t>Analista de Soporte Técnico e Implementación</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>ATCG DE COLOMBIA S.A.S</t>
-        </is>
-      </c>
-      <c r="E57" s="7" t="n">
-        <v>0.68</v>
+          <t>Manpower Group Colombia</t>
+        </is>
+      </c>
+      <c r="E57" s="4" t="n">
+        <v>0.73</v>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
@@ -3161,13 +3161,17 @@
         </is>
       </c>
       <c r="G57" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-cisco-1886760389", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H57" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-analista-de-soporte-tecnico-e-implementacion-experiencia-deseable-en-plataformas-educativas-en-bogota-dc-429E2775FD281A5261373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H57" s="6" t="inlineStr">
+        <is>
+          <t>$ 2.250.000,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I57" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 68/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 73/100 - Alta Afinidad] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J57" s="2" t="inlineStr">
@@ -3180,7 +3184,7 @@
     <row r="58" ht="22" customHeight="1">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>e29676fac3409ad6</t>
+          <t>ae736277661dc78b</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -3190,12 +3194,12 @@
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>Analista de redes y telecomunicaciones - nivel 1</t>
+          <t>Analista de redes cisco</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>MANPOWER</t>
+          <t>ATCG DE COLOMBIA S.A.S</t>
         </is>
       </c>
       <c r="E58" s="7" t="n">
@@ -3207,7 +3211,7 @@
         </is>
       </c>
       <c r="G58" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-y-telecomunicaciones-nivel-1-1886760565", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-cisco-1886760389", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H58" s="6" t="inlineStr"/>
@@ -3226,26 +3230,26 @@
     <row r="59" ht="22" customHeight="1">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>8d7f304ffb8625b5</t>
+          <t>e29676fac3409ad6</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 15:54</t>
+          <t>2026-09-24 15:23</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar de sistemas</t>
+          <t>Analista de redes y telecomunicaciones - nivel 1</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>MANPOWER</t>
         </is>
       </c>
       <c r="E59" s="7" t="n">
-        <v>0.58</v>
+        <v>0.68</v>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
@@ -3253,13 +3257,13 @@
         </is>
       </c>
       <c r="G59" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886751888", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-y-telecomunicaciones-nivel-1-1886760565", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H59" s="6" t="inlineStr"/>
       <c r="I59" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 68/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J59" s="2" t="inlineStr">
@@ -3272,7 +3276,7 @@
     <row r="60" ht="22" customHeight="1">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>3b5b26f92a305c0c</t>
+          <t>8d7f304ffb8625b5</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -3299,7 +3303,7 @@
         </is>
       </c>
       <c r="G60" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886749497", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886751888", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H60" s="6" t="inlineStr"/>
@@ -3318,7 +3322,7 @@
     <row r="61" ht="22" customHeight="1">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>e760bcd88d90fbbe</t>
+          <t>3b5b26f92a305c0c</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
@@ -3328,12 +3332,12 @@
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>Agente de mesa de ayuda</t>
+          <t>Auxiliar de sistemas</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>SELCOMP INGENIERÍA SAS</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E61" s="7" t="n">
@@ -3345,7 +3349,7 @@
         </is>
       </c>
       <c r="G61" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-de-mesa-de-ayuda-1886758623", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886749497", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H61" s="6" t="inlineStr"/>
@@ -3364,7 +3368,7 @@
     <row r="62" ht="22" customHeight="1">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>86dcab5c5d802693</t>
+          <t>e760bcd88d90fbbe</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -3374,12 +3378,12 @@
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>Analista mesa de ayuda para tunja</t>
+          <t>Agente de mesa de ayuda</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>Gestión de Seguridad Electrónica</t>
+          <t>SELCOMP INGENIERÍA SAS</t>
         </is>
       </c>
       <c r="E62" s="7" t="n">
@@ -3391,7 +3395,7 @@
         </is>
       </c>
       <c r="G62" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-para-tunja-1886766955", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-de-mesa-de-ayuda-1886758623", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H62" s="6" t="inlineStr"/>
@@ -3410,7 +3414,7 @@
     <row r="63" ht="22" customHeight="1">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>55fdaa0983ef9124</t>
+          <t>86dcab5c5d802693</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
@@ -3420,12 +3424,12 @@
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>Lider técnico con itil practice manager</t>
+          <t>Analista mesa de ayuda para tunja</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>Sinergy &amp; Lowells</t>
+          <t>Gestión de Seguridad Electrónica</t>
         </is>
       </c>
       <c r="E63" s="7" t="n">
@@ -3437,7 +3441,7 @@
         </is>
       </c>
       <c r="G63" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/lider-tecnico-con-itil-practice-manager-1886753953", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-para-tunja-1886766955", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H63" s="6" t="inlineStr"/>
@@ -3456,7 +3460,7 @@
     <row r="64" ht="22" customHeight="1">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>a1ca7bc58cd48fad</t>
+          <t>55fdaa0983ef9124</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -3466,12 +3470,12 @@
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de mesa de ayuda/mujeres contratacion inmediata</t>
+          <t>Lider técnico con itil practice manager</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Sinergy &amp; Lowells</t>
         </is>
       </c>
       <c r="E64" s="7" t="n">
@@ -3483,7 +3487,7 @@
         </is>
       </c>
       <c r="G64" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-mesa-de-ayuda-mujeres-contratacion-inmediata-1886770931", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/lider-tecnico-con-itil-practice-manager-1886753953", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H64" s="6" t="inlineStr"/>
@@ -3502,7 +3506,7 @@
     <row r="65" ht="22" customHeight="1">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>e28aba5df8a2d3ae</t>
+          <t>a1ca7bc58cd48fad</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
@@ -3529,7 +3533,7 @@
         </is>
       </c>
       <c r="G65" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-mesa-de-ayuda-mujeres-contratacion-inmediata-1886769701", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-mesa-de-ayuda-mujeres-contratacion-inmediata-1886770931", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H65" s="6" t="inlineStr"/>
@@ -3548,7 +3552,7 @@
     <row r="66" ht="22" customHeight="1">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>9326784c1a2726fb</t>
+          <t>e28aba5df8a2d3ae</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -3558,12 +3562,12 @@
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>Técnico de soporte y mesa de ayuda / medellín</t>
+          <t>Tecnico de mesa de ayuda/mujeres contratacion inmediata</t>
         </is>
       </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
-          <t>Colsof S.A.S</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E66" s="7" t="n">
@@ -3575,7 +3579,7 @@
         </is>
       </c>
       <c r="G66" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-y-mesa-de-ayuda-medellin-1886738118", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-mesa-de-ayuda-mujeres-contratacion-inmediata-1886769701", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H66" s="6" t="inlineStr"/>
@@ -3594,7 +3598,7 @@
     <row r="67" ht="22" customHeight="1">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>b67dc9a9be4a1a6f</t>
+          <t>9326784c1a2726fb</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
@@ -3604,12 +3608,12 @@
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>Service desk agent</t>
+          <t>Técnico de soporte y mesa de ayuda / medellín</t>
         </is>
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Colsof S.A.S</t>
         </is>
       </c>
       <c r="E67" s="7" t="n">
@@ -3621,13 +3625,13 @@
         </is>
       </c>
       <c r="G67" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/service-desk-agent-soporte-tecnico-nivel-1-1886755112", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-y-mesa-de-ayuda-medellin-1886738118", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H67" s="6" t="inlineStr"/>
       <c r="I67" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J67" s="2" t="inlineStr">
@@ -3640,7 +3644,7 @@
     <row r="68" ht="22" customHeight="1">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>9c65f710f43158b7</t>
+          <t>b67dc9a9be4a1a6f</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -3650,7 +3654,7 @@
       </c>
       <c r="C68" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de instalaciones cableado de redes - licencia conte</t>
+          <t>Service desk agent</t>
         </is>
       </c>
       <c r="D68" s="3" t="inlineStr">
@@ -3667,13 +3671,13 @@
         </is>
       </c>
       <c r="G68" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-1886749397", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/service-desk-agent-soporte-tecnico-nivel-1-1886755112", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H68" s="6" t="inlineStr"/>
       <c r="I68" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J68" s="2" t="inlineStr">
@@ -3686,22 +3690,22 @@
     <row r="69" ht="22" customHeight="1">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>a95003a0b1fc3d77</t>
+          <t>9c65f710f43158b7</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 15:41</t>
+          <t>2026-09-25 15:54</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>Técnico Soporte Nivel 1 Con ITIL</t>
+          <t>Tecnico de instalaciones cableado de redes - licencia conte</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>Importante empresa del sector de tecnología</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E69" s="7" t="n">
@@ -3713,14 +3717,10 @@
         </is>
       </c>
       <c r="G69" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-soporte-nivel-1-con-itil-en-bogota-dc-59E13FA64EF5843C61373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H69" s="6" t="inlineStr">
-        <is>
-          <t>$ 1.750.905,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-1886749397", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H69" s="6" t="inlineStr"/>
       <c r="I69" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -3736,7 +3736,7 @@
     <row r="70" ht="22" customHeight="1">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>96391fd564d83616</t>
+          <t>a95003a0b1fc3d77</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -3746,12 +3746,12 @@
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de soporte IT con Moto</t>
+          <t>Técnico Soporte Nivel 1 Con ITIL</t>
         </is>
       </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
-          <t>Los Hornitos</t>
+          <t>Importante empresa del sector de tecnología</t>
         </is>
       </c>
       <c r="E70" s="7" t="n">
@@ -3763,12 +3763,12 @@
         </is>
       </c>
       <c r="G70" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-it-con-moto-empresa-de-alimentos-en-bogota-dc-599938D46A6F4A8F61373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-soporte-nivel-1-con-itil-en-bogota-dc-59E13FA64EF5843C61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H70" s="6" t="inlineStr">
         <is>
-          <t>$ 2.125.947,00 (Mensual)</t>
+          <t>$ 1.750.905,00 (Mensual)</t>
         </is>
       </c>
       <c r="I70" s="3" t="inlineStr">
@@ -3786,7 +3786,7 @@
     <row r="71" ht="22" customHeight="1">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>b4f0b8c16fe5543e</t>
+          <t>96391fd564d83616</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
@@ -3796,12 +3796,12 @@
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar de Sistemas</t>
+          <t>Tecnico de soporte IT con Moto</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>ELIS COLOMBIA SAS</t>
+          <t>Los Hornitos</t>
         </is>
       </c>
       <c r="E71" s="7" t="n">
@@ -3813,12 +3813,12 @@
         </is>
       </c>
       <c r="G71" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-en-bogota-dc-48C2A0A3B050945661373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-it-con-moto-empresa-de-alimentos-en-bogota-dc-599938D46A6F4A8F61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H71" s="6" t="inlineStr">
         <is>
-          <t>$ 2.000.000,00 (Mensual)</t>
+          <t>$ 2.125.947,00 (Mensual)</t>
         </is>
       </c>
       <c r="I71" s="3" t="inlineStr">
@@ -3836,7 +3836,7 @@
     <row r="72" ht="22" customHeight="1">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>7e4b4e4f136a5e31</t>
+          <t>b4f0b8c16fe5543e</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -3846,12 +3846,12 @@
       </c>
       <c r="C72" s="3" t="inlineStr">
         <is>
-          <t>Agente Mesa de Ayuda</t>
+          <t>Auxiliar de Sistemas</t>
         </is>
       </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
-          <t>Importante empresa del sector</t>
+          <t>ELIS COLOMBIA SAS</t>
         </is>
       </c>
       <c r="E72" s="7" t="n">
@@ -3863,7 +3863,7 @@
         </is>
       </c>
       <c r="G72" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-agente-mesa-de-ayuda-en-bogota-dc-E39FE355E02E578761373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-en-bogota-dc-48C2A0A3B050945661373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H72" s="6" t="inlineStr">
@@ -3886,7 +3886,7 @@
     <row r="73" ht="22" customHeight="1">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>0ef2cd7667600919</t>
+          <t>7e4b4e4f136a5e31</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
@@ -3896,12 +3896,12 @@
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>Técnico de Soporte TI Regional</t>
+          <t>Agente Mesa de Ayuda</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>POLICOMP COLOMBIA SAS</t>
+          <t>Importante empresa del sector</t>
         </is>
       </c>
       <c r="E73" s="7" t="n">
@@ -3913,10 +3913,14 @@
         </is>
       </c>
       <c r="G73" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-ti-regional-en-bogota-dc-ACF045C94E41CCDE61373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H73" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-agente-mesa-de-ayuda-en-bogota-dc-E39FE355E02E578761373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H73" s="6" t="inlineStr">
+        <is>
+          <t>$ 2.000.000,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I73" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -3932,7 +3936,7 @@
     <row r="74" ht="22" customHeight="1">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>7784997bda962255</t>
+          <t>0ef2cd7667600919</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
@@ -3942,7 +3946,7 @@
       </c>
       <c r="C74" s="3" t="inlineStr">
         <is>
-          <t>Técnico de Soporte TI On Demand/ por horas</t>
+          <t>Técnico de Soporte TI Regional</t>
         </is>
       </c>
       <c r="D74" s="3" t="inlineStr">
@@ -3959,7 +3963,7 @@
         </is>
       </c>
       <c r="G74" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-ti-on-demand-por-horas-en-bogota-dc-C2338FA0172D59A561373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-ti-regional-en-bogota-dc-ACF045C94E41CCDE61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H74" s="6" t="inlineStr"/>
@@ -3978,7 +3982,7 @@
     <row r="75" ht="22" customHeight="1">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>29d0fe2e42e678f7</t>
+          <t>7784997bda962255</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
@@ -3988,12 +3992,12 @@
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>Técnico mantenimiento correctivo impresoras</t>
+          <t>Técnico de Soporte TI On Demand/ por horas</t>
         </is>
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>Multinacional de Impresión</t>
+          <t>POLICOMP COLOMBIA SAS</t>
         </is>
       </c>
       <c r="E75" s="7" t="n">
@@ -4005,14 +4009,10 @@
         </is>
       </c>
       <c r="G75" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-mantenimiento-correctivo-impresoras-en-guarne-BC0E775C0F25B27D61373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H75" s="6" t="inlineStr">
-        <is>
-          <t>$ 1.800.000,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-ti-on-demand-por-horas-en-bogota-dc-C2338FA0172D59A561373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H75" s="6" t="inlineStr"/>
       <c r="I75" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -4028,22 +4028,22 @@
     <row r="76" ht="22" customHeight="1">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>98c9ab11f5b1eace</t>
+          <t>29d0fe2e42e678f7</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 18:36</t>
+          <t>2026-09-27 15:41</t>
         </is>
       </c>
       <c r="C76" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar de sistemas</t>
+          <t>Técnico mantenimiento correctivo impresoras</t>
         </is>
       </c>
       <c r="D76" s="3" t="inlineStr">
         <is>
-          <t>Importante empresa del sector</t>
+          <t>Multinacional de Impresión</t>
         </is>
       </c>
       <c r="E76" s="7" t="n">
@@ -4055,12 +4055,12 @@
         </is>
       </c>
       <c r="G76" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-persona-con-discapacidad-remota-en-bogota-dc-5F2A812D014E159B61373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-mantenimiento-correctivo-impresoras-en-guarne-BC0E775C0F25B27D61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H76" s="6" t="inlineStr">
         <is>
-          <t>$ 1.750.905,00 (Mensual)</t>
+          <t>$ 1.800.000,00 (Mensual)</t>
         </is>
       </c>
       <c r="I76" s="3" t="inlineStr">
@@ -4078,7 +4078,7 @@
     <row r="77" ht="22" customHeight="1">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>58133ddc4da9c68e</t>
+          <t>98c9ab11f5b1eace</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
@@ -4105,7 +4105,7 @@
         </is>
       </c>
       <c r="G77" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-persona-con-discapacidad-remota-en-bogota-dc-A00C07C9CC9A494B61373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-persona-con-discapacidad-remota-en-bogota-dc-5F2A812D014E159B61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H77" s="6" t="inlineStr">
@@ -4128,7 +4128,7 @@
     <row r="78" ht="22" customHeight="1">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>aed3420a4cfdc248</t>
+          <t>58133ddc4da9c68e</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -4138,12 +4138,12 @@
       </c>
       <c r="C78" s="3" t="inlineStr">
         <is>
-          <t>Consultor de servicios/ mesa de ayuda nómina y erp software</t>
+          <t>Auxiliar de sistemas</t>
         </is>
       </c>
       <c r="D78" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Importante empresa del sector</t>
         </is>
       </c>
       <c r="E78" s="7" t="n">
@@ -4155,10 +4155,14 @@
         </is>
       </c>
       <c r="G78" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/consultor-de-servicios-mesa-de-ayuda-nomina-y-erp-software-inclusivo-1886716126", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H78" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-persona-con-discapacidad-remota-en-bogota-dc-A00C07C9CC9A494B61373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H78" s="6" t="inlineStr">
+        <is>
+          <t>$ 1.750.905,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I78" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -4174,22 +4178,22 @@
     <row r="79" ht="22" customHeight="1">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>2b8357189ff315da</t>
+          <t>aed3420a4cfdc248</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 17:00</t>
+          <t>2026-09-28 18:36</t>
         </is>
       </c>
       <c r="C79" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar de sistemas</t>
+          <t>Consultor de servicios/ mesa de ayuda nómina y erp software</t>
         </is>
       </c>
       <c r="D79" s="3" t="inlineStr">
         <is>
-          <t>DAVITA SAS</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E79" s="7" t="n">
@@ -4201,7 +4205,7 @@
         </is>
       </c>
       <c r="G79" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886758163", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/consultor-de-servicios-mesa-de-ayuda-nomina-y-erp-software-inclusivo-1886716126", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H79" s="6" t="inlineStr"/>
@@ -4220,7 +4224,7 @@
     <row r="80" ht="22" customHeight="1">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>a87934e7643b2c1c</t>
+          <t>2b8357189ff315da</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
@@ -4230,12 +4234,12 @@
       </c>
       <c r="C80" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de instalaciones cableado de redes - licencia conte cali</t>
+          <t>Auxiliar de sistemas</t>
         </is>
       </c>
       <c r="D80" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>DAVITA SAS</t>
         </is>
       </c>
       <c r="E80" s="7" t="n">
@@ -4247,7 +4251,7 @@
         </is>
       </c>
       <c r="G80" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-cali-1886759847", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886758163", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H80" s="6" t="inlineStr"/>
@@ -4266,7 +4270,7 @@
     <row r="81" ht="22" customHeight="1">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>10b4265e3ad11d81</t>
+          <t>a87934e7643b2c1c</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
@@ -4276,12 +4280,12 @@
       </c>
       <c r="C81" s="3" t="inlineStr">
         <is>
-          <t>Information Technology Help Desk Support</t>
+          <t>Tecnico de instalaciones cableado de redes - licencia conte cali</t>
         </is>
       </c>
       <c r="D81" s="3" t="inlineStr">
         <is>
-          <t>Booth</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E81" s="7" t="n">
@@ -4293,7 +4297,7 @@
         </is>
       </c>
       <c r="G81" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/information-technology-help-desk-support-at-booth-4471203962", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-cali-1886759847", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H81" s="6" t="inlineStr"/>
@@ -4312,52 +4316,236 @@
     <row r="82" ht="22" customHeight="1">
       <c r="A82" s="2" t="inlineStr">
         <is>
+          <t>10b4265e3ad11d81</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 17:00</t>
+        </is>
+      </c>
+      <c r="C82" s="3" t="inlineStr">
+        <is>
+          <t>Information Technology Help Desk Support</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="inlineStr">
+        <is>
+          <t>Booth</t>
+        </is>
+      </c>
+      <c r="E82" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G82" s="5">
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/information-technology-help-desk-support-at-booth-4471203962", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H82" s="6" t="inlineStr"/>
+      <c r="I82" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J82" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K82" s="3" t="inlineStr"/>
+    </row>
+    <row r="83" ht="22" customHeight="1">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>ff69ae85c8697a37</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 16:49</t>
+        </is>
+      </c>
+      <c r="C83" s="3" t="inlineStr">
+        <is>
+          <t>Técnico de soporte ti - bogota</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="inlineStr">
+        <is>
+          <t>Confidencial</t>
+        </is>
+      </c>
+      <c r="E83" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G83" s="5">
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-ti-bogota-1886774059", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H83" s="6" t="inlineStr"/>
+      <c r="I83" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J83" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K83" s="3" t="inlineStr"/>
+    </row>
+    <row r="84" ht="22" customHeight="1">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>bbacf7d69ab9084e</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 16:49</t>
+        </is>
+      </c>
+      <c r="C84" s="3" t="inlineStr">
+        <is>
+          <t>IT Helpdesk Analyst</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="inlineStr">
+        <is>
+          <t>Power Digital Marketing</t>
+        </is>
+      </c>
+      <c r="E84" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G84" s="5">
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/it-helpdesk-analyst-at-power-digital-marketing-4472601999", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H84" s="6" t="inlineStr"/>
+      <c r="I84" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J84" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K84" s="3" t="inlineStr"/>
+    </row>
+    <row r="85" ht="22" customHeight="1">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
           <t>0b0ae49f910109bb</t>
         </is>
       </c>
-      <c r="B82" s="2" t="inlineStr">
+      <c r="B85" s="2" t="inlineStr">
         <is>
           <t>2026-09-25 15:54</t>
         </is>
       </c>
-      <c r="C82" s="3" t="inlineStr">
+      <c r="C85" s="3" t="inlineStr">
         <is>
           <t>Ejecutivo Técnico Arancel Junior</t>
         </is>
       </c>
-      <c r="D82" s="3" t="inlineStr">
+      <c r="D85" s="3" t="inlineStr">
         <is>
           <t>Importante Empresa de Logística y Comercio</t>
         </is>
       </c>
-      <c r="E82" s="7" t="n">
+      <c r="E85" s="7" t="n">
         <v>0.5</v>
       </c>
-      <c r="F82" s="2" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
-      <c r="G82" s="5">
+      <c r="F85" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G85" s="5">
         <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-547866639B487E0161373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
-      <c r="H82" s="6" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
-      <c r="I82" s="3" t="inlineStr">
+      <c r="H85" s="6" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="I85" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
-      <c r="J82" s="2" t="inlineStr">
-        <is>
-          <t>Nueva</t>
-        </is>
-      </c>
-      <c r="K82" s="3" t="inlineStr"/>
+      <c r="J85" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K85" s="3" t="inlineStr"/>
+    </row>
+    <row r="86" ht="22" customHeight="1">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>582a04b3c639bfa0</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 16:49</t>
+        </is>
+      </c>
+      <c r="C86" s="3" t="inlineStr">
+        <is>
+          <t>Junior IT Support Specialist</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="inlineStr">
+        <is>
+          <t>Touch Support, Inc. &amp; SNF Back Office</t>
+        </is>
+      </c>
+      <c r="E86" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G86" s="5">
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/junior-it-support-specialist-at-touch-support-inc-snf-back-office-4472187578", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H86" s="6" t="inlineStr"/>
+      <c r="I86" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J86" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K86" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
chore(tracker): actualizacion diaria de vacantes 2026-10-01
</commit_message>
<xml_diff>
--- a/output/profile_5_tecnico_sistemas_tracker.xlsx
+++ b/output/profile_5_tecnico_sistemas_tracker.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K86"/>
+  <dimension ref="A1:K92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3184,26 +3184,26 @@
     <row r="58" ht="22" customHeight="1">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>ae736277661dc78b</t>
+          <t>343718cc539a53c2</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 15:23</t>
+          <t>2026-10-01 17:26</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>Analista de redes cisco</t>
+          <t>Analista de Soporte Tecnico Cubrimiento de Licencia</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>ATCG DE COLOMBIA S.A.S</t>
-        </is>
-      </c>
-      <c r="E58" s="7" t="n">
-        <v>0.68</v>
+          <t>ZEMSANIA COLOMBIA SAS</t>
+        </is>
+      </c>
+      <c r="E58" s="4" t="n">
+        <v>0.73</v>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
@@ -3211,13 +3211,17 @@
         </is>
       </c>
       <c r="G58" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-cisco-1886760389", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H58" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-analista-de-soporte-tecnico-cubrimiento-de-licencia-remoto-en-bogota-dc-55EB665BAC5F3EB161373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H58" s="6" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
       <c r="I58" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 68/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 73/100 - Alta Afinidad] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J58" s="2" t="inlineStr">
@@ -3230,26 +3234,26 @@
     <row r="59" ht="22" customHeight="1">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>e29676fac3409ad6</t>
+          <t>d36873ab6ad37d17</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 15:23</t>
+          <t>2026-10-01 17:26</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>Analista de redes y telecomunicaciones - nivel 1</t>
+          <t>Analista de Soporte Técnico y Mesa de Ayuda TI</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>MANPOWER</t>
-        </is>
-      </c>
-      <c r="E59" s="7" t="n">
-        <v>0.68</v>
+          <t>E-GLOBAL S.A.</t>
+        </is>
+      </c>
+      <c r="E59" s="4" t="n">
+        <v>0.73</v>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
@@ -3257,13 +3261,17 @@
         </is>
       </c>
       <c r="G59" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-y-telecomunicaciones-nivel-1-1886760565", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H59" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-analista-de-soporte-tecnico-y-mesa-de-ayuda-ti-en-medellin-2D6021D92F3B61C461373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H59" s="6" t="inlineStr">
+        <is>
+          <t>$ 2.000.000,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I59" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 68/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 73/100 - Alta Afinidad] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J59" s="2" t="inlineStr">
@@ -3276,26 +3284,26 @@
     <row r="60" ht="22" customHeight="1">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>8d7f304ffb8625b5</t>
+          <t>ae736277661dc78b</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 15:54</t>
+          <t>2026-09-24 15:23</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar de sistemas</t>
+          <t>Analista de redes cisco</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>ATCG DE COLOMBIA S.A.S</t>
         </is>
       </c>
       <c r="E60" s="7" t="n">
-        <v>0.58</v>
+        <v>0.68</v>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
@@ -3303,13 +3311,13 @@
         </is>
       </c>
       <c r="G60" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886751888", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-cisco-1886760389", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H60" s="6" t="inlineStr"/>
       <c r="I60" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 68/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J60" s="2" t="inlineStr">
@@ -3322,26 +3330,26 @@
     <row r="61" ht="22" customHeight="1">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>3b5b26f92a305c0c</t>
+          <t>e29676fac3409ad6</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 15:54</t>
+          <t>2026-09-24 15:23</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar de sistemas</t>
+          <t>Analista de redes y telecomunicaciones - nivel 1</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>MANPOWER</t>
         </is>
       </c>
       <c r="E61" s="7" t="n">
-        <v>0.58</v>
+        <v>0.68</v>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
@@ -3349,13 +3357,13 @@
         </is>
       </c>
       <c r="G61" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886749497", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-y-telecomunicaciones-nivel-1-1886760565", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H61" s="6" t="inlineStr"/>
       <c r="I61" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 68/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J61" s="2" t="inlineStr">
@@ -3368,7 +3376,7 @@
     <row r="62" ht="22" customHeight="1">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>e760bcd88d90fbbe</t>
+          <t>8d7f304ffb8625b5</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -3378,12 +3386,12 @@
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>Agente de mesa de ayuda</t>
+          <t>Auxiliar de sistemas</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>SELCOMP INGENIERÍA SAS</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E62" s="7" t="n">
@@ -3395,7 +3403,7 @@
         </is>
       </c>
       <c r="G62" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-de-mesa-de-ayuda-1886758623", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886751888", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H62" s="6" t="inlineStr"/>
@@ -3414,7 +3422,7 @@
     <row r="63" ht="22" customHeight="1">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>86dcab5c5d802693</t>
+          <t>3b5b26f92a305c0c</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
@@ -3424,12 +3432,12 @@
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>Analista mesa de ayuda para tunja</t>
+          <t>Auxiliar de sistemas</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>Gestión de Seguridad Electrónica</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E63" s="7" t="n">
@@ -3441,7 +3449,7 @@
         </is>
       </c>
       <c r="G63" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-para-tunja-1886766955", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886749497", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H63" s="6" t="inlineStr"/>
@@ -3460,7 +3468,7 @@
     <row r="64" ht="22" customHeight="1">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>55fdaa0983ef9124</t>
+          <t>e760bcd88d90fbbe</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -3470,12 +3478,12 @@
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>Lider técnico con itil practice manager</t>
+          <t>Agente de mesa de ayuda</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t>Sinergy &amp; Lowells</t>
+          <t>SELCOMP INGENIERÍA SAS</t>
         </is>
       </c>
       <c r="E64" s="7" t="n">
@@ -3487,7 +3495,7 @@
         </is>
       </c>
       <c r="G64" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/lider-tecnico-con-itil-practice-manager-1886753953", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-de-mesa-de-ayuda-1886758623", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H64" s="6" t="inlineStr"/>
@@ -3506,7 +3514,7 @@
     <row r="65" ht="22" customHeight="1">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>a1ca7bc58cd48fad</t>
+          <t>86dcab5c5d802693</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
@@ -3516,12 +3524,12 @@
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de mesa de ayuda/mujeres contratacion inmediata</t>
+          <t>Analista mesa de ayuda para tunja</t>
         </is>
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Gestión de Seguridad Electrónica</t>
         </is>
       </c>
       <c r="E65" s="7" t="n">
@@ -3533,7 +3541,7 @@
         </is>
       </c>
       <c r="G65" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-mesa-de-ayuda-mujeres-contratacion-inmediata-1886770931", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-para-tunja-1886766955", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H65" s="6" t="inlineStr"/>
@@ -3552,7 +3560,7 @@
     <row r="66" ht="22" customHeight="1">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>e28aba5df8a2d3ae</t>
+          <t>55fdaa0983ef9124</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -3562,12 +3570,12 @@
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de mesa de ayuda/mujeres contratacion inmediata</t>
+          <t>Lider técnico con itil practice manager</t>
         </is>
       </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Sinergy &amp; Lowells</t>
         </is>
       </c>
       <c r="E66" s="7" t="n">
@@ -3579,7 +3587,7 @@
         </is>
       </c>
       <c r="G66" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-mesa-de-ayuda-mujeres-contratacion-inmediata-1886769701", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/lider-tecnico-con-itil-practice-manager-1886753953", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H66" s="6" t="inlineStr"/>
@@ -3598,7 +3606,7 @@
     <row r="67" ht="22" customHeight="1">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>9326784c1a2726fb</t>
+          <t>a1ca7bc58cd48fad</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
@@ -3608,12 +3616,12 @@
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>Técnico de soporte y mesa de ayuda / medellín</t>
+          <t>Tecnico de mesa de ayuda/mujeres contratacion inmediata</t>
         </is>
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>Colsof S.A.S</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E67" s="7" t="n">
@@ -3625,7 +3633,7 @@
         </is>
       </c>
       <c r="G67" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-y-mesa-de-ayuda-medellin-1886738118", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-mesa-de-ayuda-mujeres-contratacion-inmediata-1886770931", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H67" s="6" t="inlineStr"/>
@@ -3644,7 +3652,7 @@
     <row r="68" ht="22" customHeight="1">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>b67dc9a9be4a1a6f</t>
+          <t>e28aba5df8a2d3ae</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -3654,7 +3662,7 @@
       </c>
       <c r="C68" s="3" t="inlineStr">
         <is>
-          <t>Service desk agent</t>
+          <t>Tecnico de mesa de ayuda/mujeres contratacion inmediata</t>
         </is>
       </c>
       <c r="D68" s="3" t="inlineStr">
@@ -3671,13 +3679,13 @@
         </is>
       </c>
       <c r="G68" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/service-desk-agent-soporte-tecnico-nivel-1-1886755112", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-mesa-de-ayuda-mujeres-contratacion-inmediata-1886769701", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H68" s="6" t="inlineStr"/>
       <c r="I68" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J68" s="2" t="inlineStr">
@@ -3690,7 +3698,7 @@
     <row r="69" ht="22" customHeight="1">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>9c65f710f43158b7</t>
+          <t>9326784c1a2726fb</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
@@ -3700,12 +3708,12 @@
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de instalaciones cableado de redes - licencia conte</t>
+          <t>Técnico de soporte y mesa de ayuda / medellín</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Colsof S.A.S</t>
         </is>
       </c>
       <c r="E69" s="7" t="n">
@@ -3717,7 +3725,7 @@
         </is>
       </c>
       <c r="G69" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-1886749397", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-y-mesa-de-ayuda-medellin-1886738118", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H69" s="6" t="inlineStr"/>
@@ -3736,22 +3744,22 @@
     <row r="70" ht="22" customHeight="1">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>a95003a0b1fc3d77</t>
+          <t>b67dc9a9be4a1a6f</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 15:41</t>
+          <t>2026-09-25 15:54</t>
         </is>
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>Técnico Soporte Nivel 1 Con ITIL</t>
+          <t>Service desk agent</t>
         </is>
       </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
-          <t>Importante empresa del sector de tecnología</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E70" s="7" t="n">
@@ -3763,17 +3771,13 @@
         </is>
       </c>
       <c r="G70" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-soporte-nivel-1-con-itil-en-bogota-dc-59E13FA64EF5843C61373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H70" s="6" t="inlineStr">
-        <is>
-          <t>$ 1.750.905,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/service-desk-agent-soporte-tecnico-nivel-1-1886755112", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H70" s="6" t="inlineStr"/>
       <c r="I70" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J70" s="2" t="inlineStr">
@@ -3786,22 +3790,22 @@
     <row r="71" ht="22" customHeight="1">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>96391fd564d83616</t>
+          <t>9c65f710f43158b7</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 15:41</t>
+          <t>2026-09-25 15:54</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de soporte IT con Moto</t>
+          <t>Tecnico de instalaciones cableado de redes - licencia conte</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>Los Hornitos</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E71" s="7" t="n">
@@ -3813,14 +3817,10 @@
         </is>
       </c>
       <c r="G71" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-it-con-moto-empresa-de-alimentos-en-bogota-dc-599938D46A6F4A8F61373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H71" s="6" t="inlineStr">
-        <is>
-          <t>$ 2.125.947,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-1886749397", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H71" s="6" t="inlineStr"/>
       <c r="I71" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -3836,7 +3836,7 @@
     <row r="72" ht="22" customHeight="1">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>b4f0b8c16fe5543e</t>
+          <t>a95003a0b1fc3d77</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -3846,12 +3846,12 @@
       </c>
       <c r="C72" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar de Sistemas</t>
+          <t>Técnico Soporte Nivel 1 Con ITIL</t>
         </is>
       </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
-          <t>ELIS COLOMBIA SAS</t>
+          <t>Importante empresa del sector de tecnología</t>
         </is>
       </c>
       <c r="E72" s="7" t="n">
@@ -3863,12 +3863,12 @@
         </is>
       </c>
       <c r="G72" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-en-bogota-dc-48C2A0A3B050945661373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-soporte-nivel-1-con-itil-en-bogota-dc-59E13FA64EF5843C61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H72" s="6" t="inlineStr">
         <is>
-          <t>$ 2.000.000,00 (Mensual)</t>
+          <t>$ 1.750.905,00 (Mensual)</t>
         </is>
       </c>
       <c r="I72" s="3" t="inlineStr">
@@ -3886,7 +3886,7 @@
     <row r="73" ht="22" customHeight="1">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>7e4b4e4f136a5e31</t>
+          <t>96391fd564d83616</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
@@ -3896,12 +3896,12 @@
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>Agente Mesa de Ayuda</t>
+          <t>Tecnico de soporte IT con Moto</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>Importante empresa del sector</t>
+          <t>Los Hornitos</t>
         </is>
       </c>
       <c r="E73" s="7" t="n">
@@ -3913,12 +3913,12 @@
         </is>
       </c>
       <c r="G73" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-agente-mesa-de-ayuda-en-bogota-dc-E39FE355E02E578761373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-it-con-moto-empresa-de-alimentos-en-bogota-dc-599938D46A6F4A8F61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H73" s="6" t="inlineStr">
         <is>
-          <t>$ 2.000.000,00 (Mensual)</t>
+          <t>$ 2.125.947,00 (Mensual)</t>
         </is>
       </c>
       <c r="I73" s="3" t="inlineStr">
@@ -3936,7 +3936,7 @@
     <row r="74" ht="22" customHeight="1">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>0ef2cd7667600919</t>
+          <t>b4f0b8c16fe5543e</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
@@ -3946,12 +3946,12 @@
       </c>
       <c r="C74" s="3" t="inlineStr">
         <is>
-          <t>Técnico de Soporte TI Regional</t>
+          <t>Auxiliar de Sistemas</t>
         </is>
       </c>
       <c r="D74" s="3" t="inlineStr">
         <is>
-          <t>POLICOMP COLOMBIA SAS</t>
+          <t>ELIS COLOMBIA SAS</t>
         </is>
       </c>
       <c r="E74" s="7" t="n">
@@ -3963,10 +3963,14 @@
         </is>
       </c>
       <c r="G74" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-ti-regional-en-bogota-dc-ACF045C94E41CCDE61373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H74" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-en-bogota-dc-48C2A0A3B050945661373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H74" s="6" t="inlineStr">
+        <is>
+          <t>$ 2.000.000,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I74" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -3982,7 +3986,7 @@
     <row r="75" ht="22" customHeight="1">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>7784997bda962255</t>
+          <t>7e4b4e4f136a5e31</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
@@ -3992,12 +3996,12 @@
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>Técnico de Soporte TI On Demand/ por horas</t>
+          <t>Agente Mesa de Ayuda</t>
         </is>
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>POLICOMP COLOMBIA SAS</t>
+          <t>Importante empresa del sector</t>
         </is>
       </c>
       <c r="E75" s="7" t="n">
@@ -4009,10 +4013,14 @@
         </is>
       </c>
       <c r="G75" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-ti-on-demand-por-horas-en-bogota-dc-C2338FA0172D59A561373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H75" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-agente-mesa-de-ayuda-en-bogota-dc-E39FE355E02E578761373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H75" s="6" t="inlineStr">
+        <is>
+          <t>$ 2.000.000,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I75" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -4028,7 +4036,7 @@
     <row r="76" ht="22" customHeight="1">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>29d0fe2e42e678f7</t>
+          <t>0ef2cd7667600919</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
@@ -4038,12 +4046,12 @@
       </c>
       <c r="C76" s="3" t="inlineStr">
         <is>
-          <t>Técnico mantenimiento correctivo impresoras</t>
+          <t>Técnico de Soporte TI Regional</t>
         </is>
       </c>
       <c r="D76" s="3" t="inlineStr">
         <is>
-          <t>Multinacional de Impresión</t>
+          <t>POLICOMP COLOMBIA SAS</t>
         </is>
       </c>
       <c r="E76" s="7" t="n">
@@ -4055,14 +4063,10 @@
         </is>
       </c>
       <c r="G76" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-mantenimiento-correctivo-impresoras-en-guarne-BC0E775C0F25B27D61373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H76" s="6" t="inlineStr">
-        <is>
-          <t>$ 1.800.000,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-ti-regional-en-bogota-dc-ACF045C94E41CCDE61373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H76" s="6" t="inlineStr"/>
       <c r="I76" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -4078,22 +4082,22 @@
     <row r="77" ht="22" customHeight="1">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>98c9ab11f5b1eace</t>
+          <t>7784997bda962255</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 18:36</t>
+          <t>2026-09-27 15:41</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar de sistemas</t>
+          <t>Técnico de Soporte TI On Demand/ por horas</t>
         </is>
       </c>
       <c r="D77" s="3" t="inlineStr">
         <is>
-          <t>Importante empresa del sector</t>
+          <t>POLICOMP COLOMBIA SAS</t>
         </is>
       </c>
       <c r="E77" s="7" t="n">
@@ -4105,14 +4109,10 @@
         </is>
       </c>
       <c r="G77" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-persona-con-discapacidad-remota-en-bogota-dc-5F2A812D014E159B61373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H77" s="6" t="inlineStr">
-        <is>
-          <t>$ 1.750.905,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-ti-on-demand-por-horas-en-bogota-dc-C2338FA0172D59A561373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H77" s="6" t="inlineStr"/>
       <c r="I77" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -4128,22 +4128,22 @@
     <row r="78" ht="22" customHeight="1">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>58133ddc4da9c68e</t>
+          <t>29d0fe2e42e678f7</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 18:36</t>
+          <t>2026-09-27 15:41</t>
         </is>
       </c>
       <c r="C78" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar de sistemas</t>
+          <t>Técnico mantenimiento correctivo impresoras</t>
         </is>
       </c>
       <c r="D78" s="3" t="inlineStr">
         <is>
-          <t>Importante empresa del sector</t>
+          <t>Multinacional de Impresión</t>
         </is>
       </c>
       <c r="E78" s="7" t="n">
@@ -4155,12 +4155,12 @@
         </is>
       </c>
       <c r="G78" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-persona-con-discapacidad-remota-en-bogota-dc-A00C07C9CC9A494B61373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-mantenimiento-correctivo-impresoras-en-guarne-BC0E775C0F25B27D61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H78" s="6" t="inlineStr">
         <is>
-          <t>$ 1.750.905,00 (Mensual)</t>
+          <t>$ 1.800.000,00 (Mensual)</t>
         </is>
       </c>
       <c r="I78" s="3" t="inlineStr">
@@ -4178,7 +4178,7 @@
     <row r="79" ht="22" customHeight="1">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>aed3420a4cfdc248</t>
+          <t>98c9ab11f5b1eace</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
@@ -4188,12 +4188,12 @@
       </c>
       <c r="C79" s="3" t="inlineStr">
         <is>
-          <t>Consultor de servicios/ mesa de ayuda nómina y erp software</t>
+          <t>Auxiliar de sistemas</t>
         </is>
       </c>
       <c r="D79" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Importante empresa del sector</t>
         </is>
       </c>
       <c r="E79" s="7" t="n">
@@ -4205,10 +4205,14 @@
         </is>
       </c>
       <c r="G79" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/consultor-de-servicios-mesa-de-ayuda-nomina-y-erp-software-inclusivo-1886716126", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H79" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-persona-con-discapacidad-remota-en-bogota-dc-5F2A812D014E159B61373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H79" s="6" t="inlineStr">
+        <is>
+          <t>$ 1.750.905,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I79" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -4224,12 +4228,12 @@
     <row r="80" ht="22" customHeight="1">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>2b8357189ff315da</t>
+          <t>58133ddc4da9c68e</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 17:00</t>
+          <t>2026-09-28 18:36</t>
         </is>
       </c>
       <c r="C80" s="3" t="inlineStr">
@@ -4239,7 +4243,7 @@
       </c>
       <c r="D80" s="3" t="inlineStr">
         <is>
-          <t>DAVITA SAS</t>
+          <t>Importante empresa del sector</t>
         </is>
       </c>
       <c r="E80" s="7" t="n">
@@ -4251,10 +4255,14 @@
         </is>
       </c>
       <c r="G80" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886758163", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H80" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-persona-con-discapacidad-remota-en-bogota-dc-A00C07C9CC9A494B61373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H80" s="6" t="inlineStr">
+        <is>
+          <t>$ 1.750.905,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I80" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -4270,17 +4278,17 @@
     <row r="81" ht="22" customHeight="1">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>a87934e7643b2c1c</t>
+          <t>aed3420a4cfdc248</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 17:00</t>
+          <t>2026-09-28 18:36</t>
         </is>
       </c>
       <c r="C81" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de instalaciones cableado de redes - licencia conte cali</t>
+          <t>Consultor de servicios/ mesa de ayuda nómina y erp software</t>
         </is>
       </c>
       <c r="D81" s="3" t="inlineStr">
@@ -4297,7 +4305,7 @@
         </is>
       </c>
       <c r="G81" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-cali-1886759847", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/consultor-de-servicios-mesa-de-ayuda-nomina-y-erp-software-inclusivo-1886716126", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H81" s="6" t="inlineStr"/>
@@ -4316,7 +4324,7 @@
     <row r="82" ht="22" customHeight="1">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>10b4265e3ad11d81</t>
+          <t>2b8357189ff315da</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
@@ -4326,12 +4334,12 @@
       </c>
       <c r="C82" s="3" t="inlineStr">
         <is>
-          <t>Information Technology Help Desk Support</t>
+          <t>Auxiliar de sistemas</t>
         </is>
       </c>
       <c r="D82" s="3" t="inlineStr">
         <is>
-          <t>Booth</t>
+          <t>DAVITA SAS</t>
         </is>
       </c>
       <c r="E82" s="7" t="n">
@@ -4343,7 +4351,7 @@
         </is>
       </c>
       <c r="G82" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/information-technology-help-desk-support-at-booth-4471203962", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886758163", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H82" s="6" t="inlineStr"/>
@@ -4362,17 +4370,17 @@
     <row r="83" ht="22" customHeight="1">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>ff69ae85c8697a37</t>
+          <t>a87934e7643b2c1c</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 16:49</t>
+          <t>2026-09-29 17:00</t>
         </is>
       </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t>Técnico de soporte ti - bogota</t>
+          <t>Tecnico de instalaciones cableado de redes - licencia conte cali</t>
         </is>
       </c>
       <c r="D83" s="3" t="inlineStr">
@@ -4389,7 +4397,7 @@
         </is>
       </c>
       <c r="G83" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-ti-bogota-1886774059", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-cali-1886759847", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H83" s="6" t="inlineStr"/>
@@ -4408,22 +4416,22 @@
     <row r="84" ht="22" customHeight="1">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>bbacf7d69ab9084e</t>
+          <t>10b4265e3ad11d81</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 16:49</t>
+          <t>2026-09-29 17:00</t>
         </is>
       </c>
       <c r="C84" s="3" t="inlineStr">
         <is>
-          <t>IT Helpdesk Analyst</t>
+          <t>Information Technology Help Desk Support</t>
         </is>
       </c>
       <c r="D84" s="3" t="inlineStr">
         <is>
-          <t>Power Digital Marketing</t>
+          <t>Booth</t>
         </is>
       </c>
       <c r="E84" s="7" t="n">
@@ -4435,7 +4443,7 @@
         </is>
       </c>
       <c r="G84" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/it-helpdesk-analyst-at-power-digital-marketing-4472601999", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/information-technology-help-desk-support-at-booth-4471203962", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H84" s="6" t="inlineStr"/>
@@ -4454,26 +4462,26 @@
     <row r="85" ht="22" customHeight="1">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>0b0ae49f910109bb</t>
+          <t>ff69ae85c8697a37</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 15:54</t>
+          <t>2026-09-30 16:49</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>Ejecutivo Técnico Arancel Junior</t>
+          <t>Técnico de soporte ti - bogota</t>
         </is>
       </c>
       <c r="D85" s="3" t="inlineStr">
         <is>
-          <t>Importante Empresa de Logística y Comercio</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E85" s="7" t="n">
-        <v>0.5</v>
+        <v>0.58</v>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
@@ -4481,17 +4489,13 @@
         </is>
       </c>
       <c r="G85" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-547866639B487E0161373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H85" s="6" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-ti-bogota-1886774059", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H85" s="6" t="inlineStr"/>
       <c r="I85" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J85" s="2" t="inlineStr">
@@ -4504,7 +4508,7 @@
     <row r="86" ht="22" customHeight="1">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>582a04b3c639bfa0</t>
+          <t>bbacf7d69ab9084e</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
@@ -4514,16 +4518,16 @@
       </c>
       <c r="C86" s="3" t="inlineStr">
         <is>
-          <t>Junior IT Support Specialist</t>
+          <t>IT Helpdesk Analyst</t>
         </is>
       </c>
       <c r="D86" s="3" t="inlineStr">
         <is>
-          <t>Touch Support, Inc. &amp; SNF Back Office</t>
+          <t>Power Digital Marketing</t>
         </is>
       </c>
       <c r="E86" s="7" t="n">
-        <v>0.5</v>
+        <v>0.58</v>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
@@ -4531,21 +4535,305 @@
         </is>
       </c>
       <c r="G86" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/junior-it-support-specialist-at-touch-support-inc-snf-back-office-4472187578", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/it-helpdesk-analyst-at-power-digital-marketing-4472601999", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H86" s="6" t="inlineStr"/>
       <c r="I86" s="3" t="inlineStr">
         <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J86" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K86" s="3" t="inlineStr"/>
+    </row>
+    <row r="87" ht="22" customHeight="1">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>bb848f474ff4b611</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01 17:26</t>
+        </is>
+      </c>
+      <c r="C87" s="3" t="inlineStr">
+        <is>
+          <t>Técnico de soporte ti - bogota</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="inlineStr">
+        <is>
+          <t>Confidencial</t>
+        </is>
+      </c>
+      <c r="E87" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F87" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G87" s="5">
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-ti-bogota-1886772292", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H87" s="6" t="inlineStr"/>
+      <c r="I87" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J87" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K87" s="3" t="inlineStr"/>
+    </row>
+    <row r="88" ht="22" customHeight="1">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>b44a1c6cfb004ca8</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01 17:26</t>
+        </is>
+      </c>
+      <c r="C88" s="3" t="inlineStr">
+        <is>
+          <t>Soporte ti nivel 2 - bogotá</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="inlineStr">
+        <is>
+          <t>Confidencial</t>
+        </is>
+      </c>
+      <c r="E88" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G88" s="5">
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/soporte-ti-nivel-2-bogota-1886774821", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H88" s="6" t="inlineStr"/>
+      <c r="I88" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J88" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K88" s="3" t="inlineStr"/>
+    </row>
+    <row r="89" ht="22" customHeight="1">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>fb0ad2b513afb97c</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01 17:26</t>
+        </is>
+      </c>
+      <c r="C89" s="3" t="inlineStr">
+        <is>
+          <t>IT Help Desk Support Specialist</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="inlineStr">
+        <is>
+          <t>Talento</t>
+        </is>
+      </c>
+      <c r="E89" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F89" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G89" s="5">
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/it-help-desk-support-specialist-tier-1-at-talento-4473960480", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H89" s="6" t="inlineStr"/>
+      <c r="I89" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J89" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K89" s="3" t="inlineStr"/>
+    </row>
+    <row r="90" ht="22" customHeight="1">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>0b0ae49f910109bb</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25 15:54</t>
+        </is>
+      </c>
+      <c r="C90" s="3" t="inlineStr">
+        <is>
+          <t>Ejecutivo Técnico Arancel Junior</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="inlineStr">
+        <is>
+          <t>Importante Empresa de Logística y Comercio</t>
+        </is>
+      </c>
+      <c r="E90" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G90" s="5">
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-547866639B487E0161373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H90" s="6" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="I90" s="3" t="inlineStr">
+        <is>
           <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
-      <c r="J86" s="2" t="inlineStr">
-        <is>
-          <t>Nueva</t>
-        </is>
-      </c>
-      <c r="K86" s="3" t="inlineStr"/>
+      <c r="J90" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K90" s="3" t="inlineStr"/>
+    </row>
+    <row r="91" ht="22" customHeight="1">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>582a04b3c639bfa0</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 16:49</t>
+        </is>
+      </c>
+      <c r="C91" s="3" t="inlineStr">
+        <is>
+          <t>Junior IT Support Specialist</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="inlineStr">
+        <is>
+          <t>Touch Support, Inc. &amp; SNF Back Office</t>
+        </is>
+      </c>
+      <c r="E91" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F91" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G91" s="5">
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/junior-it-support-specialist-at-touch-support-inc-snf-back-office-4472187578", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H91" s="6" t="inlineStr"/>
+      <c r="I91" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J91" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K91" s="3" t="inlineStr"/>
+    </row>
+    <row r="92" ht="22" customHeight="1">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>6e04c4d57d3fc3c7</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01 17:26</t>
+        </is>
+      </c>
+      <c r="C92" s="3" t="inlineStr">
+        <is>
+          <t>Ejecutivo Técnico Arancel Junior</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="inlineStr">
+        <is>
+          <t>Importante Empresa de Logística y Comercio</t>
+        </is>
+      </c>
+      <c r="E92" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G92" s="5">
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-8444AB594560844161373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H92" s="6" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="I92" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J92" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K92" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
chore(tracker): actualizacion diaria de vacantes 2026-10-02
</commit_message>
<xml_diff>
--- a/output/profile_5_tecnico_sistemas_tracker.xlsx
+++ b/output/profile_5_tecnico_sistemas_tracker.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K92"/>
+  <dimension ref="A1:K94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -4692,26 +4692,26 @@
     <row r="90" ht="22" customHeight="1">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>0b0ae49f910109bb</t>
+          <t>0b2067d6ae488f4c</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 15:54</t>
+          <t>2026-10-02 16:39</t>
         </is>
       </c>
       <c r="C90" s="3" t="inlineStr">
         <is>
-          <t>Ejecutivo Técnico Arancel Junior</t>
+          <t>Help Desk Technician level 1</t>
         </is>
       </c>
       <c r="D90" s="3" t="inlineStr">
         <is>
-          <t>Importante Empresa de Logística y Comercio</t>
+          <t>Solvo Global</t>
         </is>
       </c>
       <c r="E90" s="7" t="n">
-        <v>0.5</v>
+        <v>0.58</v>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
@@ -4719,17 +4719,13 @@
         </is>
       </c>
       <c r="G90" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-547866639B487E0161373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H90" s="6" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/help-desk-technician-level-1-at-solvo-global-4472590892", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H90" s="6" t="inlineStr"/>
       <c r="I90" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J90" s="2" t="inlineStr">
@@ -4742,26 +4738,26 @@
     <row r="91" ht="22" customHeight="1">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>582a04b3c639bfa0</t>
+          <t>50c79dfbfd49f52d</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 16:49</t>
+          <t>2026-10-02 16:39</t>
         </is>
       </c>
       <c r="C91" s="3" t="inlineStr">
         <is>
-          <t>Junior IT Support Specialist</t>
+          <t>Analista de redes noc 1 telecomunicaciones.</t>
         </is>
       </c>
       <c r="D91" s="3" t="inlineStr">
         <is>
-          <t>Touch Support, Inc. &amp; SNF Back Office</t>
+          <t>MANPOWER</t>
         </is>
       </c>
       <c r="E91" s="7" t="n">
-        <v>0.5</v>
+        <v>0.53</v>
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
@@ -4769,13 +4765,13 @@
         </is>
       </c>
       <c r="G91" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/junior-it-support-specialist-at-touch-support-inc-snf-back-office-4472187578", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-noc-1-telecomunicaciones-1886772075", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H91" s="6" t="inlineStr"/>
       <c r="I91" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J91" s="2" t="inlineStr">
@@ -4788,12 +4784,12 @@
     <row r="92" ht="22" customHeight="1">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>6e04c4d57d3fc3c7</t>
+          <t>0b0ae49f910109bb</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 17:26</t>
+          <t>2026-09-25 15:54</t>
         </is>
       </c>
       <c r="C92" s="3" t="inlineStr">
@@ -4815,25 +4811,121 @@
         </is>
       </c>
       <c r="G92" s="5">
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-547866639B487E0161373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H92" s="6" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="I92" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J92" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K92" s="3" t="inlineStr"/>
+    </row>
+    <row r="93" ht="22" customHeight="1">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>582a04b3c639bfa0</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 16:49</t>
+        </is>
+      </c>
+      <c r="C93" s="3" t="inlineStr">
+        <is>
+          <t>Junior IT Support Specialist</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="inlineStr">
+        <is>
+          <t>Touch Support, Inc. &amp; SNF Back Office</t>
+        </is>
+      </c>
+      <c r="E93" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F93" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G93" s="5">
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/junior-it-support-specialist-at-touch-support-inc-snf-back-office-4472187578", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H93" s="6" t="inlineStr"/>
+      <c r="I93" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J93" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K93" s="3" t="inlineStr"/>
+    </row>
+    <row r="94" ht="22" customHeight="1">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>6e04c4d57d3fc3c7</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01 17:26</t>
+        </is>
+      </c>
+      <c r="C94" s="3" t="inlineStr">
+        <is>
+          <t>Ejecutivo Técnico Arancel Junior</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="inlineStr">
+        <is>
+          <t>Importante Empresa de Logística y Comercio</t>
+        </is>
+      </c>
+      <c r="E94" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G94" s="5">
         <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-8444AB594560844161373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
-      <c r="H92" s="6" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
-      <c r="I92" s="3" t="inlineStr">
+      <c r="H94" s="6" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="I94" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
-      <c r="J92" s="2" t="inlineStr">
-        <is>
-          <t>Nueva</t>
-        </is>
-      </c>
-      <c r="K92" s="3" t="inlineStr"/>
+      <c r="J94" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K94" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
chore(tracker): actualizacion diaria de vacantes 2026-10-03
</commit_message>
<xml_diff>
--- a/output/profile_5_tecnico_sistemas_tracker.xlsx
+++ b/output/profile_5_tecnico_sistemas_tracker.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K94"/>
+  <dimension ref="A1:K95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -4738,26 +4738,26 @@
     <row r="91" ht="22" customHeight="1">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>50c79dfbfd49f52d</t>
+          <t>07acc222a3ca2ef1</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 16:39</t>
+          <t>2026-10-03 15:12</t>
         </is>
       </c>
       <c r="C91" s="3" t="inlineStr">
         <is>
-          <t>Analista de redes noc 1 telecomunicaciones.</t>
+          <t>Analista mesa de ayuda funza temporal 6 meses</t>
         </is>
       </c>
       <c r="D91" s="3" t="inlineStr">
         <is>
-          <t>MANPOWER</t>
+          <t>Axity</t>
         </is>
       </c>
       <c r="E91" s="7" t="n">
-        <v>0.53</v>
+        <v>0.58</v>
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
@@ -4765,13 +4765,13 @@
         </is>
       </c>
       <c r="G91" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-noc-1-telecomunicaciones-1886772075", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-funza-temporal-6-meses-1886774524", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H91" s="6" t="inlineStr"/>
       <c r="I91" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J91" s="2" t="inlineStr">
@@ -4784,26 +4784,26 @@
     <row r="92" ht="22" customHeight="1">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>0b0ae49f910109bb</t>
+          <t>50c79dfbfd49f52d</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 15:54</t>
+          <t>2026-10-02 16:39</t>
         </is>
       </c>
       <c r="C92" s="3" t="inlineStr">
         <is>
-          <t>Ejecutivo Técnico Arancel Junior</t>
+          <t>Analista de redes noc 1 telecomunicaciones.</t>
         </is>
       </c>
       <c r="D92" s="3" t="inlineStr">
         <is>
-          <t>Importante Empresa de Logística y Comercio</t>
+          <t>MANPOWER</t>
         </is>
       </c>
       <c r="E92" s="7" t="n">
-        <v>0.5</v>
+        <v>0.53</v>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
@@ -4811,17 +4811,13 @@
         </is>
       </c>
       <c r="G92" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-547866639B487E0161373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H92" s="6" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-noc-1-telecomunicaciones-1886772075", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H92" s="6" t="inlineStr"/>
       <c r="I92" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J92" s="2" t="inlineStr">
@@ -4834,22 +4830,22 @@
     <row r="93" ht="22" customHeight="1">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>582a04b3c639bfa0</t>
+          <t>0b0ae49f910109bb</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 16:49</t>
+          <t>2026-09-25 15:54</t>
         </is>
       </c>
       <c r="C93" s="3" t="inlineStr">
         <is>
-          <t>Junior IT Support Specialist</t>
+          <t>Ejecutivo Técnico Arancel Junior</t>
         </is>
       </c>
       <c r="D93" s="3" t="inlineStr">
         <is>
-          <t>Touch Support, Inc. &amp; SNF Back Office</t>
+          <t>Importante Empresa de Logística y Comercio</t>
         </is>
       </c>
       <c r="E93" s="7" t="n">
@@ -4861,10 +4857,14 @@
         </is>
       </c>
       <c r="G93" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/junior-it-support-specialist-at-touch-support-inc-snf-back-office-4472187578", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H93" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-547866639B487E0161373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H93" s="6" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
       <c r="I93" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -4880,22 +4880,22 @@
     <row r="94" ht="22" customHeight="1">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>6e04c4d57d3fc3c7</t>
+          <t>582a04b3c639bfa0</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 17:26</t>
+          <t>2026-09-30 16:49</t>
         </is>
       </c>
       <c r="C94" s="3" t="inlineStr">
         <is>
-          <t>Ejecutivo Técnico Arancel Junior</t>
+          <t>Junior IT Support Specialist</t>
         </is>
       </c>
       <c r="D94" s="3" t="inlineStr">
         <is>
-          <t>Importante Empresa de Logística y Comercio</t>
+          <t>Touch Support, Inc. &amp; SNF Back Office</t>
         </is>
       </c>
       <c r="E94" s="7" t="n">
@@ -4907,25 +4907,71 @@
         </is>
       </c>
       <c r="G94" s="5">
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/junior-it-support-specialist-at-touch-support-inc-snf-back-office-4472187578", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H94" s="6" t="inlineStr"/>
+      <c r="I94" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J94" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K94" s="3" t="inlineStr"/>
+    </row>
+    <row r="95" ht="22" customHeight="1">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>6e04c4d57d3fc3c7</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01 17:26</t>
+        </is>
+      </c>
+      <c r="C95" s="3" t="inlineStr">
+        <is>
+          <t>Ejecutivo Técnico Arancel Junior</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="inlineStr">
+        <is>
+          <t>Importante Empresa de Logística y Comercio</t>
+        </is>
+      </c>
+      <c r="E95" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G95" s="5">
         <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-8444AB594560844161373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
-      <c r="H94" s="6" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
-      <c r="I94" s="3" t="inlineStr">
+      <c r="H95" s="6" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="I95" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
-      <c r="J94" s="2" t="inlineStr">
-        <is>
-          <t>Nueva</t>
-        </is>
-      </c>
-      <c r="K94" s="3" t="inlineStr"/>
+      <c r="J95" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K95" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
chore(tracker): actualizacion diaria de vacantes 2026-10-05
</commit_message>
<xml_diff>
--- a/output/profile_5_tecnico_sistemas_tracker.xlsx
+++ b/output/profile_5_tecnico_sistemas_tracker.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K95"/>
+  <dimension ref="A1:K100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3284,26 +3284,26 @@
     <row r="60" ht="22" customHeight="1">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>ae736277661dc78b</t>
+          <t>21bd61491ee26e9f</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 15:23</t>
+          <t>2026-10-05 19:45</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>Analista de redes cisco</t>
+          <t>Agente de Service Desk Mesa de Ayuda – Soporte Técnico</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>ATCG DE COLOMBIA S.A.S</t>
-        </is>
-      </c>
-      <c r="E60" s="7" t="n">
-        <v>0.68</v>
+          <t>Redes Humanas</t>
+        </is>
+      </c>
+      <c r="E60" s="4" t="n">
+        <v>0.73</v>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
@@ -3311,13 +3311,17 @@
         </is>
       </c>
       <c r="G60" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-cisco-1886760389", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H60" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-agente-de-service-desk-mesa-de-ayuda-soporte-tecnico-en-bogota-dc-B1FB577FEE65D70B61373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H60" s="6" t="inlineStr">
+        <is>
+          <t>$ 1.750.905,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I60" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 68/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 73/100 - Alta Afinidad] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J60" s="2" t="inlineStr">
@@ -3330,7 +3334,7 @@
     <row r="61" ht="22" customHeight="1">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>e29676fac3409ad6</t>
+          <t>ae736277661dc78b</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
@@ -3340,12 +3344,12 @@
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>Analista de redes y telecomunicaciones - nivel 1</t>
+          <t>Analista de redes cisco</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>MANPOWER</t>
+          <t>ATCG DE COLOMBIA S.A.S</t>
         </is>
       </c>
       <c r="E61" s="7" t="n">
@@ -3357,7 +3361,7 @@
         </is>
       </c>
       <c r="G61" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-y-telecomunicaciones-nivel-1-1886760565", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-cisco-1886760389", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H61" s="6" t="inlineStr"/>
@@ -3376,26 +3380,26 @@
     <row r="62" ht="22" customHeight="1">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>8d7f304ffb8625b5</t>
+          <t>e29676fac3409ad6</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 15:54</t>
+          <t>2026-09-24 15:23</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar de sistemas</t>
+          <t>Analista de redes y telecomunicaciones - nivel 1</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>MANPOWER</t>
         </is>
       </c>
       <c r="E62" s="7" t="n">
-        <v>0.58</v>
+        <v>0.68</v>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
@@ -3403,13 +3407,13 @@
         </is>
       </c>
       <c r="G62" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886751888", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-y-telecomunicaciones-nivel-1-1886760565", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H62" s="6" t="inlineStr"/>
       <c r="I62" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 68/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J62" s="2" t="inlineStr">
@@ -3422,26 +3426,26 @@
     <row r="63" ht="22" customHeight="1">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>3b5b26f92a305c0c</t>
+          <t>73882c81e04abc7e</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 15:54</t>
+          <t>2026-10-05 19:45</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar de sistemas</t>
+          <t>Soporte L1 Junior</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Hublance</t>
         </is>
       </c>
       <c r="E63" s="7" t="n">
-        <v>0.58</v>
+        <v>0.6</v>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
@@ -3449,13 +3453,13 @@
         </is>
       </c>
       <c r="G63" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886749497", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/soporte-l1-junior-at-hublance-4475841269", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H63" s="6" t="inlineStr"/>
       <c r="I63" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 60/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J63" s="2" t="inlineStr">
@@ -3468,7 +3472,7 @@
     <row r="64" ht="22" customHeight="1">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>e760bcd88d90fbbe</t>
+          <t>8d7f304ffb8625b5</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -3478,12 +3482,12 @@
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>Agente de mesa de ayuda</t>
+          <t>Auxiliar de sistemas</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t>SELCOMP INGENIERÍA SAS</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E64" s="7" t="n">
@@ -3495,7 +3499,7 @@
         </is>
       </c>
       <c r="G64" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-de-mesa-de-ayuda-1886758623", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886751888", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H64" s="6" t="inlineStr"/>
@@ -3514,7 +3518,7 @@
     <row r="65" ht="22" customHeight="1">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>86dcab5c5d802693</t>
+          <t>3b5b26f92a305c0c</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
@@ -3524,12 +3528,12 @@
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>Analista mesa de ayuda para tunja</t>
+          <t>Auxiliar de sistemas</t>
         </is>
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>Gestión de Seguridad Electrónica</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E65" s="7" t="n">
@@ -3541,7 +3545,7 @@
         </is>
       </c>
       <c r="G65" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-para-tunja-1886766955", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886749497", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H65" s="6" t="inlineStr"/>
@@ -3560,7 +3564,7 @@
     <row r="66" ht="22" customHeight="1">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>55fdaa0983ef9124</t>
+          <t>e760bcd88d90fbbe</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -3570,12 +3574,12 @@
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>Lider técnico con itil practice manager</t>
+          <t>Agente de mesa de ayuda</t>
         </is>
       </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
-          <t>Sinergy &amp; Lowells</t>
+          <t>SELCOMP INGENIERÍA SAS</t>
         </is>
       </c>
       <c r="E66" s="7" t="n">
@@ -3587,7 +3591,7 @@
         </is>
       </c>
       <c r="G66" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/lider-tecnico-con-itil-practice-manager-1886753953", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-de-mesa-de-ayuda-1886758623", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H66" s="6" t="inlineStr"/>
@@ -3606,7 +3610,7 @@
     <row r="67" ht="22" customHeight="1">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>a1ca7bc58cd48fad</t>
+          <t>86dcab5c5d802693</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
@@ -3616,12 +3620,12 @@
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de mesa de ayuda/mujeres contratacion inmediata</t>
+          <t>Analista mesa de ayuda para tunja</t>
         </is>
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Gestión de Seguridad Electrónica</t>
         </is>
       </c>
       <c r="E67" s="7" t="n">
@@ -3633,7 +3637,7 @@
         </is>
       </c>
       <c r="G67" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-mesa-de-ayuda-mujeres-contratacion-inmediata-1886770931", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-para-tunja-1886766955", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H67" s="6" t="inlineStr"/>
@@ -3652,7 +3656,7 @@
     <row r="68" ht="22" customHeight="1">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>e28aba5df8a2d3ae</t>
+          <t>55fdaa0983ef9124</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -3662,12 +3666,12 @@
       </c>
       <c r="C68" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de mesa de ayuda/mujeres contratacion inmediata</t>
+          <t>Lider técnico con itil practice manager</t>
         </is>
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Sinergy &amp; Lowells</t>
         </is>
       </c>
       <c r="E68" s="7" t="n">
@@ -3679,7 +3683,7 @@
         </is>
       </c>
       <c r="G68" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-mesa-de-ayuda-mujeres-contratacion-inmediata-1886769701", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/lider-tecnico-con-itil-practice-manager-1886753953", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H68" s="6" t="inlineStr"/>
@@ -3698,7 +3702,7 @@
     <row r="69" ht="22" customHeight="1">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>9326784c1a2726fb</t>
+          <t>a1ca7bc58cd48fad</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
@@ -3708,12 +3712,12 @@
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>Técnico de soporte y mesa de ayuda / medellín</t>
+          <t>Tecnico de mesa de ayuda/mujeres contratacion inmediata</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>Colsof S.A.S</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E69" s="7" t="n">
@@ -3725,7 +3729,7 @@
         </is>
       </c>
       <c r="G69" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-y-mesa-de-ayuda-medellin-1886738118", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-mesa-de-ayuda-mujeres-contratacion-inmediata-1886770931", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H69" s="6" t="inlineStr"/>
@@ -3744,7 +3748,7 @@
     <row r="70" ht="22" customHeight="1">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>b67dc9a9be4a1a6f</t>
+          <t>e28aba5df8a2d3ae</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -3754,7 +3758,7 @@
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>Service desk agent</t>
+          <t>Tecnico de mesa de ayuda/mujeres contratacion inmediata</t>
         </is>
       </c>
       <c r="D70" s="3" t="inlineStr">
@@ -3771,13 +3775,13 @@
         </is>
       </c>
       <c r="G70" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/service-desk-agent-soporte-tecnico-nivel-1-1886755112", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-mesa-de-ayuda-mujeres-contratacion-inmediata-1886769701", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H70" s="6" t="inlineStr"/>
       <c r="I70" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J70" s="2" t="inlineStr">
@@ -3790,7 +3794,7 @@
     <row r="71" ht="22" customHeight="1">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>9c65f710f43158b7</t>
+          <t>9326784c1a2726fb</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
@@ -3800,12 +3804,12 @@
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de instalaciones cableado de redes - licencia conte</t>
+          <t>Técnico de soporte y mesa de ayuda / medellín</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Colsof S.A.S</t>
         </is>
       </c>
       <c r="E71" s="7" t="n">
@@ -3817,7 +3821,7 @@
         </is>
       </c>
       <c r="G71" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-1886749397", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-y-mesa-de-ayuda-medellin-1886738118", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H71" s="6" t="inlineStr"/>
@@ -3836,22 +3840,22 @@
     <row r="72" ht="22" customHeight="1">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>a95003a0b1fc3d77</t>
+          <t>b67dc9a9be4a1a6f</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 15:41</t>
+          <t>2026-09-25 15:54</t>
         </is>
       </c>
       <c r="C72" s="3" t="inlineStr">
         <is>
-          <t>Técnico Soporte Nivel 1 Con ITIL</t>
+          <t>Service desk agent</t>
         </is>
       </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
-          <t>Importante empresa del sector de tecnología</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E72" s="7" t="n">
@@ -3863,17 +3867,13 @@
         </is>
       </c>
       <c r="G72" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-soporte-nivel-1-con-itil-en-bogota-dc-59E13FA64EF5843C61373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H72" s="6" t="inlineStr">
-        <is>
-          <t>$ 1.750.905,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/service-desk-agent-soporte-tecnico-nivel-1-1886755112", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H72" s="6" t="inlineStr"/>
       <c r="I72" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J72" s="2" t="inlineStr">
@@ -3886,22 +3886,22 @@
     <row r="73" ht="22" customHeight="1">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>96391fd564d83616</t>
+          <t>9c65f710f43158b7</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 15:41</t>
+          <t>2026-09-25 15:54</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de soporte IT con Moto</t>
+          <t>Tecnico de instalaciones cableado de redes - licencia conte</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>Los Hornitos</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E73" s="7" t="n">
@@ -3913,14 +3913,10 @@
         </is>
       </c>
       <c r="G73" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-it-con-moto-empresa-de-alimentos-en-bogota-dc-599938D46A6F4A8F61373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H73" s="6" t="inlineStr">
-        <is>
-          <t>$ 2.125.947,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-1886749397", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H73" s="6" t="inlineStr"/>
       <c r="I73" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -3936,7 +3932,7 @@
     <row r="74" ht="22" customHeight="1">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>b4f0b8c16fe5543e</t>
+          <t>a95003a0b1fc3d77</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
@@ -3946,12 +3942,12 @@
       </c>
       <c r="C74" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar de Sistemas</t>
+          <t>Técnico Soporte Nivel 1 Con ITIL</t>
         </is>
       </c>
       <c r="D74" s="3" t="inlineStr">
         <is>
-          <t>ELIS COLOMBIA SAS</t>
+          <t>Importante empresa del sector de tecnología</t>
         </is>
       </c>
       <c r="E74" s="7" t="n">
@@ -3963,12 +3959,12 @@
         </is>
       </c>
       <c r="G74" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-en-bogota-dc-48C2A0A3B050945661373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-soporte-nivel-1-con-itil-en-bogota-dc-59E13FA64EF5843C61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H74" s="6" t="inlineStr">
         <is>
-          <t>$ 2.000.000,00 (Mensual)</t>
+          <t>$ 1.750.905,00 (Mensual)</t>
         </is>
       </c>
       <c r="I74" s="3" t="inlineStr">
@@ -3986,7 +3982,7 @@
     <row r="75" ht="22" customHeight="1">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>7e4b4e4f136a5e31</t>
+          <t>96391fd564d83616</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
@@ -3996,12 +3992,12 @@
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>Agente Mesa de Ayuda</t>
+          <t>Tecnico de soporte IT con Moto</t>
         </is>
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>Importante empresa del sector</t>
+          <t>Los Hornitos</t>
         </is>
       </c>
       <c r="E75" s="7" t="n">
@@ -4013,12 +4009,12 @@
         </is>
       </c>
       <c r="G75" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-agente-mesa-de-ayuda-en-bogota-dc-E39FE355E02E578761373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-it-con-moto-empresa-de-alimentos-en-bogota-dc-599938D46A6F4A8F61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H75" s="6" t="inlineStr">
         <is>
-          <t>$ 2.000.000,00 (Mensual)</t>
+          <t>$ 2.125.947,00 (Mensual)</t>
         </is>
       </c>
       <c r="I75" s="3" t="inlineStr">
@@ -4036,7 +4032,7 @@
     <row r="76" ht="22" customHeight="1">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>0ef2cd7667600919</t>
+          <t>b4f0b8c16fe5543e</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
@@ -4046,12 +4042,12 @@
       </c>
       <c r="C76" s="3" t="inlineStr">
         <is>
-          <t>Técnico de Soporte TI Regional</t>
+          <t>Auxiliar de Sistemas</t>
         </is>
       </c>
       <c r="D76" s="3" t="inlineStr">
         <is>
-          <t>POLICOMP COLOMBIA SAS</t>
+          <t>ELIS COLOMBIA SAS</t>
         </is>
       </c>
       <c r="E76" s="7" t="n">
@@ -4063,10 +4059,14 @@
         </is>
       </c>
       <c r="G76" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-ti-regional-en-bogota-dc-ACF045C94E41CCDE61373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H76" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-en-bogota-dc-48C2A0A3B050945661373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H76" s="6" t="inlineStr">
+        <is>
+          <t>$ 2.000.000,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I76" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -4082,7 +4082,7 @@
     <row r="77" ht="22" customHeight="1">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>7784997bda962255</t>
+          <t>7e4b4e4f136a5e31</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
@@ -4092,12 +4092,12 @@
       </c>
       <c r="C77" s="3" t="inlineStr">
         <is>
-          <t>Técnico de Soporte TI On Demand/ por horas</t>
+          <t>Agente Mesa de Ayuda</t>
         </is>
       </c>
       <c r="D77" s="3" t="inlineStr">
         <is>
-          <t>POLICOMP COLOMBIA SAS</t>
+          <t>Importante empresa del sector</t>
         </is>
       </c>
       <c r="E77" s="7" t="n">
@@ -4109,10 +4109,14 @@
         </is>
       </c>
       <c r="G77" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-ti-on-demand-por-horas-en-bogota-dc-C2338FA0172D59A561373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H77" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-agente-mesa-de-ayuda-en-bogota-dc-E39FE355E02E578761373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H77" s="6" t="inlineStr">
+        <is>
+          <t>$ 2.000.000,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I77" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -4128,7 +4132,7 @@
     <row r="78" ht="22" customHeight="1">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>29d0fe2e42e678f7</t>
+          <t>0ef2cd7667600919</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -4138,12 +4142,12 @@
       </c>
       <c r="C78" s="3" t="inlineStr">
         <is>
-          <t>Técnico mantenimiento correctivo impresoras</t>
+          <t>Técnico de Soporte TI Regional</t>
         </is>
       </c>
       <c r="D78" s="3" t="inlineStr">
         <is>
-          <t>Multinacional de Impresión</t>
+          <t>POLICOMP COLOMBIA SAS</t>
         </is>
       </c>
       <c r="E78" s="7" t="n">
@@ -4155,14 +4159,10 @@
         </is>
       </c>
       <c r="G78" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-mantenimiento-correctivo-impresoras-en-guarne-BC0E775C0F25B27D61373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H78" s="6" t="inlineStr">
-        <is>
-          <t>$ 1.800.000,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-ti-regional-en-bogota-dc-ACF045C94E41CCDE61373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H78" s="6" t="inlineStr"/>
       <c r="I78" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -4178,22 +4178,22 @@
     <row r="79" ht="22" customHeight="1">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>98c9ab11f5b1eace</t>
+          <t>7784997bda962255</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 18:36</t>
+          <t>2026-09-27 15:41</t>
         </is>
       </c>
       <c r="C79" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar de sistemas</t>
+          <t>Técnico de Soporte TI On Demand/ por horas</t>
         </is>
       </c>
       <c r="D79" s="3" t="inlineStr">
         <is>
-          <t>Importante empresa del sector</t>
+          <t>POLICOMP COLOMBIA SAS</t>
         </is>
       </c>
       <c r="E79" s="7" t="n">
@@ -4205,14 +4205,10 @@
         </is>
       </c>
       <c r="G79" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-persona-con-discapacidad-remota-en-bogota-dc-5F2A812D014E159B61373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H79" s="6" t="inlineStr">
-        <is>
-          <t>$ 1.750.905,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-ti-on-demand-por-horas-en-bogota-dc-C2338FA0172D59A561373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H79" s="6" t="inlineStr"/>
       <c r="I79" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -4228,22 +4224,22 @@
     <row r="80" ht="22" customHeight="1">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>58133ddc4da9c68e</t>
+          <t>29d0fe2e42e678f7</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 18:36</t>
+          <t>2026-09-27 15:41</t>
         </is>
       </c>
       <c r="C80" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar de sistemas</t>
+          <t>Técnico mantenimiento correctivo impresoras</t>
         </is>
       </c>
       <c r="D80" s="3" t="inlineStr">
         <is>
-          <t>Importante empresa del sector</t>
+          <t>Multinacional de Impresión</t>
         </is>
       </c>
       <c r="E80" s="7" t="n">
@@ -4255,12 +4251,12 @@
         </is>
       </c>
       <c r="G80" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-persona-con-discapacidad-remota-en-bogota-dc-A00C07C9CC9A494B61373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-mantenimiento-correctivo-impresoras-en-guarne-BC0E775C0F25B27D61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H80" s="6" t="inlineStr">
         <is>
-          <t>$ 1.750.905,00 (Mensual)</t>
+          <t>$ 1.800.000,00 (Mensual)</t>
         </is>
       </c>
       <c r="I80" s="3" t="inlineStr">
@@ -4278,7 +4274,7 @@
     <row r="81" ht="22" customHeight="1">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>aed3420a4cfdc248</t>
+          <t>98c9ab11f5b1eace</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
@@ -4288,12 +4284,12 @@
       </c>
       <c r="C81" s="3" t="inlineStr">
         <is>
-          <t>Consultor de servicios/ mesa de ayuda nómina y erp software</t>
+          <t>Auxiliar de sistemas</t>
         </is>
       </c>
       <c r="D81" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Importante empresa del sector</t>
         </is>
       </c>
       <c r="E81" s="7" t="n">
@@ -4305,10 +4301,14 @@
         </is>
       </c>
       <c r="G81" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/consultor-de-servicios-mesa-de-ayuda-nomina-y-erp-software-inclusivo-1886716126", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H81" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-persona-con-discapacidad-remota-en-bogota-dc-5F2A812D014E159B61373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H81" s="6" t="inlineStr">
+        <is>
+          <t>$ 1.750.905,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I81" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -4324,12 +4324,12 @@
     <row r="82" ht="22" customHeight="1">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>2b8357189ff315da</t>
+          <t>58133ddc4da9c68e</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 17:00</t>
+          <t>2026-09-28 18:36</t>
         </is>
       </c>
       <c r="C82" s="3" t="inlineStr">
@@ -4339,7 +4339,7 @@
       </c>
       <c r="D82" s="3" t="inlineStr">
         <is>
-          <t>DAVITA SAS</t>
+          <t>Importante empresa del sector</t>
         </is>
       </c>
       <c r="E82" s="7" t="n">
@@ -4351,10 +4351,14 @@
         </is>
       </c>
       <c r="G82" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886758163", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H82" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-persona-con-discapacidad-remota-en-bogota-dc-A00C07C9CC9A494B61373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H82" s="6" t="inlineStr">
+        <is>
+          <t>$ 1.750.905,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I82" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -4370,17 +4374,17 @@
     <row r="83" ht="22" customHeight="1">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>a87934e7643b2c1c</t>
+          <t>aed3420a4cfdc248</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 17:00</t>
+          <t>2026-09-28 18:36</t>
         </is>
       </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de instalaciones cableado de redes - licencia conte cali</t>
+          <t>Consultor de servicios/ mesa de ayuda nómina y erp software</t>
         </is>
       </c>
       <c r="D83" s="3" t="inlineStr">
@@ -4397,7 +4401,7 @@
         </is>
       </c>
       <c r="G83" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-cali-1886759847", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/consultor-de-servicios-mesa-de-ayuda-nomina-y-erp-software-inclusivo-1886716126", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H83" s="6" t="inlineStr"/>
@@ -4416,7 +4420,7 @@
     <row r="84" ht="22" customHeight="1">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>10b4265e3ad11d81</t>
+          <t>2b8357189ff315da</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
@@ -4426,12 +4430,12 @@
       </c>
       <c r="C84" s="3" t="inlineStr">
         <is>
-          <t>Information Technology Help Desk Support</t>
+          <t>Auxiliar de sistemas</t>
         </is>
       </c>
       <c r="D84" s="3" t="inlineStr">
         <is>
-          <t>Booth</t>
+          <t>DAVITA SAS</t>
         </is>
       </c>
       <c r="E84" s="7" t="n">
@@ -4443,7 +4447,7 @@
         </is>
       </c>
       <c r="G84" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/information-technology-help-desk-support-at-booth-4471203962", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886758163", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H84" s="6" t="inlineStr"/>
@@ -4462,17 +4466,17 @@
     <row r="85" ht="22" customHeight="1">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>ff69ae85c8697a37</t>
+          <t>a87934e7643b2c1c</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 16:49</t>
+          <t>2026-09-29 17:00</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>Técnico de soporte ti - bogota</t>
+          <t>Tecnico de instalaciones cableado de redes - licencia conte cali</t>
         </is>
       </c>
       <c r="D85" s="3" t="inlineStr">
@@ -4489,7 +4493,7 @@
         </is>
       </c>
       <c r="G85" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-ti-bogota-1886774059", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-cali-1886759847", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H85" s="6" t="inlineStr"/>
@@ -4508,22 +4512,22 @@
     <row r="86" ht="22" customHeight="1">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>bbacf7d69ab9084e</t>
+          <t>10b4265e3ad11d81</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 16:49</t>
+          <t>2026-09-29 17:00</t>
         </is>
       </c>
       <c r="C86" s="3" t="inlineStr">
         <is>
-          <t>IT Helpdesk Analyst</t>
+          <t>Information Technology Help Desk Support</t>
         </is>
       </c>
       <c r="D86" s="3" t="inlineStr">
         <is>
-          <t>Power Digital Marketing</t>
+          <t>Booth</t>
         </is>
       </c>
       <c r="E86" s="7" t="n">
@@ -4535,7 +4539,7 @@
         </is>
       </c>
       <c r="G86" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/it-helpdesk-analyst-at-power-digital-marketing-4472601999", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/information-technology-help-desk-support-at-booth-4471203962", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H86" s="6" t="inlineStr"/>
@@ -4554,12 +4558,12 @@
     <row r="87" ht="22" customHeight="1">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>bb848f474ff4b611</t>
+          <t>ff69ae85c8697a37</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 17:26</t>
+          <t>2026-09-30 16:49</t>
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
@@ -4581,7 +4585,7 @@
         </is>
       </c>
       <c r="G87" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-ti-bogota-1886772292", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-ti-bogota-1886774059", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H87" s="6" t="inlineStr"/>
@@ -4600,22 +4604,22 @@
     <row r="88" ht="22" customHeight="1">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>b44a1c6cfb004ca8</t>
+          <t>bbacf7d69ab9084e</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 17:26</t>
+          <t>2026-09-30 16:49</t>
         </is>
       </c>
       <c r="C88" s="3" t="inlineStr">
         <is>
-          <t>Soporte ti nivel 2 - bogotá</t>
+          <t>IT Helpdesk Analyst</t>
         </is>
       </c>
       <c r="D88" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Power Digital Marketing</t>
         </is>
       </c>
       <c r="E88" s="7" t="n">
@@ -4627,7 +4631,7 @@
         </is>
       </c>
       <c r="G88" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/soporte-ti-nivel-2-bogota-1886774821", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/it-helpdesk-analyst-at-power-digital-marketing-4472601999", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H88" s="6" t="inlineStr"/>
@@ -4646,7 +4650,7 @@
     <row r="89" ht="22" customHeight="1">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>fb0ad2b513afb97c</t>
+          <t>bb848f474ff4b611</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
@@ -4656,12 +4660,12 @@
       </c>
       <c r="C89" s="3" t="inlineStr">
         <is>
-          <t>IT Help Desk Support Specialist</t>
+          <t>Técnico de soporte ti - bogota</t>
         </is>
       </c>
       <c r="D89" s="3" t="inlineStr">
         <is>
-          <t>Talento</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E89" s="7" t="n">
@@ -4673,7 +4677,7 @@
         </is>
       </c>
       <c r="G89" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/it-help-desk-support-specialist-tier-1-at-talento-4473960480", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-ti-bogota-1886772292", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H89" s="6" t="inlineStr"/>
@@ -4692,22 +4696,22 @@
     <row r="90" ht="22" customHeight="1">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>0b2067d6ae488f4c</t>
+          <t>b44a1c6cfb004ca8</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 16:39</t>
+          <t>2026-10-01 17:26</t>
         </is>
       </c>
       <c r="C90" s="3" t="inlineStr">
         <is>
-          <t>Help Desk Technician level 1</t>
+          <t>Soporte ti nivel 2 - bogotá</t>
         </is>
       </c>
       <c r="D90" s="3" t="inlineStr">
         <is>
-          <t>Solvo Global</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E90" s="7" t="n">
@@ -4719,7 +4723,7 @@
         </is>
       </c>
       <c r="G90" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/help-desk-technician-level-1-at-solvo-global-4472590892", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/soporte-ti-nivel-2-bogota-1886774821", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H90" s="6" t="inlineStr"/>
@@ -4738,22 +4742,22 @@
     <row r="91" ht="22" customHeight="1">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>07acc222a3ca2ef1</t>
+          <t>fb0ad2b513afb97c</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03 15:12</t>
+          <t>2026-10-01 17:26</t>
         </is>
       </c>
       <c r="C91" s="3" t="inlineStr">
         <is>
-          <t>Analista mesa de ayuda funza temporal 6 meses</t>
+          <t>IT Help Desk Support Specialist</t>
         </is>
       </c>
       <c r="D91" s="3" t="inlineStr">
         <is>
-          <t>Axity</t>
+          <t>Talento</t>
         </is>
       </c>
       <c r="E91" s="7" t="n">
@@ -4765,7 +4769,7 @@
         </is>
       </c>
       <c r="G91" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-funza-temporal-6-meses-1886774524", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/it-help-desk-support-specialist-tier-1-at-talento-4473960480", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H91" s="6" t="inlineStr"/>
@@ -4784,7 +4788,7 @@
     <row r="92" ht="22" customHeight="1">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>50c79dfbfd49f52d</t>
+          <t>0b2067d6ae488f4c</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
@@ -4794,16 +4798,16 @@
       </c>
       <c r="C92" s="3" t="inlineStr">
         <is>
-          <t>Analista de redes noc 1 telecomunicaciones.</t>
+          <t>Help Desk Technician level 1</t>
         </is>
       </c>
       <c r="D92" s="3" t="inlineStr">
         <is>
-          <t>MANPOWER</t>
+          <t>Solvo Global</t>
         </is>
       </c>
       <c r="E92" s="7" t="n">
-        <v>0.53</v>
+        <v>0.58</v>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
@@ -4811,13 +4815,13 @@
         </is>
       </c>
       <c r="G92" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-noc-1-telecomunicaciones-1886772075", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/help-desk-technician-level-1-at-solvo-global-4472590892", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H92" s="6" t="inlineStr"/>
       <c r="I92" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J92" s="2" t="inlineStr">
@@ -4830,26 +4834,26 @@
     <row r="93" ht="22" customHeight="1">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>0b0ae49f910109bb</t>
+          <t>07acc222a3ca2ef1</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 15:54</t>
+          <t>2026-10-03 15:12</t>
         </is>
       </c>
       <c r="C93" s="3" t="inlineStr">
         <is>
-          <t>Ejecutivo Técnico Arancel Junior</t>
+          <t>Analista mesa de ayuda funza temporal 6 meses</t>
         </is>
       </c>
       <c r="D93" s="3" t="inlineStr">
         <is>
-          <t>Importante Empresa de Logística y Comercio</t>
+          <t>Axity</t>
         </is>
       </c>
       <c r="E93" s="7" t="n">
-        <v>0.5</v>
+        <v>0.58</v>
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
@@ -4857,17 +4861,13 @@
         </is>
       </c>
       <c r="G93" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-547866639B487E0161373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H93" s="6" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-funza-temporal-6-meses-1886774524", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H93" s="6" t="inlineStr"/>
       <c r="I93" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J93" s="2" t="inlineStr">
@@ -4880,26 +4880,26 @@
     <row r="94" ht="22" customHeight="1">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>582a04b3c639bfa0</t>
+          <t>5ec0ea33876ba2b5</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 16:49</t>
+          <t>2026-10-05 19:45</t>
         </is>
       </c>
       <c r="C94" s="3" t="inlineStr">
         <is>
-          <t>Junior IT Support Specialist</t>
+          <t>Help desk analyst l1</t>
         </is>
       </c>
       <c r="D94" s="3" t="inlineStr">
         <is>
-          <t>Touch Support, Inc. &amp; SNF Back Office</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E94" s="7" t="n">
-        <v>0.5</v>
+        <v>0.58</v>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
@@ -4907,13 +4907,13 @@
         </is>
       </c>
       <c r="G94" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/junior-it-support-specialist-at-touch-support-inc-snf-back-office-4472187578", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/help-desk-analyst-l1-medellin-1886776156", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H94" s="6" t="inlineStr"/>
       <c r="I94" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J94" s="2" t="inlineStr">
@@ -4926,52 +4926,286 @@
     <row r="95" ht="22" customHeight="1">
       <c r="A95" s="2" t="inlineStr">
         <is>
+          <t>e8bdf2094d1c9817</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05 19:45</t>
+        </is>
+      </c>
+      <c r="C95" s="3" t="inlineStr">
+        <is>
+          <t>Administrador de herramienta de gestión de mesa de ayuda-</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="inlineStr">
+        <is>
+          <t>SELCOMP INGENIERÍA SAS</t>
+        </is>
+      </c>
+      <c r="E95" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G95" s="5">
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/administrador-de-herramienta-de-gestion-de-mesa-de-ayuda-1886776286", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H95" s="6" t="inlineStr"/>
+      <c r="I95" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J95" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K95" s="3" t="inlineStr"/>
+    </row>
+    <row r="96" ht="22" customHeight="1">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>6e9a077b42879470</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05 19:45</t>
+        </is>
+      </c>
+      <c r="C96" s="3" t="inlineStr">
+        <is>
+          <t>Analista de soporte de aplicaciones nivel 3</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="inlineStr">
+        <is>
+          <t>TALYCAP GLOBAL SAS</t>
+        </is>
+      </c>
+      <c r="E96" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G96" s="5">
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-soporte-de-aplicaciones-nivel-3-1886776104", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H96" s="6" t="inlineStr"/>
+      <c r="I96" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J96" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K96" s="3" t="inlineStr"/>
+    </row>
+    <row r="97" ht="22" customHeight="1">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>50c79dfbfd49f52d</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02 16:39</t>
+        </is>
+      </c>
+      <c r="C97" s="3" t="inlineStr">
+        <is>
+          <t>Analista de redes noc 1 telecomunicaciones.</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="inlineStr">
+        <is>
+          <t>MANPOWER</t>
+        </is>
+      </c>
+      <c r="E97" s="7" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="F97" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G97" s="5">
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-noc-1-telecomunicaciones-1886772075", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H97" s="6" t="inlineStr"/>
+      <c r="I97" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J97" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K97" s="3" t="inlineStr"/>
+    </row>
+    <row r="98" ht="22" customHeight="1">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>0b0ae49f910109bb</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25 15:54</t>
+        </is>
+      </c>
+      <c r="C98" s="3" t="inlineStr">
+        <is>
+          <t>Ejecutivo Técnico Arancel Junior</t>
+        </is>
+      </c>
+      <c r="D98" s="3" t="inlineStr">
+        <is>
+          <t>Importante Empresa de Logística y Comercio</t>
+        </is>
+      </c>
+      <c r="E98" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F98" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G98" s="5">
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-547866639B487E0161373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H98" s="6" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="I98" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J98" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K98" s="3" t="inlineStr"/>
+    </row>
+    <row r="99" ht="22" customHeight="1">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>582a04b3c639bfa0</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 16:49</t>
+        </is>
+      </c>
+      <c r="C99" s="3" t="inlineStr">
+        <is>
+          <t>Junior IT Support Specialist</t>
+        </is>
+      </c>
+      <c r="D99" s="3" t="inlineStr">
+        <is>
+          <t>Touch Support, Inc. &amp; SNF Back Office</t>
+        </is>
+      </c>
+      <c r="E99" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F99" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G99" s="5">
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/junior-it-support-specialist-at-touch-support-inc-snf-back-office-4472187578", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H99" s="6" t="inlineStr"/>
+      <c r="I99" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J99" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K99" s="3" t="inlineStr"/>
+    </row>
+    <row r="100" ht="22" customHeight="1">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
           <t>6e04c4d57d3fc3c7</t>
         </is>
       </c>
-      <c r="B95" s="2" t="inlineStr">
+      <c r="B100" s="2" t="inlineStr">
         <is>
           <t>2026-10-01 17:26</t>
         </is>
       </c>
-      <c r="C95" s="3" t="inlineStr">
+      <c r="C100" s="3" t="inlineStr">
         <is>
           <t>Ejecutivo Técnico Arancel Junior</t>
         </is>
       </c>
-      <c r="D95" s="3" t="inlineStr">
+      <c r="D100" s="3" t="inlineStr">
         <is>
           <t>Importante Empresa de Logística y Comercio</t>
         </is>
       </c>
-      <c r="E95" s="7" t="n">
+      <c r="E100" s="7" t="n">
         <v>0.5</v>
       </c>
-      <c r="F95" s="2" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
-      <c r="G95" s="5">
+      <c r="F100" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G100" s="5">
         <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-8444AB594560844161373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
-      <c r="H95" s="6" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
-      <c r="I95" s="3" t="inlineStr">
+      <c r="H100" s="6" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="I100" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
-      <c r="J95" s="2" t="inlineStr">
-        <is>
-          <t>Nueva</t>
-        </is>
-      </c>
-      <c r="K95" s="3" t="inlineStr"/>
+      <c r="J100" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K100" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
chore(tracker): actualizacion diaria de vacantes 2026-10-06
</commit_message>
<xml_diff>
--- a/output/profile_5_tecnico_sistemas_tracker.xlsx
+++ b/output/profile_5_tecnico_sistemas_tracker.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K100"/>
+  <dimension ref="A1:K101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -5018,26 +5018,26 @@
     <row r="97" ht="22" customHeight="1">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>50c79dfbfd49f52d</t>
+          <t>447afec244b20f9b</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 16:39</t>
+          <t>2026-10-06 17:12</t>
         </is>
       </c>
       <c r="C97" s="3" t="inlineStr">
         <is>
-          <t>Analista de redes noc 1 telecomunicaciones.</t>
+          <t>Técnico de soporte ti - bogota</t>
         </is>
       </c>
       <c r="D97" s="3" t="inlineStr">
         <is>
-          <t>MANPOWER</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E97" s="7" t="n">
-        <v>0.53</v>
+        <v>0.58</v>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
@@ -5045,13 +5045,13 @@
         </is>
       </c>
       <c r="G97" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-noc-1-telecomunicaciones-1886772075", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-ti-bogota-1886775990", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H97" s="6" t="inlineStr"/>
       <c r="I97" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J97" s="2" t="inlineStr">
@@ -5064,26 +5064,26 @@
     <row r="98" ht="22" customHeight="1">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>0b0ae49f910109bb</t>
+          <t>50c79dfbfd49f52d</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 15:54</t>
+          <t>2026-10-02 16:39</t>
         </is>
       </c>
       <c r="C98" s="3" t="inlineStr">
         <is>
-          <t>Ejecutivo Técnico Arancel Junior</t>
+          <t>Analista de redes noc 1 telecomunicaciones.</t>
         </is>
       </c>
       <c r="D98" s="3" t="inlineStr">
         <is>
-          <t>Importante Empresa de Logística y Comercio</t>
+          <t>MANPOWER</t>
         </is>
       </c>
       <c r="E98" s="7" t="n">
-        <v>0.5</v>
+        <v>0.53</v>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
@@ -5091,17 +5091,13 @@
         </is>
       </c>
       <c r="G98" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-547866639B487E0161373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H98" s="6" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-noc-1-telecomunicaciones-1886772075", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H98" s="6" t="inlineStr"/>
       <c r="I98" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J98" s="2" t="inlineStr">
@@ -5114,22 +5110,22 @@
     <row r="99" ht="22" customHeight="1">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>582a04b3c639bfa0</t>
+          <t>0b0ae49f910109bb</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 16:49</t>
+          <t>2026-09-25 15:54</t>
         </is>
       </c>
       <c r="C99" s="3" t="inlineStr">
         <is>
-          <t>Junior IT Support Specialist</t>
+          <t>Ejecutivo Técnico Arancel Junior</t>
         </is>
       </c>
       <c r="D99" s="3" t="inlineStr">
         <is>
-          <t>Touch Support, Inc. &amp; SNF Back Office</t>
+          <t>Importante Empresa de Logística y Comercio</t>
         </is>
       </c>
       <c r="E99" s="7" t="n">
@@ -5141,10 +5137,14 @@
         </is>
       </c>
       <c r="G99" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/junior-it-support-specialist-at-touch-support-inc-snf-back-office-4472187578", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H99" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-547866639B487E0161373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H99" s="6" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
       <c r="I99" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -5160,22 +5160,22 @@
     <row r="100" ht="22" customHeight="1">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>6e04c4d57d3fc3c7</t>
+          <t>582a04b3c639bfa0</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 17:26</t>
+          <t>2026-09-30 16:49</t>
         </is>
       </c>
       <c r="C100" s="3" t="inlineStr">
         <is>
-          <t>Ejecutivo Técnico Arancel Junior</t>
+          <t>Junior IT Support Specialist</t>
         </is>
       </c>
       <c r="D100" s="3" t="inlineStr">
         <is>
-          <t>Importante Empresa de Logística y Comercio</t>
+          <t>Touch Support, Inc. &amp; SNF Back Office</t>
         </is>
       </c>
       <c r="E100" s="7" t="n">
@@ -5187,25 +5187,71 @@
         </is>
       </c>
       <c r="G100" s="5">
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/junior-it-support-specialist-at-touch-support-inc-snf-back-office-4472187578", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H100" s="6" t="inlineStr"/>
+      <c r="I100" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J100" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K100" s="3" t="inlineStr"/>
+    </row>
+    <row r="101" ht="22" customHeight="1">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>6e04c4d57d3fc3c7</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01 17:26</t>
+        </is>
+      </c>
+      <c r="C101" s="3" t="inlineStr">
+        <is>
+          <t>Ejecutivo Técnico Arancel Junior</t>
+        </is>
+      </c>
+      <c r="D101" s="3" t="inlineStr">
+        <is>
+          <t>Importante Empresa de Logística y Comercio</t>
+        </is>
+      </c>
+      <c r="E101" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F101" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G101" s="5">
         <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-8444AB594560844161373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
-      <c r="H100" s="6" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
-      <c r="I100" s="3" t="inlineStr">
+      <c r="H101" s="6" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="I101" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
-      <c r="J100" s="2" t="inlineStr">
-        <is>
-          <t>Nueva</t>
-        </is>
-      </c>
-      <c r="K100" s="3" t="inlineStr"/>
+      <c r="J101" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K101" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
chore(tracker): actualizacion diaria de vacantes 2026-10-07
</commit_message>
<xml_diff>
--- a/output/profile_5_tecnico_sistemas_tracker.xlsx
+++ b/output/profile_5_tecnico_sistemas_tracker.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K101"/>
+  <dimension ref="A1:K107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3334,26 +3334,26 @@
     <row r="61" ht="22" customHeight="1">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>ae736277661dc78b</t>
+          <t>771146d163019cc0</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 15:23</t>
+          <t>2026-10-07 17:50</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>Analista de redes cisco</t>
+          <t>Soporte tecnico</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>ATCG DE COLOMBIA S.A.S</t>
-        </is>
-      </c>
-      <c r="E61" s="7" t="n">
-        <v>0.68</v>
+          <t>AGENCIA DE EMPLEO COLSUBSIDIO</t>
+        </is>
+      </c>
+      <c r="E61" s="4" t="n">
+        <v>0.73</v>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
@@ -3361,13 +3361,13 @@
         </is>
       </c>
       <c r="G61" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-cisco-1886760389", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/soporte-tecnico-1886776352", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H61" s="6" t="inlineStr"/>
       <c r="I61" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 68/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 73/100 - Alta Afinidad] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J61" s="2" t="inlineStr">
@@ -3380,7 +3380,7 @@
     <row r="62" ht="22" customHeight="1">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>e29676fac3409ad6</t>
+          <t>ae736277661dc78b</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -3390,12 +3390,12 @@
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>Analista de redes y telecomunicaciones - nivel 1</t>
+          <t>Analista de redes cisco</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>MANPOWER</t>
+          <t>ATCG DE COLOMBIA S.A.S</t>
         </is>
       </c>
       <c r="E62" s="7" t="n">
@@ -3407,7 +3407,7 @@
         </is>
       </c>
       <c r="G62" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-y-telecomunicaciones-nivel-1-1886760565", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-cisco-1886760389", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H62" s="6" t="inlineStr"/>
@@ -3426,26 +3426,26 @@
     <row r="63" ht="22" customHeight="1">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>73882c81e04abc7e</t>
+          <t>e29676fac3409ad6</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 19:45</t>
+          <t>2026-09-24 15:23</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>Soporte L1 Junior</t>
+          <t>Analista de redes y telecomunicaciones - nivel 1</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>Hublance</t>
+          <t>MANPOWER</t>
         </is>
       </c>
       <c r="E63" s="7" t="n">
-        <v>0.6</v>
+        <v>0.68</v>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
@@ -3453,13 +3453,13 @@
         </is>
       </c>
       <c r="G63" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/soporte-l1-junior-at-hublance-4475841269", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-y-telecomunicaciones-nivel-1-1886760565", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H63" s="6" t="inlineStr"/>
       <c r="I63" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 60/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 68/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J63" s="2" t="inlineStr">
@@ -3472,26 +3472,26 @@
     <row r="64" ht="22" customHeight="1">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>8d7f304ffb8625b5</t>
+          <t>baf000f38713dc11</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 15:54</t>
+          <t>2026-10-07 17:50</t>
         </is>
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar de sistemas</t>
+          <t>Helpdesk / Analista soporte TI / trilingüe</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Confidential</t>
         </is>
       </c>
       <c r="E64" s="7" t="n">
-        <v>0.58</v>
+        <v>0.66</v>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
@@ -3499,13 +3499,13 @@
         </is>
       </c>
       <c r="G64" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886751888", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/helpdesk-analista-soporte-ti-triling%C3%BCe-ingles-portugu%C3%A9s-at-confidential-4469673592", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H64" s="6" t="inlineStr"/>
       <c r="I64" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 66/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr">
@@ -3518,26 +3518,26 @@
     <row r="65" ht="22" customHeight="1">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>3b5b26f92a305c0c</t>
+          <t>73882c81e04abc7e</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 15:54</t>
+          <t>2026-10-05 19:45</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar de sistemas</t>
+          <t>Soporte L1 Junior</t>
         </is>
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Hublance</t>
         </is>
       </c>
       <c r="E65" s="7" t="n">
-        <v>0.58</v>
+        <v>0.6</v>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
@@ -3545,13 +3545,13 @@
         </is>
       </c>
       <c r="G65" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886749497", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/soporte-l1-junior-at-hublance-4475841269", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H65" s="6" t="inlineStr"/>
       <c r="I65" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 60/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J65" s="2" t="inlineStr">
@@ -3564,7 +3564,7 @@
     <row r="66" ht="22" customHeight="1">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>e760bcd88d90fbbe</t>
+          <t>8d7f304ffb8625b5</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -3574,12 +3574,12 @@
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>Agente de mesa de ayuda</t>
+          <t>Auxiliar de sistemas</t>
         </is>
       </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
-          <t>SELCOMP INGENIERÍA SAS</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E66" s="7" t="n">
@@ -3591,7 +3591,7 @@
         </is>
       </c>
       <c r="G66" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-de-mesa-de-ayuda-1886758623", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886751888", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H66" s="6" t="inlineStr"/>
@@ -3610,7 +3610,7 @@
     <row r="67" ht="22" customHeight="1">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>86dcab5c5d802693</t>
+          <t>3b5b26f92a305c0c</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
@@ -3620,12 +3620,12 @@
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>Analista mesa de ayuda para tunja</t>
+          <t>Auxiliar de sistemas</t>
         </is>
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>Gestión de Seguridad Electrónica</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E67" s="7" t="n">
@@ -3637,7 +3637,7 @@
         </is>
       </c>
       <c r="G67" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-para-tunja-1886766955", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886749497", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H67" s="6" t="inlineStr"/>
@@ -3656,7 +3656,7 @@
     <row r="68" ht="22" customHeight="1">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>55fdaa0983ef9124</t>
+          <t>e760bcd88d90fbbe</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -3666,12 +3666,12 @@
       </c>
       <c r="C68" s="3" t="inlineStr">
         <is>
-          <t>Lider técnico con itil practice manager</t>
+          <t>Agente de mesa de ayuda</t>
         </is>
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
-          <t>Sinergy &amp; Lowells</t>
+          <t>SELCOMP INGENIERÍA SAS</t>
         </is>
       </c>
       <c r="E68" s="7" t="n">
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="G68" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/lider-tecnico-con-itil-practice-manager-1886753953", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-de-mesa-de-ayuda-1886758623", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H68" s="6" t="inlineStr"/>
@@ -3702,7 +3702,7 @@
     <row r="69" ht="22" customHeight="1">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>a1ca7bc58cd48fad</t>
+          <t>86dcab5c5d802693</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
@@ -3712,12 +3712,12 @@
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de mesa de ayuda/mujeres contratacion inmediata</t>
+          <t>Analista mesa de ayuda para tunja</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Gestión de Seguridad Electrónica</t>
         </is>
       </c>
       <c r="E69" s="7" t="n">
@@ -3729,7 +3729,7 @@
         </is>
       </c>
       <c r="G69" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-mesa-de-ayuda-mujeres-contratacion-inmediata-1886770931", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-para-tunja-1886766955", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H69" s="6" t="inlineStr"/>
@@ -3748,7 +3748,7 @@
     <row r="70" ht="22" customHeight="1">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>e28aba5df8a2d3ae</t>
+          <t>55fdaa0983ef9124</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -3758,12 +3758,12 @@
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de mesa de ayuda/mujeres contratacion inmediata</t>
+          <t>Lider técnico con itil practice manager</t>
         </is>
       </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Sinergy &amp; Lowells</t>
         </is>
       </c>
       <c r="E70" s="7" t="n">
@@ -3775,7 +3775,7 @@
         </is>
       </c>
       <c r="G70" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-mesa-de-ayuda-mujeres-contratacion-inmediata-1886769701", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/lider-tecnico-con-itil-practice-manager-1886753953", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H70" s="6" t="inlineStr"/>
@@ -3794,7 +3794,7 @@
     <row r="71" ht="22" customHeight="1">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>9326784c1a2726fb</t>
+          <t>a1ca7bc58cd48fad</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
@@ -3804,12 +3804,12 @@
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>Técnico de soporte y mesa de ayuda / medellín</t>
+          <t>Tecnico de mesa de ayuda/mujeres contratacion inmediata</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>Colsof S.A.S</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E71" s="7" t="n">
@@ -3821,7 +3821,7 @@
         </is>
       </c>
       <c r="G71" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-y-mesa-de-ayuda-medellin-1886738118", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-mesa-de-ayuda-mujeres-contratacion-inmediata-1886770931", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H71" s="6" t="inlineStr"/>
@@ -3840,7 +3840,7 @@
     <row r="72" ht="22" customHeight="1">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>b67dc9a9be4a1a6f</t>
+          <t>e28aba5df8a2d3ae</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -3850,7 +3850,7 @@
       </c>
       <c r="C72" s="3" t="inlineStr">
         <is>
-          <t>Service desk agent</t>
+          <t>Tecnico de mesa de ayuda/mujeres contratacion inmediata</t>
         </is>
       </c>
       <c r="D72" s="3" t="inlineStr">
@@ -3867,13 +3867,13 @@
         </is>
       </c>
       <c r="G72" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/service-desk-agent-soporte-tecnico-nivel-1-1886755112", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-mesa-de-ayuda-mujeres-contratacion-inmediata-1886769701", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H72" s="6" t="inlineStr"/>
       <c r="I72" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J72" s="2" t="inlineStr">
@@ -3886,7 +3886,7 @@
     <row r="73" ht="22" customHeight="1">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>9c65f710f43158b7</t>
+          <t>9326784c1a2726fb</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
@@ -3896,12 +3896,12 @@
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de instalaciones cableado de redes - licencia conte</t>
+          <t>Técnico de soporte y mesa de ayuda / medellín</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Colsof S.A.S</t>
         </is>
       </c>
       <c r="E73" s="7" t="n">
@@ -3913,7 +3913,7 @@
         </is>
       </c>
       <c r="G73" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-1886749397", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-y-mesa-de-ayuda-medellin-1886738118", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H73" s="6" t="inlineStr"/>
@@ -3932,22 +3932,22 @@
     <row r="74" ht="22" customHeight="1">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>a95003a0b1fc3d77</t>
+          <t>b67dc9a9be4a1a6f</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 15:41</t>
+          <t>2026-09-25 15:54</t>
         </is>
       </c>
       <c r="C74" s="3" t="inlineStr">
         <is>
-          <t>Técnico Soporte Nivel 1 Con ITIL</t>
+          <t>Service desk agent</t>
         </is>
       </c>
       <c r="D74" s="3" t="inlineStr">
         <is>
-          <t>Importante empresa del sector de tecnología</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E74" s="7" t="n">
@@ -3959,17 +3959,13 @@
         </is>
       </c>
       <c r="G74" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-soporte-nivel-1-con-itil-en-bogota-dc-59E13FA64EF5843C61373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H74" s="6" t="inlineStr">
-        <is>
-          <t>$ 1.750.905,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/service-desk-agent-soporte-tecnico-nivel-1-1886755112", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H74" s="6" t="inlineStr"/>
       <c r="I74" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J74" s="2" t="inlineStr">
@@ -3982,22 +3978,22 @@
     <row r="75" ht="22" customHeight="1">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>96391fd564d83616</t>
+          <t>9c65f710f43158b7</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 15:41</t>
+          <t>2026-09-25 15:54</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de soporte IT con Moto</t>
+          <t>Tecnico de instalaciones cableado de redes - licencia conte</t>
         </is>
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>Los Hornitos</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E75" s="7" t="n">
@@ -4009,14 +4005,10 @@
         </is>
       </c>
       <c r="G75" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-it-con-moto-empresa-de-alimentos-en-bogota-dc-599938D46A6F4A8F61373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H75" s="6" t="inlineStr">
-        <is>
-          <t>$ 2.125.947,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-1886749397", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H75" s="6" t="inlineStr"/>
       <c r="I75" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -4032,7 +4024,7 @@
     <row r="76" ht="22" customHeight="1">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>b4f0b8c16fe5543e</t>
+          <t>a95003a0b1fc3d77</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
@@ -4042,12 +4034,12 @@
       </c>
       <c r="C76" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar de Sistemas</t>
+          <t>Técnico Soporte Nivel 1 Con ITIL</t>
         </is>
       </c>
       <c r="D76" s="3" t="inlineStr">
         <is>
-          <t>ELIS COLOMBIA SAS</t>
+          <t>Importante empresa del sector de tecnología</t>
         </is>
       </c>
       <c r="E76" s="7" t="n">
@@ -4059,12 +4051,12 @@
         </is>
       </c>
       <c r="G76" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-en-bogota-dc-48C2A0A3B050945661373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-soporte-nivel-1-con-itil-en-bogota-dc-59E13FA64EF5843C61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H76" s="6" t="inlineStr">
         <is>
-          <t>$ 2.000.000,00 (Mensual)</t>
+          <t>$ 1.750.905,00 (Mensual)</t>
         </is>
       </c>
       <c r="I76" s="3" t="inlineStr">
@@ -4082,7 +4074,7 @@
     <row r="77" ht="22" customHeight="1">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>7e4b4e4f136a5e31</t>
+          <t>96391fd564d83616</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
@@ -4092,12 +4084,12 @@
       </c>
       <c r="C77" s="3" t="inlineStr">
         <is>
-          <t>Agente Mesa de Ayuda</t>
+          <t>Tecnico de soporte IT con Moto</t>
         </is>
       </c>
       <c r="D77" s="3" t="inlineStr">
         <is>
-          <t>Importante empresa del sector</t>
+          <t>Los Hornitos</t>
         </is>
       </c>
       <c r="E77" s="7" t="n">
@@ -4109,12 +4101,12 @@
         </is>
       </c>
       <c r="G77" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-agente-mesa-de-ayuda-en-bogota-dc-E39FE355E02E578761373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-it-con-moto-empresa-de-alimentos-en-bogota-dc-599938D46A6F4A8F61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H77" s="6" t="inlineStr">
         <is>
-          <t>$ 2.000.000,00 (Mensual)</t>
+          <t>$ 2.125.947,00 (Mensual)</t>
         </is>
       </c>
       <c r="I77" s="3" t="inlineStr">
@@ -4132,7 +4124,7 @@
     <row r="78" ht="22" customHeight="1">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>0ef2cd7667600919</t>
+          <t>b4f0b8c16fe5543e</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -4142,12 +4134,12 @@
       </c>
       <c r="C78" s="3" t="inlineStr">
         <is>
-          <t>Técnico de Soporte TI Regional</t>
+          <t>Auxiliar de Sistemas</t>
         </is>
       </c>
       <c r="D78" s="3" t="inlineStr">
         <is>
-          <t>POLICOMP COLOMBIA SAS</t>
+          <t>ELIS COLOMBIA SAS</t>
         </is>
       </c>
       <c r="E78" s="7" t="n">
@@ -4159,10 +4151,14 @@
         </is>
       </c>
       <c r="G78" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-ti-regional-en-bogota-dc-ACF045C94E41CCDE61373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H78" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-en-bogota-dc-48C2A0A3B050945661373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H78" s="6" t="inlineStr">
+        <is>
+          <t>$ 2.000.000,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I78" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -4178,7 +4174,7 @@
     <row r="79" ht="22" customHeight="1">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>7784997bda962255</t>
+          <t>7e4b4e4f136a5e31</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
@@ -4188,12 +4184,12 @@
       </c>
       <c r="C79" s="3" t="inlineStr">
         <is>
-          <t>Técnico de Soporte TI On Demand/ por horas</t>
+          <t>Agente Mesa de Ayuda</t>
         </is>
       </c>
       <c r="D79" s="3" t="inlineStr">
         <is>
-          <t>POLICOMP COLOMBIA SAS</t>
+          <t>Importante empresa del sector</t>
         </is>
       </c>
       <c r="E79" s="7" t="n">
@@ -4205,10 +4201,14 @@
         </is>
       </c>
       <c r="G79" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-ti-on-demand-por-horas-en-bogota-dc-C2338FA0172D59A561373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H79" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-agente-mesa-de-ayuda-en-bogota-dc-E39FE355E02E578761373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H79" s="6" t="inlineStr">
+        <is>
+          <t>$ 2.000.000,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I79" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -4224,7 +4224,7 @@
     <row r="80" ht="22" customHeight="1">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>29d0fe2e42e678f7</t>
+          <t>0ef2cd7667600919</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
@@ -4234,12 +4234,12 @@
       </c>
       <c r="C80" s="3" t="inlineStr">
         <is>
-          <t>Técnico mantenimiento correctivo impresoras</t>
+          <t>Técnico de Soporte TI Regional</t>
         </is>
       </c>
       <c r="D80" s="3" t="inlineStr">
         <is>
-          <t>Multinacional de Impresión</t>
+          <t>POLICOMP COLOMBIA SAS</t>
         </is>
       </c>
       <c r="E80" s="7" t="n">
@@ -4251,14 +4251,10 @@
         </is>
       </c>
       <c r="G80" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-mantenimiento-correctivo-impresoras-en-guarne-BC0E775C0F25B27D61373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H80" s="6" t="inlineStr">
-        <is>
-          <t>$ 1.800.000,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-ti-regional-en-bogota-dc-ACF045C94E41CCDE61373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H80" s="6" t="inlineStr"/>
       <c r="I80" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -4274,22 +4270,22 @@
     <row r="81" ht="22" customHeight="1">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>98c9ab11f5b1eace</t>
+          <t>7784997bda962255</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 18:36</t>
+          <t>2026-09-27 15:41</t>
         </is>
       </c>
       <c r="C81" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar de sistemas</t>
+          <t>Técnico de Soporte TI On Demand/ por horas</t>
         </is>
       </c>
       <c r="D81" s="3" t="inlineStr">
         <is>
-          <t>Importante empresa del sector</t>
+          <t>POLICOMP COLOMBIA SAS</t>
         </is>
       </c>
       <c r="E81" s="7" t="n">
@@ -4301,14 +4297,10 @@
         </is>
       </c>
       <c r="G81" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-persona-con-discapacidad-remota-en-bogota-dc-5F2A812D014E159B61373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H81" s="6" t="inlineStr">
-        <is>
-          <t>$ 1.750.905,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-ti-on-demand-por-horas-en-bogota-dc-C2338FA0172D59A561373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H81" s="6" t="inlineStr"/>
       <c r="I81" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -4324,22 +4316,22 @@
     <row r="82" ht="22" customHeight="1">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>58133ddc4da9c68e</t>
+          <t>29d0fe2e42e678f7</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 18:36</t>
+          <t>2026-09-27 15:41</t>
         </is>
       </c>
       <c r="C82" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar de sistemas</t>
+          <t>Técnico mantenimiento correctivo impresoras</t>
         </is>
       </c>
       <c r="D82" s="3" t="inlineStr">
         <is>
-          <t>Importante empresa del sector</t>
+          <t>Multinacional de Impresión</t>
         </is>
       </c>
       <c r="E82" s="7" t="n">
@@ -4351,12 +4343,12 @@
         </is>
       </c>
       <c r="G82" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-persona-con-discapacidad-remota-en-bogota-dc-A00C07C9CC9A494B61373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-mantenimiento-correctivo-impresoras-en-guarne-BC0E775C0F25B27D61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H82" s="6" t="inlineStr">
         <is>
-          <t>$ 1.750.905,00 (Mensual)</t>
+          <t>$ 1.800.000,00 (Mensual)</t>
         </is>
       </c>
       <c r="I82" s="3" t="inlineStr">
@@ -4374,7 +4366,7 @@
     <row r="83" ht="22" customHeight="1">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>aed3420a4cfdc248</t>
+          <t>98c9ab11f5b1eace</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
@@ -4384,12 +4376,12 @@
       </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t>Consultor de servicios/ mesa de ayuda nómina y erp software</t>
+          <t>Auxiliar de sistemas</t>
         </is>
       </c>
       <c r="D83" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Importante empresa del sector</t>
         </is>
       </c>
       <c r="E83" s="7" t="n">
@@ -4401,10 +4393,14 @@
         </is>
       </c>
       <c r="G83" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/consultor-de-servicios-mesa-de-ayuda-nomina-y-erp-software-inclusivo-1886716126", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H83" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-persona-con-discapacidad-remota-en-bogota-dc-5F2A812D014E159B61373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H83" s="6" t="inlineStr">
+        <is>
+          <t>$ 1.750.905,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I83" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -4420,12 +4416,12 @@
     <row r="84" ht="22" customHeight="1">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>2b8357189ff315da</t>
+          <t>58133ddc4da9c68e</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 17:00</t>
+          <t>2026-09-28 18:36</t>
         </is>
       </c>
       <c r="C84" s="3" t="inlineStr">
@@ -4435,7 +4431,7 @@
       </c>
       <c r="D84" s="3" t="inlineStr">
         <is>
-          <t>DAVITA SAS</t>
+          <t>Importante empresa del sector</t>
         </is>
       </c>
       <c r="E84" s="7" t="n">
@@ -4447,10 +4443,14 @@
         </is>
       </c>
       <c r="G84" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886758163", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H84" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-persona-con-discapacidad-remota-en-bogota-dc-A00C07C9CC9A494B61373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H84" s="6" t="inlineStr">
+        <is>
+          <t>$ 1.750.905,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I84" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -4466,17 +4466,17 @@
     <row r="85" ht="22" customHeight="1">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>a87934e7643b2c1c</t>
+          <t>aed3420a4cfdc248</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 17:00</t>
+          <t>2026-09-28 18:36</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de instalaciones cableado de redes - licencia conte cali</t>
+          <t>Consultor de servicios/ mesa de ayuda nómina y erp software</t>
         </is>
       </c>
       <c r="D85" s="3" t="inlineStr">
@@ -4493,7 +4493,7 @@
         </is>
       </c>
       <c r="G85" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-cali-1886759847", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/consultor-de-servicios-mesa-de-ayuda-nomina-y-erp-software-inclusivo-1886716126", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H85" s="6" t="inlineStr"/>
@@ -4512,7 +4512,7 @@
     <row r="86" ht="22" customHeight="1">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>10b4265e3ad11d81</t>
+          <t>2b8357189ff315da</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
@@ -4522,12 +4522,12 @@
       </c>
       <c r="C86" s="3" t="inlineStr">
         <is>
-          <t>Information Technology Help Desk Support</t>
+          <t>Auxiliar de sistemas</t>
         </is>
       </c>
       <c r="D86" s="3" t="inlineStr">
         <is>
-          <t>Booth</t>
+          <t>DAVITA SAS</t>
         </is>
       </c>
       <c r="E86" s="7" t="n">
@@ -4539,7 +4539,7 @@
         </is>
       </c>
       <c r="G86" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/information-technology-help-desk-support-at-booth-4471203962", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886758163", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H86" s="6" t="inlineStr"/>
@@ -4558,17 +4558,17 @@
     <row r="87" ht="22" customHeight="1">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>ff69ae85c8697a37</t>
+          <t>a87934e7643b2c1c</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 16:49</t>
+          <t>2026-09-29 17:00</t>
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>Técnico de soporte ti - bogota</t>
+          <t>Tecnico de instalaciones cableado de redes - licencia conte cali</t>
         </is>
       </c>
       <c r="D87" s="3" t="inlineStr">
@@ -4585,7 +4585,7 @@
         </is>
       </c>
       <c r="G87" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-ti-bogota-1886774059", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-cali-1886759847", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H87" s="6" t="inlineStr"/>
@@ -4604,22 +4604,22 @@
     <row r="88" ht="22" customHeight="1">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>bbacf7d69ab9084e</t>
+          <t>10b4265e3ad11d81</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 16:49</t>
+          <t>2026-09-29 17:00</t>
         </is>
       </c>
       <c r="C88" s="3" t="inlineStr">
         <is>
-          <t>IT Helpdesk Analyst</t>
+          <t>Information Technology Help Desk Support</t>
         </is>
       </c>
       <c r="D88" s="3" t="inlineStr">
         <is>
-          <t>Power Digital Marketing</t>
+          <t>Booth</t>
         </is>
       </c>
       <c r="E88" s="7" t="n">
@@ -4631,7 +4631,7 @@
         </is>
       </c>
       <c r="G88" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/it-helpdesk-analyst-at-power-digital-marketing-4472601999", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/information-technology-help-desk-support-at-booth-4471203962", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H88" s="6" t="inlineStr"/>
@@ -4650,12 +4650,12 @@
     <row r="89" ht="22" customHeight="1">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>bb848f474ff4b611</t>
+          <t>ff69ae85c8697a37</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 17:26</t>
+          <t>2026-09-30 16:49</t>
         </is>
       </c>
       <c r="C89" s="3" t="inlineStr">
@@ -4677,7 +4677,7 @@
         </is>
       </c>
       <c r="G89" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-ti-bogota-1886772292", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-ti-bogota-1886774059", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H89" s="6" t="inlineStr"/>
@@ -4696,22 +4696,22 @@
     <row r="90" ht="22" customHeight="1">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>b44a1c6cfb004ca8</t>
+          <t>bbacf7d69ab9084e</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 17:26</t>
+          <t>2026-09-30 16:49</t>
         </is>
       </c>
       <c r="C90" s="3" t="inlineStr">
         <is>
-          <t>Soporte ti nivel 2 - bogotá</t>
+          <t>IT Helpdesk Analyst</t>
         </is>
       </c>
       <c r="D90" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Power Digital Marketing</t>
         </is>
       </c>
       <c r="E90" s="7" t="n">
@@ -4723,7 +4723,7 @@
         </is>
       </c>
       <c r="G90" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/soporte-ti-nivel-2-bogota-1886774821", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/it-helpdesk-analyst-at-power-digital-marketing-4472601999", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H90" s="6" t="inlineStr"/>
@@ -4742,7 +4742,7 @@
     <row r="91" ht="22" customHeight="1">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>fb0ad2b513afb97c</t>
+          <t>bb848f474ff4b611</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
@@ -4752,12 +4752,12 @@
       </c>
       <c r="C91" s="3" t="inlineStr">
         <is>
-          <t>IT Help Desk Support Specialist</t>
+          <t>Técnico de soporte ti - bogota</t>
         </is>
       </c>
       <c r="D91" s="3" t="inlineStr">
         <is>
-          <t>Talento</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E91" s="7" t="n">
@@ -4769,7 +4769,7 @@
         </is>
       </c>
       <c r="G91" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/it-help-desk-support-specialist-tier-1-at-talento-4473960480", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-ti-bogota-1886772292", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H91" s="6" t="inlineStr"/>
@@ -4788,22 +4788,22 @@
     <row r="92" ht="22" customHeight="1">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>0b2067d6ae488f4c</t>
+          <t>b44a1c6cfb004ca8</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 16:39</t>
+          <t>2026-10-01 17:26</t>
         </is>
       </c>
       <c r="C92" s="3" t="inlineStr">
         <is>
-          <t>Help Desk Technician level 1</t>
+          <t>Soporte ti nivel 2 - bogotá</t>
         </is>
       </c>
       <c r="D92" s="3" t="inlineStr">
         <is>
-          <t>Solvo Global</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E92" s="7" t="n">
@@ -4815,7 +4815,7 @@
         </is>
       </c>
       <c r="G92" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/help-desk-technician-level-1-at-solvo-global-4472590892", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/soporte-ti-nivel-2-bogota-1886774821", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H92" s="6" t="inlineStr"/>
@@ -4834,22 +4834,22 @@
     <row r="93" ht="22" customHeight="1">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>07acc222a3ca2ef1</t>
+          <t>fb0ad2b513afb97c</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03 15:12</t>
+          <t>2026-10-01 17:26</t>
         </is>
       </c>
       <c r="C93" s="3" t="inlineStr">
         <is>
-          <t>Analista mesa de ayuda funza temporal 6 meses</t>
+          <t>IT Help Desk Support Specialist</t>
         </is>
       </c>
       <c r="D93" s="3" t="inlineStr">
         <is>
-          <t>Axity</t>
+          <t>Talento</t>
         </is>
       </c>
       <c r="E93" s="7" t="n">
@@ -4861,7 +4861,7 @@
         </is>
       </c>
       <c r="G93" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-funza-temporal-6-meses-1886774524", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/it-help-desk-support-specialist-tier-1-at-talento-4473960480", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H93" s="6" t="inlineStr"/>
@@ -4880,22 +4880,22 @@
     <row r="94" ht="22" customHeight="1">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>5ec0ea33876ba2b5</t>
+          <t>0b2067d6ae488f4c</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 19:45</t>
+          <t>2026-10-02 16:39</t>
         </is>
       </c>
       <c r="C94" s="3" t="inlineStr">
         <is>
-          <t>Help desk analyst l1</t>
+          <t>Help Desk Technician level 1</t>
         </is>
       </c>
       <c r="D94" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Solvo Global</t>
         </is>
       </c>
       <c r="E94" s="7" t="n">
@@ -4907,7 +4907,7 @@
         </is>
       </c>
       <c r="G94" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/help-desk-analyst-l1-medellin-1886776156", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/help-desk-technician-level-1-at-solvo-global-4472590892", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H94" s="6" t="inlineStr"/>
@@ -4926,22 +4926,22 @@
     <row r="95" ht="22" customHeight="1">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>e8bdf2094d1c9817</t>
+          <t>07acc222a3ca2ef1</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 19:45</t>
+          <t>2026-10-03 15:12</t>
         </is>
       </c>
       <c r="C95" s="3" t="inlineStr">
         <is>
-          <t>Administrador de herramienta de gestión de mesa de ayuda-</t>
+          <t>Analista mesa de ayuda funza temporal 6 meses</t>
         </is>
       </c>
       <c r="D95" s="3" t="inlineStr">
         <is>
-          <t>SELCOMP INGENIERÍA SAS</t>
+          <t>Axity</t>
         </is>
       </c>
       <c r="E95" s="7" t="n">
@@ -4953,7 +4953,7 @@
         </is>
       </c>
       <c r="G95" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/administrador-de-herramienta-de-gestion-de-mesa-de-ayuda-1886776286", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-funza-temporal-6-meses-1886774524", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H95" s="6" t="inlineStr"/>
@@ -4972,7 +4972,7 @@
     <row r="96" ht="22" customHeight="1">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>6e9a077b42879470</t>
+          <t>5ec0ea33876ba2b5</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
@@ -4982,12 +4982,12 @@
       </c>
       <c r="C96" s="3" t="inlineStr">
         <is>
-          <t>Analista de soporte de aplicaciones nivel 3</t>
+          <t>Help desk analyst l1</t>
         </is>
       </c>
       <c r="D96" s="3" t="inlineStr">
         <is>
-          <t>TALYCAP GLOBAL SAS</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E96" s="7" t="n">
@@ -4999,7 +4999,7 @@
         </is>
       </c>
       <c r="G96" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-soporte-de-aplicaciones-nivel-3-1886776104", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/help-desk-analyst-l1-medellin-1886776156", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H96" s="6" t="inlineStr"/>
@@ -5018,22 +5018,22 @@
     <row r="97" ht="22" customHeight="1">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>447afec244b20f9b</t>
+          <t>e8bdf2094d1c9817</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06 17:12</t>
+          <t>2026-10-05 19:45</t>
         </is>
       </c>
       <c r="C97" s="3" t="inlineStr">
         <is>
-          <t>Técnico de soporte ti - bogota</t>
+          <t>Administrador de herramienta de gestión de mesa de ayuda-</t>
         </is>
       </c>
       <c r="D97" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>SELCOMP INGENIERÍA SAS</t>
         </is>
       </c>
       <c r="E97" s="7" t="n">
@@ -5045,7 +5045,7 @@
         </is>
       </c>
       <c r="G97" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-ti-bogota-1886775990", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/administrador-de-herramienta-de-gestion-de-mesa-de-ayuda-1886776286", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H97" s="6" t="inlineStr"/>
@@ -5064,26 +5064,26 @@
     <row r="98" ht="22" customHeight="1">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>50c79dfbfd49f52d</t>
+          <t>6e9a077b42879470</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 16:39</t>
+          <t>2026-10-05 19:45</t>
         </is>
       </c>
       <c r="C98" s="3" t="inlineStr">
         <is>
-          <t>Analista de redes noc 1 telecomunicaciones.</t>
+          <t>Analista de soporte de aplicaciones nivel 3</t>
         </is>
       </c>
       <c r="D98" s="3" t="inlineStr">
         <is>
-          <t>MANPOWER</t>
+          <t>TALYCAP GLOBAL SAS</t>
         </is>
       </c>
       <c r="E98" s="7" t="n">
-        <v>0.53</v>
+        <v>0.58</v>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
@@ -5091,13 +5091,13 @@
         </is>
       </c>
       <c r="G98" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-noc-1-telecomunicaciones-1886772075", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-soporte-de-aplicaciones-nivel-3-1886776104", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H98" s="6" t="inlineStr"/>
       <c r="I98" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J98" s="2" t="inlineStr">
@@ -5110,26 +5110,26 @@
     <row r="99" ht="22" customHeight="1">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>0b0ae49f910109bb</t>
+          <t>447afec244b20f9b</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 15:54</t>
+          <t>2026-10-06 17:12</t>
         </is>
       </c>
       <c r="C99" s="3" t="inlineStr">
         <is>
-          <t>Ejecutivo Técnico Arancel Junior</t>
+          <t>Técnico de soporte ti - bogota</t>
         </is>
       </c>
       <c r="D99" s="3" t="inlineStr">
         <is>
-          <t>Importante Empresa de Logística y Comercio</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E99" s="7" t="n">
-        <v>0.5</v>
+        <v>0.58</v>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
@@ -5137,17 +5137,13 @@
         </is>
       </c>
       <c r="G99" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-547866639B487E0161373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H99" s="6" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-ti-bogota-1886775990", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H99" s="6" t="inlineStr"/>
       <c r="I99" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J99" s="2" t="inlineStr">
@@ -5160,26 +5156,26 @@
     <row r="100" ht="22" customHeight="1">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>582a04b3c639bfa0</t>
+          <t>8f14c41f3b443ac0</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 16:49</t>
+          <t>2026-10-07 17:50</t>
         </is>
       </c>
       <c r="C100" s="3" t="inlineStr">
         <is>
-          <t>Junior IT Support Specialist</t>
+          <t>Soporte mesa de ayuda</t>
         </is>
       </c>
       <c r="D100" s="3" t="inlineStr">
         <is>
-          <t>Touch Support, Inc. &amp; SNF Back Office</t>
+          <t>MANPOWER</t>
         </is>
       </c>
       <c r="E100" s="7" t="n">
-        <v>0.5</v>
+        <v>0.58</v>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
@@ -5187,13 +5183,13 @@
         </is>
       </c>
       <c r="G100" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/junior-it-support-specialist-at-touch-support-inc-snf-back-office-4472187578", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/soporte-mesa-de-ayuda-vacaciones-1886776917", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H100" s="6" t="inlineStr"/>
       <c r="I100" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J100" s="2" t="inlineStr">
@@ -5206,52 +5202,332 @@
     <row r="101" ht="22" customHeight="1">
       <c r="A101" s="2" t="inlineStr">
         <is>
+          <t>b1a9e03967fff91e</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07 17:50</t>
+        </is>
+      </c>
+      <c r="C101" s="3" t="inlineStr">
+        <is>
+          <t>Tecnólogo de soporte pl - mesa de ayuda</t>
+        </is>
+      </c>
+      <c r="D101" s="3" t="inlineStr">
+        <is>
+          <t>Positivo S+</t>
+        </is>
+      </c>
+      <c r="E101" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F101" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G101" s="5">
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnologo-de-soporte-pl-mesa-de-ayuda-1886775546", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H101" s="6" t="inlineStr"/>
+      <c r="I101" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J101" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K101" s="3" t="inlineStr"/>
+    </row>
+    <row r="102" ht="22" customHeight="1">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>eb49981c97933d93</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07 17:50</t>
+        </is>
+      </c>
+      <c r="C102" s="3" t="inlineStr">
+        <is>
+          <t>Tecnico de instalaciones cableado de redes - licencia conte</t>
+        </is>
+      </c>
+      <c r="D102" s="3" t="inlineStr">
+        <is>
+          <t>Confidencial</t>
+        </is>
+      </c>
+      <c r="E102" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F102" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G102" s="5">
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-1886777333", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H102" s="6" t="inlineStr"/>
+      <c r="I102" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J102" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K102" s="3" t="inlineStr"/>
+    </row>
+    <row r="103" ht="22" customHeight="1">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>d39af22b6e937d28</t>
+        </is>
+      </c>
+      <c r="B103" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07 17:50</t>
+        </is>
+      </c>
+      <c r="C103" s="3" t="inlineStr">
+        <is>
+          <t>Analista Mesa de Ayuda Funza</t>
+        </is>
+      </c>
+      <c r="D103" s="3" t="inlineStr">
+        <is>
+          <t>axity</t>
+        </is>
+      </c>
+      <c r="E103" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F103" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G103" s="5">
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/analista-mesa-de-ayuda-funza-at-axity-4471985006", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H103" s="6" t="inlineStr"/>
+      <c r="I103" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J103" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K103" s="3" t="inlineStr"/>
+    </row>
+    <row r="104" ht="22" customHeight="1">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>50c79dfbfd49f52d</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02 16:39</t>
+        </is>
+      </c>
+      <c r="C104" s="3" t="inlineStr">
+        <is>
+          <t>Analista de redes noc 1 telecomunicaciones.</t>
+        </is>
+      </c>
+      <c r="D104" s="3" t="inlineStr">
+        <is>
+          <t>MANPOWER</t>
+        </is>
+      </c>
+      <c r="E104" s="7" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="F104" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G104" s="5">
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-noc-1-telecomunicaciones-1886772075", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H104" s="6" t="inlineStr"/>
+      <c r="I104" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J104" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K104" s="3" t="inlineStr"/>
+    </row>
+    <row r="105" ht="22" customHeight="1">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>0b0ae49f910109bb</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25 15:54</t>
+        </is>
+      </c>
+      <c r="C105" s="3" t="inlineStr">
+        <is>
+          <t>Ejecutivo Técnico Arancel Junior</t>
+        </is>
+      </c>
+      <c r="D105" s="3" t="inlineStr">
+        <is>
+          <t>Importante Empresa de Logística y Comercio</t>
+        </is>
+      </c>
+      <c r="E105" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F105" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G105" s="5">
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-547866639B487E0161373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H105" s="6" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="I105" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J105" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K105" s="3" t="inlineStr"/>
+    </row>
+    <row r="106" ht="22" customHeight="1">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>582a04b3c639bfa0</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 16:49</t>
+        </is>
+      </c>
+      <c r="C106" s="3" t="inlineStr">
+        <is>
+          <t>Junior IT Support Specialist</t>
+        </is>
+      </c>
+      <c r="D106" s="3" t="inlineStr">
+        <is>
+          <t>Touch Support, Inc. &amp; SNF Back Office</t>
+        </is>
+      </c>
+      <c r="E106" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F106" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G106" s="5">
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/junior-it-support-specialist-at-touch-support-inc-snf-back-office-4472187578", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H106" s="6" t="inlineStr"/>
+      <c r="I106" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J106" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K106" s="3" t="inlineStr"/>
+    </row>
+    <row r="107" ht="22" customHeight="1">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
           <t>6e04c4d57d3fc3c7</t>
         </is>
       </c>
-      <c r="B101" s="2" t="inlineStr">
+      <c r="B107" s="2" t="inlineStr">
         <is>
           <t>2026-10-01 17:26</t>
         </is>
       </c>
-      <c r="C101" s="3" t="inlineStr">
+      <c r="C107" s="3" t="inlineStr">
         <is>
           <t>Ejecutivo Técnico Arancel Junior</t>
         </is>
       </c>
-      <c r="D101" s="3" t="inlineStr">
+      <c r="D107" s="3" t="inlineStr">
         <is>
           <t>Importante Empresa de Logística y Comercio</t>
         </is>
       </c>
-      <c r="E101" s="7" t="n">
+      <c r="E107" s="7" t="n">
         <v>0.5</v>
       </c>
-      <c r="F101" s="2" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
-      <c r="G101" s="5">
+      <c r="F107" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G107" s="5">
         <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-8444AB594560844161373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
-      <c r="H101" s="6" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
-      <c r="I101" s="3" t="inlineStr">
+      <c r="H107" s="6" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="I107" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
-      <c r="J101" s="2" t="inlineStr">
-        <is>
-          <t>Nueva</t>
-        </is>
-      </c>
-      <c r="K101" s="3" t="inlineStr"/>
+      <c r="J107" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K107" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
chore(tracker): actualizacion diaria de vacantes 2026-10-08
</commit_message>
<xml_diff>
--- a/output/profile_5_tecnico_sistemas_tracker.xlsx
+++ b/output/profile_5_tecnico_sistemas_tracker.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K107"/>
+  <dimension ref="A1:K108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -5340,26 +5340,26 @@
     <row r="104" ht="22" customHeight="1">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>50c79dfbfd49f52d</t>
+          <t>0904912d51c5cd61</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 16:39</t>
+          <t>2026-10-08 17:52</t>
         </is>
       </c>
       <c r="C104" s="3" t="inlineStr">
         <is>
-          <t>Analista de redes noc 1 telecomunicaciones.</t>
+          <t>Analista mesa de ayuda</t>
         </is>
       </c>
       <c r="D104" s="3" t="inlineStr">
         <is>
-          <t>MANPOWER</t>
+          <t>Desarrollo de Sistemas y Servicios SAS</t>
         </is>
       </c>
       <c r="E104" s="7" t="n">
-        <v>0.53</v>
+        <v>0.58</v>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
@@ -5367,13 +5367,13 @@
         </is>
       </c>
       <c r="G104" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-noc-1-telecomunicaciones-1886772075", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-1886778032", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H104" s="6" t="inlineStr"/>
       <c r="I104" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J104" s="2" t="inlineStr">
@@ -5386,26 +5386,26 @@
     <row r="105" ht="22" customHeight="1">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>0b0ae49f910109bb</t>
+          <t>50c79dfbfd49f52d</t>
         </is>
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 15:54</t>
+          <t>2026-10-02 16:39</t>
         </is>
       </c>
       <c r="C105" s="3" t="inlineStr">
         <is>
-          <t>Ejecutivo Técnico Arancel Junior</t>
+          <t>Analista de redes noc 1 telecomunicaciones.</t>
         </is>
       </c>
       <c r="D105" s="3" t="inlineStr">
         <is>
-          <t>Importante Empresa de Logística y Comercio</t>
+          <t>MANPOWER</t>
         </is>
       </c>
       <c r="E105" s="7" t="n">
-        <v>0.5</v>
+        <v>0.53</v>
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
@@ -5413,17 +5413,13 @@
         </is>
       </c>
       <c r="G105" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-547866639B487E0161373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H105" s="6" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-noc-1-telecomunicaciones-1886772075", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H105" s="6" t="inlineStr"/>
       <c r="I105" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J105" s="2" t="inlineStr">
@@ -5436,22 +5432,22 @@
     <row r="106" ht="22" customHeight="1">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>582a04b3c639bfa0</t>
+          <t>0b0ae49f910109bb</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 16:49</t>
+          <t>2026-09-25 15:54</t>
         </is>
       </c>
       <c r="C106" s="3" t="inlineStr">
         <is>
-          <t>Junior IT Support Specialist</t>
+          <t>Ejecutivo Técnico Arancel Junior</t>
         </is>
       </c>
       <c r="D106" s="3" t="inlineStr">
         <is>
-          <t>Touch Support, Inc. &amp; SNF Back Office</t>
+          <t>Importante Empresa de Logística y Comercio</t>
         </is>
       </c>
       <c r="E106" s="7" t="n">
@@ -5463,10 +5459,14 @@
         </is>
       </c>
       <c r="G106" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/junior-it-support-specialist-at-touch-support-inc-snf-back-office-4472187578", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H106" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-547866639B487E0161373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H106" s="6" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
       <c r="I106" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -5482,22 +5482,22 @@
     <row r="107" ht="22" customHeight="1">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>6e04c4d57d3fc3c7</t>
+          <t>582a04b3c639bfa0</t>
         </is>
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 17:26</t>
+          <t>2026-09-30 16:49</t>
         </is>
       </c>
       <c r="C107" s="3" t="inlineStr">
         <is>
-          <t>Ejecutivo Técnico Arancel Junior</t>
+          <t>Junior IT Support Specialist</t>
         </is>
       </c>
       <c r="D107" s="3" t="inlineStr">
         <is>
-          <t>Importante Empresa de Logística y Comercio</t>
+          <t>Touch Support, Inc. &amp; SNF Back Office</t>
         </is>
       </c>
       <c r="E107" s="7" t="n">
@@ -5509,25 +5509,71 @@
         </is>
       </c>
       <c r="G107" s="5">
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/junior-it-support-specialist-at-touch-support-inc-snf-back-office-4472187578", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H107" s="6" t="inlineStr"/>
+      <c r="I107" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J107" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K107" s="3" t="inlineStr"/>
+    </row>
+    <row r="108" ht="22" customHeight="1">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>6e04c4d57d3fc3c7</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01 17:26</t>
+        </is>
+      </c>
+      <c r="C108" s="3" t="inlineStr">
+        <is>
+          <t>Ejecutivo Técnico Arancel Junior</t>
+        </is>
+      </c>
+      <c r="D108" s="3" t="inlineStr">
+        <is>
+          <t>Importante Empresa de Logística y Comercio</t>
+        </is>
+      </c>
+      <c r="E108" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F108" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G108" s="5">
         <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-8444AB594560844161373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
-      <c r="H107" s="6" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
-      <c r="I107" s="3" t="inlineStr">
+      <c r="H108" s="6" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="I108" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
-      <c r="J107" s="2" t="inlineStr">
-        <is>
-          <t>Nueva</t>
-        </is>
-      </c>
-      <c r="K107" s="3" t="inlineStr"/>
+      <c r="J108" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K108" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
chore(tracker): actualizacion diaria de vacantes 2026-10-09
</commit_message>
<xml_diff>
--- a/output/profile_5_tecnico_sistemas_tracker.xlsx
+++ b/output/profile_5_tecnico_sistemas_tracker.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -5386,26 +5386,26 @@
     <row r="105" ht="22" customHeight="1">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>50c79dfbfd49f52d</t>
+          <t>c665ada630270dce</t>
         </is>
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 16:39</t>
+          <t>2026-10-09 17:28</t>
         </is>
       </c>
       <c r="C105" s="3" t="inlineStr">
         <is>
-          <t>Analista de redes noc 1 telecomunicaciones.</t>
+          <t>Técnico(a) / tecnólogo(a) / profesional de telecomunicaciones - redes de fibra óptica</t>
         </is>
       </c>
       <c r="D105" s="3" t="inlineStr">
         <is>
-          <t>MANPOWER</t>
+          <t>JAHV MC GREGOR S.A.S</t>
         </is>
       </c>
       <c r="E105" s="7" t="n">
-        <v>0.53</v>
+        <v>0.58</v>
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
@@ -5413,13 +5413,13 @@
         </is>
       </c>
       <c r="G105" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-noc-1-telecomunicaciones-1886772075", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnicoa-tecnologoa-profesional-de-telecomunicaciones-redes-de-fibra-optica-1886768691", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H105" s="6" t="inlineStr"/>
       <c r="I105" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J105" s="2" t="inlineStr">
@@ -5432,26 +5432,26 @@
     <row r="106" ht="22" customHeight="1">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>0b0ae49f910109bb</t>
+          <t>4e5b3128aa7f8f9b</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 15:54</t>
+          <t>2026-10-09 17:28</t>
         </is>
       </c>
       <c r="C106" s="3" t="inlineStr">
         <is>
-          <t>Ejecutivo Técnico Arancel Junior</t>
+          <t>Gestor de servicios mesa de ayuda sap</t>
         </is>
       </c>
       <c r="D106" s="3" t="inlineStr">
         <is>
-          <t>Importante Empresa de Logística y Comercio</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E106" s="7" t="n">
-        <v>0.5</v>
+        <v>0.58</v>
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
@@ -5459,17 +5459,13 @@
         </is>
       </c>
       <c r="G106" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-547866639B487E0161373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H106" s="6" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/gestor-de-servicios-mesa-de-ayuda-sap-1886775732", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H106" s="6" t="inlineStr"/>
       <c r="I106" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J106" s="2" t="inlineStr">
@@ -5482,26 +5478,26 @@
     <row r="107" ht="22" customHeight="1">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>582a04b3c639bfa0</t>
+          <t>1c92f7ef9b7af696</t>
         </is>
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 16:49</t>
+          <t>2026-10-09 17:28</t>
         </is>
       </c>
       <c r="C107" s="3" t="inlineStr">
         <is>
-          <t>Junior IT Support Specialist</t>
+          <t>Agente de mesa de ayuda nivel 1</t>
         </is>
       </c>
       <c r="D107" s="3" t="inlineStr">
         <is>
-          <t>Touch Support, Inc. &amp; SNF Back Office</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E107" s="7" t="n">
-        <v>0.5</v>
+        <v>0.58</v>
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
@@ -5509,13 +5505,13 @@
         </is>
       </c>
       <c r="G107" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/junior-it-support-specialist-at-touch-support-inc-snf-back-office-4472187578", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-de-mesa-de-ayuda-nivel-1-1886778506", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H107" s="6" t="inlineStr"/>
       <c r="I107" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J107" s="2" t="inlineStr">
@@ -5528,52 +5524,194 @@
     <row r="108" ht="22" customHeight="1">
       <c r="A108" s="2" t="inlineStr">
         <is>
+          <t>50c79dfbfd49f52d</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02 16:39</t>
+        </is>
+      </c>
+      <c r="C108" s="3" t="inlineStr">
+        <is>
+          <t>Analista de redes noc 1 telecomunicaciones.</t>
+        </is>
+      </c>
+      <c r="D108" s="3" t="inlineStr">
+        <is>
+          <t>MANPOWER</t>
+        </is>
+      </c>
+      <c r="E108" s="7" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="F108" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G108" s="5">
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-noc-1-telecomunicaciones-1886772075", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H108" s="6" t="inlineStr"/>
+      <c r="I108" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J108" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K108" s="3" t="inlineStr"/>
+    </row>
+    <row r="109" ht="22" customHeight="1">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>0b0ae49f910109bb</t>
+        </is>
+      </c>
+      <c r="B109" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25 15:54</t>
+        </is>
+      </c>
+      <c r="C109" s="3" t="inlineStr">
+        <is>
+          <t>Ejecutivo Técnico Arancel Junior</t>
+        </is>
+      </c>
+      <c r="D109" s="3" t="inlineStr">
+        <is>
+          <t>Importante Empresa de Logística y Comercio</t>
+        </is>
+      </c>
+      <c r="E109" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F109" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G109" s="5">
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-547866639B487E0161373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H109" s="6" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="I109" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J109" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K109" s="3" t="inlineStr"/>
+    </row>
+    <row r="110" ht="22" customHeight="1">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>582a04b3c639bfa0</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 16:49</t>
+        </is>
+      </c>
+      <c r="C110" s="3" t="inlineStr">
+        <is>
+          <t>Junior IT Support Specialist</t>
+        </is>
+      </c>
+      <c r="D110" s="3" t="inlineStr">
+        <is>
+          <t>Touch Support, Inc. &amp; SNF Back Office</t>
+        </is>
+      </c>
+      <c r="E110" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F110" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G110" s="5">
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/junior-it-support-specialist-at-touch-support-inc-snf-back-office-4472187578", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H110" s="6" t="inlineStr"/>
+      <c r="I110" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J110" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K110" s="3" t="inlineStr"/>
+    </row>
+    <row r="111" ht="22" customHeight="1">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
           <t>6e04c4d57d3fc3c7</t>
         </is>
       </c>
-      <c r="B108" s="2" t="inlineStr">
+      <c r="B111" s="2" t="inlineStr">
         <is>
           <t>2026-10-01 17:26</t>
         </is>
       </c>
-      <c r="C108" s="3" t="inlineStr">
+      <c r="C111" s="3" t="inlineStr">
         <is>
           <t>Ejecutivo Técnico Arancel Junior</t>
         </is>
       </c>
-      <c r="D108" s="3" t="inlineStr">
+      <c r="D111" s="3" t="inlineStr">
         <is>
           <t>Importante Empresa de Logística y Comercio</t>
         </is>
       </c>
-      <c r="E108" s="7" t="n">
+      <c r="E111" s="7" t="n">
         <v>0.5</v>
       </c>
-      <c r="F108" s="2" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
-      <c r="G108" s="5">
+      <c r="F111" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G111" s="5">
         <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-8444AB594560844161373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
-      <c r="H108" s="6" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
-      <c r="I108" s="3" t="inlineStr">
+      <c r="H111" s="6" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="I111" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
-      <c r="J108" s="2" t="inlineStr">
-        <is>
-          <t>Nueva</t>
-        </is>
-      </c>
-      <c r="K108" s="3" t="inlineStr"/>
+      <c r="J111" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K111" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
chore(tracker): actualizacion diaria de vacantes 2026-10-10
</commit_message>
<xml_diff>
--- a/output/profile_5_tecnico_sistemas_tracker.xlsx
+++ b/output/profile_5_tecnico_sistemas_tracker.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K111"/>
+  <dimension ref="A1:K112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -5524,26 +5524,26 @@
     <row r="108" ht="22" customHeight="1">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>50c79dfbfd49f52d</t>
+          <t>718ceee355d457ea</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 16:39</t>
+          <t>2026-10-10 16:16</t>
         </is>
       </c>
       <c r="C108" s="3" t="inlineStr">
         <is>
-          <t>Analista de redes noc 1 telecomunicaciones.</t>
+          <t>IT Help Desk Support</t>
         </is>
       </c>
       <c r="D108" s="3" t="inlineStr">
         <is>
-          <t>MANPOWER</t>
+          <t>Booth</t>
         </is>
       </c>
       <c r="E108" s="7" t="n">
-        <v>0.53</v>
+        <v>0.58</v>
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
@@ -5551,13 +5551,13 @@
         </is>
       </c>
       <c r="G108" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-noc-1-telecomunicaciones-1886772075", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/it-help-desk-support-at-booth-4471203962", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H108" s="6" t="inlineStr"/>
       <c r="I108" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J108" s="2" t="inlineStr">
@@ -5570,26 +5570,26 @@
     <row r="109" ht="22" customHeight="1">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>0b0ae49f910109bb</t>
+          <t>50c79dfbfd49f52d</t>
         </is>
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 15:54</t>
+          <t>2026-10-02 16:39</t>
         </is>
       </c>
       <c r="C109" s="3" t="inlineStr">
         <is>
-          <t>Ejecutivo Técnico Arancel Junior</t>
+          <t>Analista de redes noc 1 telecomunicaciones.</t>
         </is>
       </c>
       <c r="D109" s="3" t="inlineStr">
         <is>
-          <t>Importante Empresa de Logística y Comercio</t>
+          <t>MANPOWER</t>
         </is>
       </c>
       <c r="E109" s="7" t="n">
-        <v>0.5</v>
+        <v>0.53</v>
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
@@ -5597,17 +5597,13 @@
         </is>
       </c>
       <c r="G109" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-547866639B487E0161373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H109" s="6" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-noc-1-telecomunicaciones-1886772075", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H109" s="6" t="inlineStr"/>
       <c r="I109" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J109" s="2" t="inlineStr">
@@ -5620,22 +5616,22 @@
     <row r="110" ht="22" customHeight="1">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>582a04b3c639bfa0</t>
+          <t>0b0ae49f910109bb</t>
         </is>
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 16:49</t>
+          <t>2026-09-25 15:54</t>
         </is>
       </c>
       <c r="C110" s="3" t="inlineStr">
         <is>
-          <t>Junior IT Support Specialist</t>
+          <t>Ejecutivo Técnico Arancel Junior</t>
         </is>
       </c>
       <c r="D110" s="3" t="inlineStr">
         <is>
-          <t>Touch Support, Inc. &amp; SNF Back Office</t>
+          <t>Importante Empresa de Logística y Comercio</t>
         </is>
       </c>
       <c r="E110" s="7" t="n">
@@ -5647,10 +5643,14 @@
         </is>
       </c>
       <c r="G110" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/junior-it-support-specialist-at-touch-support-inc-snf-back-office-4472187578", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H110" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-547866639B487E0161373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H110" s="6" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
       <c r="I110" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -5666,22 +5666,22 @@
     <row r="111" ht="22" customHeight="1">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>6e04c4d57d3fc3c7</t>
+          <t>582a04b3c639bfa0</t>
         </is>
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 17:26</t>
+          <t>2026-09-30 16:49</t>
         </is>
       </c>
       <c r="C111" s="3" t="inlineStr">
         <is>
-          <t>Ejecutivo Técnico Arancel Junior</t>
+          <t>Junior IT Support Specialist</t>
         </is>
       </c>
       <c r="D111" s="3" t="inlineStr">
         <is>
-          <t>Importante Empresa de Logística y Comercio</t>
+          <t>Touch Support, Inc. &amp; SNF Back Office</t>
         </is>
       </c>
       <c r="E111" s="7" t="n">
@@ -5693,25 +5693,71 @@
         </is>
       </c>
       <c r="G111" s="5">
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/junior-it-support-specialist-at-touch-support-inc-snf-back-office-4472187578", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H111" s="6" t="inlineStr"/>
+      <c r="I111" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J111" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K111" s="3" t="inlineStr"/>
+    </row>
+    <row r="112" ht="22" customHeight="1">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>6e04c4d57d3fc3c7</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01 17:26</t>
+        </is>
+      </c>
+      <c r="C112" s="3" t="inlineStr">
+        <is>
+          <t>Ejecutivo Técnico Arancel Junior</t>
+        </is>
+      </c>
+      <c r="D112" s="3" t="inlineStr">
+        <is>
+          <t>Importante Empresa de Logística y Comercio</t>
+        </is>
+      </c>
+      <c r="E112" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F112" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G112" s="5">
         <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-8444AB594560844161373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
-      <c r="H111" s="6" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
-      <c r="I111" s="3" t="inlineStr">
+      <c r="H112" s="6" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="I112" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
-      <c r="J111" s="2" t="inlineStr">
-        <is>
-          <t>Nueva</t>
-        </is>
-      </c>
-      <c r="K111" s="3" t="inlineStr"/>
+      <c r="J112" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K112" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
chore(tracker): actualizacion diaria de vacantes 2026-10-12
</commit_message>
<xml_diff>
--- a/output/profile_5_tecnico_sistemas_tracker.xlsx
+++ b/output/profile_5_tecnico_sistemas_tracker.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K112"/>
+  <dimension ref="A1:K114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3380,26 +3380,26 @@
     <row r="62" ht="22" customHeight="1">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>ae736277661dc78b</t>
+          <t>625a5609a531ab02</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 15:23</t>
+          <t>2026-10-12 20:17</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>Analista de redes cisco</t>
+          <t>Soporte técnico</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>ATCG DE COLOMBIA S.A.S</t>
-        </is>
-      </c>
-      <c r="E62" s="7" t="n">
-        <v>0.68</v>
+          <t>Méderi</t>
+        </is>
+      </c>
+      <c r="E62" s="4" t="n">
+        <v>0.73</v>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
@@ -3407,13 +3407,13 @@
         </is>
       </c>
       <c r="G62" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-cisco-1886760389", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/soporte-tecnico-1886774861", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H62" s="6" t="inlineStr"/>
       <c r="I62" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 68/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 73/100 - Alta Afinidad] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J62" s="2" t="inlineStr">
@@ -3426,7 +3426,7 @@
     <row r="63" ht="22" customHeight="1">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>e29676fac3409ad6</t>
+          <t>ae736277661dc78b</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
@@ -3436,12 +3436,12 @@
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>Analista de redes y telecomunicaciones - nivel 1</t>
+          <t>Analista de redes cisco</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>MANPOWER</t>
+          <t>ATCG DE COLOMBIA S.A.S</t>
         </is>
       </c>
       <c r="E63" s="7" t="n">
@@ -3453,7 +3453,7 @@
         </is>
       </c>
       <c r="G63" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-y-telecomunicaciones-nivel-1-1886760565", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-cisco-1886760389", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H63" s="6" t="inlineStr"/>
@@ -3472,26 +3472,26 @@
     <row r="64" ht="22" customHeight="1">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>baf000f38713dc11</t>
+          <t>e29676fac3409ad6</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07 17:50</t>
+          <t>2026-09-24 15:23</t>
         </is>
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>Helpdesk / Analista soporte TI / trilingüe</t>
+          <t>Analista de redes y telecomunicaciones - nivel 1</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t>Confidential</t>
+          <t>MANPOWER</t>
         </is>
       </c>
       <c r="E64" s="7" t="n">
-        <v>0.66</v>
+        <v>0.68</v>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
@@ -3499,13 +3499,13 @@
         </is>
       </c>
       <c r="G64" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/helpdesk-analista-soporte-ti-triling%C3%BCe-ingles-portugu%C3%A9s-at-confidential-4469673592", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-y-telecomunicaciones-nivel-1-1886760565", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H64" s="6" t="inlineStr"/>
       <c r="I64" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 66/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 68/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr">
@@ -3518,26 +3518,26 @@
     <row r="65" ht="22" customHeight="1">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>73882c81e04abc7e</t>
+          <t>baf000f38713dc11</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 19:45</t>
+          <t>2026-10-07 17:50</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>Soporte L1 Junior</t>
+          <t>Helpdesk / Analista soporte TI / trilingüe</t>
         </is>
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>Hublance</t>
+          <t>Confidential</t>
         </is>
       </c>
       <c r="E65" s="7" t="n">
-        <v>0.6</v>
+        <v>0.66</v>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
@@ -3545,13 +3545,13 @@
         </is>
       </c>
       <c r="G65" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/soporte-l1-junior-at-hublance-4475841269", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/helpdesk-analista-soporte-ti-triling%C3%BCe-ingles-portugu%C3%A9s-at-confidential-4469673592", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H65" s="6" t="inlineStr"/>
       <c r="I65" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 60/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 66/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J65" s="2" t="inlineStr">
@@ -3564,26 +3564,26 @@
     <row r="66" ht="22" customHeight="1">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>8d7f304ffb8625b5</t>
+          <t>73882c81e04abc7e</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 15:54</t>
+          <t>2026-10-05 19:45</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar de sistemas</t>
+          <t>Soporte L1 Junior</t>
         </is>
       </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Hublance</t>
         </is>
       </c>
       <c r="E66" s="7" t="n">
-        <v>0.58</v>
+        <v>0.6</v>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
@@ -3591,13 +3591,13 @@
         </is>
       </c>
       <c r="G66" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886751888", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/soporte-l1-junior-at-hublance-4475841269", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H66" s="6" t="inlineStr"/>
       <c r="I66" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 60/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J66" s="2" t="inlineStr">
@@ -3610,7 +3610,7 @@
     <row r="67" ht="22" customHeight="1">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>3b5b26f92a305c0c</t>
+          <t>8d7f304ffb8625b5</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
@@ -3637,7 +3637,7 @@
         </is>
       </c>
       <c r="G67" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886749497", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886751888", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H67" s="6" t="inlineStr"/>
@@ -3656,7 +3656,7 @@
     <row r="68" ht="22" customHeight="1">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>e760bcd88d90fbbe</t>
+          <t>3b5b26f92a305c0c</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -3666,12 +3666,12 @@
       </c>
       <c r="C68" s="3" t="inlineStr">
         <is>
-          <t>Agente de mesa de ayuda</t>
+          <t>Auxiliar de sistemas</t>
         </is>
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
-          <t>SELCOMP INGENIERÍA SAS</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E68" s="7" t="n">
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="G68" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-de-mesa-de-ayuda-1886758623", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886749497", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H68" s="6" t="inlineStr"/>
@@ -3702,7 +3702,7 @@
     <row r="69" ht="22" customHeight="1">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>86dcab5c5d802693</t>
+          <t>e760bcd88d90fbbe</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
@@ -3712,12 +3712,12 @@
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>Analista mesa de ayuda para tunja</t>
+          <t>Agente de mesa de ayuda</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>Gestión de Seguridad Electrónica</t>
+          <t>SELCOMP INGENIERÍA SAS</t>
         </is>
       </c>
       <c r="E69" s="7" t="n">
@@ -3729,7 +3729,7 @@
         </is>
       </c>
       <c r="G69" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-para-tunja-1886766955", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-de-mesa-de-ayuda-1886758623", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H69" s="6" t="inlineStr"/>
@@ -3748,7 +3748,7 @@
     <row r="70" ht="22" customHeight="1">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>55fdaa0983ef9124</t>
+          <t>86dcab5c5d802693</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -3758,12 +3758,12 @@
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>Lider técnico con itil practice manager</t>
+          <t>Analista mesa de ayuda para tunja</t>
         </is>
       </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
-          <t>Sinergy &amp; Lowells</t>
+          <t>Gestión de Seguridad Electrónica</t>
         </is>
       </c>
       <c r="E70" s="7" t="n">
@@ -3775,7 +3775,7 @@
         </is>
       </c>
       <c r="G70" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/lider-tecnico-con-itil-practice-manager-1886753953", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-para-tunja-1886766955", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H70" s="6" t="inlineStr"/>
@@ -3794,7 +3794,7 @@
     <row r="71" ht="22" customHeight="1">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>a1ca7bc58cd48fad</t>
+          <t>55fdaa0983ef9124</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
@@ -3804,12 +3804,12 @@
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de mesa de ayuda/mujeres contratacion inmediata</t>
+          <t>Lider técnico con itil practice manager</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Sinergy &amp; Lowells</t>
         </is>
       </c>
       <c r="E71" s="7" t="n">
@@ -3821,7 +3821,7 @@
         </is>
       </c>
       <c r="G71" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-mesa-de-ayuda-mujeres-contratacion-inmediata-1886770931", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/lider-tecnico-con-itil-practice-manager-1886753953", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H71" s="6" t="inlineStr"/>
@@ -3840,7 +3840,7 @@
     <row r="72" ht="22" customHeight="1">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>e28aba5df8a2d3ae</t>
+          <t>a1ca7bc58cd48fad</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -3867,7 +3867,7 @@
         </is>
       </c>
       <c r="G72" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-mesa-de-ayuda-mujeres-contratacion-inmediata-1886769701", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-mesa-de-ayuda-mujeres-contratacion-inmediata-1886770931", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H72" s="6" t="inlineStr"/>
@@ -3886,7 +3886,7 @@
     <row r="73" ht="22" customHeight="1">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>9326784c1a2726fb</t>
+          <t>e28aba5df8a2d3ae</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
@@ -3896,12 +3896,12 @@
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>Técnico de soporte y mesa de ayuda / medellín</t>
+          <t>Tecnico de mesa de ayuda/mujeres contratacion inmediata</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>Colsof S.A.S</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E73" s="7" t="n">
@@ -3913,7 +3913,7 @@
         </is>
       </c>
       <c r="G73" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-y-mesa-de-ayuda-medellin-1886738118", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-mesa-de-ayuda-mujeres-contratacion-inmediata-1886769701", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H73" s="6" t="inlineStr"/>
@@ -3932,7 +3932,7 @@
     <row r="74" ht="22" customHeight="1">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>b67dc9a9be4a1a6f</t>
+          <t>9326784c1a2726fb</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
@@ -3942,12 +3942,12 @@
       </c>
       <c r="C74" s="3" t="inlineStr">
         <is>
-          <t>Service desk agent</t>
+          <t>Técnico de soporte y mesa de ayuda / medellín</t>
         </is>
       </c>
       <c r="D74" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Colsof S.A.S</t>
         </is>
       </c>
       <c r="E74" s="7" t="n">
@@ -3959,13 +3959,13 @@
         </is>
       </c>
       <c r="G74" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/service-desk-agent-soporte-tecnico-nivel-1-1886755112", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-y-mesa-de-ayuda-medellin-1886738118", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H74" s="6" t="inlineStr"/>
       <c r="I74" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J74" s="2" t="inlineStr">
@@ -3978,7 +3978,7 @@
     <row r="75" ht="22" customHeight="1">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>9c65f710f43158b7</t>
+          <t>b67dc9a9be4a1a6f</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
@@ -3988,7 +3988,7 @@
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de instalaciones cableado de redes - licencia conte</t>
+          <t>Service desk agent</t>
         </is>
       </c>
       <c r="D75" s="3" t="inlineStr">
@@ -4005,13 +4005,13 @@
         </is>
       </c>
       <c r="G75" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-1886749397", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/service-desk-agent-soporte-tecnico-nivel-1-1886755112", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H75" s="6" t="inlineStr"/>
       <c r="I75" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J75" s="2" t="inlineStr">
@@ -4024,22 +4024,22 @@
     <row r="76" ht="22" customHeight="1">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>a95003a0b1fc3d77</t>
+          <t>9c65f710f43158b7</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 15:41</t>
+          <t>2026-09-25 15:54</t>
         </is>
       </c>
       <c r="C76" s="3" t="inlineStr">
         <is>
-          <t>Técnico Soporte Nivel 1 Con ITIL</t>
+          <t>Tecnico de instalaciones cableado de redes - licencia conte</t>
         </is>
       </c>
       <c r="D76" s="3" t="inlineStr">
         <is>
-          <t>Importante empresa del sector de tecnología</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E76" s="7" t="n">
@@ -4051,14 +4051,10 @@
         </is>
       </c>
       <c r="G76" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-soporte-nivel-1-con-itil-en-bogota-dc-59E13FA64EF5843C61373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H76" s="6" t="inlineStr">
-        <is>
-          <t>$ 1.750.905,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-1886749397", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H76" s="6" t="inlineStr"/>
       <c r="I76" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -4074,7 +4070,7 @@
     <row r="77" ht="22" customHeight="1">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>96391fd564d83616</t>
+          <t>a95003a0b1fc3d77</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
@@ -4084,12 +4080,12 @@
       </c>
       <c r="C77" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de soporte IT con Moto</t>
+          <t>Técnico Soporte Nivel 1 Con ITIL</t>
         </is>
       </c>
       <c r="D77" s="3" t="inlineStr">
         <is>
-          <t>Los Hornitos</t>
+          <t>Importante empresa del sector de tecnología</t>
         </is>
       </c>
       <c r="E77" s="7" t="n">
@@ -4101,12 +4097,12 @@
         </is>
       </c>
       <c r="G77" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-it-con-moto-empresa-de-alimentos-en-bogota-dc-599938D46A6F4A8F61373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-soporte-nivel-1-con-itil-en-bogota-dc-59E13FA64EF5843C61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H77" s="6" t="inlineStr">
         <is>
-          <t>$ 2.125.947,00 (Mensual)</t>
+          <t>$ 1.750.905,00 (Mensual)</t>
         </is>
       </c>
       <c r="I77" s="3" t="inlineStr">
@@ -4124,7 +4120,7 @@
     <row r="78" ht="22" customHeight="1">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>b4f0b8c16fe5543e</t>
+          <t>96391fd564d83616</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -4134,12 +4130,12 @@
       </c>
       <c r="C78" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar de Sistemas</t>
+          <t>Tecnico de soporte IT con Moto</t>
         </is>
       </c>
       <c r="D78" s="3" t="inlineStr">
         <is>
-          <t>ELIS COLOMBIA SAS</t>
+          <t>Los Hornitos</t>
         </is>
       </c>
       <c r="E78" s="7" t="n">
@@ -4151,12 +4147,12 @@
         </is>
       </c>
       <c r="G78" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-en-bogota-dc-48C2A0A3B050945661373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-it-con-moto-empresa-de-alimentos-en-bogota-dc-599938D46A6F4A8F61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H78" s="6" t="inlineStr">
         <is>
-          <t>$ 2.000.000,00 (Mensual)</t>
+          <t>$ 2.125.947,00 (Mensual)</t>
         </is>
       </c>
       <c r="I78" s="3" t="inlineStr">
@@ -4174,7 +4170,7 @@
     <row r="79" ht="22" customHeight="1">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>7e4b4e4f136a5e31</t>
+          <t>b4f0b8c16fe5543e</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
@@ -4184,12 +4180,12 @@
       </c>
       <c r="C79" s="3" t="inlineStr">
         <is>
-          <t>Agente Mesa de Ayuda</t>
+          <t>Auxiliar de Sistemas</t>
         </is>
       </c>
       <c r="D79" s="3" t="inlineStr">
         <is>
-          <t>Importante empresa del sector</t>
+          <t>ELIS COLOMBIA SAS</t>
         </is>
       </c>
       <c r="E79" s="7" t="n">
@@ -4201,7 +4197,7 @@
         </is>
       </c>
       <c r="G79" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-agente-mesa-de-ayuda-en-bogota-dc-E39FE355E02E578761373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-en-bogota-dc-48C2A0A3B050945661373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H79" s="6" t="inlineStr">
@@ -4224,7 +4220,7 @@
     <row r="80" ht="22" customHeight="1">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>0ef2cd7667600919</t>
+          <t>7e4b4e4f136a5e31</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
@@ -4234,12 +4230,12 @@
       </c>
       <c r="C80" s="3" t="inlineStr">
         <is>
-          <t>Técnico de Soporte TI Regional</t>
+          <t>Agente Mesa de Ayuda</t>
         </is>
       </c>
       <c r="D80" s="3" t="inlineStr">
         <is>
-          <t>POLICOMP COLOMBIA SAS</t>
+          <t>Importante empresa del sector</t>
         </is>
       </c>
       <c r="E80" s="7" t="n">
@@ -4251,10 +4247,14 @@
         </is>
       </c>
       <c r="G80" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-ti-regional-en-bogota-dc-ACF045C94E41CCDE61373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H80" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-agente-mesa-de-ayuda-en-bogota-dc-E39FE355E02E578761373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H80" s="6" t="inlineStr">
+        <is>
+          <t>$ 2.000.000,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I80" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -4270,7 +4270,7 @@
     <row r="81" ht="22" customHeight="1">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>7784997bda962255</t>
+          <t>0ef2cd7667600919</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
@@ -4280,7 +4280,7 @@
       </c>
       <c r="C81" s="3" t="inlineStr">
         <is>
-          <t>Técnico de Soporte TI On Demand/ por horas</t>
+          <t>Técnico de Soporte TI Regional</t>
         </is>
       </c>
       <c r="D81" s="3" t="inlineStr">
@@ -4297,7 +4297,7 @@
         </is>
       </c>
       <c r="G81" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-ti-on-demand-por-horas-en-bogota-dc-C2338FA0172D59A561373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-ti-regional-en-bogota-dc-ACF045C94E41CCDE61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H81" s="6" t="inlineStr"/>
@@ -4316,7 +4316,7 @@
     <row r="82" ht="22" customHeight="1">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>29d0fe2e42e678f7</t>
+          <t>7784997bda962255</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
@@ -4326,12 +4326,12 @@
       </c>
       <c r="C82" s="3" t="inlineStr">
         <is>
-          <t>Técnico mantenimiento correctivo impresoras</t>
+          <t>Técnico de Soporte TI On Demand/ por horas</t>
         </is>
       </c>
       <c r="D82" s="3" t="inlineStr">
         <is>
-          <t>Multinacional de Impresión</t>
+          <t>POLICOMP COLOMBIA SAS</t>
         </is>
       </c>
       <c r="E82" s="7" t="n">
@@ -4343,14 +4343,10 @@
         </is>
       </c>
       <c r="G82" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-mantenimiento-correctivo-impresoras-en-guarne-BC0E775C0F25B27D61373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H82" s="6" t="inlineStr">
-        <is>
-          <t>$ 1.800.000,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-ti-on-demand-por-horas-en-bogota-dc-C2338FA0172D59A561373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H82" s="6" t="inlineStr"/>
       <c r="I82" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -4366,22 +4362,22 @@
     <row r="83" ht="22" customHeight="1">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>98c9ab11f5b1eace</t>
+          <t>29d0fe2e42e678f7</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 18:36</t>
+          <t>2026-09-27 15:41</t>
         </is>
       </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar de sistemas</t>
+          <t>Técnico mantenimiento correctivo impresoras</t>
         </is>
       </c>
       <c r="D83" s="3" t="inlineStr">
         <is>
-          <t>Importante empresa del sector</t>
+          <t>Multinacional de Impresión</t>
         </is>
       </c>
       <c r="E83" s="7" t="n">
@@ -4393,12 +4389,12 @@
         </is>
       </c>
       <c r="G83" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-persona-con-discapacidad-remota-en-bogota-dc-5F2A812D014E159B61373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-mantenimiento-correctivo-impresoras-en-guarne-BC0E775C0F25B27D61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H83" s="6" t="inlineStr">
         <is>
-          <t>$ 1.750.905,00 (Mensual)</t>
+          <t>$ 1.800.000,00 (Mensual)</t>
         </is>
       </c>
       <c r="I83" s="3" t="inlineStr">
@@ -4416,7 +4412,7 @@
     <row r="84" ht="22" customHeight="1">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>58133ddc4da9c68e</t>
+          <t>98c9ab11f5b1eace</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
@@ -4443,7 +4439,7 @@
         </is>
       </c>
       <c r="G84" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-persona-con-discapacidad-remota-en-bogota-dc-A00C07C9CC9A494B61373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-persona-con-discapacidad-remota-en-bogota-dc-5F2A812D014E159B61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H84" s="6" t="inlineStr">
@@ -4466,7 +4462,7 @@
     <row r="85" ht="22" customHeight="1">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>aed3420a4cfdc248</t>
+          <t>58133ddc4da9c68e</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
@@ -4476,12 +4472,12 @@
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>Consultor de servicios/ mesa de ayuda nómina y erp software</t>
+          <t>Auxiliar de sistemas</t>
         </is>
       </c>
       <c r="D85" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Importante empresa del sector</t>
         </is>
       </c>
       <c r="E85" s="7" t="n">
@@ -4493,10 +4489,14 @@
         </is>
       </c>
       <c r="G85" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/consultor-de-servicios-mesa-de-ayuda-nomina-y-erp-software-inclusivo-1886716126", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H85" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-persona-con-discapacidad-remota-en-bogota-dc-A00C07C9CC9A494B61373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H85" s="6" t="inlineStr">
+        <is>
+          <t>$ 1.750.905,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I85" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -4512,22 +4512,22 @@
     <row r="86" ht="22" customHeight="1">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>2b8357189ff315da</t>
+          <t>aed3420a4cfdc248</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 17:00</t>
+          <t>2026-09-28 18:36</t>
         </is>
       </c>
       <c r="C86" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar de sistemas</t>
+          <t>Consultor de servicios/ mesa de ayuda nómina y erp software</t>
         </is>
       </c>
       <c r="D86" s="3" t="inlineStr">
         <is>
-          <t>DAVITA SAS</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E86" s="7" t="n">
@@ -4539,7 +4539,7 @@
         </is>
       </c>
       <c r="G86" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886758163", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/consultor-de-servicios-mesa-de-ayuda-nomina-y-erp-software-inclusivo-1886716126", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H86" s="6" t="inlineStr"/>
@@ -4558,7 +4558,7 @@
     <row r="87" ht="22" customHeight="1">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>a87934e7643b2c1c</t>
+          <t>2b8357189ff315da</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
@@ -4568,12 +4568,12 @@
       </c>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de instalaciones cableado de redes - licencia conte cali</t>
+          <t>Auxiliar de sistemas</t>
         </is>
       </c>
       <c r="D87" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>DAVITA SAS</t>
         </is>
       </c>
       <c r="E87" s="7" t="n">
@@ -4585,7 +4585,7 @@
         </is>
       </c>
       <c r="G87" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-cali-1886759847", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886758163", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H87" s="6" t="inlineStr"/>
@@ -4604,7 +4604,7 @@
     <row r="88" ht="22" customHeight="1">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>10b4265e3ad11d81</t>
+          <t>a87934e7643b2c1c</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
@@ -4614,12 +4614,12 @@
       </c>
       <c r="C88" s="3" t="inlineStr">
         <is>
-          <t>Information Technology Help Desk Support</t>
+          <t>Tecnico de instalaciones cableado de redes - licencia conte cali</t>
         </is>
       </c>
       <c r="D88" s="3" t="inlineStr">
         <is>
-          <t>Booth</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E88" s="7" t="n">
@@ -4631,7 +4631,7 @@
         </is>
       </c>
       <c r="G88" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/information-technology-help-desk-support-at-booth-4471203962", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-cali-1886759847", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H88" s="6" t="inlineStr"/>
@@ -4650,22 +4650,22 @@
     <row r="89" ht="22" customHeight="1">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>ff69ae85c8697a37</t>
+          <t>10b4265e3ad11d81</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 16:49</t>
+          <t>2026-09-29 17:00</t>
         </is>
       </c>
       <c r="C89" s="3" t="inlineStr">
         <is>
-          <t>Técnico de soporte ti - bogota</t>
+          <t>Information Technology Help Desk Support</t>
         </is>
       </c>
       <c r="D89" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Booth</t>
         </is>
       </c>
       <c r="E89" s="7" t="n">
@@ -4677,7 +4677,7 @@
         </is>
       </c>
       <c r="G89" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-ti-bogota-1886774059", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/information-technology-help-desk-support-at-booth-4471203962", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H89" s="6" t="inlineStr"/>
@@ -4696,7 +4696,7 @@
     <row r="90" ht="22" customHeight="1">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>bbacf7d69ab9084e</t>
+          <t>ff69ae85c8697a37</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
@@ -4706,12 +4706,12 @@
       </c>
       <c r="C90" s="3" t="inlineStr">
         <is>
-          <t>IT Helpdesk Analyst</t>
+          <t>Técnico de soporte ti - bogota</t>
         </is>
       </c>
       <c r="D90" s="3" t="inlineStr">
         <is>
-          <t>Power Digital Marketing</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E90" s="7" t="n">
@@ -4723,7 +4723,7 @@
         </is>
       </c>
       <c r="G90" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/it-helpdesk-analyst-at-power-digital-marketing-4472601999", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-ti-bogota-1886774059", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H90" s="6" t="inlineStr"/>
@@ -4742,22 +4742,22 @@
     <row r="91" ht="22" customHeight="1">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>bb848f474ff4b611</t>
+          <t>bbacf7d69ab9084e</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 17:26</t>
+          <t>2026-09-30 16:49</t>
         </is>
       </c>
       <c r="C91" s="3" t="inlineStr">
         <is>
-          <t>Técnico de soporte ti - bogota</t>
+          <t>IT Helpdesk Analyst</t>
         </is>
       </c>
       <c r="D91" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Power Digital Marketing</t>
         </is>
       </c>
       <c r="E91" s="7" t="n">
@@ -4769,7 +4769,7 @@
         </is>
       </c>
       <c r="G91" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-ti-bogota-1886772292", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/it-helpdesk-analyst-at-power-digital-marketing-4472601999", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H91" s="6" t="inlineStr"/>
@@ -4788,7 +4788,7 @@
     <row r="92" ht="22" customHeight="1">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>b44a1c6cfb004ca8</t>
+          <t>bb848f474ff4b611</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
@@ -4798,7 +4798,7 @@
       </c>
       <c r="C92" s="3" t="inlineStr">
         <is>
-          <t>Soporte ti nivel 2 - bogotá</t>
+          <t>Técnico de soporte ti - bogota</t>
         </is>
       </c>
       <c r="D92" s="3" t="inlineStr">
@@ -4815,7 +4815,7 @@
         </is>
       </c>
       <c r="G92" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/soporte-ti-nivel-2-bogota-1886774821", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-ti-bogota-1886772292", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H92" s="6" t="inlineStr"/>
@@ -4834,7 +4834,7 @@
     <row r="93" ht="22" customHeight="1">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>fb0ad2b513afb97c</t>
+          <t>b44a1c6cfb004ca8</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
@@ -4844,12 +4844,12 @@
       </c>
       <c r="C93" s="3" t="inlineStr">
         <is>
-          <t>IT Help Desk Support Specialist</t>
+          <t>Soporte ti nivel 2 - bogotá</t>
         </is>
       </c>
       <c r="D93" s="3" t="inlineStr">
         <is>
-          <t>Talento</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E93" s="7" t="n">
@@ -4861,7 +4861,7 @@
         </is>
       </c>
       <c r="G93" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/it-help-desk-support-specialist-tier-1-at-talento-4473960480", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/soporte-ti-nivel-2-bogota-1886774821", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H93" s="6" t="inlineStr"/>
@@ -4880,22 +4880,22 @@
     <row r="94" ht="22" customHeight="1">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>0b2067d6ae488f4c</t>
+          <t>fb0ad2b513afb97c</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 16:39</t>
+          <t>2026-10-01 17:26</t>
         </is>
       </c>
       <c r="C94" s="3" t="inlineStr">
         <is>
-          <t>Help Desk Technician level 1</t>
+          <t>IT Help Desk Support Specialist</t>
         </is>
       </c>
       <c r="D94" s="3" t="inlineStr">
         <is>
-          <t>Solvo Global</t>
+          <t>Talento</t>
         </is>
       </c>
       <c r="E94" s="7" t="n">
@@ -4907,7 +4907,7 @@
         </is>
       </c>
       <c r="G94" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/help-desk-technician-level-1-at-solvo-global-4472590892", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/it-help-desk-support-specialist-tier-1-at-talento-4473960480", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H94" s="6" t="inlineStr"/>
@@ -4926,22 +4926,22 @@
     <row r="95" ht="22" customHeight="1">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>07acc222a3ca2ef1</t>
+          <t>0b2067d6ae488f4c</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03 15:12</t>
+          <t>2026-10-02 16:39</t>
         </is>
       </c>
       <c r="C95" s="3" t="inlineStr">
         <is>
-          <t>Analista mesa de ayuda funza temporal 6 meses</t>
+          <t>Help Desk Technician level 1</t>
         </is>
       </c>
       <c r="D95" s="3" t="inlineStr">
         <is>
-          <t>Axity</t>
+          <t>Solvo Global</t>
         </is>
       </c>
       <c r="E95" s="7" t="n">
@@ -4953,7 +4953,7 @@
         </is>
       </c>
       <c r="G95" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-funza-temporal-6-meses-1886774524", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/help-desk-technician-level-1-at-solvo-global-4472590892", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H95" s="6" t="inlineStr"/>
@@ -4972,22 +4972,22 @@
     <row r="96" ht="22" customHeight="1">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>5ec0ea33876ba2b5</t>
+          <t>07acc222a3ca2ef1</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 19:45</t>
+          <t>2026-10-03 15:12</t>
         </is>
       </c>
       <c r="C96" s="3" t="inlineStr">
         <is>
-          <t>Help desk analyst l1</t>
+          <t>Analista mesa de ayuda funza temporal 6 meses</t>
         </is>
       </c>
       <c r="D96" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Axity</t>
         </is>
       </c>
       <c r="E96" s="7" t="n">
@@ -4999,7 +4999,7 @@
         </is>
       </c>
       <c r="G96" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/help-desk-analyst-l1-medellin-1886776156", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-funza-temporal-6-meses-1886774524", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H96" s="6" t="inlineStr"/>
@@ -5018,7 +5018,7 @@
     <row r="97" ht="22" customHeight="1">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>e8bdf2094d1c9817</t>
+          <t>5ec0ea33876ba2b5</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
@@ -5028,12 +5028,12 @@
       </c>
       <c r="C97" s="3" t="inlineStr">
         <is>
-          <t>Administrador de herramienta de gestión de mesa de ayuda-</t>
+          <t>Help desk analyst l1</t>
         </is>
       </c>
       <c r="D97" s="3" t="inlineStr">
         <is>
-          <t>SELCOMP INGENIERÍA SAS</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E97" s="7" t="n">
@@ -5045,7 +5045,7 @@
         </is>
       </c>
       <c r="G97" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/administrador-de-herramienta-de-gestion-de-mesa-de-ayuda-1886776286", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/help-desk-analyst-l1-medellin-1886776156", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H97" s="6" t="inlineStr"/>
@@ -5064,7 +5064,7 @@
     <row r="98" ht="22" customHeight="1">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>6e9a077b42879470</t>
+          <t>e8bdf2094d1c9817</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
@@ -5074,12 +5074,12 @@
       </c>
       <c r="C98" s="3" t="inlineStr">
         <is>
-          <t>Analista de soporte de aplicaciones nivel 3</t>
+          <t>Administrador de herramienta de gestión de mesa de ayuda-</t>
         </is>
       </c>
       <c r="D98" s="3" t="inlineStr">
         <is>
-          <t>TALYCAP GLOBAL SAS</t>
+          <t>SELCOMP INGENIERÍA SAS</t>
         </is>
       </c>
       <c r="E98" s="7" t="n">
@@ -5091,7 +5091,7 @@
         </is>
       </c>
       <c r="G98" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-soporte-de-aplicaciones-nivel-3-1886776104", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/administrador-de-herramienta-de-gestion-de-mesa-de-ayuda-1886776286", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H98" s="6" t="inlineStr"/>
@@ -5110,22 +5110,22 @@
     <row r="99" ht="22" customHeight="1">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>447afec244b20f9b</t>
+          <t>6e9a077b42879470</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06 17:12</t>
+          <t>2026-10-05 19:45</t>
         </is>
       </c>
       <c r="C99" s="3" t="inlineStr">
         <is>
-          <t>Técnico de soporte ti - bogota</t>
+          <t>Analista de soporte de aplicaciones nivel 3</t>
         </is>
       </c>
       <c r="D99" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>TALYCAP GLOBAL SAS</t>
         </is>
       </c>
       <c r="E99" s="7" t="n">
@@ -5137,7 +5137,7 @@
         </is>
       </c>
       <c r="G99" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-ti-bogota-1886775990", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-soporte-de-aplicaciones-nivel-3-1886776104", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H99" s="6" t="inlineStr"/>
@@ -5156,22 +5156,22 @@
     <row r="100" ht="22" customHeight="1">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>8f14c41f3b443ac0</t>
+          <t>447afec244b20f9b</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07 17:50</t>
+          <t>2026-10-06 17:12</t>
         </is>
       </c>
       <c r="C100" s="3" t="inlineStr">
         <is>
-          <t>Soporte mesa de ayuda</t>
+          <t>Técnico de soporte ti - bogota</t>
         </is>
       </c>
       <c r="D100" s="3" t="inlineStr">
         <is>
-          <t>MANPOWER</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E100" s="7" t="n">
@@ -5183,7 +5183,7 @@
         </is>
       </c>
       <c r="G100" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/soporte-mesa-de-ayuda-vacaciones-1886776917", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-ti-bogota-1886775990", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H100" s="6" t="inlineStr"/>
@@ -5202,7 +5202,7 @@
     <row r="101" ht="22" customHeight="1">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>b1a9e03967fff91e</t>
+          <t>8f14c41f3b443ac0</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr">
@@ -5212,12 +5212,12 @@
       </c>
       <c r="C101" s="3" t="inlineStr">
         <is>
-          <t>Tecnólogo de soporte pl - mesa de ayuda</t>
+          <t>Soporte mesa de ayuda</t>
         </is>
       </c>
       <c r="D101" s="3" t="inlineStr">
         <is>
-          <t>Positivo S+</t>
+          <t>MANPOWER</t>
         </is>
       </c>
       <c r="E101" s="7" t="n">
@@ -5229,7 +5229,7 @@
         </is>
       </c>
       <c r="G101" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnologo-de-soporte-pl-mesa-de-ayuda-1886775546", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/soporte-mesa-de-ayuda-vacaciones-1886776917", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H101" s="6" t="inlineStr"/>
@@ -5248,7 +5248,7 @@
     <row r="102" ht="22" customHeight="1">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>eb49981c97933d93</t>
+          <t>b1a9e03967fff91e</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
@@ -5258,12 +5258,12 @@
       </c>
       <c r="C102" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de instalaciones cableado de redes - licencia conte</t>
+          <t>Tecnólogo de soporte pl - mesa de ayuda</t>
         </is>
       </c>
       <c r="D102" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Positivo S+</t>
         </is>
       </c>
       <c r="E102" s="7" t="n">
@@ -5275,7 +5275,7 @@
         </is>
       </c>
       <c r="G102" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-1886777333", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnologo-de-soporte-pl-mesa-de-ayuda-1886775546", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H102" s="6" t="inlineStr"/>
@@ -5294,7 +5294,7 @@
     <row r="103" ht="22" customHeight="1">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>d39af22b6e937d28</t>
+          <t>eb49981c97933d93</t>
         </is>
       </c>
       <c r="B103" s="2" t="inlineStr">
@@ -5304,12 +5304,12 @@
       </c>
       <c r="C103" s="3" t="inlineStr">
         <is>
-          <t>Analista Mesa de Ayuda Funza</t>
+          <t>Tecnico de instalaciones cableado de redes - licencia conte</t>
         </is>
       </c>
       <c r="D103" s="3" t="inlineStr">
         <is>
-          <t>axity</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E103" s="7" t="n">
@@ -5321,7 +5321,7 @@
         </is>
       </c>
       <c r="G103" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/analista-mesa-de-ayuda-funza-at-axity-4471985006", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-1886777333", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H103" s="6" t="inlineStr"/>
@@ -5340,22 +5340,22 @@
     <row r="104" ht="22" customHeight="1">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>0904912d51c5cd61</t>
+          <t>d39af22b6e937d28</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08 17:52</t>
+          <t>2026-10-07 17:50</t>
         </is>
       </c>
       <c r="C104" s="3" t="inlineStr">
         <is>
-          <t>Analista mesa de ayuda</t>
+          <t>Analista Mesa de Ayuda Funza</t>
         </is>
       </c>
       <c r="D104" s="3" t="inlineStr">
         <is>
-          <t>Desarrollo de Sistemas y Servicios SAS</t>
+          <t>axity</t>
         </is>
       </c>
       <c r="E104" s="7" t="n">
@@ -5367,7 +5367,7 @@
         </is>
       </c>
       <c r="G104" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-1886778032", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/analista-mesa-de-ayuda-funza-at-axity-4471985006", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H104" s="6" t="inlineStr"/>
@@ -5386,22 +5386,22 @@
     <row r="105" ht="22" customHeight="1">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>c665ada630270dce</t>
+          <t>0904912d51c5cd61</t>
         </is>
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09 17:28</t>
+          <t>2026-10-08 17:52</t>
         </is>
       </c>
       <c r="C105" s="3" t="inlineStr">
         <is>
-          <t>Técnico(a) / tecnólogo(a) / profesional de telecomunicaciones - redes de fibra óptica</t>
+          <t>Analista mesa de ayuda</t>
         </is>
       </c>
       <c r="D105" s="3" t="inlineStr">
         <is>
-          <t>JAHV MC GREGOR S.A.S</t>
+          <t>Desarrollo de Sistemas y Servicios SAS</t>
         </is>
       </c>
       <c r="E105" s="7" t="n">
@@ -5413,7 +5413,7 @@
         </is>
       </c>
       <c r="G105" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnicoa-tecnologoa-profesional-de-telecomunicaciones-redes-de-fibra-optica-1886768691", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-1886778032", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H105" s="6" t="inlineStr"/>
@@ -5432,7 +5432,7 @@
     <row r="106" ht="22" customHeight="1">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>4e5b3128aa7f8f9b</t>
+          <t>c665ada630270dce</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
@@ -5442,12 +5442,12 @@
       </c>
       <c r="C106" s="3" t="inlineStr">
         <is>
-          <t>Gestor de servicios mesa de ayuda sap</t>
+          <t>Técnico(a) / tecnólogo(a) / profesional de telecomunicaciones - redes de fibra óptica</t>
         </is>
       </c>
       <c r="D106" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>JAHV MC GREGOR S.A.S</t>
         </is>
       </c>
       <c r="E106" s="7" t="n">
@@ -5459,7 +5459,7 @@
         </is>
       </c>
       <c r="G106" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/gestor-de-servicios-mesa-de-ayuda-sap-1886775732", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnicoa-tecnologoa-profesional-de-telecomunicaciones-redes-de-fibra-optica-1886768691", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H106" s="6" t="inlineStr"/>
@@ -5478,7 +5478,7 @@
     <row r="107" ht="22" customHeight="1">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>1c92f7ef9b7af696</t>
+          <t>4e5b3128aa7f8f9b</t>
         </is>
       </c>
       <c r="B107" s="2" t="inlineStr">
@@ -5488,7 +5488,7 @@
       </c>
       <c r="C107" s="3" t="inlineStr">
         <is>
-          <t>Agente de mesa de ayuda nivel 1</t>
+          <t>Gestor de servicios mesa de ayuda sap</t>
         </is>
       </c>
       <c r="D107" s="3" t="inlineStr">
@@ -5505,7 +5505,7 @@
         </is>
       </c>
       <c r="G107" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-de-mesa-de-ayuda-nivel-1-1886778506", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/gestor-de-servicios-mesa-de-ayuda-sap-1886775732", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H107" s="6" t="inlineStr"/>
@@ -5524,22 +5524,22 @@
     <row r="108" ht="22" customHeight="1">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>718ceee355d457ea</t>
+          <t>1c92f7ef9b7af696</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10 16:16</t>
+          <t>2026-10-09 17:28</t>
         </is>
       </c>
       <c r="C108" s="3" t="inlineStr">
         <is>
-          <t>IT Help Desk Support</t>
+          <t>Agente de mesa de ayuda nivel 1</t>
         </is>
       </c>
       <c r="D108" s="3" t="inlineStr">
         <is>
-          <t>Booth</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E108" s="7" t="n">
@@ -5551,7 +5551,7 @@
         </is>
       </c>
       <c r="G108" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/it-help-desk-support-at-booth-4471203962", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-de-mesa-de-ayuda-nivel-1-1886778506", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H108" s="6" t="inlineStr"/>
@@ -5570,26 +5570,26 @@
     <row r="109" ht="22" customHeight="1">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>50c79dfbfd49f52d</t>
+          <t>718ceee355d457ea</t>
         </is>
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 16:39</t>
+          <t>2026-10-10 16:16</t>
         </is>
       </c>
       <c r="C109" s="3" t="inlineStr">
         <is>
-          <t>Analista de redes noc 1 telecomunicaciones.</t>
+          <t>IT Help Desk Support</t>
         </is>
       </c>
       <c r="D109" s="3" t="inlineStr">
         <is>
-          <t>MANPOWER</t>
+          <t>Booth</t>
         </is>
       </c>
       <c r="E109" s="7" t="n">
-        <v>0.53</v>
+        <v>0.58</v>
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
@@ -5597,13 +5597,13 @@
         </is>
       </c>
       <c r="G109" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-noc-1-telecomunicaciones-1886772075", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/it-help-desk-support-at-booth-4471203962", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H109" s="6" t="inlineStr"/>
       <c r="I109" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J109" s="2" t="inlineStr">
@@ -5616,26 +5616,26 @@
     <row r="110" ht="22" customHeight="1">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>0b0ae49f910109bb</t>
+          <t>925f43273b78f188</t>
         </is>
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 15:54</t>
+          <t>2026-10-12 20:17</t>
         </is>
       </c>
       <c r="C110" s="3" t="inlineStr">
         <is>
-          <t>Ejecutivo Técnico Arancel Junior</t>
+          <t>Mesa de ayuda ti - girón</t>
         </is>
       </c>
       <c r="D110" s="3" t="inlineStr">
         <is>
-          <t>Importante Empresa de Logística y Comercio</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E110" s="7" t="n">
-        <v>0.5</v>
+        <v>0.58</v>
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
@@ -5643,17 +5643,13 @@
         </is>
       </c>
       <c r="G110" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-547866639B487E0161373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H110" s="6" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/mesa-de-ayuda-ti-giron-1886745168", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H110" s="6" t="inlineStr"/>
       <c r="I110" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J110" s="2" t="inlineStr">
@@ -5666,26 +5662,26 @@
     <row r="111" ht="22" customHeight="1">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>582a04b3c639bfa0</t>
+          <t>50c79dfbfd49f52d</t>
         </is>
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 16:49</t>
+          <t>2026-10-02 16:39</t>
         </is>
       </c>
       <c r="C111" s="3" t="inlineStr">
         <is>
-          <t>Junior IT Support Specialist</t>
+          <t>Analista de redes noc 1 telecomunicaciones.</t>
         </is>
       </c>
       <c r="D111" s="3" t="inlineStr">
         <is>
-          <t>Touch Support, Inc. &amp; SNF Back Office</t>
+          <t>MANPOWER</t>
         </is>
       </c>
       <c r="E111" s="7" t="n">
-        <v>0.5</v>
+        <v>0.53</v>
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
@@ -5693,13 +5689,13 @@
         </is>
       </c>
       <c r="G111" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/junior-it-support-specialist-at-touch-support-inc-snf-back-office-4472187578", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-noc-1-telecomunicaciones-1886772075", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H111" s="6" t="inlineStr"/>
       <c r="I111" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J111" s="2" t="inlineStr">
@@ -5712,12 +5708,12 @@
     <row r="112" ht="22" customHeight="1">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>6e04c4d57d3fc3c7</t>
+          <t>0b0ae49f910109bb</t>
         </is>
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 17:26</t>
+          <t>2026-09-25 15:54</t>
         </is>
       </c>
       <c r="C112" s="3" t="inlineStr">
@@ -5739,25 +5735,121 @@
         </is>
       </c>
       <c r="G112" s="5">
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-547866639B487E0161373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H112" s="6" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="I112" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J112" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K112" s="3" t="inlineStr"/>
+    </row>
+    <row r="113" ht="22" customHeight="1">
+      <c r="A113" s="2" t="inlineStr">
+        <is>
+          <t>582a04b3c639bfa0</t>
+        </is>
+      </c>
+      <c r="B113" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 16:49</t>
+        </is>
+      </c>
+      <c r="C113" s="3" t="inlineStr">
+        <is>
+          <t>Junior IT Support Specialist</t>
+        </is>
+      </c>
+      <c r="D113" s="3" t="inlineStr">
+        <is>
+          <t>Touch Support, Inc. &amp; SNF Back Office</t>
+        </is>
+      </c>
+      <c r="E113" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F113" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G113" s="5">
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/junior-it-support-specialist-at-touch-support-inc-snf-back-office-4472187578", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H113" s="6" t="inlineStr"/>
+      <c r="I113" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J113" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K113" s="3" t="inlineStr"/>
+    </row>
+    <row r="114" ht="22" customHeight="1">
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t>6e04c4d57d3fc3c7</t>
+        </is>
+      </c>
+      <c r="B114" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01 17:26</t>
+        </is>
+      </c>
+      <c r="C114" s="3" t="inlineStr">
+        <is>
+          <t>Ejecutivo Técnico Arancel Junior</t>
+        </is>
+      </c>
+      <c r="D114" s="3" t="inlineStr">
+        <is>
+          <t>Importante Empresa de Logística y Comercio</t>
+        </is>
+      </c>
+      <c r="E114" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F114" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G114" s="5">
         <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-8444AB594560844161373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
-      <c r="H112" s="6" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
-      <c r="I112" s="3" t="inlineStr">
+      <c r="H114" s="6" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="I114" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
-      <c r="J112" s="2" t="inlineStr">
-        <is>
-          <t>Nueva</t>
-        </is>
-      </c>
-      <c r="K112" s="3" t="inlineStr"/>
+      <c r="J114" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K114" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
chore(tracker): actualizacion diaria de vacantes 2026-10-13
</commit_message>
<xml_diff>
--- a/output/profile_5_tecnico_sistemas_tracker.xlsx
+++ b/output/profile_5_tecnico_sistemas_tracker.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K114"/>
+  <dimension ref="A1:K116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -5662,26 +5662,26 @@
     <row r="111" ht="22" customHeight="1">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>50c79dfbfd49f52d</t>
+          <t>ec0c8875e04f4933</t>
         </is>
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 16:39</t>
+          <t>2026-10-13 18:08</t>
         </is>
       </c>
       <c r="C111" s="3" t="inlineStr">
         <is>
-          <t>Analista de redes noc 1 telecomunicaciones.</t>
+          <t>Analista de mesa de ayuda.</t>
         </is>
       </c>
       <c r="D111" s="3" t="inlineStr">
         <is>
-          <t>MANPOWER</t>
+          <t>Softtek Colombia</t>
         </is>
       </c>
       <c r="E111" s="7" t="n">
-        <v>0.53</v>
+        <v>0.58</v>
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
@@ -5689,13 +5689,13 @@
         </is>
       </c>
       <c r="G111" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-noc-1-telecomunicaciones-1886772075", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-mesa-de-ayuda-1886754207", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H111" s="6" t="inlineStr"/>
       <c r="I111" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J111" s="2" t="inlineStr">
@@ -5708,26 +5708,26 @@
     <row r="112" ht="22" customHeight="1">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>0b0ae49f910109bb</t>
+          <t>87fac63aa714f401</t>
         </is>
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 15:54</t>
+          <t>2026-10-13 18:08</t>
         </is>
       </c>
       <c r="C112" s="3" t="inlineStr">
         <is>
-          <t>Ejecutivo Técnico Arancel Junior</t>
+          <t>Agente mesa de ayuda.</t>
         </is>
       </c>
       <c r="D112" s="3" t="inlineStr">
         <is>
-          <t>Importante Empresa de Logística y Comercio</t>
+          <t>Softtek Colombia</t>
         </is>
       </c>
       <c r="E112" s="7" t="n">
-        <v>0.5</v>
+        <v>0.58</v>
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
@@ -5735,17 +5735,13 @@
         </is>
       </c>
       <c r="G112" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-547866639B487E0161373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H112" s="6" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-mesa-de-ayuda-1886753535", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H112" s="6" t="inlineStr"/>
       <c r="I112" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J112" s="2" t="inlineStr">
@@ -5758,26 +5754,26 @@
     <row r="113" ht="22" customHeight="1">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>582a04b3c639bfa0</t>
+          <t>50c79dfbfd49f52d</t>
         </is>
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 16:49</t>
+          <t>2026-10-02 16:39</t>
         </is>
       </c>
       <c r="C113" s="3" t="inlineStr">
         <is>
-          <t>Junior IT Support Specialist</t>
+          <t>Analista de redes noc 1 telecomunicaciones.</t>
         </is>
       </c>
       <c r="D113" s="3" t="inlineStr">
         <is>
-          <t>Touch Support, Inc. &amp; SNF Back Office</t>
+          <t>MANPOWER</t>
         </is>
       </c>
       <c r="E113" s="7" t="n">
-        <v>0.5</v>
+        <v>0.53</v>
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
@@ -5785,13 +5781,13 @@
         </is>
       </c>
       <c r="G113" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/junior-it-support-specialist-at-touch-support-inc-snf-back-office-4472187578", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-noc-1-telecomunicaciones-1886772075", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H113" s="6" t="inlineStr"/>
       <c r="I113" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J113" s="2" t="inlineStr">
@@ -5804,12 +5800,12 @@
     <row r="114" ht="22" customHeight="1">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>6e04c4d57d3fc3c7</t>
+          <t>0b0ae49f910109bb</t>
         </is>
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 17:26</t>
+          <t>2026-09-25 15:54</t>
         </is>
       </c>
       <c r="C114" s="3" t="inlineStr">
@@ -5831,25 +5827,121 @@
         </is>
       </c>
       <c r="G114" s="5">
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-547866639B487E0161373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H114" s="6" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="I114" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J114" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K114" s="3" t="inlineStr"/>
+    </row>
+    <row r="115" ht="22" customHeight="1">
+      <c r="A115" s="2" t="inlineStr">
+        <is>
+          <t>582a04b3c639bfa0</t>
+        </is>
+      </c>
+      <c r="B115" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 16:49</t>
+        </is>
+      </c>
+      <c r="C115" s="3" t="inlineStr">
+        <is>
+          <t>Junior IT Support Specialist</t>
+        </is>
+      </c>
+      <c r="D115" s="3" t="inlineStr">
+        <is>
+          <t>Touch Support, Inc. &amp; SNF Back Office</t>
+        </is>
+      </c>
+      <c r="E115" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F115" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G115" s="5">
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/junior-it-support-specialist-at-touch-support-inc-snf-back-office-4472187578", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H115" s="6" t="inlineStr"/>
+      <c r="I115" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J115" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K115" s="3" t="inlineStr"/>
+    </row>
+    <row r="116" ht="22" customHeight="1">
+      <c r="A116" s="2" t="inlineStr">
+        <is>
+          <t>6e04c4d57d3fc3c7</t>
+        </is>
+      </c>
+      <c r="B116" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01 17:26</t>
+        </is>
+      </c>
+      <c r="C116" s="3" t="inlineStr">
+        <is>
+          <t>Ejecutivo Técnico Arancel Junior</t>
+        </is>
+      </c>
+      <c r="D116" s="3" t="inlineStr">
+        <is>
+          <t>Importante Empresa de Logística y Comercio</t>
+        </is>
+      </c>
+      <c r="E116" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F116" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G116" s="5">
         <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-8444AB594560844161373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
-      <c r="H114" s="6" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
-      <c r="I114" s="3" t="inlineStr">
+      <c r="H116" s="6" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="I116" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
-      <c r="J114" s="2" t="inlineStr">
-        <is>
-          <t>Nueva</t>
-        </is>
-      </c>
-      <c r="K114" s="3" t="inlineStr"/>
+      <c r="J116" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K116" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
chore(tracker): actualizacion diaria de vacantes 2026-10-14
</commit_message>
<xml_diff>
--- a/output/profile_5_tecnico_sistemas_tracker.xlsx
+++ b/output/profile_5_tecnico_sistemas_tracker.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K116"/>
+  <dimension ref="A1:K117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3564,26 +3564,26 @@
     <row r="66" ht="22" customHeight="1">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>73882c81e04abc7e</t>
+          <t>422a27df3967ecbb</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 19:45</t>
+          <t>2026-10-14 15:52</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>Soporte L1 Junior</t>
+          <t>Técnico de sistemas y soporte ti</t>
         </is>
       </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
-          <t>Hublance</t>
+          <t>AGENCIA DE EMPLEO CAFAM</t>
         </is>
       </c>
       <c r="E66" s="7" t="n">
-        <v>0.6</v>
+        <v>0.66</v>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
@@ -3591,13 +3591,13 @@
         </is>
       </c>
       <c r="G66" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/soporte-l1-junior-at-hublance-4475841269", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-sistemas-y-soporte-ti-1886780022", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H66" s="6" t="inlineStr"/>
       <c r="I66" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 60/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 66/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J66" s="2" t="inlineStr">
@@ -3610,26 +3610,26 @@
     <row r="67" ht="22" customHeight="1">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>8d7f304ffb8625b5</t>
+          <t>73882c81e04abc7e</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 15:54</t>
+          <t>2026-10-05 19:45</t>
         </is>
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar de sistemas</t>
+          <t>Soporte L1 Junior</t>
         </is>
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Hublance</t>
         </is>
       </c>
       <c r="E67" s="7" t="n">
-        <v>0.58</v>
+        <v>0.6</v>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
@@ -3637,13 +3637,13 @@
         </is>
       </c>
       <c r="G67" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886751888", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/soporte-l1-junior-at-hublance-4475841269", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H67" s="6" t="inlineStr"/>
       <c r="I67" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 60/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J67" s="2" t="inlineStr">
@@ -3656,7 +3656,7 @@
     <row r="68" ht="22" customHeight="1">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>3b5b26f92a305c0c</t>
+          <t>8d7f304ffb8625b5</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="G68" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886749497", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886751888", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H68" s="6" t="inlineStr"/>
@@ -3702,7 +3702,7 @@
     <row r="69" ht="22" customHeight="1">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>e760bcd88d90fbbe</t>
+          <t>3b5b26f92a305c0c</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
@@ -3712,12 +3712,12 @@
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>Agente de mesa de ayuda</t>
+          <t>Auxiliar de sistemas</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>SELCOMP INGENIERÍA SAS</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E69" s="7" t="n">
@@ -3729,7 +3729,7 @@
         </is>
       </c>
       <c r="G69" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-de-mesa-de-ayuda-1886758623", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886749497", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H69" s="6" t="inlineStr"/>
@@ -3748,7 +3748,7 @@
     <row r="70" ht="22" customHeight="1">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>86dcab5c5d802693</t>
+          <t>e760bcd88d90fbbe</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -3758,12 +3758,12 @@
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>Analista mesa de ayuda para tunja</t>
+          <t>Agente de mesa de ayuda</t>
         </is>
       </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
-          <t>Gestión de Seguridad Electrónica</t>
+          <t>SELCOMP INGENIERÍA SAS</t>
         </is>
       </c>
       <c r="E70" s="7" t="n">
@@ -3775,7 +3775,7 @@
         </is>
       </c>
       <c r="G70" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-para-tunja-1886766955", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-de-mesa-de-ayuda-1886758623", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H70" s="6" t="inlineStr"/>
@@ -3794,7 +3794,7 @@
     <row r="71" ht="22" customHeight="1">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>55fdaa0983ef9124</t>
+          <t>86dcab5c5d802693</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
@@ -3804,12 +3804,12 @@
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>Lider técnico con itil practice manager</t>
+          <t>Analista mesa de ayuda para tunja</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>Sinergy &amp; Lowells</t>
+          <t>Gestión de Seguridad Electrónica</t>
         </is>
       </c>
       <c r="E71" s="7" t="n">
@@ -3821,7 +3821,7 @@
         </is>
       </c>
       <c r="G71" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/lider-tecnico-con-itil-practice-manager-1886753953", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-para-tunja-1886766955", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H71" s="6" t="inlineStr"/>
@@ -3840,7 +3840,7 @@
     <row r="72" ht="22" customHeight="1">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>a1ca7bc58cd48fad</t>
+          <t>55fdaa0983ef9124</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -3850,12 +3850,12 @@
       </c>
       <c r="C72" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de mesa de ayuda/mujeres contratacion inmediata</t>
+          <t>Lider técnico con itil practice manager</t>
         </is>
       </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Sinergy &amp; Lowells</t>
         </is>
       </c>
       <c r="E72" s="7" t="n">
@@ -3867,7 +3867,7 @@
         </is>
       </c>
       <c r="G72" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-mesa-de-ayuda-mujeres-contratacion-inmediata-1886770931", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/lider-tecnico-con-itil-practice-manager-1886753953", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H72" s="6" t="inlineStr"/>
@@ -3886,7 +3886,7 @@
     <row r="73" ht="22" customHeight="1">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>e28aba5df8a2d3ae</t>
+          <t>a1ca7bc58cd48fad</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
@@ -3913,7 +3913,7 @@
         </is>
       </c>
       <c r="G73" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-mesa-de-ayuda-mujeres-contratacion-inmediata-1886769701", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-mesa-de-ayuda-mujeres-contratacion-inmediata-1886770931", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H73" s="6" t="inlineStr"/>
@@ -3932,7 +3932,7 @@
     <row r="74" ht="22" customHeight="1">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>9326784c1a2726fb</t>
+          <t>e28aba5df8a2d3ae</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
@@ -3942,12 +3942,12 @@
       </c>
       <c r="C74" s="3" t="inlineStr">
         <is>
-          <t>Técnico de soporte y mesa de ayuda / medellín</t>
+          <t>Tecnico de mesa de ayuda/mujeres contratacion inmediata</t>
         </is>
       </c>
       <c r="D74" s="3" t="inlineStr">
         <is>
-          <t>Colsof S.A.S</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E74" s="7" t="n">
@@ -3959,7 +3959,7 @@
         </is>
       </c>
       <c r="G74" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-y-mesa-de-ayuda-medellin-1886738118", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-mesa-de-ayuda-mujeres-contratacion-inmediata-1886769701", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H74" s="6" t="inlineStr"/>
@@ -3978,7 +3978,7 @@
     <row r="75" ht="22" customHeight="1">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>b67dc9a9be4a1a6f</t>
+          <t>9326784c1a2726fb</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
@@ -3988,12 +3988,12 @@
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>Service desk agent</t>
+          <t>Técnico de soporte y mesa de ayuda / medellín</t>
         </is>
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Colsof S.A.S</t>
         </is>
       </c>
       <c r="E75" s="7" t="n">
@@ -4005,13 +4005,13 @@
         </is>
       </c>
       <c r="G75" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/service-desk-agent-soporte-tecnico-nivel-1-1886755112", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-y-mesa-de-ayuda-medellin-1886738118", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H75" s="6" t="inlineStr"/>
       <c r="I75" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J75" s="2" t="inlineStr">
@@ -4024,7 +4024,7 @@
     <row r="76" ht="22" customHeight="1">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>9c65f710f43158b7</t>
+          <t>b67dc9a9be4a1a6f</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
@@ -4034,7 +4034,7 @@
       </c>
       <c r="C76" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de instalaciones cableado de redes - licencia conte</t>
+          <t>Service desk agent</t>
         </is>
       </c>
       <c r="D76" s="3" t="inlineStr">
@@ -4051,13 +4051,13 @@
         </is>
       </c>
       <c r="G76" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-1886749397", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/service-desk-agent-soporte-tecnico-nivel-1-1886755112", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H76" s="6" t="inlineStr"/>
       <c r="I76" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J76" s="2" t="inlineStr">
@@ -4070,22 +4070,22 @@
     <row r="77" ht="22" customHeight="1">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>a95003a0b1fc3d77</t>
+          <t>9c65f710f43158b7</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 15:41</t>
+          <t>2026-09-25 15:54</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
         <is>
-          <t>Técnico Soporte Nivel 1 Con ITIL</t>
+          <t>Tecnico de instalaciones cableado de redes - licencia conte</t>
         </is>
       </c>
       <c r="D77" s="3" t="inlineStr">
         <is>
-          <t>Importante empresa del sector de tecnología</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E77" s="7" t="n">
@@ -4097,14 +4097,10 @@
         </is>
       </c>
       <c r="G77" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-soporte-nivel-1-con-itil-en-bogota-dc-59E13FA64EF5843C61373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H77" s="6" t="inlineStr">
-        <is>
-          <t>$ 1.750.905,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-1886749397", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H77" s="6" t="inlineStr"/>
       <c r="I77" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -4120,7 +4116,7 @@
     <row r="78" ht="22" customHeight="1">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>96391fd564d83616</t>
+          <t>a95003a0b1fc3d77</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -4130,12 +4126,12 @@
       </c>
       <c r="C78" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de soporte IT con Moto</t>
+          <t>Técnico Soporte Nivel 1 Con ITIL</t>
         </is>
       </c>
       <c r="D78" s="3" t="inlineStr">
         <is>
-          <t>Los Hornitos</t>
+          <t>Importante empresa del sector de tecnología</t>
         </is>
       </c>
       <c r="E78" s="7" t="n">
@@ -4147,12 +4143,12 @@
         </is>
       </c>
       <c r="G78" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-it-con-moto-empresa-de-alimentos-en-bogota-dc-599938D46A6F4A8F61373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-soporte-nivel-1-con-itil-en-bogota-dc-59E13FA64EF5843C61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H78" s="6" t="inlineStr">
         <is>
-          <t>$ 2.125.947,00 (Mensual)</t>
+          <t>$ 1.750.905,00 (Mensual)</t>
         </is>
       </c>
       <c r="I78" s="3" t="inlineStr">
@@ -4170,7 +4166,7 @@
     <row r="79" ht="22" customHeight="1">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>b4f0b8c16fe5543e</t>
+          <t>96391fd564d83616</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
@@ -4180,12 +4176,12 @@
       </c>
       <c r="C79" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar de Sistemas</t>
+          <t>Tecnico de soporte IT con Moto</t>
         </is>
       </c>
       <c r="D79" s="3" t="inlineStr">
         <is>
-          <t>ELIS COLOMBIA SAS</t>
+          <t>Los Hornitos</t>
         </is>
       </c>
       <c r="E79" s="7" t="n">
@@ -4197,12 +4193,12 @@
         </is>
       </c>
       <c r="G79" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-en-bogota-dc-48C2A0A3B050945661373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-it-con-moto-empresa-de-alimentos-en-bogota-dc-599938D46A6F4A8F61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H79" s="6" t="inlineStr">
         <is>
-          <t>$ 2.000.000,00 (Mensual)</t>
+          <t>$ 2.125.947,00 (Mensual)</t>
         </is>
       </c>
       <c r="I79" s="3" t="inlineStr">
@@ -4220,7 +4216,7 @@
     <row r="80" ht="22" customHeight="1">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>7e4b4e4f136a5e31</t>
+          <t>b4f0b8c16fe5543e</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
@@ -4230,12 +4226,12 @@
       </c>
       <c r="C80" s="3" t="inlineStr">
         <is>
-          <t>Agente Mesa de Ayuda</t>
+          <t>Auxiliar de Sistemas</t>
         </is>
       </c>
       <c r="D80" s="3" t="inlineStr">
         <is>
-          <t>Importante empresa del sector</t>
+          <t>ELIS COLOMBIA SAS</t>
         </is>
       </c>
       <c r="E80" s="7" t="n">
@@ -4247,7 +4243,7 @@
         </is>
       </c>
       <c r="G80" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-agente-mesa-de-ayuda-en-bogota-dc-E39FE355E02E578761373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-en-bogota-dc-48C2A0A3B050945661373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H80" s="6" t="inlineStr">
@@ -4270,7 +4266,7 @@
     <row r="81" ht="22" customHeight="1">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>0ef2cd7667600919</t>
+          <t>7e4b4e4f136a5e31</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
@@ -4280,12 +4276,12 @@
       </c>
       <c r="C81" s="3" t="inlineStr">
         <is>
-          <t>Técnico de Soporte TI Regional</t>
+          <t>Agente Mesa de Ayuda</t>
         </is>
       </c>
       <c r="D81" s="3" t="inlineStr">
         <is>
-          <t>POLICOMP COLOMBIA SAS</t>
+          <t>Importante empresa del sector</t>
         </is>
       </c>
       <c r="E81" s="7" t="n">
@@ -4297,10 +4293,14 @@
         </is>
       </c>
       <c r="G81" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-ti-regional-en-bogota-dc-ACF045C94E41CCDE61373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H81" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-agente-mesa-de-ayuda-en-bogota-dc-E39FE355E02E578761373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H81" s="6" t="inlineStr">
+        <is>
+          <t>$ 2.000.000,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I81" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -4316,7 +4316,7 @@
     <row r="82" ht="22" customHeight="1">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>7784997bda962255</t>
+          <t>0ef2cd7667600919</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
@@ -4326,7 +4326,7 @@
       </c>
       <c r="C82" s="3" t="inlineStr">
         <is>
-          <t>Técnico de Soporte TI On Demand/ por horas</t>
+          <t>Técnico de Soporte TI Regional</t>
         </is>
       </c>
       <c r="D82" s="3" t="inlineStr">
@@ -4343,7 +4343,7 @@
         </is>
       </c>
       <c r="G82" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-ti-on-demand-por-horas-en-bogota-dc-C2338FA0172D59A561373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-ti-regional-en-bogota-dc-ACF045C94E41CCDE61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H82" s="6" t="inlineStr"/>
@@ -4362,7 +4362,7 @@
     <row r="83" ht="22" customHeight="1">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>29d0fe2e42e678f7</t>
+          <t>7784997bda962255</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
@@ -4372,12 +4372,12 @@
       </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t>Técnico mantenimiento correctivo impresoras</t>
+          <t>Técnico de Soporte TI On Demand/ por horas</t>
         </is>
       </c>
       <c r="D83" s="3" t="inlineStr">
         <is>
-          <t>Multinacional de Impresión</t>
+          <t>POLICOMP COLOMBIA SAS</t>
         </is>
       </c>
       <c r="E83" s="7" t="n">
@@ -4389,14 +4389,10 @@
         </is>
       </c>
       <c r="G83" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-mantenimiento-correctivo-impresoras-en-guarne-BC0E775C0F25B27D61373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H83" s="6" t="inlineStr">
-        <is>
-          <t>$ 1.800.000,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-ti-on-demand-por-horas-en-bogota-dc-C2338FA0172D59A561373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H83" s="6" t="inlineStr"/>
       <c r="I83" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -4412,22 +4408,22 @@
     <row r="84" ht="22" customHeight="1">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>98c9ab11f5b1eace</t>
+          <t>29d0fe2e42e678f7</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 18:36</t>
+          <t>2026-09-27 15:41</t>
         </is>
       </c>
       <c r="C84" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar de sistemas</t>
+          <t>Técnico mantenimiento correctivo impresoras</t>
         </is>
       </c>
       <c r="D84" s="3" t="inlineStr">
         <is>
-          <t>Importante empresa del sector</t>
+          <t>Multinacional de Impresión</t>
         </is>
       </c>
       <c r="E84" s="7" t="n">
@@ -4439,12 +4435,12 @@
         </is>
       </c>
       <c r="G84" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-persona-con-discapacidad-remota-en-bogota-dc-5F2A812D014E159B61373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-mantenimiento-correctivo-impresoras-en-guarne-BC0E775C0F25B27D61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H84" s="6" t="inlineStr">
         <is>
-          <t>$ 1.750.905,00 (Mensual)</t>
+          <t>$ 1.800.000,00 (Mensual)</t>
         </is>
       </c>
       <c r="I84" s="3" t="inlineStr">
@@ -4462,7 +4458,7 @@
     <row r="85" ht="22" customHeight="1">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>58133ddc4da9c68e</t>
+          <t>98c9ab11f5b1eace</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
@@ -4489,7 +4485,7 @@
         </is>
       </c>
       <c r="G85" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-persona-con-discapacidad-remota-en-bogota-dc-A00C07C9CC9A494B61373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-persona-con-discapacidad-remota-en-bogota-dc-5F2A812D014E159B61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H85" s="6" t="inlineStr">
@@ -4512,7 +4508,7 @@
     <row r="86" ht="22" customHeight="1">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>aed3420a4cfdc248</t>
+          <t>58133ddc4da9c68e</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
@@ -4522,12 +4518,12 @@
       </c>
       <c r="C86" s="3" t="inlineStr">
         <is>
-          <t>Consultor de servicios/ mesa de ayuda nómina y erp software</t>
+          <t>Auxiliar de sistemas</t>
         </is>
       </c>
       <c r="D86" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Importante empresa del sector</t>
         </is>
       </c>
       <c r="E86" s="7" t="n">
@@ -4539,10 +4535,14 @@
         </is>
       </c>
       <c r="G86" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/consultor-de-servicios-mesa-de-ayuda-nomina-y-erp-software-inclusivo-1886716126", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H86" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-persona-con-discapacidad-remota-en-bogota-dc-A00C07C9CC9A494B61373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H86" s="6" t="inlineStr">
+        <is>
+          <t>$ 1.750.905,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I86" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -4558,22 +4558,22 @@
     <row r="87" ht="22" customHeight="1">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>2b8357189ff315da</t>
+          <t>aed3420a4cfdc248</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 17:00</t>
+          <t>2026-09-28 18:36</t>
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar de sistemas</t>
+          <t>Consultor de servicios/ mesa de ayuda nómina y erp software</t>
         </is>
       </c>
       <c r="D87" s="3" t="inlineStr">
         <is>
-          <t>DAVITA SAS</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E87" s="7" t="n">
@@ -4585,7 +4585,7 @@
         </is>
       </c>
       <c r="G87" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886758163", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/consultor-de-servicios-mesa-de-ayuda-nomina-y-erp-software-inclusivo-1886716126", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H87" s="6" t="inlineStr"/>
@@ -4604,7 +4604,7 @@
     <row r="88" ht="22" customHeight="1">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>a87934e7643b2c1c</t>
+          <t>2b8357189ff315da</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
@@ -4614,12 +4614,12 @@
       </c>
       <c r="C88" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de instalaciones cableado de redes - licencia conte cali</t>
+          <t>Auxiliar de sistemas</t>
         </is>
       </c>
       <c r="D88" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>DAVITA SAS</t>
         </is>
       </c>
       <c r="E88" s="7" t="n">
@@ -4631,7 +4631,7 @@
         </is>
       </c>
       <c r="G88" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-cali-1886759847", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886758163", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H88" s="6" t="inlineStr"/>
@@ -4650,7 +4650,7 @@
     <row r="89" ht="22" customHeight="1">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>10b4265e3ad11d81</t>
+          <t>a87934e7643b2c1c</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
@@ -4660,12 +4660,12 @@
       </c>
       <c r="C89" s="3" t="inlineStr">
         <is>
-          <t>Information Technology Help Desk Support</t>
+          <t>Tecnico de instalaciones cableado de redes - licencia conte cali</t>
         </is>
       </c>
       <c r="D89" s="3" t="inlineStr">
         <is>
-          <t>Booth</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E89" s="7" t="n">
@@ -4677,7 +4677,7 @@
         </is>
       </c>
       <c r="G89" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/information-technology-help-desk-support-at-booth-4471203962", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-cali-1886759847", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H89" s="6" t="inlineStr"/>
@@ -4696,22 +4696,22 @@
     <row r="90" ht="22" customHeight="1">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>ff69ae85c8697a37</t>
+          <t>10b4265e3ad11d81</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 16:49</t>
+          <t>2026-09-29 17:00</t>
         </is>
       </c>
       <c r="C90" s="3" t="inlineStr">
         <is>
-          <t>Técnico de soporte ti - bogota</t>
+          <t>Information Technology Help Desk Support</t>
         </is>
       </c>
       <c r="D90" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Booth</t>
         </is>
       </c>
       <c r="E90" s="7" t="n">
@@ -4723,7 +4723,7 @@
         </is>
       </c>
       <c r="G90" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-ti-bogota-1886774059", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/information-technology-help-desk-support-at-booth-4471203962", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H90" s="6" t="inlineStr"/>
@@ -4742,7 +4742,7 @@
     <row r="91" ht="22" customHeight="1">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>bbacf7d69ab9084e</t>
+          <t>ff69ae85c8697a37</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
@@ -4752,12 +4752,12 @@
       </c>
       <c r="C91" s="3" t="inlineStr">
         <is>
-          <t>IT Helpdesk Analyst</t>
+          <t>Técnico de soporte ti - bogota</t>
         </is>
       </c>
       <c r="D91" s="3" t="inlineStr">
         <is>
-          <t>Power Digital Marketing</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E91" s="7" t="n">
@@ -4769,7 +4769,7 @@
         </is>
       </c>
       <c r="G91" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/it-helpdesk-analyst-at-power-digital-marketing-4472601999", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-ti-bogota-1886774059", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H91" s="6" t="inlineStr"/>
@@ -4788,22 +4788,22 @@
     <row r="92" ht="22" customHeight="1">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>bb848f474ff4b611</t>
+          <t>bbacf7d69ab9084e</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 17:26</t>
+          <t>2026-09-30 16:49</t>
         </is>
       </c>
       <c r="C92" s="3" t="inlineStr">
         <is>
-          <t>Técnico de soporte ti - bogota</t>
+          <t>IT Helpdesk Analyst</t>
         </is>
       </c>
       <c r="D92" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Power Digital Marketing</t>
         </is>
       </c>
       <c r="E92" s="7" t="n">
@@ -4815,7 +4815,7 @@
         </is>
       </c>
       <c r="G92" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-ti-bogota-1886772292", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/it-helpdesk-analyst-at-power-digital-marketing-4472601999", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H92" s="6" t="inlineStr"/>
@@ -4834,7 +4834,7 @@
     <row r="93" ht="22" customHeight="1">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>b44a1c6cfb004ca8</t>
+          <t>bb848f474ff4b611</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
@@ -4844,7 +4844,7 @@
       </c>
       <c r="C93" s="3" t="inlineStr">
         <is>
-          <t>Soporte ti nivel 2 - bogotá</t>
+          <t>Técnico de soporte ti - bogota</t>
         </is>
       </c>
       <c r="D93" s="3" t="inlineStr">
@@ -4861,7 +4861,7 @@
         </is>
       </c>
       <c r="G93" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/soporte-ti-nivel-2-bogota-1886774821", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-ti-bogota-1886772292", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H93" s="6" t="inlineStr"/>
@@ -4880,7 +4880,7 @@
     <row r="94" ht="22" customHeight="1">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>fb0ad2b513afb97c</t>
+          <t>b44a1c6cfb004ca8</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
@@ -4890,12 +4890,12 @@
       </c>
       <c r="C94" s="3" t="inlineStr">
         <is>
-          <t>IT Help Desk Support Specialist</t>
+          <t>Soporte ti nivel 2 - bogotá</t>
         </is>
       </c>
       <c r="D94" s="3" t="inlineStr">
         <is>
-          <t>Talento</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E94" s="7" t="n">
@@ -4907,7 +4907,7 @@
         </is>
       </c>
       <c r="G94" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/it-help-desk-support-specialist-tier-1-at-talento-4473960480", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/soporte-ti-nivel-2-bogota-1886774821", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H94" s="6" t="inlineStr"/>
@@ -4926,22 +4926,22 @@
     <row r="95" ht="22" customHeight="1">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>0b2067d6ae488f4c</t>
+          <t>fb0ad2b513afb97c</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 16:39</t>
+          <t>2026-10-01 17:26</t>
         </is>
       </c>
       <c r="C95" s="3" t="inlineStr">
         <is>
-          <t>Help Desk Technician level 1</t>
+          <t>IT Help Desk Support Specialist</t>
         </is>
       </c>
       <c r="D95" s="3" t="inlineStr">
         <is>
-          <t>Solvo Global</t>
+          <t>Talento</t>
         </is>
       </c>
       <c r="E95" s="7" t="n">
@@ -4953,7 +4953,7 @@
         </is>
       </c>
       <c r="G95" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/help-desk-technician-level-1-at-solvo-global-4472590892", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/it-help-desk-support-specialist-tier-1-at-talento-4473960480", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H95" s="6" t="inlineStr"/>
@@ -4972,22 +4972,22 @@
     <row r="96" ht="22" customHeight="1">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>07acc222a3ca2ef1</t>
+          <t>0b2067d6ae488f4c</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03 15:12</t>
+          <t>2026-10-02 16:39</t>
         </is>
       </c>
       <c r="C96" s="3" t="inlineStr">
         <is>
-          <t>Analista mesa de ayuda funza temporal 6 meses</t>
+          <t>Help Desk Technician level 1</t>
         </is>
       </c>
       <c r="D96" s="3" t="inlineStr">
         <is>
-          <t>Axity</t>
+          <t>Solvo Global</t>
         </is>
       </c>
       <c r="E96" s="7" t="n">
@@ -4999,7 +4999,7 @@
         </is>
       </c>
       <c r="G96" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-funza-temporal-6-meses-1886774524", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/help-desk-technician-level-1-at-solvo-global-4472590892", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H96" s="6" t="inlineStr"/>
@@ -5018,22 +5018,22 @@
     <row r="97" ht="22" customHeight="1">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>5ec0ea33876ba2b5</t>
+          <t>07acc222a3ca2ef1</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 19:45</t>
+          <t>2026-10-03 15:12</t>
         </is>
       </c>
       <c r="C97" s="3" t="inlineStr">
         <is>
-          <t>Help desk analyst l1</t>
+          <t>Analista mesa de ayuda funza temporal 6 meses</t>
         </is>
       </c>
       <c r="D97" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Axity</t>
         </is>
       </c>
       <c r="E97" s="7" t="n">
@@ -5045,7 +5045,7 @@
         </is>
       </c>
       <c r="G97" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/help-desk-analyst-l1-medellin-1886776156", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-funza-temporal-6-meses-1886774524", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H97" s="6" t="inlineStr"/>
@@ -5064,7 +5064,7 @@
     <row r="98" ht="22" customHeight="1">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>e8bdf2094d1c9817</t>
+          <t>5ec0ea33876ba2b5</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
@@ -5074,12 +5074,12 @@
       </c>
       <c r="C98" s="3" t="inlineStr">
         <is>
-          <t>Administrador de herramienta de gestión de mesa de ayuda-</t>
+          <t>Help desk analyst l1</t>
         </is>
       </c>
       <c r="D98" s="3" t="inlineStr">
         <is>
-          <t>SELCOMP INGENIERÍA SAS</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E98" s="7" t="n">
@@ -5091,7 +5091,7 @@
         </is>
       </c>
       <c r="G98" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/administrador-de-herramienta-de-gestion-de-mesa-de-ayuda-1886776286", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/help-desk-analyst-l1-medellin-1886776156", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H98" s="6" t="inlineStr"/>
@@ -5110,7 +5110,7 @@
     <row r="99" ht="22" customHeight="1">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>6e9a077b42879470</t>
+          <t>e8bdf2094d1c9817</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
@@ -5120,12 +5120,12 @@
       </c>
       <c r="C99" s="3" t="inlineStr">
         <is>
-          <t>Analista de soporte de aplicaciones nivel 3</t>
+          <t>Administrador de herramienta de gestión de mesa de ayuda-</t>
         </is>
       </c>
       <c r="D99" s="3" t="inlineStr">
         <is>
-          <t>TALYCAP GLOBAL SAS</t>
+          <t>SELCOMP INGENIERÍA SAS</t>
         </is>
       </c>
       <c r="E99" s="7" t="n">
@@ -5137,7 +5137,7 @@
         </is>
       </c>
       <c r="G99" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-soporte-de-aplicaciones-nivel-3-1886776104", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/administrador-de-herramienta-de-gestion-de-mesa-de-ayuda-1886776286", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H99" s="6" t="inlineStr"/>
@@ -5156,22 +5156,22 @@
     <row r="100" ht="22" customHeight="1">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>447afec244b20f9b</t>
+          <t>6e9a077b42879470</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06 17:12</t>
+          <t>2026-10-05 19:45</t>
         </is>
       </c>
       <c r="C100" s="3" t="inlineStr">
         <is>
-          <t>Técnico de soporte ti - bogota</t>
+          <t>Analista de soporte de aplicaciones nivel 3</t>
         </is>
       </c>
       <c r="D100" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>TALYCAP GLOBAL SAS</t>
         </is>
       </c>
       <c r="E100" s="7" t="n">
@@ -5183,7 +5183,7 @@
         </is>
       </c>
       <c r="G100" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-ti-bogota-1886775990", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-soporte-de-aplicaciones-nivel-3-1886776104", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H100" s="6" t="inlineStr"/>
@@ -5202,22 +5202,22 @@
     <row r="101" ht="22" customHeight="1">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>8f14c41f3b443ac0</t>
+          <t>447afec244b20f9b</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07 17:50</t>
+          <t>2026-10-06 17:12</t>
         </is>
       </c>
       <c r="C101" s="3" t="inlineStr">
         <is>
-          <t>Soporte mesa de ayuda</t>
+          <t>Técnico de soporte ti - bogota</t>
         </is>
       </c>
       <c r="D101" s="3" t="inlineStr">
         <is>
-          <t>MANPOWER</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E101" s="7" t="n">
@@ -5229,7 +5229,7 @@
         </is>
       </c>
       <c r="G101" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/soporte-mesa-de-ayuda-vacaciones-1886776917", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-ti-bogota-1886775990", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H101" s="6" t="inlineStr"/>
@@ -5248,7 +5248,7 @@
     <row r="102" ht="22" customHeight="1">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>b1a9e03967fff91e</t>
+          <t>8f14c41f3b443ac0</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
@@ -5258,12 +5258,12 @@
       </c>
       <c r="C102" s="3" t="inlineStr">
         <is>
-          <t>Tecnólogo de soporte pl - mesa de ayuda</t>
+          <t>Soporte mesa de ayuda</t>
         </is>
       </c>
       <c r="D102" s="3" t="inlineStr">
         <is>
-          <t>Positivo S+</t>
+          <t>MANPOWER</t>
         </is>
       </c>
       <c r="E102" s="7" t="n">
@@ -5275,7 +5275,7 @@
         </is>
       </c>
       <c r="G102" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnologo-de-soporte-pl-mesa-de-ayuda-1886775546", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/soporte-mesa-de-ayuda-vacaciones-1886776917", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H102" s="6" t="inlineStr"/>
@@ -5294,7 +5294,7 @@
     <row r="103" ht="22" customHeight="1">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>eb49981c97933d93</t>
+          <t>b1a9e03967fff91e</t>
         </is>
       </c>
       <c r="B103" s="2" t="inlineStr">
@@ -5304,12 +5304,12 @@
       </c>
       <c r="C103" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de instalaciones cableado de redes - licencia conte</t>
+          <t>Tecnólogo de soporte pl - mesa de ayuda</t>
         </is>
       </c>
       <c r="D103" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Positivo S+</t>
         </is>
       </c>
       <c r="E103" s="7" t="n">
@@ -5321,7 +5321,7 @@
         </is>
       </c>
       <c r="G103" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-1886777333", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnologo-de-soporte-pl-mesa-de-ayuda-1886775546", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H103" s="6" t="inlineStr"/>
@@ -5340,7 +5340,7 @@
     <row r="104" ht="22" customHeight="1">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>d39af22b6e937d28</t>
+          <t>eb49981c97933d93</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
@@ -5350,12 +5350,12 @@
       </c>
       <c r="C104" s="3" t="inlineStr">
         <is>
-          <t>Analista Mesa de Ayuda Funza</t>
+          <t>Tecnico de instalaciones cableado de redes - licencia conte</t>
         </is>
       </c>
       <c r="D104" s="3" t="inlineStr">
         <is>
-          <t>axity</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E104" s="7" t="n">
@@ -5367,7 +5367,7 @@
         </is>
       </c>
       <c r="G104" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/analista-mesa-de-ayuda-funza-at-axity-4471985006", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-1886777333", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H104" s="6" t="inlineStr"/>
@@ -5386,22 +5386,22 @@
     <row r="105" ht="22" customHeight="1">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>0904912d51c5cd61</t>
+          <t>d39af22b6e937d28</t>
         </is>
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08 17:52</t>
+          <t>2026-10-07 17:50</t>
         </is>
       </c>
       <c r="C105" s="3" t="inlineStr">
         <is>
-          <t>Analista mesa de ayuda</t>
+          <t>Analista Mesa de Ayuda Funza</t>
         </is>
       </c>
       <c r="D105" s="3" t="inlineStr">
         <is>
-          <t>Desarrollo de Sistemas y Servicios SAS</t>
+          <t>axity</t>
         </is>
       </c>
       <c r="E105" s="7" t="n">
@@ -5413,7 +5413,7 @@
         </is>
       </c>
       <c r="G105" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-1886778032", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/analista-mesa-de-ayuda-funza-at-axity-4471985006", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H105" s="6" t="inlineStr"/>
@@ -5432,22 +5432,22 @@
     <row r="106" ht="22" customHeight="1">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>c665ada630270dce</t>
+          <t>0904912d51c5cd61</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09 17:28</t>
+          <t>2026-10-08 17:52</t>
         </is>
       </c>
       <c r="C106" s="3" t="inlineStr">
         <is>
-          <t>Técnico(a) / tecnólogo(a) / profesional de telecomunicaciones - redes de fibra óptica</t>
+          <t>Analista mesa de ayuda</t>
         </is>
       </c>
       <c r="D106" s="3" t="inlineStr">
         <is>
-          <t>JAHV MC GREGOR S.A.S</t>
+          <t>Desarrollo de Sistemas y Servicios SAS</t>
         </is>
       </c>
       <c r="E106" s="7" t="n">
@@ -5459,7 +5459,7 @@
         </is>
       </c>
       <c r="G106" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnicoa-tecnologoa-profesional-de-telecomunicaciones-redes-de-fibra-optica-1886768691", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-1886778032", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H106" s="6" t="inlineStr"/>
@@ -5478,7 +5478,7 @@
     <row r="107" ht="22" customHeight="1">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>4e5b3128aa7f8f9b</t>
+          <t>c665ada630270dce</t>
         </is>
       </c>
       <c r="B107" s="2" t="inlineStr">
@@ -5488,12 +5488,12 @@
       </c>
       <c r="C107" s="3" t="inlineStr">
         <is>
-          <t>Gestor de servicios mesa de ayuda sap</t>
+          <t>Técnico(a) / tecnólogo(a) / profesional de telecomunicaciones - redes de fibra óptica</t>
         </is>
       </c>
       <c r="D107" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>JAHV MC GREGOR S.A.S</t>
         </is>
       </c>
       <c r="E107" s="7" t="n">
@@ -5505,7 +5505,7 @@
         </is>
       </c>
       <c r="G107" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/gestor-de-servicios-mesa-de-ayuda-sap-1886775732", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnicoa-tecnologoa-profesional-de-telecomunicaciones-redes-de-fibra-optica-1886768691", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H107" s="6" t="inlineStr"/>
@@ -5524,7 +5524,7 @@
     <row r="108" ht="22" customHeight="1">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>1c92f7ef9b7af696</t>
+          <t>4e5b3128aa7f8f9b</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr">
@@ -5534,7 +5534,7 @@
       </c>
       <c r="C108" s="3" t="inlineStr">
         <is>
-          <t>Agente de mesa de ayuda nivel 1</t>
+          <t>Gestor de servicios mesa de ayuda sap</t>
         </is>
       </c>
       <c r="D108" s="3" t="inlineStr">
@@ -5551,7 +5551,7 @@
         </is>
       </c>
       <c r="G108" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-de-mesa-de-ayuda-nivel-1-1886778506", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/gestor-de-servicios-mesa-de-ayuda-sap-1886775732", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H108" s="6" t="inlineStr"/>
@@ -5570,22 +5570,22 @@
     <row r="109" ht="22" customHeight="1">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>718ceee355d457ea</t>
+          <t>1c92f7ef9b7af696</t>
         </is>
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10 16:16</t>
+          <t>2026-10-09 17:28</t>
         </is>
       </c>
       <c r="C109" s="3" t="inlineStr">
         <is>
-          <t>IT Help Desk Support</t>
+          <t>Agente de mesa de ayuda nivel 1</t>
         </is>
       </c>
       <c r="D109" s="3" t="inlineStr">
         <is>
-          <t>Booth</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E109" s="7" t="n">
@@ -5597,7 +5597,7 @@
         </is>
       </c>
       <c r="G109" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/it-help-desk-support-at-booth-4471203962", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-de-mesa-de-ayuda-nivel-1-1886778506", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H109" s="6" t="inlineStr"/>
@@ -5616,22 +5616,22 @@
     <row r="110" ht="22" customHeight="1">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>925f43273b78f188</t>
+          <t>718ceee355d457ea</t>
         </is>
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12 20:17</t>
+          <t>2026-10-10 16:16</t>
         </is>
       </c>
       <c r="C110" s="3" t="inlineStr">
         <is>
-          <t>Mesa de ayuda ti - girón</t>
+          <t>IT Help Desk Support</t>
         </is>
       </c>
       <c r="D110" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Booth</t>
         </is>
       </c>
       <c r="E110" s="7" t="n">
@@ -5643,7 +5643,7 @@
         </is>
       </c>
       <c r="G110" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/mesa-de-ayuda-ti-giron-1886745168", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/it-help-desk-support-at-booth-4471203962", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H110" s="6" t="inlineStr"/>
@@ -5662,22 +5662,22 @@
     <row r="111" ht="22" customHeight="1">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>ec0c8875e04f4933</t>
+          <t>925f43273b78f188</t>
         </is>
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13 18:08</t>
+          <t>2026-10-12 20:17</t>
         </is>
       </c>
       <c r="C111" s="3" t="inlineStr">
         <is>
-          <t>Analista de mesa de ayuda.</t>
+          <t>Mesa de ayuda ti - girón</t>
         </is>
       </c>
       <c r="D111" s="3" t="inlineStr">
         <is>
-          <t>Softtek Colombia</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E111" s="7" t="n">
@@ -5689,7 +5689,7 @@
         </is>
       </c>
       <c r="G111" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-mesa-de-ayuda-1886754207", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/mesa-de-ayuda-ti-giron-1886745168", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H111" s="6" t="inlineStr"/>
@@ -5708,7 +5708,7 @@
     <row r="112" ht="22" customHeight="1">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>87fac63aa714f401</t>
+          <t>ec0c8875e04f4933</t>
         </is>
       </c>
       <c r="B112" s="2" t="inlineStr">
@@ -5718,7 +5718,7 @@
       </c>
       <c r="C112" s="3" t="inlineStr">
         <is>
-          <t>Agente mesa de ayuda.</t>
+          <t>Analista de mesa de ayuda.</t>
         </is>
       </c>
       <c r="D112" s="3" t="inlineStr">
@@ -5735,7 +5735,7 @@
         </is>
       </c>
       <c r="G112" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-mesa-de-ayuda-1886753535", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-mesa-de-ayuda-1886754207", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H112" s="6" t="inlineStr"/>
@@ -5754,26 +5754,26 @@
     <row r="113" ht="22" customHeight="1">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>50c79dfbfd49f52d</t>
+          <t>87fac63aa714f401</t>
         </is>
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 16:39</t>
+          <t>2026-10-13 18:08</t>
         </is>
       </c>
       <c r="C113" s="3" t="inlineStr">
         <is>
-          <t>Analista de redes noc 1 telecomunicaciones.</t>
+          <t>Agente mesa de ayuda.</t>
         </is>
       </c>
       <c r="D113" s="3" t="inlineStr">
         <is>
-          <t>MANPOWER</t>
+          <t>Softtek Colombia</t>
         </is>
       </c>
       <c r="E113" s="7" t="n">
-        <v>0.53</v>
+        <v>0.58</v>
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
@@ -5781,13 +5781,13 @@
         </is>
       </c>
       <c r="G113" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-noc-1-telecomunicaciones-1886772075", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-mesa-de-ayuda-1886753535", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H113" s="6" t="inlineStr"/>
       <c r="I113" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J113" s="2" t="inlineStr">
@@ -5800,26 +5800,26 @@
     <row r="114" ht="22" customHeight="1">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>0b0ae49f910109bb</t>
+          <t>50c79dfbfd49f52d</t>
         </is>
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 15:54</t>
+          <t>2026-10-02 16:39</t>
         </is>
       </c>
       <c r="C114" s="3" t="inlineStr">
         <is>
-          <t>Ejecutivo Técnico Arancel Junior</t>
+          <t>Analista de redes noc 1 telecomunicaciones.</t>
         </is>
       </c>
       <c r="D114" s="3" t="inlineStr">
         <is>
-          <t>Importante Empresa de Logística y Comercio</t>
+          <t>MANPOWER</t>
         </is>
       </c>
       <c r="E114" s="7" t="n">
-        <v>0.5</v>
+        <v>0.53</v>
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
@@ -5827,17 +5827,13 @@
         </is>
       </c>
       <c r="G114" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-547866639B487E0161373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H114" s="6" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-noc-1-telecomunicaciones-1886772075", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H114" s="6" t="inlineStr"/>
       <c r="I114" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J114" s="2" t="inlineStr">
@@ -5850,22 +5846,22 @@
     <row r="115" ht="22" customHeight="1">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>582a04b3c639bfa0</t>
+          <t>0b0ae49f910109bb</t>
         </is>
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 16:49</t>
+          <t>2026-09-25 15:54</t>
         </is>
       </c>
       <c r="C115" s="3" t="inlineStr">
         <is>
-          <t>Junior IT Support Specialist</t>
+          <t>Ejecutivo Técnico Arancel Junior</t>
         </is>
       </c>
       <c r="D115" s="3" t="inlineStr">
         <is>
-          <t>Touch Support, Inc. &amp; SNF Back Office</t>
+          <t>Importante Empresa de Logística y Comercio</t>
         </is>
       </c>
       <c r="E115" s="7" t="n">
@@ -5877,10 +5873,14 @@
         </is>
       </c>
       <c r="G115" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/junior-it-support-specialist-at-touch-support-inc-snf-back-office-4472187578", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H115" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-547866639B487E0161373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H115" s="6" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
       <c r="I115" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -5896,22 +5896,22 @@
     <row r="116" ht="22" customHeight="1">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>6e04c4d57d3fc3c7</t>
+          <t>582a04b3c639bfa0</t>
         </is>
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 17:26</t>
+          <t>2026-09-30 16:49</t>
         </is>
       </c>
       <c r="C116" s="3" t="inlineStr">
         <is>
-          <t>Ejecutivo Técnico Arancel Junior</t>
+          <t>Junior IT Support Specialist</t>
         </is>
       </c>
       <c r="D116" s="3" t="inlineStr">
         <is>
-          <t>Importante Empresa de Logística y Comercio</t>
+          <t>Touch Support, Inc. &amp; SNF Back Office</t>
         </is>
       </c>
       <c r="E116" s="7" t="n">
@@ -5923,25 +5923,71 @@
         </is>
       </c>
       <c r="G116" s="5">
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/junior-it-support-specialist-at-touch-support-inc-snf-back-office-4472187578", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H116" s="6" t="inlineStr"/>
+      <c r="I116" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J116" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K116" s="3" t="inlineStr"/>
+    </row>
+    <row r="117" ht="22" customHeight="1">
+      <c r="A117" s="2" t="inlineStr">
+        <is>
+          <t>6e04c4d57d3fc3c7</t>
+        </is>
+      </c>
+      <c r="B117" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01 17:26</t>
+        </is>
+      </c>
+      <c r="C117" s="3" t="inlineStr">
+        <is>
+          <t>Ejecutivo Técnico Arancel Junior</t>
+        </is>
+      </c>
+      <c r="D117" s="3" t="inlineStr">
+        <is>
+          <t>Importante Empresa de Logística y Comercio</t>
+        </is>
+      </c>
+      <c r="E117" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F117" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G117" s="5">
         <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-8444AB594560844161373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
-      <c r="H116" s="6" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
-      <c r="I116" s="3" t="inlineStr">
+      <c r="H117" s="6" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="I117" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
-      <c r="J116" s="2" t="inlineStr">
-        <is>
-          <t>Nueva</t>
-        </is>
-      </c>
-      <c r="K116" s="3" t="inlineStr"/>
+      <c r="J117" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K117" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
chore(tracker): actualizacion diaria de vacantes 2026-10-15
</commit_message>
<xml_diff>
--- a/output/profile_5_tecnico_sistemas_tracker.xlsx
+++ b/output/profile_5_tecnico_sistemas_tracker.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K117"/>
+  <dimension ref="A1:K118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -5800,26 +5800,26 @@
     <row r="114" ht="22" customHeight="1">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>50c79dfbfd49f52d</t>
+          <t>dfa7dd88fd24afb4</t>
         </is>
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 16:39</t>
+          <t>2026-10-15 15:40</t>
         </is>
       </c>
       <c r="C114" s="3" t="inlineStr">
         <is>
-          <t>Analista de redes noc 1 telecomunicaciones.</t>
+          <t>Agente mesa de ayuda nivel 1 ingles avanzado</t>
         </is>
       </c>
       <c r="D114" s="3" t="inlineStr">
         <is>
-          <t>MANPOWER</t>
+          <t>SUSTS Colombia Ltda.</t>
         </is>
       </c>
       <c r="E114" s="7" t="n">
-        <v>0.53</v>
+        <v>0.58</v>
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
@@ -5827,13 +5827,13 @@
         </is>
       </c>
       <c r="G114" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-noc-1-telecomunicaciones-1886772075", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-mesa-de-ayuda-nivel-1-ingles-avanzado-1886780371", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H114" s="6" t="inlineStr"/>
       <c r="I114" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J114" s="2" t="inlineStr">
@@ -5846,26 +5846,26 @@
     <row r="115" ht="22" customHeight="1">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>0b0ae49f910109bb</t>
+          <t>50c79dfbfd49f52d</t>
         </is>
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 15:54</t>
+          <t>2026-10-02 16:39</t>
         </is>
       </c>
       <c r="C115" s="3" t="inlineStr">
         <is>
-          <t>Ejecutivo Técnico Arancel Junior</t>
+          <t>Analista de redes noc 1 telecomunicaciones.</t>
         </is>
       </c>
       <c r="D115" s="3" t="inlineStr">
         <is>
-          <t>Importante Empresa de Logística y Comercio</t>
+          <t>MANPOWER</t>
         </is>
       </c>
       <c r="E115" s="7" t="n">
-        <v>0.5</v>
+        <v>0.53</v>
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
@@ -5873,17 +5873,13 @@
         </is>
       </c>
       <c r="G115" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-547866639B487E0161373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H115" s="6" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-noc-1-telecomunicaciones-1886772075", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H115" s="6" t="inlineStr"/>
       <c r="I115" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J115" s="2" t="inlineStr">
@@ -5896,22 +5892,22 @@
     <row r="116" ht="22" customHeight="1">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>582a04b3c639bfa0</t>
+          <t>0b0ae49f910109bb</t>
         </is>
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 16:49</t>
+          <t>2026-09-25 15:54</t>
         </is>
       </c>
       <c r="C116" s="3" t="inlineStr">
         <is>
-          <t>Junior IT Support Specialist</t>
+          <t>Ejecutivo Técnico Arancel Junior</t>
         </is>
       </c>
       <c r="D116" s="3" t="inlineStr">
         <is>
-          <t>Touch Support, Inc. &amp; SNF Back Office</t>
+          <t>Importante Empresa de Logística y Comercio</t>
         </is>
       </c>
       <c r="E116" s="7" t="n">
@@ -5923,10 +5919,14 @@
         </is>
       </c>
       <c r="G116" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/junior-it-support-specialist-at-touch-support-inc-snf-back-office-4472187578", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H116" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-547866639B487E0161373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H116" s="6" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
       <c r="I116" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -5942,22 +5942,22 @@
     <row r="117" ht="22" customHeight="1">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>6e04c4d57d3fc3c7</t>
+          <t>582a04b3c639bfa0</t>
         </is>
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 17:26</t>
+          <t>2026-09-30 16:49</t>
         </is>
       </c>
       <c r="C117" s="3" t="inlineStr">
         <is>
-          <t>Ejecutivo Técnico Arancel Junior</t>
+          <t>Junior IT Support Specialist</t>
         </is>
       </c>
       <c r="D117" s="3" t="inlineStr">
         <is>
-          <t>Importante Empresa de Logística y Comercio</t>
+          <t>Touch Support, Inc. &amp; SNF Back Office</t>
         </is>
       </c>
       <c r="E117" s="7" t="n">
@@ -5969,25 +5969,71 @@
         </is>
       </c>
       <c r="G117" s="5">
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/junior-it-support-specialist-at-touch-support-inc-snf-back-office-4472187578", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H117" s="6" t="inlineStr"/>
+      <c r="I117" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J117" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K117" s="3" t="inlineStr"/>
+    </row>
+    <row r="118" ht="22" customHeight="1">
+      <c r="A118" s="2" t="inlineStr">
+        <is>
+          <t>6e04c4d57d3fc3c7</t>
+        </is>
+      </c>
+      <c r="B118" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01 17:26</t>
+        </is>
+      </c>
+      <c r="C118" s="3" t="inlineStr">
+        <is>
+          <t>Ejecutivo Técnico Arancel Junior</t>
+        </is>
+      </c>
+      <c r="D118" s="3" t="inlineStr">
+        <is>
+          <t>Importante Empresa de Logística y Comercio</t>
+        </is>
+      </c>
+      <c r="E118" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F118" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G118" s="5">
         <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-8444AB594560844161373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
-      <c r="H117" s="6" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
-      <c r="I117" s="3" t="inlineStr">
+      <c r="H118" s="6" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="I118" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
-      <c r="J117" s="2" t="inlineStr">
-        <is>
-          <t>Nueva</t>
-        </is>
-      </c>
-      <c r="K117" s="3" t="inlineStr"/>
+      <c r="J118" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K118" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
chore(tracker): actualizacion diaria de vacantes 2026-10-16
</commit_message>
<xml_diff>
--- a/output/profile_5_tecnico_sistemas_tracker.xlsx
+++ b/output/profile_5_tecnico_sistemas_tracker.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K118"/>
+  <dimension ref="A1:K124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3426,26 +3426,26 @@
     <row r="63" ht="22" customHeight="1">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>ae736277661dc78b</t>
+          <t>1495b0203ce51c84</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 15:23</t>
+          <t>2026-10-16 15:22</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>Analista de redes cisco</t>
+          <t>Analista de soporte técnico TI</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>ATCG DE COLOMBIA S.A.S</t>
-        </is>
-      </c>
-      <c r="E63" s="7" t="n">
-        <v>0.68</v>
+          <t>Salesland Colombia</t>
+        </is>
+      </c>
+      <c r="E63" s="4" t="n">
+        <v>0.73</v>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
@@ -3453,13 +3453,17 @@
         </is>
       </c>
       <c r="G63" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-cisco-1886760389", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H63" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-analista-de-soporte-tecnico-ti-en-bogota-dc-AB1F1A0EC252EFA061373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H63" s="6" t="inlineStr">
+        <is>
+          <t>$ 3.600.000,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I63" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 68/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 73/100 - Alta Afinidad] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J63" s="2" t="inlineStr">
@@ -3472,26 +3476,26 @@
     <row r="64" ht="22" customHeight="1">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>e29676fac3409ad6</t>
+          <t>77ab2968500ab26e</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 15:23</t>
+          <t>2026-10-16 15:22</t>
         </is>
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>Analista de redes y telecomunicaciones - nivel 1</t>
+          <t>Auxiliar de Soporte Técnico – Equipos y Dispositivos Móviles</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t>MANPOWER</t>
-        </is>
-      </c>
-      <c r="E64" s="7" t="n">
-        <v>0.68</v>
+          <t>Nases EST</t>
+        </is>
+      </c>
+      <c r="E64" s="4" t="n">
+        <v>0.73</v>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
@@ -3499,13 +3503,17 @@
         </is>
       </c>
       <c r="G64" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-y-telecomunicaciones-nivel-1-1886760565", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H64" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-soporte-tecnico-equipos-y-dispositivos-moviles-multinacional-de-consumo-masivo-en-bogota-dc-4F6AAF66DBFB586861373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H64" s="6" t="inlineStr">
+        <is>
+          <t>$ 2.573.000,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I64" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 68/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 73/100 - Alta Afinidad] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr">
@@ -3518,26 +3526,26 @@
     <row r="65" ht="22" customHeight="1">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>baf000f38713dc11</t>
+          <t>d391690839cf39de</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07 17:50</t>
+          <t>2026-10-16 15:22</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>Helpdesk / Analista soporte TI / trilingüe</t>
+          <t>Analista de Soporte Técnico y Mesa de Ayuda TI</t>
         </is>
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>Confidential</t>
-        </is>
-      </c>
-      <c r="E65" s="7" t="n">
-        <v>0.66</v>
+          <t>E-GLOBAL S.A.</t>
+        </is>
+      </c>
+      <c r="E65" s="4" t="n">
+        <v>0.73</v>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
@@ -3545,13 +3553,17 @@
         </is>
       </c>
       <c r="G65" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/helpdesk-analista-soporte-ti-triling%C3%BCe-ingles-portugu%C3%A9s-at-confidential-4469673592", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H65" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-analista-de-soporte-tecnico-y-mesa-de-ayuda-ti-en-medellin-1DDB06FA36E0C3B361373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H65" s="6" t="inlineStr">
+        <is>
+          <t>$ 2.101.215,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I65" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 66/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 73/100 - Alta Afinidad] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J65" s="2" t="inlineStr">
@@ -3564,26 +3576,26 @@
     <row r="66" ht="22" customHeight="1">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>422a27df3967ecbb</t>
+          <t>92dec0af0aaf5cbf</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14 15:52</t>
+          <t>2026-10-16 15:22</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>Técnico de sistemas y soporte ti</t>
+          <t>Agente de soporte técnico</t>
         </is>
       </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
-          <t>AGENCIA DE EMPLEO CAFAM</t>
-        </is>
-      </c>
-      <c r="E66" s="7" t="n">
-        <v>0.66</v>
+          <t>SUMMAR PRODUCTIVIDAD S.A.S</t>
+        </is>
+      </c>
+      <c r="E66" s="4" t="n">
+        <v>0.73</v>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
@@ -3591,13 +3603,13 @@
         </is>
       </c>
       <c r="G66" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-sistemas-y-soporte-ti-1886780022", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-de-soporte-tecnico-1886779162", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H66" s="6" t="inlineStr"/>
       <c r="I66" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 66/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 73/100 - Alta Afinidad] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J66" s="2" t="inlineStr">
@@ -3610,26 +3622,26 @@
     <row r="67" ht="22" customHeight="1">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>73882c81e04abc7e</t>
+          <t>ae736277661dc78b</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 19:45</t>
+          <t>2026-09-24 15:23</t>
         </is>
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>Soporte L1 Junior</t>
+          <t>Analista de redes cisco</t>
         </is>
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>Hublance</t>
+          <t>ATCG DE COLOMBIA S.A.S</t>
         </is>
       </c>
       <c r="E67" s="7" t="n">
-        <v>0.6</v>
+        <v>0.68</v>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
@@ -3637,13 +3649,13 @@
         </is>
       </c>
       <c r="G67" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/soporte-l1-junior-at-hublance-4475841269", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-cisco-1886760389", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H67" s="6" t="inlineStr"/>
       <c r="I67" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 60/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 68/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J67" s="2" t="inlineStr">
@@ -3656,26 +3668,26 @@
     <row r="68" ht="22" customHeight="1">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>8d7f304ffb8625b5</t>
+          <t>e29676fac3409ad6</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 15:54</t>
+          <t>2026-09-24 15:23</t>
         </is>
       </c>
       <c r="C68" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar de sistemas</t>
+          <t>Analista de redes y telecomunicaciones - nivel 1</t>
         </is>
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>MANPOWER</t>
         </is>
       </c>
       <c r="E68" s="7" t="n">
-        <v>0.58</v>
+        <v>0.68</v>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
@@ -3683,13 +3695,13 @@
         </is>
       </c>
       <c r="G68" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886751888", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-y-telecomunicaciones-nivel-1-1886760565", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H68" s="6" t="inlineStr"/>
       <c r="I68" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 68/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J68" s="2" t="inlineStr">
@@ -3702,26 +3714,26 @@
     <row r="69" ht="22" customHeight="1">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>3b5b26f92a305c0c</t>
+          <t>baf000f38713dc11</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 15:54</t>
+          <t>2026-10-07 17:50</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar de sistemas</t>
+          <t>Helpdesk / Analista soporte TI / trilingüe</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Confidential</t>
         </is>
       </c>
       <c r="E69" s="7" t="n">
-        <v>0.58</v>
+        <v>0.66</v>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
@@ -3729,13 +3741,13 @@
         </is>
       </c>
       <c r="G69" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886749497", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/helpdesk-analista-soporte-ti-triling%C3%BCe-ingles-portugu%C3%A9s-at-confidential-4469673592", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H69" s="6" t="inlineStr"/>
       <c r="I69" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 66/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J69" s="2" t="inlineStr">
@@ -3748,26 +3760,26 @@
     <row r="70" ht="22" customHeight="1">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>e760bcd88d90fbbe</t>
+          <t>422a27df3967ecbb</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 15:54</t>
+          <t>2026-10-14 15:52</t>
         </is>
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>Agente de mesa de ayuda</t>
+          <t>Técnico de sistemas y soporte ti</t>
         </is>
       </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
-          <t>SELCOMP INGENIERÍA SAS</t>
+          <t>AGENCIA DE EMPLEO CAFAM</t>
         </is>
       </c>
       <c r="E70" s="7" t="n">
-        <v>0.58</v>
+        <v>0.66</v>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
@@ -3775,13 +3787,13 @@
         </is>
       </c>
       <c r="G70" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-de-mesa-de-ayuda-1886758623", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-sistemas-y-soporte-ti-1886780022", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H70" s="6" t="inlineStr"/>
       <c r="I70" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 66/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J70" s="2" t="inlineStr">
@@ -3794,26 +3806,26 @@
     <row r="71" ht="22" customHeight="1">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>86dcab5c5d802693</t>
+          <t>73882c81e04abc7e</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 15:54</t>
+          <t>2026-10-05 19:45</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>Analista mesa de ayuda para tunja</t>
+          <t>Soporte L1 Junior</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>Gestión de Seguridad Electrónica</t>
+          <t>Hublance</t>
         </is>
       </c>
       <c r="E71" s="7" t="n">
-        <v>0.58</v>
+        <v>0.6</v>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
@@ -3821,13 +3833,13 @@
         </is>
       </c>
       <c r="G71" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-para-tunja-1886766955", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/soporte-l1-junior-at-hublance-4475841269", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H71" s="6" t="inlineStr"/>
       <c r="I71" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 60/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J71" s="2" t="inlineStr">
@@ -3840,7 +3852,7 @@
     <row r="72" ht="22" customHeight="1">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>55fdaa0983ef9124</t>
+          <t>8d7f304ffb8625b5</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -3850,12 +3862,12 @@
       </c>
       <c r="C72" s="3" t="inlineStr">
         <is>
-          <t>Lider técnico con itil practice manager</t>
+          <t>Auxiliar de sistemas</t>
         </is>
       </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
-          <t>Sinergy &amp; Lowells</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E72" s="7" t="n">
@@ -3867,7 +3879,7 @@
         </is>
       </c>
       <c r="G72" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/lider-tecnico-con-itil-practice-manager-1886753953", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886751888", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H72" s="6" t="inlineStr"/>
@@ -3886,7 +3898,7 @@
     <row r="73" ht="22" customHeight="1">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>a1ca7bc58cd48fad</t>
+          <t>3b5b26f92a305c0c</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
@@ -3896,7 +3908,7 @@
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de mesa de ayuda/mujeres contratacion inmediata</t>
+          <t>Auxiliar de sistemas</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr">
@@ -3913,7 +3925,7 @@
         </is>
       </c>
       <c r="G73" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-mesa-de-ayuda-mujeres-contratacion-inmediata-1886770931", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886749497", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H73" s="6" t="inlineStr"/>
@@ -3932,7 +3944,7 @@
     <row r="74" ht="22" customHeight="1">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>e28aba5df8a2d3ae</t>
+          <t>e760bcd88d90fbbe</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
@@ -3942,12 +3954,12 @@
       </c>
       <c r="C74" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de mesa de ayuda/mujeres contratacion inmediata</t>
+          <t>Agente de mesa de ayuda</t>
         </is>
       </c>
       <c r="D74" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>SELCOMP INGENIERÍA SAS</t>
         </is>
       </c>
       <c r="E74" s="7" t="n">
@@ -3959,7 +3971,7 @@
         </is>
       </c>
       <c r="G74" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-mesa-de-ayuda-mujeres-contratacion-inmediata-1886769701", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-de-mesa-de-ayuda-1886758623", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H74" s="6" t="inlineStr"/>
@@ -3978,7 +3990,7 @@
     <row r="75" ht="22" customHeight="1">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>9326784c1a2726fb</t>
+          <t>86dcab5c5d802693</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
@@ -3988,12 +4000,12 @@
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>Técnico de soporte y mesa de ayuda / medellín</t>
+          <t>Analista mesa de ayuda para tunja</t>
         </is>
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>Colsof S.A.S</t>
+          <t>Gestión de Seguridad Electrónica</t>
         </is>
       </c>
       <c r="E75" s="7" t="n">
@@ -4005,7 +4017,7 @@
         </is>
       </c>
       <c r="G75" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-y-mesa-de-ayuda-medellin-1886738118", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-para-tunja-1886766955", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H75" s="6" t="inlineStr"/>
@@ -4024,7 +4036,7 @@
     <row r="76" ht="22" customHeight="1">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>b67dc9a9be4a1a6f</t>
+          <t>55fdaa0983ef9124</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
@@ -4034,12 +4046,12 @@
       </c>
       <c r="C76" s="3" t="inlineStr">
         <is>
-          <t>Service desk agent</t>
+          <t>Lider técnico con itil practice manager</t>
         </is>
       </c>
       <c r="D76" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Sinergy &amp; Lowells</t>
         </is>
       </c>
       <c r="E76" s="7" t="n">
@@ -4051,13 +4063,13 @@
         </is>
       </c>
       <c r="G76" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/service-desk-agent-soporte-tecnico-nivel-1-1886755112", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/lider-tecnico-con-itil-practice-manager-1886753953", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H76" s="6" t="inlineStr"/>
       <c r="I76" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J76" s="2" t="inlineStr">
@@ -4070,7 +4082,7 @@
     <row r="77" ht="22" customHeight="1">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>9c65f710f43158b7</t>
+          <t>a1ca7bc58cd48fad</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
@@ -4080,7 +4092,7 @@
       </c>
       <c r="C77" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de instalaciones cableado de redes - licencia conte</t>
+          <t>Tecnico de mesa de ayuda/mujeres contratacion inmediata</t>
         </is>
       </c>
       <c r="D77" s="3" t="inlineStr">
@@ -4097,7 +4109,7 @@
         </is>
       </c>
       <c r="G77" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-1886749397", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-mesa-de-ayuda-mujeres-contratacion-inmediata-1886770931", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H77" s="6" t="inlineStr"/>
@@ -4116,22 +4128,22 @@
     <row r="78" ht="22" customHeight="1">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>a95003a0b1fc3d77</t>
+          <t>e28aba5df8a2d3ae</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 15:41</t>
+          <t>2026-09-25 15:54</t>
         </is>
       </c>
       <c r="C78" s="3" t="inlineStr">
         <is>
-          <t>Técnico Soporte Nivel 1 Con ITIL</t>
+          <t>Tecnico de mesa de ayuda/mujeres contratacion inmediata</t>
         </is>
       </c>
       <c r="D78" s="3" t="inlineStr">
         <is>
-          <t>Importante empresa del sector de tecnología</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E78" s="7" t="n">
@@ -4143,14 +4155,10 @@
         </is>
       </c>
       <c r="G78" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-soporte-nivel-1-con-itil-en-bogota-dc-59E13FA64EF5843C61373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H78" s="6" t="inlineStr">
-        <is>
-          <t>$ 1.750.905,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-mesa-de-ayuda-mujeres-contratacion-inmediata-1886769701", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H78" s="6" t="inlineStr"/>
       <c r="I78" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -4166,22 +4174,22 @@
     <row r="79" ht="22" customHeight="1">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>96391fd564d83616</t>
+          <t>9326784c1a2726fb</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 15:41</t>
+          <t>2026-09-25 15:54</t>
         </is>
       </c>
       <c r="C79" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de soporte IT con Moto</t>
+          <t>Técnico de soporte y mesa de ayuda / medellín</t>
         </is>
       </c>
       <c r="D79" s="3" t="inlineStr">
         <is>
-          <t>Los Hornitos</t>
+          <t>Colsof S.A.S</t>
         </is>
       </c>
       <c r="E79" s="7" t="n">
@@ -4193,14 +4201,10 @@
         </is>
       </c>
       <c r="G79" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-it-con-moto-empresa-de-alimentos-en-bogota-dc-599938D46A6F4A8F61373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H79" s="6" t="inlineStr">
-        <is>
-          <t>$ 2.125.947,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-y-mesa-de-ayuda-medellin-1886738118", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H79" s="6" t="inlineStr"/>
       <c r="I79" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -4216,22 +4220,22 @@
     <row r="80" ht="22" customHeight="1">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>b4f0b8c16fe5543e</t>
+          <t>b67dc9a9be4a1a6f</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 15:41</t>
+          <t>2026-09-25 15:54</t>
         </is>
       </c>
       <c r="C80" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar de Sistemas</t>
+          <t>Service desk agent</t>
         </is>
       </c>
       <c r="D80" s="3" t="inlineStr">
         <is>
-          <t>ELIS COLOMBIA SAS</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E80" s="7" t="n">
@@ -4243,17 +4247,13 @@
         </is>
       </c>
       <c r="G80" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-en-bogota-dc-48C2A0A3B050945661373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H80" s="6" t="inlineStr">
-        <is>
-          <t>$ 2.000.000,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/service-desk-agent-soporte-tecnico-nivel-1-1886755112", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H80" s="6" t="inlineStr"/>
       <c r="I80" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J80" s="2" t="inlineStr">
@@ -4266,22 +4266,22 @@
     <row r="81" ht="22" customHeight="1">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>7e4b4e4f136a5e31</t>
+          <t>9c65f710f43158b7</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 15:41</t>
+          <t>2026-09-25 15:54</t>
         </is>
       </c>
       <c r="C81" s="3" t="inlineStr">
         <is>
-          <t>Agente Mesa de Ayuda</t>
+          <t>Tecnico de instalaciones cableado de redes - licencia conte</t>
         </is>
       </c>
       <c r="D81" s="3" t="inlineStr">
         <is>
-          <t>Importante empresa del sector</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E81" s="7" t="n">
@@ -4293,14 +4293,10 @@
         </is>
       </c>
       <c r="G81" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-agente-mesa-de-ayuda-en-bogota-dc-E39FE355E02E578761373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H81" s="6" t="inlineStr">
-        <is>
-          <t>$ 2.000.000,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-1886749397", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H81" s="6" t="inlineStr"/>
       <c r="I81" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -4316,7 +4312,7 @@
     <row r="82" ht="22" customHeight="1">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>0ef2cd7667600919</t>
+          <t>a95003a0b1fc3d77</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
@@ -4326,12 +4322,12 @@
       </c>
       <c r="C82" s="3" t="inlineStr">
         <is>
-          <t>Técnico de Soporte TI Regional</t>
+          <t>Técnico Soporte Nivel 1 Con ITIL</t>
         </is>
       </c>
       <c r="D82" s="3" t="inlineStr">
         <is>
-          <t>POLICOMP COLOMBIA SAS</t>
+          <t>Importante empresa del sector de tecnología</t>
         </is>
       </c>
       <c r="E82" s="7" t="n">
@@ -4343,10 +4339,14 @@
         </is>
       </c>
       <c r="G82" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-ti-regional-en-bogota-dc-ACF045C94E41CCDE61373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H82" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-soporte-nivel-1-con-itil-en-bogota-dc-59E13FA64EF5843C61373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H82" s="6" t="inlineStr">
+        <is>
+          <t>$ 1.750.905,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I82" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -4362,7 +4362,7 @@
     <row r="83" ht="22" customHeight="1">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>7784997bda962255</t>
+          <t>96391fd564d83616</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
@@ -4372,12 +4372,12 @@
       </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t>Técnico de Soporte TI On Demand/ por horas</t>
+          <t>Tecnico de soporte IT con Moto</t>
         </is>
       </c>
       <c r="D83" s="3" t="inlineStr">
         <is>
-          <t>POLICOMP COLOMBIA SAS</t>
+          <t>Los Hornitos</t>
         </is>
       </c>
       <c r="E83" s="7" t="n">
@@ -4389,10 +4389,14 @@
         </is>
       </c>
       <c r="G83" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-ti-on-demand-por-horas-en-bogota-dc-C2338FA0172D59A561373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H83" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-it-con-moto-empresa-de-alimentos-en-bogota-dc-599938D46A6F4A8F61373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H83" s="6" t="inlineStr">
+        <is>
+          <t>$ 2.125.947,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I83" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -4408,7 +4412,7 @@
     <row r="84" ht="22" customHeight="1">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>29d0fe2e42e678f7</t>
+          <t>b4f0b8c16fe5543e</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
@@ -4418,12 +4422,12 @@
       </c>
       <c r="C84" s="3" t="inlineStr">
         <is>
-          <t>Técnico mantenimiento correctivo impresoras</t>
+          <t>Auxiliar de Sistemas</t>
         </is>
       </c>
       <c r="D84" s="3" t="inlineStr">
         <is>
-          <t>Multinacional de Impresión</t>
+          <t>ELIS COLOMBIA SAS</t>
         </is>
       </c>
       <c r="E84" s="7" t="n">
@@ -4435,12 +4439,12 @@
         </is>
       </c>
       <c r="G84" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-mantenimiento-correctivo-impresoras-en-guarne-BC0E775C0F25B27D61373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-en-bogota-dc-48C2A0A3B050945661373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H84" s="6" t="inlineStr">
         <is>
-          <t>$ 1.800.000,00 (Mensual)</t>
+          <t>$ 2.000.000,00 (Mensual)</t>
         </is>
       </c>
       <c r="I84" s="3" t="inlineStr">
@@ -4458,17 +4462,17 @@
     <row r="85" ht="22" customHeight="1">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>98c9ab11f5b1eace</t>
+          <t>7e4b4e4f136a5e31</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 18:36</t>
+          <t>2026-09-27 15:41</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar de sistemas</t>
+          <t>Agente Mesa de Ayuda</t>
         </is>
       </c>
       <c r="D85" s="3" t="inlineStr">
@@ -4485,12 +4489,12 @@
         </is>
       </c>
       <c r="G85" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-persona-con-discapacidad-remota-en-bogota-dc-5F2A812D014E159B61373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-agente-mesa-de-ayuda-en-bogota-dc-E39FE355E02E578761373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H85" s="6" t="inlineStr">
         <is>
-          <t>$ 1.750.905,00 (Mensual)</t>
+          <t>$ 2.000.000,00 (Mensual)</t>
         </is>
       </c>
       <c r="I85" s="3" t="inlineStr">
@@ -4508,22 +4512,22 @@
     <row r="86" ht="22" customHeight="1">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>58133ddc4da9c68e</t>
+          <t>0ef2cd7667600919</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 18:36</t>
+          <t>2026-09-27 15:41</t>
         </is>
       </c>
       <c r="C86" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar de sistemas</t>
+          <t>Técnico de Soporte TI Regional</t>
         </is>
       </c>
       <c r="D86" s="3" t="inlineStr">
         <is>
-          <t>Importante empresa del sector</t>
+          <t>POLICOMP COLOMBIA SAS</t>
         </is>
       </c>
       <c r="E86" s="7" t="n">
@@ -4535,14 +4539,10 @@
         </is>
       </c>
       <c r="G86" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-persona-con-discapacidad-remota-en-bogota-dc-A00C07C9CC9A494B61373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H86" s="6" t="inlineStr">
-        <is>
-          <t>$ 1.750.905,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-ti-regional-en-bogota-dc-ACF045C94E41CCDE61373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H86" s="6" t="inlineStr"/>
       <c r="I86" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -4558,22 +4558,22 @@
     <row r="87" ht="22" customHeight="1">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>aed3420a4cfdc248</t>
+          <t>7784997bda962255</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 18:36</t>
+          <t>2026-09-27 15:41</t>
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>Consultor de servicios/ mesa de ayuda nómina y erp software</t>
+          <t>Técnico de Soporte TI On Demand/ por horas</t>
         </is>
       </c>
       <c r="D87" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>POLICOMP COLOMBIA SAS</t>
         </is>
       </c>
       <c r="E87" s="7" t="n">
@@ -4585,7 +4585,7 @@
         </is>
       </c>
       <c r="G87" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/consultor-de-servicios-mesa-de-ayuda-nomina-y-erp-software-inclusivo-1886716126", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-ti-on-demand-por-horas-en-bogota-dc-C2338FA0172D59A561373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H87" s="6" t="inlineStr"/>
@@ -4604,22 +4604,22 @@
     <row r="88" ht="22" customHeight="1">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>2b8357189ff315da</t>
+          <t>29d0fe2e42e678f7</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 17:00</t>
+          <t>2026-09-27 15:41</t>
         </is>
       </c>
       <c r="C88" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar de sistemas</t>
+          <t>Técnico mantenimiento correctivo impresoras</t>
         </is>
       </c>
       <c r="D88" s="3" t="inlineStr">
         <is>
-          <t>DAVITA SAS</t>
+          <t>Multinacional de Impresión</t>
         </is>
       </c>
       <c r="E88" s="7" t="n">
@@ -4631,10 +4631,14 @@
         </is>
       </c>
       <c r="G88" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886758163", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H88" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-mantenimiento-correctivo-impresoras-en-guarne-BC0E775C0F25B27D61373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H88" s="6" t="inlineStr">
+        <is>
+          <t>$ 1.800.000,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I88" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -4650,22 +4654,22 @@
     <row r="89" ht="22" customHeight="1">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>a87934e7643b2c1c</t>
+          <t>98c9ab11f5b1eace</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 17:00</t>
+          <t>2026-09-28 18:36</t>
         </is>
       </c>
       <c r="C89" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de instalaciones cableado de redes - licencia conte cali</t>
+          <t>Auxiliar de sistemas</t>
         </is>
       </c>
       <c r="D89" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Importante empresa del sector</t>
         </is>
       </c>
       <c r="E89" s="7" t="n">
@@ -4677,10 +4681,14 @@
         </is>
       </c>
       <c r="G89" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-cali-1886759847", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H89" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-persona-con-discapacidad-remota-en-bogota-dc-5F2A812D014E159B61373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H89" s="6" t="inlineStr">
+        <is>
+          <t>$ 1.750.905,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I89" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -4696,22 +4704,22 @@
     <row r="90" ht="22" customHeight="1">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>10b4265e3ad11d81</t>
+          <t>58133ddc4da9c68e</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 17:00</t>
+          <t>2026-09-28 18:36</t>
         </is>
       </c>
       <c r="C90" s="3" t="inlineStr">
         <is>
-          <t>Information Technology Help Desk Support</t>
+          <t>Auxiliar de sistemas</t>
         </is>
       </c>
       <c r="D90" s="3" t="inlineStr">
         <is>
-          <t>Booth</t>
+          <t>Importante empresa del sector</t>
         </is>
       </c>
       <c r="E90" s="7" t="n">
@@ -4723,10 +4731,14 @@
         </is>
       </c>
       <c r="G90" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/information-technology-help-desk-support-at-booth-4471203962", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H90" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-persona-con-discapacidad-remota-en-bogota-dc-A00C07C9CC9A494B61373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H90" s="6" t="inlineStr">
+        <is>
+          <t>$ 1.750.905,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I90" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -4742,17 +4754,17 @@
     <row r="91" ht="22" customHeight="1">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>ff69ae85c8697a37</t>
+          <t>aed3420a4cfdc248</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 16:49</t>
+          <t>2026-09-28 18:36</t>
         </is>
       </c>
       <c r="C91" s="3" t="inlineStr">
         <is>
-          <t>Técnico de soporte ti - bogota</t>
+          <t>Consultor de servicios/ mesa de ayuda nómina y erp software</t>
         </is>
       </c>
       <c r="D91" s="3" t="inlineStr">
@@ -4769,7 +4781,7 @@
         </is>
       </c>
       <c r="G91" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-ti-bogota-1886774059", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/consultor-de-servicios-mesa-de-ayuda-nomina-y-erp-software-inclusivo-1886716126", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H91" s="6" t="inlineStr"/>
@@ -4788,22 +4800,22 @@
     <row r="92" ht="22" customHeight="1">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>bbacf7d69ab9084e</t>
+          <t>2b8357189ff315da</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 16:49</t>
+          <t>2026-09-29 17:00</t>
         </is>
       </c>
       <c r="C92" s="3" t="inlineStr">
         <is>
-          <t>IT Helpdesk Analyst</t>
+          <t>Auxiliar de sistemas</t>
         </is>
       </c>
       <c r="D92" s="3" t="inlineStr">
         <is>
-          <t>Power Digital Marketing</t>
+          <t>DAVITA SAS</t>
         </is>
       </c>
       <c r="E92" s="7" t="n">
@@ -4815,7 +4827,7 @@
         </is>
       </c>
       <c r="G92" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/it-helpdesk-analyst-at-power-digital-marketing-4472601999", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886758163", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H92" s="6" t="inlineStr"/>
@@ -4834,17 +4846,17 @@
     <row r="93" ht="22" customHeight="1">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>bb848f474ff4b611</t>
+          <t>a87934e7643b2c1c</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 17:26</t>
+          <t>2026-09-29 17:00</t>
         </is>
       </c>
       <c r="C93" s="3" t="inlineStr">
         <is>
-          <t>Técnico de soporte ti - bogota</t>
+          <t>Tecnico de instalaciones cableado de redes - licencia conte cali</t>
         </is>
       </c>
       <c r="D93" s="3" t="inlineStr">
@@ -4861,7 +4873,7 @@
         </is>
       </c>
       <c r="G93" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-ti-bogota-1886772292", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-cali-1886759847", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H93" s="6" t="inlineStr"/>
@@ -4880,22 +4892,22 @@
     <row r="94" ht="22" customHeight="1">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>b44a1c6cfb004ca8</t>
+          <t>10b4265e3ad11d81</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 17:26</t>
+          <t>2026-09-29 17:00</t>
         </is>
       </c>
       <c r="C94" s="3" t="inlineStr">
         <is>
-          <t>Soporte ti nivel 2 - bogotá</t>
+          <t>Information Technology Help Desk Support</t>
         </is>
       </c>
       <c r="D94" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Booth</t>
         </is>
       </c>
       <c r="E94" s="7" t="n">
@@ -4907,7 +4919,7 @@
         </is>
       </c>
       <c r="G94" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/soporte-ti-nivel-2-bogota-1886774821", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/information-technology-help-desk-support-at-booth-4471203962", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H94" s="6" t="inlineStr"/>
@@ -4926,22 +4938,22 @@
     <row r="95" ht="22" customHeight="1">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>fb0ad2b513afb97c</t>
+          <t>ff69ae85c8697a37</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 17:26</t>
+          <t>2026-09-30 16:49</t>
         </is>
       </c>
       <c r="C95" s="3" t="inlineStr">
         <is>
-          <t>IT Help Desk Support Specialist</t>
+          <t>Técnico de soporte ti - bogota</t>
         </is>
       </c>
       <c r="D95" s="3" t="inlineStr">
         <is>
-          <t>Talento</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E95" s="7" t="n">
@@ -4953,7 +4965,7 @@
         </is>
       </c>
       <c r="G95" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/it-help-desk-support-specialist-tier-1-at-talento-4473960480", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-ti-bogota-1886774059", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H95" s="6" t="inlineStr"/>
@@ -4972,22 +4984,22 @@
     <row r="96" ht="22" customHeight="1">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>0b2067d6ae488f4c</t>
+          <t>bbacf7d69ab9084e</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 16:39</t>
+          <t>2026-09-30 16:49</t>
         </is>
       </c>
       <c r="C96" s="3" t="inlineStr">
         <is>
-          <t>Help Desk Technician level 1</t>
+          <t>IT Helpdesk Analyst</t>
         </is>
       </c>
       <c r="D96" s="3" t="inlineStr">
         <is>
-          <t>Solvo Global</t>
+          <t>Power Digital Marketing</t>
         </is>
       </c>
       <c r="E96" s="7" t="n">
@@ -4999,7 +5011,7 @@
         </is>
       </c>
       <c r="G96" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/help-desk-technician-level-1-at-solvo-global-4472590892", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/it-helpdesk-analyst-at-power-digital-marketing-4472601999", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H96" s="6" t="inlineStr"/>
@@ -5018,22 +5030,22 @@
     <row r="97" ht="22" customHeight="1">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>07acc222a3ca2ef1</t>
+          <t>bb848f474ff4b611</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03 15:12</t>
+          <t>2026-10-01 17:26</t>
         </is>
       </c>
       <c r="C97" s="3" t="inlineStr">
         <is>
-          <t>Analista mesa de ayuda funza temporal 6 meses</t>
+          <t>Técnico de soporte ti - bogota</t>
         </is>
       </c>
       <c r="D97" s="3" t="inlineStr">
         <is>
-          <t>Axity</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E97" s="7" t="n">
@@ -5045,7 +5057,7 @@
         </is>
       </c>
       <c r="G97" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-funza-temporal-6-meses-1886774524", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-ti-bogota-1886772292", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H97" s="6" t="inlineStr"/>
@@ -5064,17 +5076,17 @@
     <row r="98" ht="22" customHeight="1">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>5ec0ea33876ba2b5</t>
+          <t>b44a1c6cfb004ca8</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 19:45</t>
+          <t>2026-10-01 17:26</t>
         </is>
       </c>
       <c r="C98" s="3" t="inlineStr">
         <is>
-          <t>Help desk analyst l1</t>
+          <t>Soporte ti nivel 2 - bogotá</t>
         </is>
       </c>
       <c r="D98" s="3" t="inlineStr">
@@ -5091,7 +5103,7 @@
         </is>
       </c>
       <c r="G98" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/help-desk-analyst-l1-medellin-1886776156", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/soporte-ti-nivel-2-bogota-1886774821", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H98" s="6" t="inlineStr"/>
@@ -5110,22 +5122,22 @@
     <row r="99" ht="22" customHeight="1">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>e8bdf2094d1c9817</t>
+          <t>fb0ad2b513afb97c</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 19:45</t>
+          <t>2026-10-01 17:26</t>
         </is>
       </c>
       <c r="C99" s="3" t="inlineStr">
         <is>
-          <t>Administrador de herramienta de gestión de mesa de ayuda-</t>
+          <t>IT Help Desk Support Specialist</t>
         </is>
       </c>
       <c r="D99" s="3" t="inlineStr">
         <is>
-          <t>SELCOMP INGENIERÍA SAS</t>
+          <t>Talento</t>
         </is>
       </c>
       <c r="E99" s="7" t="n">
@@ -5137,7 +5149,7 @@
         </is>
       </c>
       <c r="G99" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/administrador-de-herramienta-de-gestion-de-mesa-de-ayuda-1886776286", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/it-help-desk-support-specialist-tier-1-at-talento-4473960480", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H99" s="6" t="inlineStr"/>
@@ -5156,22 +5168,22 @@
     <row r="100" ht="22" customHeight="1">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>6e9a077b42879470</t>
+          <t>0b2067d6ae488f4c</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 19:45</t>
+          <t>2026-10-02 16:39</t>
         </is>
       </c>
       <c r="C100" s="3" t="inlineStr">
         <is>
-          <t>Analista de soporte de aplicaciones nivel 3</t>
+          <t>Help Desk Technician level 1</t>
         </is>
       </c>
       <c r="D100" s="3" t="inlineStr">
         <is>
-          <t>TALYCAP GLOBAL SAS</t>
+          <t>Solvo Global</t>
         </is>
       </c>
       <c r="E100" s="7" t="n">
@@ -5183,7 +5195,7 @@
         </is>
       </c>
       <c r="G100" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-soporte-de-aplicaciones-nivel-3-1886776104", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/help-desk-technician-level-1-at-solvo-global-4472590892", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H100" s="6" t="inlineStr"/>
@@ -5202,22 +5214,22 @@
     <row r="101" ht="22" customHeight="1">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>447afec244b20f9b</t>
+          <t>07acc222a3ca2ef1</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06 17:12</t>
+          <t>2026-10-03 15:12</t>
         </is>
       </c>
       <c r="C101" s="3" t="inlineStr">
         <is>
-          <t>Técnico de soporte ti - bogota</t>
+          <t>Analista mesa de ayuda funza temporal 6 meses</t>
         </is>
       </c>
       <c r="D101" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Axity</t>
         </is>
       </c>
       <c r="E101" s="7" t="n">
@@ -5229,7 +5241,7 @@
         </is>
       </c>
       <c r="G101" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-ti-bogota-1886775990", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-funza-temporal-6-meses-1886774524", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H101" s="6" t="inlineStr"/>
@@ -5248,22 +5260,22 @@
     <row r="102" ht="22" customHeight="1">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>8f14c41f3b443ac0</t>
+          <t>5ec0ea33876ba2b5</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07 17:50</t>
+          <t>2026-10-05 19:45</t>
         </is>
       </c>
       <c r="C102" s="3" t="inlineStr">
         <is>
-          <t>Soporte mesa de ayuda</t>
+          <t>Help desk analyst l1</t>
         </is>
       </c>
       <c r="D102" s="3" t="inlineStr">
         <is>
-          <t>MANPOWER</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E102" s="7" t="n">
@@ -5275,7 +5287,7 @@
         </is>
       </c>
       <c r="G102" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/soporte-mesa-de-ayuda-vacaciones-1886776917", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/help-desk-analyst-l1-medellin-1886776156", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H102" s="6" t="inlineStr"/>
@@ -5294,22 +5306,22 @@
     <row r="103" ht="22" customHeight="1">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>b1a9e03967fff91e</t>
+          <t>e8bdf2094d1c9817</t>
         </is>
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07 17:50</t>
+          <t>2026-10-05 19:45</t>
         </is>
       </c>
       <c r="C103" s="3" t="inlineStr">
         <is>
-          <t>Tecnólogo de soporte pl - mesa de ayuda</t>
+          <t>Administrador de herramienta de gestión de mesa de ayuda-</t>
         </is>
       </c>
       <c r="D103" s="3" t="inlineStr">
         <is>
-          <t>Positivo S+</t>
+          <t>SELCOMP INGENIERÍA SAS</t>
         </is>
       </c>
       <c r="E103" s="7" t="n">
@@ -5321,7 +5333,7 @@
         </is>
       </c>
       <c r="G103" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnologo-de-soporte-pl-mesa-de-ayuda-1886775546", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/administrador-de-herramienta-de-gestion-de-mesa-de-ayuda-1886776286", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H103" s="6" t="inlineStr"/>
@@ -5340,22 +5352,22 @@
     <row r="104" ht="22" customHeight="1">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>eb49981c97933d93</t>
+          <t>6e9a077b42879470</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07 17:50</t>
+          <t>2026-10-05 19:45</t>
         </is>
       </c>
       <c r="C104" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de instalaciones cableado de redes - licencia conte</t>
+          <t>Analista de soporte de aplicaciones nivel 3</t>
         </is>
       </c>
       <c r="D104" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>TALYCAP GLOBAL SAS</t>
         </is>
       </c>
       <c r="E104" s="7" t="n">
@@ -5367,7 +5379,7 @@
         </is>
       </c>
       <c r="G104" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-1886777333", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-soporte-de-aplicaciones-nivel-3-1886776104", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H104" s="6" t="inlineStr"/>
@@ -5386,22 +5398,22 @@
     <row r="105" ht="22" customHeight="1">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>d39af22b6e937d28</t>
+          <t>447afec244b20f9b</t>
         </is>
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07 17:50</t>
+          <t>2026-10-06 17:12</t>
         </is>
       </c>
       <c r="C105" s="3" t="inlineStr">
         <is>
-          <t>Analista Mesa de Ayuda Funza</t>
+          <t>Técnico de soporte ti - bogota</t>
         </is>
       </c>
       <c r="D105" s="3" t="inlineStr">
         <is>
-          <t>axity</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E105" s="7" t="n">
@@ -5413,7 +5425,7 @@
         </is>
       </c>
       <c r="G105" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/analista-mesa-de-ayuda-funza-at-axity-4471985006", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-ti-bogota-1886775990", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H105" s="6" t="inlineStr"/>
@@ -5432,22 +5444,22 @@
     <row r="106" ht="22" customHeight="1">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>0904912d51c5cd61</t>
+          <t>8f14c41f3b443ac0</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08 17:52</t>
+          <t>2026-10-07 17:50</t>
         </is>
       </c>
       <c r="C106" s="3" t="inlineStr">
         <is>
-          <t>Analista mesa de ayuda</t>
+          <t>Soporte mesa de ayuda</t>
         </is>
       </c>
       <c r="D106" s="3" t="inlineStr">
         <is>
-          <t>Desarrollo de Sistemas y Servicios SAS</t>
+          <t>MANPOWER</t>
         </is>
       </c>
       <c r="E106" s="7" t="n">
@@ -5459,7 +5471,7 @@
         </is>
       </c>
       <c r="G106" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-1886778032", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/soporte-mesa-de-ayuda-vacaciones-1886776917", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H106" s="6" t="inlineStr"/>
@@ -5478,22 +5490,22 @@
     <row r="107" ht="22" customHeight="1">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>c665ada630270dce</t>
+          <t>b1a9e03967fff91e</t>
         </is>
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09 17:28</t>
+          <t>2026-10-07 17:50</t>
         </is>
       </c>
       <c r="C107" s="3" t="inlineStr">
         <is>
-          <t>Técnico(a) / tecnólogo(a) / profesional de telecomunicaciones - redes de fibra óptica</t>
+          <t>Tecnólogo de soporte pl - mesa de ayuda</t>
         </is>
       </c>
       <c r="D107" s="3" t="inlineStr">
         <is>
-          <t>JAHV MC GREGOR S.A.S</t>
+          <t>Positivo S+</t>
         </is>
       </c>
       <c r="E107" s="7" t="n">
@@ -5505,7 +5517,7 @@
         </is>
       </c>
       <c r="G107" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnicoa-tecnologoa-profesional-de-telecomunicaciones-redes-de-fibra-optica-1886768691", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnologo-de-soporte-pl-mesa-de-ayuda-1886775546", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H107" s="6" t="inlineStr"/>
@@ -5524,17 +5536,17 @@
     <row r="108" ht="22" customHeight="1">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>4e5b3128aa7f8f9b</t>
+          <t>eb49981c97933d93</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09 17:28</t>
+          <t>2026-10-07 17:50</t>
         </is>
       </c>
       <c r="C108" s="3" t="inlineStr">
         <is>
-          <t>Gestor de servicios mesa de ayuda sap</t>
+          <t>Tecnico de instalaciones cableado de redes - licencia conte</t>
         </is>
       </c>
       <c r="D108" s="3" t="inlineStr">
@@ -5551,7 +5563,7 @@
         </is>
       </c>
       <c r="G108" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/gestor-de-servicios-mesa-de-ayuda-sap-1886775732", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-1886777333", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H108" s="6" t="inlineStr"/>
@@ -5570,22 +5582,22 @@
     <row r="109" ht="22" customHeight="1">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>1c92f7ef9b7af696</t>
+          <t>d39af22b6e937d28</t>
         </is>
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09 17:28</t>
+          <t>2026-10-07 17:50</t>
         </is>
       </c>
       <c r="C109" s="3" t="inlineStr">
         <is>
-          <t>Agente de mesa de ayuda nivel 1</t>
+          <t>Analista Mesa de Ayuda Funza</t>
         </is>
       </c>
       <c r="D109" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>axity</t>
         </is>
       </c>
       <c r="E109" s="7" t="n">
@@ -5597,7 +5609,7 @@
         </is>
       </c>
       <c r="G109" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-de-mesa-de-ayuda-nivel-1-1886778506", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/analista-mesa-de-ayuda-funza-at-axity-4471985006", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H109" s="6" t="inlineStr"/>
@@ -5616,22 +5628,22 @@
     <row r="110" ht="22" customHeight="1">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>718ceee355d457ea</t>
+          <t>0904912d51c5cd61</t>
         </is>
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10 16:16</t>
+          <t>2026-10-08 17:52</t>
         </is>
       </c>
       <c r="C110" s="3" t="inlineStr">
         <is>
-          <t>IT Help Desk Support</t>
+          <t>Analista mesa de ayuda</t>
         </is>
       </c>
       <c r="D110" s="3" t="inlineStr">
         <is>
-          <t>Booth</t>
+          <t>Desarrollo de Sistemas y Servicios SAS</t>
         </is>
       </c>
       <c r="E110" s="7" t="n">
@@ -5643,7 +5655,7 @@
         </is>
       </c>
       <c r="G110" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/it-help-desk-support-at-booth-4471203962", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-1886778032", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H110" s="6" t="inlineStr"/>
@@ -5662,22 +5674,22 @@
     <row r="111" ht="22" customHeight="1">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>925f43273b78f188</t>
+          <t>c665ada630270dce</t>
         </is>
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12 20:17</t>
+          <t>2026-10-09 17:28</t>
         </is>
       </c>
       <c r="C111" s="3" t="inlineStr">
         <is>
-          <t>Mesa de ayuda ti - girón</t>
+          <t>Técnico(a) / tecnólogo(a) / profesional de telecomunicaciones - redes de fibra óptica</t>
         </is>
       </c>
       <c r="D111" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>JAHV MC GREGOR S.A.S</t>
         </is>
       </c>
       <c r="E111" s="7" t="n">
@@ -5689,7 +5701,7 @@
         </is>
       </c>
       <c r="G111" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/mesa-de-ayuda-ti-giron-1886745168", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnicoa-tecnologoa-profesional-de-telecomunicaciones-redes-de-fibra-optica-1886768691", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H111" s="6" t="inlineStr"/>
@@ -5708,22 +5720,22 @@
     <row r="112" ht="22" customHeight="1">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>ec0c8875e04f4933</t>
+          <t>4e5b3128aa7f8f9b</t>
         </is>
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13 18:08</t>
+          <t>2026-10-09 17:28</t>
         </is>
       </c>
       <c r="C112" s="3" t="inlineStr">
         <is>
-          <t>Analista de mesa de ayuda.</t>
+          <t>Gestor de servicios mesa de ayuda sap</t>
         </is>
       </c>
       <c r="D112" s="3" t="inlineStr">
         <is>
-          <t>Softtek Colombia</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E112" s="7" t="n">
@@ -5735,7 +5747,7 @@
         </is>
       </c>
       <c r="G112" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-mesa-de-ayuda-1886754207", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/gestor-de-servicios-mesa-de-ayuda-sap-1886775732", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H112" s="6" t="inlineStr"/>
@@ -5754,22 +5766,22 @@
     <row r="113" ht="22" customHeight="1">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>87fac63aa714f401</t>
+          <t>1c92f7ef9b7af696</t>
         </is>
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13 18:08</t>
+          <t>2026-10-09 17:28</t>
         </is>
       </c>
       <c r="C113" s="3" t="inlineStr">
         <is>
-          <t>Agente mesa de ayuda.</t>
+          <t>Agente de mesa de ayuda nivel 1</t>
         </is>
       </c>
       <c r="D113" s="3" t="inlineStr">
         <is>
-          <t>Softtek Colombia</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E113" s="7" t="n">
@@ -5781,7 +5793,7 @@
         </is>
       </c>
       <c r="G113" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-mesa-de-ayuda-1886753535", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-de-mesa-de-ayuda-nivel-1-1886778506", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H113" s="6" t="inlineStr"/>
@@ -5800,22 +5812,22 @@
     <row r="114" ht="22" customHeight="1">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>dfa7dd88fd24afb4</t>
+          <t>718ceee355d457ea</t>
         </is>
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15 15:40</t>
+          <t>2026-10-10 16:16</t>
         </is>
       </c>
       <c r="C114" s="3" t="inlineStr">
         <is>
-          <t>Agente mesa de ayuda nivel 1 ingles avanzado</t>
+          <t>IT Help Desk Support</t>
         </is>
       </c>
       <c r="D114" s="3" t="inlineStr">
         <is>
-          <t>SUSTS Colombia Ltda.</t>
+          <t>Booth</t>
         </is>
       </c>
       <c r="E114" s="7" t="n">
@@ -5827,7 +5839,7 @@
         </is>
       </c>
       <c r="G114" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-mesa-de-ayuda-nivel-1-ingles-avanzado-1886780371", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/it-help-desk-support-at-booth-4471203962", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H114" s="6" t="inlineStr"/>
@@ -5846,26 +5858,26 @@
     <row r="115" ht="22" customHeight="1">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>50c79dfbfd49f52d</t>
+          <t>925f43273b78f188</t>
         </is>
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 16:39</t>
+          <t>2026-10-12 20:17</t>
         </is>
       </c>
       <c r="C115" s="3" t="inlineStr">
         <is>
-          <t>Analista de redes noc 1 telecomunicaciones.</t>
+          <t>Mesa de ayuda ti - girón</t>
         </is>
       </c>
       <c r="D115" s="3" t="inlineStr">
         <is>
-          <t>MANPOWER</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E115" s="7" t="n">
-        <v>0.53</v>
+        <v>0.58</v>
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
@@ -5873,13 +5885,13 @@
         </is>
       </c>
       <c r="G115" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-noc-1-telecomunicaciones-1886772075", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/mesa-de-ayuda-ti-giron-1886745168", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H115" s="6" t="inlineStr"/>
       <c r="I115" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J115" s="2" t="inlineStr">
@@ -5892,26 +5904,26 @@
     <row r="116" ht="22" customHeight="1">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>0b0ae49f910109bb</t>
+          <t>ec0c8875e04f4933</t>
         </is>
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 15:54</t>
+          <t>2026-10-13 18:08</t>
         </is>
       </c>
       <c r="C116" s="3" t="inlineStr">
         <is>
-          <t>Ejecutivo Técnico Arancel Junior</t>
+          <t>Analista de mesa de ayuda.</t>
         </is>
       </c>
       <c r="D116" s="3" t="inlineStr">
         <is>
-          <t>Importante Empresa de Logística y Comercio</t>
+          <t>Softtek Colombia</t>
         </is>
       </c>
       <c r="E116" s="7" t="n">
-        <v>0.5</v>
+        <v>0.58</v>
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
@@ -5919,17 +5931,13 @@
         </is>
       </c>
       <c r="G116" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-547866639B487E0161373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H116" s="6" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-mesa-de-ayuda-1886754207", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H116" s="6" t="inlineStr"/>
       <c r="I116" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J116" s="2" t="inlineStr">
@@ -5942,26 +5950,26 @@
     <row r="117" ht="22" customHeight="1">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>582a04b3c639bfa0</t>
+          <t>87fac63aa714f401</t>
         </is>
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 16:49</t>
+          <t>2026-10-13 18:08</t>
         </is>
       </c>
       <c r="C117" s="3" t="inlineStr">
         <is>
-          <t>Junior IT Support Specialist</t>
+          <t>Agente mesa de ayuda.</t>
         </is>
       </c>
       <c r="D117" s="3" t="inlineStr">
         <is>
-          <t>Touch Support, Inc. &amp; SNF Back Office</t>
+          <t>Softtek Colombia</t>
         </is>
       </c>
       <c r="E117" s="7" t="n">
-        <v>0.5</v>
+        <v>0.58</v>
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
@@ -5969,13 +5977,13 @@
         </is>
       </c>
       <c r="G117" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/junior-it-support-specialist-at-touch-support-inc-snf-back-office-4472187578", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-mesa-de-ayuda-1886753535", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H117" s="6" t="inlineStr"/>
       <c r="I117" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J117" s="2" t="inlineStr">
@@ -5988,52 +5996,336 @@
     <row r="118" ht="22" customHeight="1">
       <c r="A118" s="2" t="inlineStr">
         <is>
+          <t>dfa7dd88fd24afb4</t>
+        </is>
+      </c>
+      <c r="B118" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15 15:40</t>
+        </is>
+      </c>
+      <c r="C118" s="3" t="inlineStr">
+        <is>
+          <t>Agente mesa de ayuda nivel 1 ingles avanzado</t>
+        </is>
+      </c>
+      <c r="D118" s="3" t="inlineStr">
+        <is>
+          <t>SUSTS Colombia Ltda.</t>
+        </is>
+      </c>
+      <c r="E118" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F118" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G118" s="5">
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-mesa-de-ayuda-nivel-1-ingles-avanzado-1886780371", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H118" s="6" t="inlineStr"/>
+      <c r="I118" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J118" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K118" s="3" t="inlineStr"/>
+    </row>
+    <row r="119" ht="22" customHeight="1">
+      <c r="A119" s="2" t="inlineStr">
+        <is>
+          <t>6ec1aeac55104810</t>
+        </is>
+      </c>
+      <c r="B119" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16 15:22</t>
+        </is>
+      </c>
+      <c r="C119" s="3" t="inlineStr">
+        <is>
+          <t>Analista de Mesa de Ayuda</t>
+        </is>
+      </c>
+      <c r="D119" s="3" t="inlineStr">
+        <is>
+          <t>INSEPET S.A.S</t>
+        </is>
+      </c>
+      <c r="E119" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F119" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G119" s="5">
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-analista-de-mesa-de-ayuda-en-bogota-dc-731E37A9EEFEA71561373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H119" s="6" t="inlineStr">
+        <is>
+          <t>$ 1.800.000,00 (Mensual)</t>
+        </is>
+      </c>
+      <c r="I119" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J119" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K119" s="3" t="inlineStr"/>
+    </row>
+    <row r="120" ht="22" customHeight="1">
+      <c r="A120" s="2" t="inlineStr">
+        <is>
+          <t>c03a3cc06e28c7bb</t>
+        </is>
+      </c>
+      <c r="B120" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16 15:22</t>
+        </is>
+      </c>
+      <c r="C120" s="3" t="inlineStr">
+        <is>
+          <t>Agente de mesa de ayuda portugues</t>
+        </is>
+      </c>
+      <c r="D120" s="3" t="inlineStr">
+        <is>
+          <t>COMWARE S.A.</t>
+        </is>
+      </c>
+      <c r="E120" s="7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F120" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G120" s="5">
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-de-mesa-de-ayuda-portugues-1886781202", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H120" s="6" t="inlineStr"/>
+      <c r="I120" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J120" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K120" s="3" t="inlineStr"/>
+    </row>
+    <row r="121" ht="22" customHeight="1">
+      <c r="A121" s="2" t="inlineStr">
+        <is>
+          <t>50c79dfbfd49f52d</t>
+        </is>
+      </c>
+      <c r="B121" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02 16:39</t>
+        </is>
+      </c>
+      <c r="C121" s="3" t="inlineStr">
+        <is>
+          <t>Analista de redes noc 1 telecomunicaciones.</t>
+        </is>
+      </c>
+      <c r="D121" s="3" t="inlineStr">
+        <is>
+          <t>MANPOWER</t>
+        </is>
+      </c>
+      <c r="E121" s="7" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="F121" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G121" s="5">
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-noc-1-telecomunicaciones-1886772075", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H121" s="6" t="inlineStr"/>
+      <c r="I121" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J121" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K121" s="3" t="inlineStr"/>
+    </row>
+    <row r="122" ht="22" customHeight="1">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
+          <t>0b0ae49f910109bb</t>
+        </is>
+      </c>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25 15:54</t>
+        </is>
+      </c>
+      <c r="C122" s="3" t="inlineStr">
+        <is>
+          <t>Ejecutivo Técnico Arancel Junior</t>
+        </is>
+      </c>
+      <c r="D122" s="3" t="inlineStr">
+        <is>
+          <t>Importante Empresa de Logística y Comercio</t>
+        </is>
+      </c>
+      <c r="E122" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F122" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G122" s="5">
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-547866639B487E0161373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H122" s="6" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="I122" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J122" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K122" s="3" t="inlineStr"/>
+    </row>
+    <row r="123" ht="22" customHeight="1">
+      <c r="A123" s="2" t="inlineStr">
+        <is>
+          <t>582a04b3c639bfa0</t>
+        </is>
+      </c>
+      <c r="B123" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 16:49</t>
+        </is>
+      </c>
+      <c r="C123" s="3" t="inlineStr">
+        <is>
+          <t>Junior IT Support Specialist</t>
+        </is>
+      </c>
+      <c r="D123" s="3" t="inlineStr">
+        <is>
+          <t>Touch Support, Inc. &amp; SNF Back Office</t>
+        </is>
+      </c>
+      <c r="E123" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F123" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G123" s="5">
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/junior-it-support-specialist-at-touch-support-inc-snf-back-office-4472187578", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H123" s="6" t="inlineStr"/>
+      <c r="I123" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J123" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K123" s="3" t="inlineStr"/>
+    </row>
+    <row r="124" ht="22" customHeight="1">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
           <t>6e04c4d57d3fc3c7</t>
         </is>
       </c>
-      <c r="B118" s="2" t="inlineStr">
+      <c r="B124" s="2" t="inlineStr">
         <is>
           <t>2026-10-01 17:26</t>
         </is>
       </c>
-      <c r="C118" s="3" t="inlineStr">
+      <c r="C124" s="3" t="inlineStr">
         <is>
           <t>Ejecutivo Técnico Arancel Junior</t>
         </is>
       </c>
-      <c r="D118" s="3" t="inlineStr">
+      <c r="D124" s="3" t="inlineStr">
         <is>
           <t>Importante Empresa de Logística y Comercio</t>
         </is>
       </c>
-      <c r="E118" s="7" t="n">
+      <c r="E124" s="7" t="n">
         <v>0.5</v>
       </c>
-      <c r="F118" s="2" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
-      <c r="G118" s="5">
+      <c r="F124" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G124" s="5">
         <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-8444AB594560844161373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
-      <c r="H118" s="6" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
-      <c r="I118" s="3" t="inlineStr">
+      <c r="H124" s="6" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="I124" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
-      <c r="J118" s="2" t="inlineStr">
-        <is>
-          <t>Nueva</t>
-        </is>
-      </c>
-      <c r="K118" s="3" t="inlineStr"/>
+      <c r="J124" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K124" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
chore(tracker): actualizacion diaria de vacantes 2026-10-17
</commit_message>
<xml_diff>
--- a/output/profile_5_tecnico_sistemas_tracker.xlsx
+++ b/output/profile_5_tecnico_sistemas_tracker.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K124"/>
+  <dimension ref="A1:K125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -6138,26 +6138,26 @@
     <row r="121" ht="22" customHeight="1">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>50c79dfbfd49f52d</t>
+          <t>2ecdc22edf2ff172</t>
         </is>
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 16:39</t>
+          <t>2026-10-17 14:15</t>
         </is>
       </c>
       <c r="C121" s="3" t="inlineStr">
         <is>
-          <t>Analista de redes noc 1 telecomunicaciones.</t>
+          <t>Agente Mesa de ayuda Portugués</t>
         </is>
       </c>
       <c r="D121" s="3" t="inlineStr">
         <is>
-          <t>MANPOWER</t>
+          <t>COMWARE S.A</t>
         </is>
       </c>
       <c r="E121" s="7" t="n">
-        <v>0.53</v>
+        <v>0.58</v>
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
@@ -6165,13 +6165,17 @@
         </is>
       </c>
       <c r="G121" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-noc-1-telecomunicaciones-1886772075", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H121" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-agente-mesa-de-ayuda-portugues-en-bogota-dc-D31C231B9F8EFFCA61373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H121" s="6" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
       <c r="I121" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J121" s="2" t="inlineStr">
@@ -6184,26 +6188,26 @@
     <row r="122" ht="22" customHeight="1">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>0b0ae49f910109bb</t>
+          <t>50c79dfbfd49f52d</t>
         </is>
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 15:54</t>
+          <t>2026-10-02 16:39</t>
         </is>
       </c>
       <c r="C122" s="3" t="inlineStr">
         <is>
-          <t>Ejecutivo Técnico Arancel Junior</t>
+          <t>Analista de redes noc 1 telecomunicaciones.</t>
         </is>
       </c>
       <c r="D122" s="3" t="inlineStr">
         <is>
-          <t>Importante Empresa de Logística y Comercio</t>
+          <t>MANPOWER</t>
         </is>
       </c>
       <c r="E122" s="7" t="n">
-        <v>0.5</v>
+        <v>0.53</v>
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
@@ -6211,17 +6215,13 @@
         </is>
       </c>
       <c r="G122" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-547866639B487E0161373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H122" s="6" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-noc-1-telecomunicaciones-1886772075", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H122" s="6" t="inlineStr"/>
       <c r="I122" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J122" s="2" t="inlineStr">
@@ -6234,22 +6234,22 @@
     <row r="123" ht="22" customHeight="1">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>582a04b3c639bfa0</t>
+          <t>0b0ae49f910109bb</t>
         </is>
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 16:49</t>
+          <t>2026-09-25 15:54</t>
         </is>
       </c>
       <c r="C123" s="3" t="inlineStr">
         <is>
-          <t>Junior IT Support Specialist</t>
+          <t>Ejecutivo Técnico Arancel Junior</t>
         </is>
       </c>
       <c r="D123" s="3" t="inlineStr">
         <is>
-          <t>Touch Support, Inc. &amp; SNF Back Office</t>
+          <t>Importante Empresa de Logística y Comercio</t>
         </is>
       </c>
       <c r="E123" s="7" t="n">
@@ -6261,10 +6261,14 @@
         </is>
       </c>
       <c r="G123" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/junior-it-support-specialist-at-touch-support-inc-snf-back-office-4472187578", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H123" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-547866639B487E0161373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H123" s="6" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
       <c r="I123" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -6280,22 +6284,22 @@
     <row r="124" ht="22" customHeight="1">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>6e04c4d57d3fc3c7</t>
+          <t>582a04b3c639bfa0</t>
         </is>
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 17:26</t>
+          <t>2026-09-30 16:49</t>
         </is>
       </c>
       <c r="C124" s="3" t="inlineStr">
         <is>
-          <t>Ejecutivo Técnico Arancel Junior</t>
+          <t>Junior IT Support Specialist</t>
         </is>
       </c>
       <c r="D124" s="3" t="inlineStr">
         <is>
-          <t>Importante Empresa de Logística y Comercio</t>
+          <t>Touch Support, Inc. &amp; SNF Back Office</t>
         </is>
       </c>
       <c r="E124" s="7" t="n">
@@ -6307,25 +6311,71 @@
         </is>
       </c>
       <c r="G124" s="5">
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/junior-it-support-specialist-at-touch-support-inc-snf-back-office-4472187578", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H124" s="6" t="inlineStr"/>
+      <c r="I124" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J124" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K124" s="3" t="inlineStr"/>
+    </row>
+    <row r="125" ht="22" customHeight="1">
+      <c r="A125" s="2" t="inlineStr">
+        <is>
+          <t>6e04c4d57d3fc3c7</t>
+        </is>
+      </c>
+      <c r="B125" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01 17:26</t>
+        </is>
+      </c>
+      <c r="C125" s="3" t="inlineStr">
+        <is>
+          <t>Ejecutivo Técnico Arancel Junior</t>
+        </is>
+      </c>
+      <c r="D125" s="3" t="inlineStr">
+        <is>
+          <t>Importante Empresa de Logística y Comercio</t>
+        </is>
+      </c>
+      <c r="E125" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F125" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G125" s="5">
         <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-8444AB594560844161373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
-      <c r="H124" s="6" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
-      <c r="I124" s="3" t="inlineStr">
+      <c r="H125" s="6" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="I125" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
-      <c r="J124" s="2" t="inlineStr">
-        <is>
-          <t>Nueva</t>
-        </is>
-      </c>
-      <c r="K124" s="3" t="inlineStr"/>
+      <c r="J125" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K125" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
chore(tracker): actualizacion diaria de vacantes 2026-10-20
</commit_message>
<xml_diff>
--- a/output/profile_5_tecnico_sistemas_tracker.xlsx
+++ b/output/profile_5_tecnico_sistemas_tracker.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K126"/>
+  <dimension ref="A1:K129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="29" customWidth="1" min="8" max="8"/>
     <col width="65" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
     <col width="32" customWidth="1" min="11" max="11"/>
@@ -3672,26 +3672,26 @@
     <row r="68" ht="22" customHeight="1">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>ae736277661dc78b</t>
+          <t>4f7da6e4dec08863</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 15:23</t>
+          <t>2026-10-20 15:43</t>
         </is>
       </c>
       <c r="C68" s="3" t="inlineStr">
         <is>
-          <t>Analista de redes cisco</t>
+          <t>Buscamos Bachilleres con experiencia en Soporte Técnico // Teletrabajo</t>
         </is>
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
-          <t>ATCG DE COLOMBIA S.A.S</t>
-        </is>
-      </c>
-      <c r="E68" s="7" t="n">
-        <v>0.68</v>
+          <t>emtelco</t>
+        </is>
+      </c>
+      <c r="E68" s="4" t="n">
+        <v>0.73</v>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
@@ -3699,13 +3699,17 @@
         </is>
       </c>
       <c r="G68" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-cisco-1886760389", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H68" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-buscamos-bachilleres-con-experiencia-en-soporte-tecnico-teletrabajo-bachilleres-con-experiencia-en-el-area-en-medellin-1B5720BBA7ED612461373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H68" s="6" t="inlineStr">
+        <is>
+          <t>$ 1.750.905,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I68" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 68/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 73/100 - Alta Afinidad] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J68" s="2" t="inlineStr">
@@ -3718,7 +3722,7 @@
     <row r="69" ht="22" customHeight="1">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>e29676fac3409ad6</t>
+          <t>ae736277661dc78b</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
@@ -3728,12 +3732,12 @@
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>Analista de redes y telecomunicaciones - nivel 1</t>
+          <t>Analista de redes cisco</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>MANPOWER</t>
+          <t>ATCG DE COLOMBIA S.A.S</t>
         </is>
       </c>
       <c r="E69" s="7" t="n">
@@ -3745,7 +3749,7 @@
         </is>
       </c>
       <c r="G69" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-y-telecomunicaciones-nivel-1-1886760565", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-cisco-1886760389", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H69" s="6" t="inlineStr"/>
@@ -3764,26 +3768,26 @@
     <row r="70" ht="22" customHeight="1">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>baf000f38713dc11</t>
+          <t>e29676fac3409ad6</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07 17:50</t>
+          <t>2026-09-24 15:23</t>
         </is>
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>Helpdesk / Analista soporte TI / trilingüe</t>
+          <t>Analista de redes y telecomunicaciones - nivel 1</t>
         </is>
       </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
-          <t>Confidential</t>
+          <t>MANPOWER</t>
         </is>
       </c>
       <c r="E70" s="7" t="n">
-        <v>0.66</v>
+        <v>0.68</v>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
@@ -3791,13 +3795,13 @@
         </is>
       </c>
       <c r="G70" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/helpdesk-analista-soporte-ti-triling%C3%BCe-ingles-portugu%C3%A9s-at-confidential-4469673592", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-y-telecomunicaciones-nivel-1-1886760565", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H70" s="6" t="inlineStr"/>
       <c r="I70" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 66/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 68/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J70" s="2" t="inlineStr">
@@ -3810,22 +3814,22 @@
     <row r="71" ht="22" customHeight="1">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>422a27df3967ecbb</t>
+          <t>baf000f38713dc11</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14 15:52</t>
+          <t>2026-10-07 17:50</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>Técnico de sistemas y soporte ti</t>
+          <t>Helpdesk / Analista soporte TI / trilingüe</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>AGENCIA DE EMPLEO CAFAM</t>
+          <t>Confidential</t>
         </is>
       </c>
       <c r="E71" s="7" t="n">
@@ -3837,7 +3841,7 @@
         </is>
       </c>
       <c r="G71" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-sistemas-y-soporte-ti-1886780022", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/helpdesk-analista-soporte-ti-triling%C3%BCe-ingles-portugu%C3%A9s-at-confidential-4469673592", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H71" s="6" t="inlineStr"/>
@@ -3856,26 +3860,26 @@
     <row r="72" ht="22" customHeight="1">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>73882c81e04abc7e</t>
+          <t>422a27df3967ecbb</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 19:45</t>
+          <t>2026-10-14 15:52</t>
         </is>
       </c>
       <c r="C72" s="3" t="inlineStr">
         <is>
-          <t>Soporte L1 Junior</t>
+          <t>Técnico de sistemas y soporte ti</t>
         </is>
       </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
-          <t>Hublance</t>
+          <t>AGENCIA DE EMPLEO CAFAM</t>
         </is>
       </c>
       <c r="E72" s="7" t="n">
-        <v>0.6</v>
+        <v>0.66</v>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
@@ -3883,13 +3887,13 @@
         </is>
       </c>
       <c r="G72" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/soporte-l1-junior-at-hublance-4475841269", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-sistemas-y-soporte-ti-1886780022", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H72" s="6" t="inlineStr"/>
       <c r="I72" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 60/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 66/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J72" s="2" t="inlineStr">
@@ -3902,26 +3906,26 @@
     <row r="73" ht="22" customHeight="1">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>8d7f304ffb8625b5</t>
+          <t>73882c81e04abc7e</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 15:54</t>
+          <t>2026-10-05 19:45</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar de sistemas</t>
+          <t>Soporte L1 Junior</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Hublance</t>
         </is>
       </c>
       <c r="E73" s="7" t="n">
-        <v>0.58</v>
+        <v>0.6</v>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
@@ -3929,13 +3933,13 @@
         </is>
       </c>
       <c r="G73" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886751888", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/soporte-l1-junior-at-hublance-4475841269", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H73" s="6" t="inlineStr"/>
       <c r="I73" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 60/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J73" s="2" t="inlineStr">
@@ -3948,7 +3952,7 @@
     <row r="74" ht="22" customHeight="1">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>3b5b26f92a305c0c</t>
+          <t>8d7f304ffb8625b5</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
@@ -3975,7 +3979,7 @@
         </is>
       </c>
       <c r="G74" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886749497", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886751888", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H74" s="6" t="inlineStr"/>
@@ -3994,7 +3998,7 @@
     <row r="75" ht="22" customHeight="1">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>e760bcd88d90fbbe</t>
+          <t>3b5b26f92a305c0c</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
@@ -4004,12 +4008,12 @@
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>Agente de mesa de ayuda</t>
+          <t>Auxiliar de sistemas</t>
         </is>
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>SELCOMP INGENIERÍA SAS</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E75" s="7" t="n">
@@ -4021,7 +4025,7 @@
         </is>
       </c>
       <c r="G75" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-de-mesa-de-ayuda-1886758623", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886749497", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H75" s="6" t="inlineStr"/>
@@ -4040,7 +4044,7 @@
     <row r="76" ht="22" customHeight="1">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>86dcab5c5d802693</t>
+          <t>e760bcd88d90fbbe</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
@@ -4050,12 +4054,12 @@
       </c>
       <c r="C76" s="3" t="inlineStr">
         <is>
-          <t>Analista mesa de ayuda para tunja</t>
+          <t>Agente de mesa de ayuda</t>
         </is>
       </c>
       <c r="D76" s="3" t="inlineStr">
         <is>
-          <t>Gestión de Seguridad Electrónica</t>
+          <t>SELCOMP INGENIERÍA SAS</t>
         </is>
       </c>
       <c r="E76" s="7" t="n">
@@ -4067,7 +4071,7 @@
         </is>
       </c>
       <c r="G76" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-para-tunja-1886766955", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-de-mesa-de-ayuda-1886758623", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H76" s="6" t="inlineStr"/>
@@ -4086,7 +4090,7 @@
     <row r="77" ht="22" customHeight="1">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>55fdaa0983ef9124</t>
+          <t>86dcab5c5d802693</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
@@ -4096,12 +4100,12 @@
       </c>
       <c r="C77" s="3" t="inlineStr">
         <is>
-          <t>Lider técnico con itil practice manager</t>
+          <t>Analista mesa de ayuda para tunja</t>
         </is>
       </c>
       <c r="D77" s="3" t="inlineStr">
         <is>
-          <t>Sinergy &amp; Lowells</t>
+          <t>Gestión de Seguridad Electrónica</t>
         </is>
       </c>
       <c r="E77" s="7" t="n">
@@ -4113,7 +4117,7 @@
         </is>
       </c>
       <c r="G77" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/lider-tecnico-con-itil-practice-manager-1886753953", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-para-tunja-1886766955", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H77" s="6" t="inlineStr"/>
@@ -4132,7 +4136,7 @@
     <row r="78" ht="22" customHeight="1">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>a1ca7bc58cd48fad</t>
+          <t>55fdaa0983ef9124</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -4142,12 +4146,12 @@
       </c>
       <c r="C78" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de mesa de ayuda/mujeres contratacion inmediata</t>
+          <t>Lider técnico con itil practice manager</t>
         </is>
       </c>
       <c r="D78" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Sinergy &amp; Lowells</t>
         </is>
       </c>
       <c r="E78" s="7" t="n">
@@ -4159,7 +4163,7 @@
         </is>
       </c>
       <c r="G78" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-mesa-de-ayuda-mujeres-contratacion-inmediata-1886770931", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/lider-tecnico-con-itil-practice-manager-1886753953", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H78" s="6" t="inlineStr"/>
@@ -4178,7 +4182,7 @@
     <row r="79" ht="22" customHeight="1">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>e28aba5df8a2d3ae</t>
+          <t>a1ca7bc58cd48fad</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
@@ -4205,7 +4209,7 @@
         </is>
       </c>
       <c r="G79" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-mesa-de-ayuda-mujeres-contratacion-inmediata-1886769701", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-mesa-de-ayuda-mujeres-contratacion-inmediata-1886770931", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H79" s="6" t="inlineStr"/>
@@ -4224,7 +4228,7 @@
     <row r="80" ht="22" customHeight="1">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>9326784c1a2726fb</t>
+          <t>e28aba5df8a2d3ae</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
@@ -4234,12 +4238,12 @@
       </c>
       <c r="C80" s="3" t="inlineStr">
         <is>
-          <t>Técnico de soporte y mesa de ayuda / medellín</t>
+          <t>Tecnico de mesa de ayuda/mujeres contratacion inmediata</t>
         </is>
       </c>
       <c r="D80" s="3" t="inlineStr">
         <is>
-          <t>Colsof S.A.S</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E80" s="7" t="n">
@@ -4251,7 +4255,7 @@
         </is>
       </c>
       <c r="G80" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-y-mesa-de-ayuda-medellin-1886738118", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-mesa-de-ayuda-mujeres-contratacion-inmediata-1886769701", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H80" s="6" t="inlineStr"/>
@@ -4270,7 +4274,7 @@
     <row r="81" ht="22" customHeight="1">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>b67dc9a9be4a1a6f</t>
+          <t>9326784c1a2726fb</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
@@ -4280,12 +4284,12 @@
       </c>
       <c r="C81" s="3" t="inlineStr">
         <is>
-          <t>Service desk agent</t>
+          <t>Técnico de soporte y mesa de ayuda / medellín</t>
         </is>
       </c>
       <c r="D81" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Colsof S.A.S</t>
         </is>
       </c>
       <c r="E81" s="7" t="n">
@@ -4297,13 +4301,13 @@
         </is>
       </c>
       <c r="G81" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/service-desk-agent-soporte-tecnico-nivel-1-1886755112", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-y-mesa-de-ayuda-medellin-1886738118", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H81" s="6" t="inlineStr"/>
       <c r="I81" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J81" s="2" t="inlineStr">
@@ -4316,7 +4320,7 @@
     <row r="82" ht="22" customHeight="1">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>9c65f710f43158b7</t>
+          <t>b67dc9a9be4a1a6f</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
@@ -4326,7 +4330,7 @@
       </c>
       <c r="C82" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de instalaciones cableado de redes - licencia conte</t>
+          <t>Service desk agent</t>
         </is>
       </c>
       <c r="D82" s="3" t="inlineStr">
@@ -4343,13 +4347,13 @@
         </is>
       </c>
       <c r="G82" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-1886749397", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/service-desk-agent-soporte-tecnico-nivel-1-1886755112", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H82" s="6" t="inlineStr"/>
       <c r="I82" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J82" s="2" t="inlineStr">
@@ -4362,22 +4366,22 @@
     <row r="83" ht="22" customHeight="1">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>a95003a0b1fc3d77</t>
+          <t>9c65f710f43158b7</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 15:41</t>
+          <t>2026-09-25 15:54</t>
         </is>
       </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t>Técnico Soporte Nivel 1 Con ITIL</t>
+          <t>Tecnico de instalaciones cableado de redes - licencia conte</t>
         </is>
       </c>
       <c r="D83" s="3" t="inlineStr">
         <is>
-          <t>Importante empresa del sector de tecnología</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E83" s="7" t="n">
@@ -4389,14 +4393,10 @@
         </is>
       </c>
       <c r="G83" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-soporte-nivel-1-con-itil-en-bogota-dc-59E13FA64EF5843C61373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H83" s="6" t="inlineStr">
-        <is>
-          <t>$ 1.750.905,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-1886749397", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H83" s="6" t="inlineStr"/>
       <c r="I83" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -4412,7 +4412,7 @@
     <row r="84" ht="22" customHeight="1">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>96391fd564d83616</t>
+          <t>a95003a0b1fc3d77</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
@@ -4422,12 +4422,12 @@
       </c>
       <c r="C84" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de soporte IT con Moto</t>
+          <t>Técnico Soporte Nivel 1 Con ITIL</t>
         </is>
       </c>
       <c r="D84" s="3" t="inlineStr">
         <is>
-          <t>Los Hornitos</t>
+          <t>Importante empresa del sector de tecnología</t>
         </is>
       </c>
       <c r="E84" s="7" t="n">
@@ -4439,12 +4439,12 @@
         </is>
       </c>
       <c r="G84" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-it-con-moto-empresa-de-alimentos-en-bogota-dc-599938D46A6F4A8F61373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-soporte-nivel-1-con-itil-en-bogota-dc-59E13FA64EF5843C61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H84" s="6" t="inlineStr">
         <is>
-          <t>$ 2.125.947,00 (Mensual)</t>
+          <t>$ 1.750.905,00 (Mensual)</t>
         </is>
       </c>
       <c r="I84" s="3" t="inlineStr">
@@ -4462,7 +4462,7 @@
     <row r="85" ht="22" customHeight="1">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>b4f0b8c16fe5543e</t>
+          <t>96391fd564d83616</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
@@ -4472,12 +4472,12 @@
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar de Sistemas</t>
+          <t>Tecnico de soporte IT con Moto</t>
         </is>
       </c>
       <c r="D85" s="3" t="inlineStr">
         <is>
-          <t>ELIS COLOMBIA SAS</t>
+          <t>Los Hornitos</t>
         </is>
       </c>
       <c r="E85" s="7" t="n">
@@ -4489,12 +4489,12 @@
         </is>
       </c>
       <c r="G85" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-en-bogota-dc-48C2A0A3B050945661373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-it-con-moto-empresa-de-alimentos-en-bogota-dc-599938D46A6F4A8F61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H85" s="6" t="inlineStr">
         <is>
-          <t>$ 2.000.000,00 (Mensual)</t>
+          <t>$ 2.125.947,00 (Mensual)</t>
         </is>
       </c>
       <c r="I85" s="3" t="inlineStr">
@@ -4512,7 +4512,7 @@
     <row r="86" ht="22" customHeight="1">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>7e4b4e4f136a5e31</t>
+          <t>b4f0b8c16fe5543e</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
@@ -4522,12 +4522,12 @@
       </c>
       <c r="C86" s="3" t="inlineStr">
         <is>
-          <t>Agente Mesa de Ayuda</t>
+          <t>Auxiliar de Sistemas</t>
         </is>
       </c>
       <c r="D86" s="3" t="inlineStr">
         <is>
-          <t>Importante empresa del sector</t>
+          <t>ELIS COLOMBIA SAS</t>
         </is>
       </c>
       <c r="E86" s="7" t="n">
@@ -4539,7 +4539,7 @@
         </is>
       </c>
       <c r="G86" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-agente-mesa-de-ayuda-en-bogota-dc-E39FE355E02E578761373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-en-bogota-dc-48C2A0A3B050945661373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H86" s="6" t="inlineStr">
@@ -4562,7 +4562,7 @@
     <row r="87" ht="22" customHeight="1">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>0ef2cd7667600919</t>
+          <t>7e4b4e4f136a5e31</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
@@ -4572,12 +4572,12 @@
       </c>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>Técnico de Soporte TI Regional</t>
+          <t>Agente Mesa de Ayuda</t>
         </is>
       </c>
       <c r="D87" s="3" t="inlineStr">
         <is>
-          <t>POLICOMP COLOMBIA SAS</t>
+          <t>Importante empresa del sector</t>
         </is>
       </c>
       <c r="E87" s="7" t="n">
@@ -4589,10 +4589,14 @@
         </is>
       </c>
       <c r="G87" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-ti-regional-en-bogota-dc-ACF045C94E41CCDE61373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H87" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-agente-mesa-de-ayuda-en-bogota-dc-E39FE355E02E578761373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H87" s="6" t="inlineStr">
+        <is>
+          <t>$ 2.000.000,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I87" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -4608,7 +4612,7 @@
     <row r="88" ht="22" customHeight="1">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>7784997bda962255</t>
+          <t>0ef2cd7667600919</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
@@ -4618,7 +4622,7 @@
       </c>
       <c r="C88" s="3" t="inlineStr">
         <is>
-          <t>Técnico de Soporte TI On Demand/ por horas</t>
+          <t>Técnico de Soporte TI Regional</t>
         </is>
       </c>
       <c r="D88" s="3" t="inlineStr">
@@ -4635,7 +4639,7 @@
         </is>
       </c>
       <c r="G88" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-ti-on-demand-por-horas-en-bogota-dc-C2338FA0172D59A561373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-ti-regional-en-bogota-dc-ACF045C94E41CCDE61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H88" s="6" t="inlineStr"/>
@@ -4654,7 +4658,7 @@
     <row r="89" ht="22" customHeight="1">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>29d0fe2e42e678f7</t>
+          <t>7784997bda962255</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
@@ -4664,12 +4668,12 @@
       </c>
       <c r="C89" s="3" t="inlineStr">
         <is>
-          <t>Técnico mantenimiento correctivo impresoras</t>
+          <t>Técnico de Soporte TI On Demand/ por horas</t>
         </is>
       </c>
       <c r="D89" s="3" t="inlineStr">
         <is>
-          <t>Multinacional de Impresión</t>
+          <t>POLICOMP COLOMBIA SAS</t>
         </is>
       </c>
       <c r="E89" s="7" t="n">
@@ -4681,14 +4685,10 @@
         </is>
       </c>
       <c r="G89" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-mantenimiento-correctivo-impresoras-en-guarne-BC0E775C0F25B27D61373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H89" s="6" t="inlineStr">
-        <is>
-          <t>$ 1.800.000,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-ti-on-demand-por-horas-en-bogota-dc-C2338FA0172D59A561373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H89" s="6" t="inlineStr"/>
       <c r="I89" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -4704,22 +4704,22 @@
     <row r="90" ht="22" customHeight="1">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>98c9ab11f5b1eace</t>
+          <t>29d0fe2e42e678f7</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 18:36</t>
+          <t>2026-09-27 15:41</t>
         </is>
       </c>
       <c r="C90" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar de sistemas</t>
+          <t>Técnico mantenimiento correctivo impresoras</t>
         </is>
       </c>
       <c r="D90" s="3" t="inlineStr">
         <is>
-          <t>Importante empresa del sector</t>
+          <t>Multinacional de Impresión</t>
         </is>
       </c>
       <c r="E90" s="7" t="n">
@@ -4731,12 +4731,12 @@
         </is>
       </c>
       <c r="G90" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-persona-con-discapacidad-remota-en-bogota-dc-5F2A812D014E159B61373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-mantenimiento-correctivo-impresoras-en-guarne-BC0E775C0F25B27D61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H90" s="6" t="inlineStr">
         <is>
-          <t>$ 1.750.905,00 (Mensual)</t>
+          <t>$ 1.800.000,00 (Mensual)</t>
         </is>
       </c>
       <c r="I90" s="3" t="inlineStr">
@@ -4754,7 +4754,7 @@
     <row r="91" ht="22" customHeight="1">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>58133ddc4da9c68e</t>
+          <t>98c9ab11f5b1eace</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
@@ -4781,7 +4781,7 @@
         </is>
       </c>
       <c r="G91" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-persona-con-discapacidad-remota-en-bogota-dc-A00C07C9CC9A494B61373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-persona-con-discapacidad-remota-en-bogota-dc-5F2A812D014E159B61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H91" s="6" t="inlineStr">
@@ -4804,7 +4804,7 @@
     <row r="92" ht="22" customHeight="1">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>aed3420a4cfdc248</t>
+          <t>58133ddc4da9c68e</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
@@ -4814,12 +4814,12 @@
       </c>
       <c r="C92" s="3" t="inlineStr">
         <is>
-          <t>Consultor de servicios/ mesa de ayuda nómina y erp software</t>
+          <t>Auxiliar de sistemas</t>
         </is>
       </c>
       <c r="D92" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Importante empresa del sector</t>
         </is>
       </c>
       <c r="E92" s="7" t="n">
@@ -4831,10 +4831,14 @@
         </is>
       </c>
       <c r="G92" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/consultor-de-servicios-mesa-de-ayuda-nomina-y-erp-software-inclusivo-1886716126", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H92" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-persona-con-discapacidad-remota-en-bogota-dc-A00C07C9CC9A494B61373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H92" s="6" t="inlineStr">
+        <is>
+          <t>$ 1.750.905,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I92" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -4850,22 +4854,22 @@
     <row r="93" ht="22" customHeight="1">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>2b8357189ff315da</t>
+          <t>aed3420a4cfdc248</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 17:00</t>
+          <t>2026-09-28 18:36</t>
         </is>
       </c>
       <c r="C93" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar de sistemas</t>
+          <t>Consultor de servicios/ mesa de ayuda nómina y erp software</t>
         </is>
       </c>
       <c r="D93" s="3" t="inlineStr">
         <is>
-          <t>DAVITA SAS</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E93" s="7" t="n">
@@ -4877,7 +4881,7 @@
         </is>
       </c>
       <c r="G93" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886758163", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/consultor-de-servicios-mesa-de-ayuda-nomina-y-erp-software-inclusivo-1886716126", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H93" s="6" t="inlineStr"/>
@@ -4896,7 +4900,7 @@
     <row r="94" ht="22" customHeight="1">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>a87934e7643b2c1c</t>
+          <t>2b8357189ff315da</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
@@ -4906,12 +4910,12 @@
       </c>
       <c r="C94" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de instalaciones cableado de redes - licencia conte cali</t>
+          <t>Auxiliar de sistemas</t>
         </is>
       </c>
       <c r="D94" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>DAVITA SAS</t>
         </is>
       </c>
       <c r="E94" s="7" t="n">
@@ -4923,7 +4927,7 @@
         </is>
       </c>
       <c r="G94" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-cali-1886759847", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886758163", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H94" s="6" t="inlineStr"/>
@@ -4942,7 +4946,7 @@
     <row r="95" ht="22" customHeight="1">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>10b4265e3ad11d81</t>
+          <t>a87934e7643b2c1c</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr">
@@ -4952,12 +4956,12 @@
       </c>
       <c r="C95" s="3" t="inlineStr">
         <is>
-          <t>Information Technology Help Desk Support</t>
+          <t>Tecnico de instalaciones cableado de redes - licencia conte cali</t>
         </is>
       </c>
       <c r="D95" s="3" t="inlineStr">
         <is>
-          <t>Booth</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E95" s="7" t="n">
@@ -4969,7 +4973,7 @@
         </is>
       </c>
       <c r="G95" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/information-technology-help-desk-support-at-booth-4471203962", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-cali-1886759847", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H95" s="6" t="inlineStr"/>
@@ -4988,22 +4992,22 @@
     <row r="96" ht="22" customHeight="1">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>ff69ae85c8697a37</t>
+          <t>10b4265e3ad11d81</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 16:49</t>
+          <t>2026-09-29 17:00</t>
         </is>
       </c>
       <c r="C96" s="3" t="inlineStr">
         <is>
-          <t>Técnico de soporte ti - bogota</t>
+          <t>Information Technology Help Desk Support</t>
         </is>
       </c>
       <c r="D96" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Booth</t>
         </is>
       </c>
       <c r="E96" s="7" t="n">
@@ -5015,7 +5019,7 @@
         </is>
       </c>
       <c r="G96" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-ti-bogota-1886774059", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/information-technology-help-desk-support-at-booth-4471203962", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H96" s="6" t="inlineStr"/>
@@ -5034,7 +5038,7 @@
     <row r="97" ht="22" customHeight="1">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>bbacf7d69ab9084e</t>
+          <t>ff69ae85c8697a37</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
@@ -5044,12 +5048,12 @@
       </c>
       <c r="C97" s="3" t="inlineStr">
         <is>
-          <t>IT Helpdesk Analyst</t>
+          <t>Técnico de soporte ti - bogota</t>
         </is>
       </c>
       <c r="D97" s="3" t="inlineStr">
         <is>
-          <t>Power Digital Marketing</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E97" s="7" t="n">
@@ -5061,7 +5065,7 @@
         </is>
       </c>
       <c r="G97" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/it-helpdesk-analyst-at-power-digital-marketing-4472601999", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-ti-bogota-1886774059", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H97" s="6" t="inlineStr"/>
@@ -5080,22 +5084,22 @@
     <row r="98" ht="22" customHeight="1">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>bb848f474ff4b611</t>
+          <t>bbacf7d69ab9084e</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 17:26</t>
+          <t>2026-09-30 16:49</t>
         </is>
       </c>
       <c r="C98" s="3" t="inlineStr">
         <is>
-          <t>Técnico de soporte ti - bogota</t>
+          <t>IT Helpdesk Analyst</t>
         </is>
       </c>
       <c r="D98" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Power Digital Marketing</t>
         </is>
       </c>
       <c r="E98" s="7" t="n">
@@ -5107,7 +5111,7 @@
         </is>
       </c>
       <c r="G98" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-ti-bogota-1886772292", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/it-helpdesk-analyst-at-power-digital-marketing-4472601999", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H98" s="6" t="inlineStr"/>
@@ -5126,7 +5130,7 @@
     <row r="99" ht="22" customHeight="1">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>b44a1c6cfb004ca8</t>
+          <t>bb848f474ff4b611</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
@@ -5136,7 +5140,7 @@
       </c>
       <c r="C99" s="3" t="inlineStr">
         <is>
-          <t>Soporte ti nivel 2 - bogotá</t>
+          <t>Técnico de soporte ti - bogota</t>
         </is>
       </c>
       <c r="D99" s="3" t="inlineStr">
@@ -5153,7 +5157,7 @@
         </is>
       </c>
       <c r="G99" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/soporte-ti-nivel-2-bogota-1886774821", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-ti-bogota-1886772292", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H99" s="6" t="inlineStr"/>
@@ -5172,7 +5176,7 @@
     <row r="100" ht="22" customHeight="1">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>fb0ad2b513afb97c</t>
+          <t>b44a1c6cfb004ca8</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
@@ -5182,12 +5186,12 @@
       </c>
       <c r="C100" s="3" t="inlineStr">
         <is>
-          <t>IT Help Desk Support Specialist</t>
+          <t>Soporte ti nivel 2 - bogotá</t>
         </is>
       </c>
       <c r="D100" s="3" t="inlineStr">
         <is>
-          <t>Talento</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E100" s="7" t="n">
@@ -5199,7 +5203,7 @@
         </is>
       </c>
       <c r="G100" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/it-help-desk-support-specialist-tier-1-at-talento-4473960480", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/soporte-ti-nivel-2-bogota-1886774821", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H100" s="6" t="inlineStr"/>
@@ -5218,22 +5222,22 @@
     <row r="101" ht="22" customHeight="1">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>0b2067d6ae488f4c</t>
+          <t>fb0ad2b513afb97c</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 16:39</t>
+          <t>2026-10-01 17:26</t>
         </is>
       </c>
       <c r="C101" s="3" t="inlineStr">
         <is>
-          <t>Help Desk Technician level 1</t>
+          <t>IT Help Desk Support Specialist</t>
         </is>
       </c>
       <c r="D101" s="3" t="inlineStr">
         <is>
-          <t>Solvo Global</t>
+          <t>Talento</t>
         </is>
       </c>
       <c r="E101" s="7" t="n">
@@ -5245,7 +5249,7 @@
         </is>
       </c>
       <c r="G101" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/help-desk-technician-level-1-at-solvo-global-4472590892", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/it-help-desk-support-specialist-tier-1-at-talento-4473960480", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H101" s="6" t="inlineStr"/>
@@ -5264,22 +5268,22 @@
     <row r="102" ht="22" customHeight="1">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>07acc222a3ca2ef1</t>
+          <t>0b2067d6ae488f4c</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03 15:12</t>
+          <t>2026-10-02 16:39</t>
         </is>
       </c>
       <c r="C102" s="3" t="inlineStr">
         <is>
-          <t>Analista mesa de ayuda funza temporal 6 meses</t>
+          <t>Help Desk Technician level 1</t>
         </is>
       </c>
       <c r="D102" s="3" t="inlineStr">
         <is>
-          <t>Axity</t>
+          <t>Solvo Global</t>
         </is>
       </c>
       <c r="E102" s="7" t="n">
@@ -5291,7 +5295,7 @@
         </is>
       </c>
       <c r="G102" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-funza-temporal-6-meses-1886774524", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/help-desk-technician-level-1-at-solvo-global-4472590892", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H102" s="6" t="inlineStr"/>
@@ -5310,22 +5314,22 @@
     <row r="103" ht="22" customHeight="1">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>5ec0ea33876ba2b5</t>
+          <t>07acc222a3ca2ef1</t>
         </is>
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 19:45</t>
+          <t>2026-10-03 15:12</t>
         </is>
       </c>
       <c r="C103" s="3" t="inlineStr">
         <is>
-          <t>Help desk analyst l1</t>
+          <t>Analista mesa de ayuda funza temporal 6 meses</t>
         </is>
       </c>
       <c r="D103" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Axity</t>
         </is>
       </c>
       <c r="E103" s="7" t="n">
@@ -5337,7 +5341,7 @@
         </is>
       </c>
       <c r="G103" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/help-desk-analyst-l1-medellin-1886776156", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-funza-temporal-6-meses-1886774524", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H103" s="6" t="inlineStr"/>
@@ -5356,7 +5360,7 @@
     <row r="104" ht="22" customHeight="1">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>e8bdf2094d1c9817</t>
+          <t>5ec0ea33876ba2b5</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
@@ -5366,12 +5370,12 @@
       </c>
       <c r="C104" s="3" t="inlineStr">
         <is>
-          <t>Administrador de herramienta de gestión de mesa de ayuda-</t>
+          <t>Help desk analyst l1</t>
         </is>
       </c>
       <c r="D104" s="3" t="inlineStr">
         <is>
-          <t>SELCOMP INGENIERÍA SAS</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E104" s="7" t="n">
@@ -5383,7 +5387,7 @@
         </is>
       </c>
       <c r="G104" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/administrador-de-herramienta-de-gestion-de-mesa-de-ayuda-1886776286", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/help-desk-analyst-l1-medellin-1886776156", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H104" s="6" t="inlineStr"/>
@@ -5402,7 +5406,7 @@
     <row r="105" ht="22" customHeight="1">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>6e9a077b42879470</t>
+          <t>e8bdf2094d1c9817</t>
         </is>
       </c>
       <c r="B105" s="2" t="inlineStr">
@@ -5412,12 +5416,12 @@
       </c>
       <c r="C105" s="3" t="inlineStr">
         <is>
-          <t>Analista de soporte de aplicaciones nivel 3</t>
+          <t>Administrador de herramienta de gestión de mesa de ayuda-</t>
         </is>
       </c>
       <c r="D105" s="3" t="inlineStr">
         <is>
-          <t>TALYCAP GLOBAL SAS</t>
+          <t>SELCOMP INGENIERÍA SAS</t>
         </is>
       </c>
       <c r="E105" s="7" t="n">
@@ -5429,7 +5433,7 @@
         </is>
       </c>
       <c r="G105" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-soporte-de-aplicaciones-nivel-3-1886776104", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/administrador-de-herramienta-de-gestion-de-mesa-de-ayuda-1886776286", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H105" s="6" t="inlineStr"/>
@@ -5448,22 +5452,22 @@
     <row r="106" ht="22" customHeight="1">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>447afec244b20f9b</t>
+          <t>6e9a077b42879470</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06 17:12</t>
+          <t>2026-10-05 19:45</t>
         </is>
       </c>
       <c r="C106" s="3" t="inlineStr">
         <is>
-          <t>Técnico de soporte ti - bogota</t>
+          <t>Analista de soporte de aplicaciones nivel 3</t>
         </is>
       </c>
       <c r="D106" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>TALYCAP GLOBAL SAS</t>
         </is>
       </c>
       <c r="E106" s="7" t="n">
@@ -5475,7 +5479,7 @@
         </is>
       </c>
       <c r="G106" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-ti-bogota-1886775990", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-soporte-de-aplicaciones-nivel-3-1886776104", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H106" s="6" t="inlineStr"/>
@@ -5494,22 +5498,22 @@
     <row r="107" ht="22" customHeight="1">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>8f14c41f3b443ac0</t>
+          <t>447afec244b20f9b</t>
         </is>
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07 17:50</t>
+          <t>2026-10-06 17:12</t>
         </is>
       </c>
       <c r="C107" s="3" t="inlineStr">
         <is>
-          <t>Soporte mesa de ayuda</t>
+          <t>Técnico de soporte ti - bogota</t>
         </is>
       </c>
       <c r="D107" s="3" t="inlineStr">
         <is>
-          <t>MANPOWER</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E107" s="7" t="n">
@@ -5521,7 +5525,7 @@
         </is>
       </c>
       <c r="G107" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/soporte-mesa-de-ayuda-vacaciones-1886776917", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-ti-bogota-1886775990", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H107" s="6" t="inlineStr"/>
@@ -5540,7 +5544,7 @@
     <row r="108" ht="22" customHeight="1">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>b1a9e03967fff91e</t>
+          <t>8f14c41f3b443ac0</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr">
@@ -5550,12 +5554,12 @@
       </c>
       <c r="C108" s="3" t="inlineStr">
         <is>
-          <t>Tecnólogo de soporte pl - mesa de ayuda</t>
+          <t>Soporte mesa de ayuda</t>
         </is>
       </c>
       <c r="D108" s="3" t="inlineStr">
         <is>
-          <t>Positivo S+</t>
+          <t>MANPOWER</t>
         </is>
       </c>
       <c r="E108" s="7" t="n">
@@ -5567,7 +5571,7 @@
         </is>
       </c>
       <c r="G108" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnologo-de-soporte-pl-mesa-de-ayuda-1886775546", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/soporte-mesa-de-ayuda-vacaciones-1886776917", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H108" s="6" t="inlineStr"/>
@@ -5586,7 +5590,7 @@
     <row r="109" ht="22" customHeight="1">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>eb49981c97933d93</t>
+          <t>b1a9e03967fff91e</t>
         </is>
       </c>
       <c r="B109" s="2" t="inlineStr">
@@ -5596,12 +5600,12 @@
       </c>
       <c r="C109" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de instalaciones cableado de redes - licencia conte</t>
+          <t>Tecnólogo de soporte pl - mesa de ayuda</t>
         </is>
       </c>
       <c r="D109" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Positivo S+</t>
         </is>
       </c>
       <c r="E109" s="7" t="n">
@@ -5613,7 +5617,7 @@
         </is>
       </c>
       <c r="G109" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-1886777333", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnologo-de-soporte-pl-mesa-de-ayuda-1886775546", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H109" s="6" t="inlineStr"/>
@@ -5632,7 +5636,7 @@
     <row r="110" ht="22" customHeight="1">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>d39af22b6e937d28</t>
+          <t>eb49981c97933d93</t>
         </is>
       </c>
       <c r="B110" s="2" t="inlineStr">
@@ -5642,12 +5646,12 @@
       </c>
       <c r="C110" s="3" t="inlineStr">
         <is>
-          <t>Analista Mesa de Ayuda Funza</t>
+          <t>Tecnico de instalaciones cableado de redes - licencia conte</t>
         </is>
       </c>
       <c r="D110" s="3" t="inlineStr">
         <is>
-          <t>axity</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E110" s="7" t="n">
@@ -5659,7 +5663,7 @@
         </is>
       </c>
       <c r="G110" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/analista-mesa-de-ayuda-funza-at-axity-4471985006", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-1886777333", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H110" s="6" t="inlineStr"/>
@@ -5678,22 +5682,22 @@
     <row r="111" ht="22" customHeight="1">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>0904912d51c5cd61</t>
+          <t>d39af22b6e937d28</t>
         </is>
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08 17:52</t>
+          <t>2026-10-07 17:50</t>
         </is>
       </c>
       <c r="C111" s="3" t="inlineStr">
         <is>
-          <t>Analista mesa de ayuda</t>
+          <t>Analista Mesa de Ayuda Funza</t>
         </is>
       </c>
       <c r="D111" s="3" t="inlineStr">
         <is>
-          <t>Desarrollo de Sistemas y Servicios SAS</t>
+          <t>axity</t>
         </is>
       </c>
       <c r="E111" s="7" t="n">
@@ -5705,7 +5709,7 @@
         </is>
       </c>
       <c r="G111" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-1886778032", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/analista-mesa-de-ayuda-funza-at-axity-4471985006", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H111" s="6" t="inlineStr"/>
@@ -5724,22 +5728,22 @@
     <row r="112" ht="22" customHeight="1">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>c665ada630270dce</t>
+          <t>0904912d51c5cd61</t>
         </is>
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09 17:28</t>
+          <t>2026-10-08 17:52</t>
         </is>
       </c>
       <c r="C112" s="3" t="inlineStr">
         <is>
-          <t>Técnico(a) / tecnólogo(a) / profesional de telecomunicaciones - redes de fibra óptica</t>
+          <t>Analista mesa de ayuda</t>
         </is>
       </c>
       <c r="D112" s="3" t="inlineStr">
         <is>
-          <t>JAHV MC GREGOR S.A.S</t>
+          <t>Desarrollo de Sistemas y Servicios SAS</t>
         </is>
       </c>
       <c r="E112" s="7" t="n">
@@ -5751,7 +5755,7 @@
         </is>
       </c>
       <c r="G112" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnicoa-tecnologoa-profesional-de-telecomunicaciones-redes-de-fibra-optica-1886768691", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-1886778032", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H112" s="6" t="inlineStr"/>
@@ -5770,7 +5774,7 @@
     <row r="113" ht="22" customHeight="1">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>4e5b3128aa7f8f9b</t>
+          <t>c665ada630270dce</t>
         </is>
       </c>
       <c r="B113" s="2" t="inlineStr">
@@ -5780,12 +5784,12 @@
       </c>
       <c r="C113" s="3" t="inlineStr">
         <is>
-          <t>Gestor de servicios mesa de ayuda sap</t>
+          <t>Técnico(a) / tecnólogo(a) / profesional de telecomunicaciones - redes de fibra óptica</t>
         </is>
       </c>
       <c r="D113" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>JAHV MC GREGOR S.A.S</t>
         </is>
       </c>
       <c r="E113" s="7" t="n">
@@ -5797,7 +5801,7 @@
         </is>
       </c>
       <c r="G113" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/gestor-de-servicios-mesa-de-ayuda-sap-1886775732", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnicoa-tecnologoa-profesional-de-telecomunicaciones-redes-de-fibra-optica-1886768691", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H113" s="6" t="inlineStr"/>
@@ -5816,7 +5820,7 @@
     <row r="114" ht="22" customHeight="1">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>1c92f7ef9b7af696</t>
+          <t>4e5b3128aa7f8f9b</t>
         </is>
       </c>
       <c r="B114" s="2" t="inlineStr">
@@ -5826,7 +5830,7 @@
       </c>
       <c r="C114" s="3" t="inlineStr">
         <is>
-          <t>Agente de mesa de ayuda nivel 1</t>
+          <t>Gestor de servicios mesa de ayuda sap</t>
         </is>
       </c>
       <c r="D114" s="3" t="inlineStr">
@@ -5843,7 +5847,7 @@
         </is>
       </c>
       <c r="G114" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-de-mesa-de-ayuda-nivel-1-1886778506", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/gestor-de-servicios-mesa-de-ayuda-sap-1886775732", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H114" s="6" t="inlineStr"/>
@@ -5862,22 +5866,22 @@
     <row r="115" ht="22" customHeight="1">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>718ceee355d457ea</t>
+          <t>1c92f7ef9b7af696</t>
         </is>
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10 16:16</t>
+          <t>2026-10-09 17:28</t>
         </is>
       </c>
       <c r="C115" s="3" t="inlineStr">
         <is>
-          <t>IT Help Desk Support</t>
+          <t>Agente de mesa de ayuda nivel 1</t>
         </is>
       </c>
       <c r="D115" s="3" t="inlineStr">
         <is>
-          <t>Booth</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E115" s="7" t="n">
@@ -5889,7 +5893,7 @@
         </is>
       </c>
       <c r="G115" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/it-help-desk-support-at-booth-4471203962", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-de-mesa-de-ayuda-nivel-1-1886778506", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H115" s="6" t="inlineStr"/>
@@ -5908,22 +5912,22 @@
     <row r="116" ht="22" customHeight="1">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>925f43273b78f188</t>
+          <t>718ceee355d457ea</t>
         </is>
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12 20:17</t>
+          <t>2026-10-10 16:16</t>
         </is>
       </c>
       <c r="C116" s="3" t="inlineStr">
         <is>
-          <t>Mesa de ayuda ti - girón</t>
+          <t>IT Help Desk Support</t>
         </is>
       </c>
       <c r="D116" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Booth</t>
         </is>
       </c>
       <c r="E116" s="7" t="n">
@@ -5935,7 +5939,7 @@
         </is>
       </c>
       <c r="G116" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/mesa-de-ayuda-ti-giron-1886745168", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/it-help-desk-support-at-booth-4471203962", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H116" s="6" t="inlineStr"/>
@@ -5954,22 +5958,22 @@
     <row r="117" ht="22" customHeight="1">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>ec0c8875e04f4933</t>
+          <t>925f43273b78f188</t>
         </is>
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13 18:08</t>
+          <t>2026-10-12 20:17</t>
         </is>
       </c>
       <c r="C117" s="3" t="inlineStr">
         <is>
-          <t>Analista de mesa de ayuda.</t>
+          <t>Mesa de ayuda ti - girón</t>
         </is>
       </c>
       <c r="D117" s="3" t="inlineStr">
         <is>
-          <t>Softtek Colombia</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E117" s="7" t="n">
@@ -5981,7 +5985,7 @@
         </is>
       </c>
       <c r="G117" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-mesa-de-ayuda-1886754207", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/mesa-de-ayuda-ti-giron-1886745168", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H117" s="6" t="inlineStr"/>
@@ -6000,7 +6004,7 @@
     <row r="118" ht="22" customHeight="1">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>87fac63aa714f401</t>
+          <t>ec0c8875e04f4933</t>
         </is>
       </c>
       <c r="B118" s="2" t="inlineStr">
@@ -6010,7 +6014,7 @@
       </c>
       <c r="C118" s="3" t="inlineStr">
         <is>
-          <t>Agente mesa de ayuda.</t>
+          <t>Analista de mesa de ayuda.</t>
         </is>
       </c>
       <c r="D118" s="3" t="inlineStr">
@@ -6027,7 +6031,7 @@
         </is>
       </c>
       <c r="G118" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-mesa-de-ayuda-1886753535", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-mesa-de-ayuda-1886754207", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H118" s="6" t="inlineStr"/>
@@ -6046,22 +6050,22 @@
     <row r="119" ht="22" customHeight="1">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>dfa7dd88fd24afb4</t>
+          <t>87fac63aa714f401</t>
         </is>
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15 15:40</t>
+          <t>2026-10-13 18:08</t>
         </is>
       </c>
       <c r="C119" s="3" t="inlineStr">
         <is>
-          <t>Agente mesa de ayuda nivel 1 ingles avanzado</t>
+          <t>Agente mesa de ayuda.</t>
         </is>
       </c>
       <c r="D119" s="3" t="inlineStr">
         <is>
-          <t>SUSTS Colombia Ltda.</t>
+          <t>Softtek Colombia</t>
         </is>
       </c>
       <c r="E119" s="7" t="n">
@@ -6073,7 +6077,7 @@
         </is>
       </c>
       <c r="G119" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-mesa-de-ayuda-nivel-1-ingles-avanzado-1886780371", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-mesa-de-ayuda-1886753535", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H119" s="6" t="inlineStr"/>
@@ -6092,22 +6096,22 @@
     <row r="120" ht="22" customHeight="1">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>6ec1aeac55104810</t>
+          <t>dfa7dd88fd24afb4</t>
         </is>
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16 15:22</t>
+          <t>2026-10-15 15:40</t>
         </is>
       </c>
       <c r="C120" s="3" t="inlineStr">
         <is>
-          <t>Analista de Mesa de Ayuda</t>
+          <t>Agente mesa de ayuda nivel 1 ingles avanzado</t>
         </is>
       </c>
       <c r="D120" s="3" t="inlineStr">
         <is>
-          <t>INSEPET S.A.S</t>
+          <t>SUSTS Colombia Ltda.</t>
         </is>
       </c>
       <c r="E120" s="7" t="n">
@@ -6119,14 +6123,10 @@
         </is>
       </c>
       <c r="G120" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-analista-de-mesa-de-ayuda-en-bogota-dc-731E37A9EEFEA71561373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H120" s="6" t="inlineStr">
-        <is>
-          <t>$ 1.800.000,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-mesa-de-ayuda-nivel-1-ingles-avanzado-1886780371", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H120" s="6" t="inlineStr"/>
       <c r="I120" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -6142,7 +6142,7 @@
     <row r="121" ht="22" customHeight="1">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>c03a3cc06e28c7bb</t>
+          <t>6ec1aeac55104810</t>
         </is>
       </c>
       <c r="B121" s="2" t="inlineStr">
@@ -6152,12 +6152,12 @@
       </c>
       <c r="C121" s="3" t="inlineStr">
         <is>
-          <t>Agente de mesa de ayuda portugues</t>
+          <t>Analista de Mesa de Ayuda</t>
         </is>
       </c>
       <c r="D121" s="3" t="inlineStr">
         <is>
-          <t>COMWARE S.A.</t>
+          <t>INSEPET S.A.S</t>
         </is>
       </c>
       <c r="E121" s="7" t="n">
@@ -6169,10 +6169,14 @@
         </is>
       </c>
       <c r="G121" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-de-mesa-de-ayuda-portugues-1886781202", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H121" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-analista-de-mesa-de-ayuda-en-bogota-dc-731E37A9EEFEA71561373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H121" s="6" t="inlineStr">
+        <is>
+          <t>$ 1.800.000,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I121" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -6188,22 +6192,22 @@
     <row r="122" ht="22" customHeight="1">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>2ecdc22edf2ff172</t>
+          <t>c03a3cc06e28c7bb</t>
         </is>
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17 14:15</t>
+          <t>2026-10-16 15:22</t>
         </is>
       </c>
       <c r="C122" s="3" t="inlineStr">
         <is>
-          <t>Agente Mesa de ayuda Portugués</t>
+          <t>Agente de mesa de ayuda portugues</t>
         </is>
       </c>
       <c r="D122" s="3" t="inlineStr">
         <is>
-          <t>COMWARE S.A</t>
+          <t>COMWARE S.A.</t>
         </is>
       </c>
       <c r="E122" s="7" t="n">
@@ -6215,14 +6219,10 @@
         </is>
       </c>
       <c r="G122" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-agente-mesa-de-ayuda-portugues-en-bogota-dc-D31C231B9F8EFFCA61373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H122" s="6" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-de-mesa-de-ayuda-portugues-1886781202", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H122" s="6" t="inlineStr"/>
       <c r="I122" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -6238,26 +6238,26 @@
     <row r="123" ht="22" customHeight="1">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>50c79dfbfd49f52d</t>
+          <t>2ecdc22edf2ff172</t>
         </is>
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 16:39</t>
+          <t>2026-10-17 14:15</t>
         </is>
       </c>
       <c r="C123" s="3" t="inlineStr">
         <is>
-          <t>Analista de redes noc 1 telecomunicaciones.</t>
+          <t>Agente Mesa de ayuda Portugués</t>
         </is>
       </c>
       <c r="D123" s="3" t="inlineStr">
         <is>
-          <t>MANPOWER</t>
+          <t>COMWARE S.A</t>
         </is>
       </c>
       <c r="E123" s="7" t="n">
-        <v>0.53</v>
+        <v>0.58</v>
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
@@ -6265,13 +6265,17 @@
         </is>
       </c>
       <c r="G123" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-noc-1-telecomunicaciones-1886772075", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H123" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-agente-mesa-de-ayuda-portugues-en-bogota-dc-D31C231B9F8EFFCA61373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H123" s="6" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
       <c r="I123" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J123" s="2" t="inlineStr">
@@ -6284,26 +6288,26 @@
     <row r="124" ht="22" customHeight="1">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>0b0ae49f910109bb</t>
+          <t>50c79dfbfd49f52d</t>
         </is>
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 15:54</t>
+          <t>2026-10-02 16:39</t>
         </is>
       </c>
       <c r="C124" s="3" t="inlineStr">
         <is>
-          <t>Ejecutivo Técnico Arancel Junior</t>
+          <t>Analista de redes noc 1 telecomunicaciones.</t>
         </is>
       </c>
       <c r="D124" s="3" t="inlineStr">
         <is>
-          <t>Importante Empresa de Logística y Comercio</t>
+          <t>MANPOWER</t>
         </is>
       </c>
       <c r="E124" s="7" t="n">
-        <v>0.5</v>
+        <v>0.53</v>
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
@@ -6311,17 +6315,13 @@
         </is>
       </c>
       <c r="G124" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-547866639B487E0161373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H124" s="6" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-noc-1-telecomunicaciones-1886772075", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H124" s="6" t="inlineStr"/>
       <c r="I124" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J124" s="2" t="inlineStr">
@@ -6334,26 +6334,26 @@
     <row r="125" ht="22" customHeight="1">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>582a04b3c639bfa0</t>
+          <t>afe94b7770349744</t>
         </is>
       </c>
       <c r="B125" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 16:49</t>
+          <t>2026-10-20 15:43</t>
         </is>
       </c>
       <c r="C125" s="3" t="inlineStr">
         <is>
-          <t>Junior IT Support Specialist</t>
+          <t>Consultor de Seguridad de Redes – Akamai WAF con Inglés B2 o Superior.</t>
         </is>
       </c>
       <c r="D125" s="3" t="inlineStr">
         <is>
-          <t>Touch Support, Inc. &amp; SNF Back Office</t>
+          <t>Adecco Colombia S.A.</t>
         </is>
       </c>
       <c r="E125" s="7" t="n">
-        <v>0.5</v>
+        <v>0.53</v>
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
@@ -6361,13 +6361,17 @@
         </is>
       </c>
       <c r="G125" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/junior-it-support-specialist-at-touch-support-inc-snf-back-office-4472187578", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H125" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-consultor-de-seguridad-de-redes-akamai-waf-con-ingles-b2-o-superior-en-bogota-dc-50B87E7E33B988D461373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H125" s="6" t="inlineStr">
+        <is>
+          <t>$ 10.000.000,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I125" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J125" s="2" t="inlineStr">
@@ -6380,12 +6384,12 @@
     <row r="126" ht="22" customHeight="1">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>6e04c4d57d3fc3c7</t>
+          <t>0b0ae49f910109bb</t>
         </is>
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 17:26</t>
+          <t>2026-09-25 15:54</t>
         </is>
       </c>
       <c r="C126" s="3" t="inlineStr">
@@ -6407,25 +6411,171 @@
         </is>
       </c>
       <c r="G126" s="5">
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-547866639B487E0161373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H126" s="6" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="I126" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J126" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K126" s="3" t="inlineStr"/>
+    </row>
+    <row r="127" ht="22" customHeight="1">
+      <c r="A127" s="2" t="inlineStr">
+        <is>
+          <t>582a04b3c639bfa0</t>
+        </is>
+      </c>
+      <c r="B127" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 16:49</t>
+        </is>
+      </c>
+      <c r="C127" s="3" t="inlineStr">
+        <is>
+          <t>Junior IT Support Specialist</t>
+        </is>
+      </c>
+      <c r="D127" s="3" t="inlineStr">
+        <is>
+          <t>Touch Support, Inc. &amp; SNF Back Office</t>
+        </is>
+      </c>
+      <c r="E127" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F127" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G127" s="5">
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/junior-it-support-specialist-at-touch-support-inc-snf-back-office-4472187578", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H127" s="6" t="inlineStr"/>
+      <c r="I127" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J127" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K127" s="3" t="inlineStr"/>
+    </row>
+    <row r="128" ht="22" customHeight="1">
+      <c r="A128" s="2" t="inlineStr">
+        <is>
+          <t>6e04c4d57d3fc3c7</t>
+        </is>
+      </c>
+      <c r="B128" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01 17:26</t>
+        </is>
+      </c>
+      <c r="C128" s="3" t="inlineStr">
+        <is>
+          <t>Ejecutivo Técnico Arancel Junior</t>
+        </is>
+      </c>
+      <c r="D128" s="3" t="inlineStr">
+        <is>
+          <t>Importante Empresa de Logística y Comercio</t>
+        </is>
+      </c>
+      <c r="E128" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F128" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G128" s="5">
         <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-8444AB594560844161373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
-      <c r="H126" s="6" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
-      <c r="I126" s="3" t="inlineStr">
+      <c r="H128" s="6" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="I128" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
-      <c r="J126" s="2" t="inlineStr">
-        <is>
-          <t>Nueva</t>
-        </is>
-      </c>
-      <c r="K126" s="3" t="inlineStr"/>
+      <c r="J128" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K128" s="3" t="inlineStr"/>
+    </row>
+    <row r="129" ht="22" customHeight="1">
+      <c r="A129" s="2" t="inlineStr">
+        <is>
+          <t>8d81bacef79435aa</t>
+        </is>
+      </c>
+      <c r="B129" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 15:43</t>
+        </is>
+      </c>
+      <c r="C129" s="3" t="inlineStr">
+        <is>
+          <t>Buscamos Estudiantes en Áreas de Sistemas, Software para trabajar desde casa // sin Experiencia</t>
+        </is>
+      </c>
+      <c r="D129" s="3" t="inlineStr">
+        <is>
+          <t>emtelco</t>
+        </is>
+      </c>
+      <c r="E129" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F129" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G129" s="5">
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-buscamos-estudiantes-en-areas-de-sistemas-software-para-trabajar-desde-casa-sin-experiencia-participa-todas-las-areas-relacionadas-con-soporte-tecnico-en-medellin-D756C734FE234C3D61373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H129" s="6" t="inlineStr">
+        <is>
+          <t>$ 1.750.905,00 (Mensual)</t>
+        </is>
+      </c>
+      <c r="I129" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J129" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K129" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
chore(tracker): actualizacion diaria de vacantes 2026-10-21
</commit_message>
<xml_diff>
--- a/output/profile_5_tecnico_sistemas_tracker.xlsx
+++ b/output/profile_5_tecnico_sistemas_tracker.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K129"/>
+  <dimension ref="A1:K132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -6288,26 +6288,26 @@
     <row r="124" ht="22" customHeight="1">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>50c79dfbfd49f52d</t>
+          <t>3807f82cb9f9ccdb</t>
         </is>
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 16:39</t>
+          <t>2026-10-21 15:59</t>
         </is>
       </c>
       <c r="C124" s="3" t="inlineStr">
         <is>
-          <t>Analista de redes noc 1 telecomunicaciones.</t>
+          <t>Analista de Soporte TI Nivel I y II</t>
         </is>
       </c>
       <c r="D124" s="3" t="inlineStr">
         <is>
-          <t>MANPOWER</t>
+          <t>Autonomic SAS</t>
         </is>
       </c>
       <c r="E124" s="7" t="n">
-        <v>0.53</v>
+        <v>0.58</v>
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
@@ -6315,13 +6315,17 @@
         </is>
       </c>
       <c r="G124" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-noc-1-telecomunicaciones-1886772075", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H124" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-analista-de-soporte-ti-nivel-i-y-ii-en-medellin-452D284A14726B6861373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H124" s="6" t="inlineStr">
+        <is>
+          <t>$ 2.000.000,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I124" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J124" s="2" t="inlineStr">
@@ -6334,26 +6338,26 @@
     <row r="125" ht="22" customHeight="1">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>afe94b7770349744</t>
+          <t>a716d4100a0f8155</t>
         </is>
       </c>
       <c r="B125" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 15:43</t>
+          <t>2026-10-21 15:59</t>
         </is>
       </c>
       <c r="C125" s="3" t="inlineStr">
         <is>
-          <t>Consultor de Seguridad de Redes – Akamai WAF con Inglés B2 o Superior.</t>
+          <t>Técnico de infraestructura y redes de telecomunicaciones - casanare</t>
         </is>
       </c>
       <c r="D125" s="3" t="inlineStr">
         <is>
-          <t>Adecco Colombia S.A.</t>
+          <t>SDT INGENIERIA</t>
         </is>
       </c>
       <c r="E125" s="7" t="n">
-        <v>0.53</v>
+        <v>0.58</v>
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
@@ -6361,17 +6365,13 @@
         </is>
       </c>
       <c r="G125" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-consultor-de-seguridad-de-redes-akamai-waf-con-ingles-b2-o-superior-en-bogota-dc-50B87E7E33B988D461373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H125" s="6" t="inlineStr">
-        <is>
-          <t>$ 10.000.000,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-infraestructura-y-redes-de-telecomunicaciones-casanare-1886779754", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H125" s="6" t="inlineStr"/>
       <c r="I125" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J125" s="2" t="inlineStr">
@@ -6384,26 +6384,26 @@
     <row r="126" ht="22" customHeight="1">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>0b0ae49f910109bb</t>
+          <t>3802f406ec698d83</t>
         </is>
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 15:54</t>
+          <t>2026-10-21 15:59</t>
         </is>
       </c>
       <c r="C126" s="3" t="inlineStr">
         <is>
-          <t>Ejecutivo Técnico Arancel Junior</t>
+          <t>Técnico de telecomunicaciones e instalación de redes - bogotá | experiencia en obra civil</t>
         </is>
       </c>
       <c r="D126" s="3" t="inlineStr">
         <is>
-          <t>Importante Empresa de Logística y Comercio</t>
+          <t>ATIEMPO S.A.S</t>
         </is>
       </c>
       <c r="E126" s="7" t="n">
-        <v>0.5</v>
+        <v>0.58</v>
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
@@ -6411,17 +6411,13 @@
         </is>
       </c>
       <c r="G126" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-547866639B487E0161373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H126" s="6" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-telecomunicaciones-e-instalacion-de-redes-bogota-experiencia-en-obra-civil-1886760957", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H126" s="6" t="inlineStr"/>
       <c r="I126" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J126" s="2" t="inlineStr">
@@ -6434,26 +6430,26 @@
     <row r="127" ht="22" customHeight="1">
       <c r="A127" s="2" t="inlineStr">
         <is>
-          <t>582a04b3c639bfa0</t>
+          <t>50c79dfbfd49f52d</t>
         </is>
       </c>
       <c r="B127" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 16:49</t>
+          <t>2026-10-02 16:39</t>
         </is>
       </c>
       <c r="C127" s="3" t="inlineStr">
         <is>
-          <t>Junior IT Support Specialist</t>
+          <t>Analista de redes noc 1 telecomunicaciones.</t>
         </is>
       </c>
       <c r="D127" s="3" t="inlineStr">
         <is>
-          <t>Touch Support, Inc. &amp; SNF Back Office</t>
+          <t>MANPOWER</t>
         </is>
       </c>
       <c r="E127" s="7" t="n">
-        <v>0.5</v>
+        <v>0.53</v>
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
@@ -6461,13 +6457,13 @@
         </is>
       </c>
       <c r="G127" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/junior-it-support-specialist-at-touch-support-inc-snf-back-office-4472187578", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-noc-1-telecomunicaciones-1886772075", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H127" s="6" t="inlineStr"/>
       <c r="I127" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J127" s="2" t="inlineStr">
@@ -6480,26 +6476,26 @@
     <row r="128" ht="22" customHeight="1">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>6e04c4d57d3fc3c7</t>
+          <t>afe94b7770349744</t>
         </is>
       </c>
       <c r="B128" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 17:26</t>
+          <t>2026-10-20 15:43</t>
         </is>
       </c>
       <c r="C128" s="3" t="inlineStr">
         <is>
-          <t>Ejecutivo Técnico Arancel Junior</t>
+          <t>Consultor de Seguridad de Redes – Akamai WAF con Inglés B2 o Superior.</t>
         </is>
       </c>
       <c r="D128" s="3" t="inlineStr">
         <is>
-          <t>Importante Empresa de Logística y Comercio</t>
+          <t>Adecco Colombia S.A.</t>
         </is>
       </c>
       <c r="E128" s="7" t="n">
-        <v>0.5</v>
+        <v>0.53</v>
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
@@ -6507,17 +6503,17 @@
         </is>
       </c>
       <c r="G128" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-8444AB594560844161373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-consultor-de-seguridad-de-redes-akamai-waf-con-ingles-b2-o-superior-en-bogota-dc-50B87E7E33B988D461373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H128" s="6" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>$ 10.000.000,00 (Mensual)</t>
         </is>
       </c>
       <c r="I128" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J128" s="2" t="inlineStr">
@@ -6530,22 +6526,22 @@
     <row r="129" ht="22" customHeight="1">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>8d81bacef79435aa</t>
+          <t>0b0ae49f910109bb</t>
         </is>
       </c>
       <c r="B129" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 15:43</t>
+          <t>2026-09-25 15:54</t>
         </is>
       </c>
       <c r="C129" s="3" t="inlineStr">
         <is>
-          <t>Buscamos Estudiantes en Áreas de Sistemas, Software para trabajar desde casa // sin Experiencia</t>
+          <t>Ejecutivo Técnico Arancel Junior</t>
         </is>
       </c>
       <c r="D129" s="3" t="inlineStr">
         <is>
-          <t>emtelco</t>
+          <t>Importante Empresa de Logística y Comercio</t>
         </is>
       </c>
       <c r="E129" s="7" t="n">
@@ -6557,25 +6553,171 @@
         </is>
       </c>
       <c r="G129" s="5">
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-547866639B487E0161373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H129" s="6" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="I129" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J129" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K129" s="3" t="inlineStr"/>
+    </row>
+    <row r="130" ht="22" customHeight="1">
+      <c r="A130" s="2" t="inlineStr">
+        <is>
+          <t>582a04b3c639bfa0</t>
+        </is>
+      </c>
+      <c r="B130" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 16:49</t>
+        </is>
+      </c>
+      <c r="C130" s="3" t="inlineStr">
+        <is>
+          <t>Junior IT Support Specialist</t>
+        </is>
+      </c>
+      <c r="D130" s="3" t="inlineStr">
+        <is>
+          <t>Touch Support, Inc. &amp; SNF Back Office</t>
+        </is>
+      </c>
+      <c r="E130" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F130" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G130" s="5">
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/junior-it-support-specialist-at-touch-support-inc-snf-back-office-4472187578", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H130" s="6" t="inlineStr"/>
+      <c r="I130" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J130" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K130" s="3" t="inlineStr"/>
+    </row>
+    <row r="131" ht="22" customHeight="1">
+      <c r="A131" s="2" t="inlineStr">
+        <is>
+          <t>6e04c4d57d3fc3c7</t>
+        </is>
+      </c>
+      <c r="B131" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01 17:26</t>
+        </is>
+      </c>
+      <c r="C131" s="3" t="inlineStr">
+        <is>
+          <t>Ejecutivo Técnico Arancel Junior</t>
+        </is>
+      </c>
+      <c r="D131" s="3" t="inlineStr">
+        <is>
+          <t>Importante Empresa de Logística y Comercio</t>
+        </is>
+      </c>
+      <c r="E131" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F131" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G131" s="5">
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-8444AB594560844161373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H131" s="6" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="I131" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J131" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K131" s="3" t="inlineStr"/>
+    </row>
+    <row r="132" ht="22" customHeight="1">
+      <c r="A132" s="2" t="inlineStr">
+        <is>
+          <t>8d81bacef79435aa</t>
+        </is>
+      </c>
+      <c r="B132" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 15:43</t>
+        </is>
+      </c>
+      <c r="C132" s="3" t="inlineStr">
+        <is>
+          <t>Buscamos Estudiantes en Áreas de Sistemas, Software para trabajar desde casa // sin Experiencia</t>
+        </is>
+      </c>
+      <c r="D132" s="3" t="inlineStr">
+        <is>
+          <t>emtelco</t>
+        </is>
+      </c>
+      <c r="E132" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F132" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G132" s="5">
         <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-buscamos-estudiantes-en-areas-de-sistemas-software-para-trabajar-desde-casa-sin-experiencia-participa-todas-las-areas-relacionadas-con-soporte-tecnico-en-medellin-D756C734FE234C3D61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
-      <c r="H129" s="6" t="inlineStr">
+      <c r="H132" s="6" t="inlineStr">
         <is>
           <t>$ 1.750.905,00 (Mensual)</t>
         </is>
       </c>
-      <c r="I129" s="3" t="inlineStr">
+      <c r="I132" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
-      <c r="J129" s="2" t="inlineStr">
-        <is>
-          <t>Nueva</t>
-        </is>
-      </c>
-      <c r="K129" s="3" t="inlineStr"/>
+      <c r="J132" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K132" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
chore(tracker): actualizacion diaria de vacantes 2026-10-22
</commit_message>
<xml_diff>
--- a/output/profile_5_tecnico_sistemas_tracker.xlsx
+++ b/output/profile_5_tecnico_sistemas_tracker.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K132"/>
+  <dimension ref="A1:K136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3722,26 +3722,26 @@
     <row r="69" ht="22" customHeight="1">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>ae736277661dc78b</t>
+          <t>623999ab44df9605</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 15:23</t>
+          <t>2026-10-22 15:57</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>Analista de redes cisco</t>
+          <t>Agente de Service Desk Mesa de Ayuda – Soporte Técnico / Zona franca</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>ATCG DE COLOMBIA S.A.S</t>
-        </is>
-      </c>
-      <c r="E69" s="7" t="n">
-        <v>0.68</v>
+          <t>Redes Humanas</t>
+        </is>
+      </c>
+      <c r="E69" s="4" t="n">
+        <v>0.73</v>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
@@ -3749,13 +3749,17 @@
         </is>
       </c>
       <c r="G69" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-cisco-1886760389", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H69" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-agente-de-service-desk-mesa-de-ayuda-soporte-tecnico-zona-franca-en-bogota-dc-2136808CA681AC2D61373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H69" s="6" t="inlineStr">
+        <is>
+          <t>$ 1.750.905,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I69" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 68/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 73/100 - Alta Afinidad] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J69" s="2" t="inlineStr">
@@ -3768,26 +3772,26 @@
     <row r="70" ht="22" customHeight="1">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>e29676fac3409ad6</t>
+          <t>2ad6be817d734484</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 15:23</t>
+          <t>2026-10-22 15:57</t>
         </is>
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>Analista de redes y telecomunicaciones - nivel 1</t>
+          <t>Auxiliar soporte tecnico - pasto</t>
         </is>
       </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
-          <t>MANPOWER</t>
-        </is>
-      </c>
-      <c r="E70" s="7" t="n">
-        <v>0.68</v>
+          <t>ALFA TRADING S.A.S.</t>
+        </is>
+      </c>
+      <c r="E70" s="4" t="n">
+        <v>0.73</v>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
@@ -3795,13 +3799,13 @@
         </is>
       </c>
       <c r="G70" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-y-telecomunicaciones-nivel-1-1886760565", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-soporte-tecnico-pasto-1886783562", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H70" s="6" t="inlineStr"/>
       <c r="I70" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 68/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 73/100 - Alta Afinidad] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J70" s="2" t="inlineStr">
@@ -3814,26 +3818,26 @@
     <row r="71" ht="22" customHeight="1">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>baf000f38713dc11</t>
+          <t>ae736277661dc78b</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07 17:50</t>
+          <t>2026-09-24 15:23</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>Helpdesk / Analista soporte TI / trilingüe</t>
+          <t>Analista de redes cisco</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>Confidential</t>
+          <t>ATCG DE COLOMBIA S.A.S</t>
         </is>
       </c>
       <c r="E71" s="7" t="n">
-        <v>0.66</v>
+        <v>0.68</v>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
@@ -3841,13 +3845,13 @@
         </is>
       </c>
       <c r="G71" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/helpdesk-analista-soporte-ti-triling%C3%BCe-ingles-portugu%C3%A9s-at-confidential-4469673592", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-cisco-1886760389", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H71" s="6" t="inlineStr"/>
       <c r="I71" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 66/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 68/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J71" s="2" t="inlineStr">
@@ -3860,26 +3864,26 @@
     <row r="72" ht="22" customHeight="1">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>422a27df3967ecbb</t>
+          <t>e29676fac3409ad6</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14 15:52</t>
+          <t>2026-09-24 15:23</t>
         </is>
       </c>
       <c r="C72" s="3" t="inlineStr">
         <is>
-          <t>Técnico de sistemas y soporte ti</t>
+          <t>Analista de redes y telecomunicaciones - nivel 1</t>
         </is>
       </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
-          <t>AGENCIA DE EMPLEO CAFAM</t>
+          <t>MANPOWER</t>
         </is>
       </c>
       <c r="E72" s="7" t="n">
-        <v>0.66</v>
+        <v>0.68</v>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
@@ -3887,13 +3891,13 @@
         </is>
       </c>
       <c r="G72" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-sistemas-y-soporte-ti-1886780022", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-y-telecomunicaciones-nivel-1-1886760565", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H72" s="6" t="inlineStr"/>
       <c r="I72" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 66/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 68/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J72" s="2" t="inlineStr">
@@ -3906,26 +3910,26 @@
     <row r="73" ht="22" customHeight="1">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>73882c81e04abc7e</t>
+          <t>baf000f38713dc11</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 19:45</t>
+          <t>2026-10-07 17:50</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>Soporte L1 Junior</t>
+          <t>Helpdesk / Analista soporte TI / trilingüe</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>Hublance</t>
+          <t>Confidential</t>
         </is>
       </c>
       <c r="E73" s="7" t="n">
-        <v>0.6</v>
+        <v>0.66</v>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
@@ -3933,13 +3937,13 @@
         </is>
       </c>
       <c r="G73" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/soporte-l1-junior-at-hublance-4475841269", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/helpdesk-analista-soporte-ti-triling%C3%BCe-ingles-portugu%C3%A9s-at-confidential-4469673592", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H73" s="6" t="inlineStr"/>
       <c r="I73" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 60/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 66/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J73" s="2" t="inlineStr">
@@ -3952,26 +3956,26 @@
     <row r="74" ht="22" customHeight="1">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>8d7f304ffb8625b5</t>
+          <t>422a27df3967ecbb</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 15:54</t>
+          <t>2026-10-14 15:52</t>
         </is>
       </c>
       <c r="C74" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar de sistemas</t>
+          <t>Técnico de sistemas y soporte ti</t>
         </is>
       </c>
       <c r="D74" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>AGENCIA DE EMPLEO CAFAM</t>
         </is>
       </c>
       <c r="E74" s="7" t="n">
-        <v>0.58</v>
+        <v>0.66</v>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
@@ -3979,13 +3983,13 @@
         </is>
       </c>
       <c r="G74" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886751888", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-sistemas-y-soporte-ti-1886780022", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H74" s="6" t="inlineStr"/>
       <c r="I74" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 66/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J74" s="2" t="inlineStr">
@@ -3998,26 +4002,26 @@
     <row r="75" ht="22" customHeight="1">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>3b5b26f92a305c0c</t>
+          <t>73882c81e04abc7e</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 15:54</t>
+          <t>2026-10-05 19:45</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar de sistemas</t>
+          <t>Soporte L1 Junior</t>
         </is>
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Hublance</t>
         </is>
       </c>
       <c r="E75" s="7" t="n">
-        <v>0.58</v>
+        <v>0.6</v>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
@@ -4025,13 +4029,13 @@
         </is>
       </c>
       <c r="G75" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886749497", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/soporte-l1-junior-at-hublance-4475841269", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H75" s="6" t="inlineStr"/>
       <c r="I75" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 60/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J75" s="2" t="inlineStr">
@@ -4044,7 +4048,7 @@
     <row r="76" ht="22" customHeight="1">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>e760bcd88d90fbbe</t>
+          <t>8d7f304ffb8625b5</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
@@ -4054,12 +4058,12 @@
       </c>
       <c r="C76" s="3" t="inlineStr">
         <is>
-          <t>Agente de mesa de ayuda</t>
+          <t>Auxiliar de sistemas</t>
         </is>
       </c>
       <c r="D76" s="3" t="inlineStr">
         <is>
-          <t>SELCOMP INGENIERÍA SAS</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E76" s="7" t="n">
@@ -4071,7 +4075,7 @@
         </is>
       </c>
       <c r="G76" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-de-mesa-de-ayuda-1886758623", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886751888", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H76" s="6" t="inlineStr"/>
@@ -4090,7 +4094,7 @@
     <row r="77" ht="22" customHeight="1">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>86dcab5c5d802693</t>
+          <t>3b5b26f92a305c0c</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
@@ -4100,12 +4104,12 @@
       </c>
       <c r="C77" s="3" t="inlineStr">
         <is>
-          <t>Analista mesa de ayuda para tunja</t>
+          <t>Auxiliar de sistemas</t>
         </is>
       </c>
       <c r="D77" s="3" t="inlineStr">
         <is>
-          <t>Gestión de Seguridad Electrónica</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E77" s="7" t="n">
@@ -4117,7 +4121,7 @@
         </is>
       </c>
       <c r="G77" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-para-tunja-1886766955", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886749497", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H77" s="6" t="inlineStr"/>
@@ -4136,7 +4140,7 @@
     <row r="78" ht="22" customHeight="1">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>55fdaa0983ef9124</t>
+          <t>e760bcd88d90fbbe</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -4146,12 +4150,12 @@
       </c>
       <c r="C78" s="3" t="inlineStr">
         <is>
-          <t>Lider técnico con itil practice manager</t>
+          <t>Agente de mesa de ayuda</t>
         </is>
       </c>
       <c r="D78" s="3" t="inlineStr">
         <is>
-          <t>Sinergy &amp; Lowells</t>
+          <t>SELCOMP INGENIERÍA SAS</t>
         </is>
       </c>
       <c r="E78" s="7" t="n">
@@ -4163,7 +4167,7 @@
         </is>
       </c>
       <c r="G78" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/lider-tecnico-con-itil-practice-manager-1886753953", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-de-mesa-de-ayuda-1886758623", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H78" s="6" t="inlineStr"/>
@@ -4182,7 +4186,7 @@
     <row r="79" ht="22" customHeight="1">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>a1ca7bc58cd48fad</t>
+          <t>86dcab5c5d802693</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
@@ -4192,12 +4196,12 @@
       </c>
       <c r="C79" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de mesa de ayuda/mujeres contratacion inmediata</t>
+          <t>Analista mesa de ayuda para tunja</t>
         </is>
       </c>
       <c r="D79" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Gestión de Seguridad Electrónica</t>
         </is>
       </c>
       <c r="E79" s="7" t="n">
@@ -4209,7 +4213,7 @@
         </is>
       </c>
       <c r="G79" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-mesa-de-ayuda-mujeres-contratacion-inmediata-1886770931", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-para-tunja-1886766955", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H79" s="6" t="inlineStr"/>
@@ -4228,7 +4232,7 @@
     <row r="80" ht="22" customHeight="1">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>e28aba5df8a2d3ae</t>
+          <t>55fdaa0983ef9124</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
@@ -4238,12 +4242,12 @@
       </c>
       <c r="C80" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de mesa de ayuda/mujeres contratacion inmediata</t>
+          <t>Lider técnico con itil practice manager</t>
         </is>
       </c>
       <c r="D80" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Sinergy &amp; Lowells</t>
         </is>
       </c>
       <c r="E80" s="7" t="n">
@@ -4255,7 +4259,7 @@
         </is>
       </c>
       <c r="G80" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-mesa-de-ayuda-mujeres-contratacion-inmediata-1886769701", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/lider-tecnico-con-itil-practice-manager-1886753953", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H80" s="6" t="inlineStr"/>
@@ -4274,7 +4278,7 @@
     <row r="81" ht="22" customHeight="1">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>9326784c1a2726fb</t>
+          <t>a1ca7bc58cd48fad</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
@@ -4284,12 +4288,12 @@
       </c>
       <c r="C81" s="3" t="inlineStr">
         <is>
-          <t>Técnico de soporte y mesa de ayuda / medellín</t>
+          <t>Tecnico de mesa de ayuda/mujeres contratacion inmediata</t>
         </is>
       </c>
       <c r="D81" s="3" t="inlineStr">
         <is>
-          <t>Colsof S.A.S</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E81" s="7" t="n">
@@ -4301,7 +4305,7 @@
         </is>
       </c>
       <c r="G81" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-y-mesa-de-ayuda-medellin-1886738118", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-mesa-de-ayuda-mujeres-contratacion-inmediata-1886770931", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H81" s="6" t="inlineStr"/>
@@ -4320,7 +4324,7 @@
     <row r="82" ht="22" customHeight="1">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>b67dc9a9be4a1a6f</t>
+          <t>e28aba5df8a2d3ae</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
@@ -4330,7 +4334,7 @@
       </c>
       <c r="C82" s="3" t="inlineStr">
         <is>
-          <t>Service desk agent</t>
+          <t>Tecnico de mesa de ayuda/mujeres contratacion inmediata</t>
         </is>
       </c>
       <c r="D82" s="3" t="inlineStr">
@@ -4347,13 +4351,13 @@
         </is>
       </c>
       <c r="G82" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/service-desk-agent-soporte-tecnico-nivel-1-1886755112", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-mesa-de-ayuda-mujeres-contratacion-inmediata-1886769701", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H82" s="6" t="inlineStr"/>
       <c r="I82" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J82" s="2" t="inlineStr">
@@ -4366,7 +4370,7 @@
     <row r="83" ht="22" customHeight="1">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>9c65f710f43158b7</t>
+          <t>9326784c1a2726fb</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
@@ -4376,12 +4380,12 @@
       </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de instalaciones cableado de redes - licencia conte</t>
+          <t>Técnico de soporte y mesa de ayuda / medellín</t>
         </is>
       </c>
       <c r="D83" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Colsof S.A.S</t>
         </is>
       </c>
       <c r="E83" s="7" t="n">
@@ -4393,7 +4397,7 @@
         </is>
       </c>
       <c r="G83" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-1886749397", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-y-mesa-de-ayuda-medellin-1886738118", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H83" s="6" t="inlineStr"/>
@@ -4412,22 +4416,22 @@
     <row r="84" ht="22" customHeight="1">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>a95003a0b1fc3d77</t>
+          <t>b67dc9a9be4a1a6f</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 15:41</t>
+          <t>2026-09-25 15:54</t>
         </is>
       </c>
       <c r="C84" s="3" t="inlineStr">
         <is>
-          <t>Técnico Soporte Nivel 1 Con ITIL</t>
+          <t>Service desk agent</t>
         </is>
       </c>
       <c r="D84" s="3" t="inlineStr">
         <is>
-          <t>Importante empresa del sector de tecnología</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E84" s="7" t="n">
@@ -4439,17 +4443,13 @@
         </is>
       </c>
       <c r="G84" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-soporte-nivel-1-con-itil-en-bogota-dc-59E13FA64EF5843C61373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H84" s="6" t="inlineStr">
-        <is>
-          <t>$ 1.750.905,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/service-desk-agent-soporte-tecnico-nivel-1-1886755112", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H84" s="6" t="inlineStr"/>
       <c r="I84" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J84" s="2" t="inlineStr">
@@ -4462,22 +4462,22 @@
     <row r="85" ht="22" customHeight="1">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>96391fd564d83616</t>
+          <t>9c65f710f43158b7</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 15:41</t>
+          <t>2026-09-25 15:54</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de soporte IT con Moto</t>
+          <t>Tecnico de instalaciones cableado de redes - licencia conte</t>
         </is>
       </c>
       <c r="D85" s="3" t="inlineStr">
         <is>
-          <t>Los Hornitos</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E85" s="7" t="n">
@@ -4489,14 +4489,10 @@
         </is>
       </c>
       <c r="G85" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-it-con-moto-empresa-de-alimentos-en-bogota-dc-599938D46A6F4A8F61373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H85" s="6" t="inlineStr">
-        <is>
-          <t>$ 2.125.947,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-1886749397", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H85" s="6" t="inlineStr"/>
       <c r="I85" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -4512,7 +4508,7 @@
     <row r="86" ht="22" customHeight="1">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>b4f0b8c16fe5543e</t>
+          <t>a95003a0b1fc3d77</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
@@ -4522,12 +4518,12 @@
       </c>
       <c r="C86" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar de Sistemas</t>
+          <t>Técnico Soporte Nivel 1 Con ITIL</t>
         </is>
       </c>
       <c r="D86" s="3" t="inlineStr">
         <is>
-          <t>ELIS COLOMBIA SAS</t>
+          <t>Importante empresa del sector de tecnología</t>
         </is>
       </c>
       <c r="E86" s="7" t="n">
@@ -4539,12 +4535,12 @@
         </is>
       </c>
       <c r="G86" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-en-bogota-dc-48C2A0A3B050945661373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-soporte-nivel-1-con-itil-en-bogota-dc-59E13FA64EF5843C61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H86" s="6" t="inlineStr">
         <is>
-          <t>$ 2.000.000,00 (Mensual)</t>
+          <t>$ 1.750.905,00 (Mensual)</t>
         </is>
       </c>
       <c r="I86" s="3" t="inlineStr">
@@ -4562,7 +4558,7 @@
     <row r="87" ht="22" customHeight="1">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>7e4b4e4f136a5e31</t>
+          <t>96391fd564d83616</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
@@ -4572,12 +4568,12 @@
       </c>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>Agente Mesa de Ayuda</t>
+          <t>Tecnico de soporte IT con Moto</t>
         </is>
       </c>
       <c r="D87" s="3" t="inlineStr">
         <is>
-          <t>Importante empresa del sector</t>
+          <t>Los Hornitos</t>
         </is>
       </c>
       <c r="E87" s="7" t="n">
@@ -4589,12 +4585,12 @@
         </is>
       </c>
       <c r="G87" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-agente-mesa-de-ayuda-en-bogota-dc-E39FE355E02E578761373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-it-con-moto-empresa-de-alimentos-en-bogota-dc-599938D46A6F4A8F61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H87" s="6" t="inlineStr">
         <is>
-          <t>$ 2.000.000,00 (Mensual)</t>
+          <t>$ 2.125.947,00 (Mensual)</t>
         </is>
       </c>
       <c r="I87" s="3" t="inlineStr">
@@ -4612,7 +4608,7 @@
     <row r="88" ht="22" customHeight="1">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>0ef2cd7667600919</t>
+          <t>b4f0b8c16fe5543e</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
@@ -4622,12 +4618,12 @@
       </c>
       <c r="C88" s="3" t="inlineStr">
         <is>
-          <t>Técnico de Soporte TI Regional</t>
+          <t>Auxiliar de Sistemas</t>
         </is>
       </c>
       <c r="D88" s="3" t="inlineStr">
         <is>
-          <t>POLICOMP COLOMBIA SAS</t>
+          <t>ELIS COLOMBIA SAS</t>
         </is>
       </c>
       <c r="E88" s="7" t="n">
@@ -4639,10 +4635,14 @@
         </is>
       </c>
       <c r="G88" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-ti-regional-en-bogota-dc-ACF045C94E41CCDE61373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H88" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-en-bogota-dc-48C2A0A3B050945661373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H88" s="6" t="inlineStr">
+        <is>
+          <t>$ 2.000.000,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I88" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -4658,7 +4658,7 @@
     <row r="89" ht="22" customHeight="1">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>7784997bda962255</t>
+          <t>7e4b4e4f136a5e31</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
@@ -4668,12 +4668,12 @@
       </c>
       <c r="C89" s="3" t="inlineStr">
         <is>
-          <t>Técnico de Soporte TI On Demand/ por horas</t>
+          <t>Agente Mesa de Ayuda</t>
         </is>
       </c>
       <c r="D89" s="3" t="inlineStr">
         <is>
-          <t>POLICOMP COLOMBIA SAS</t>
+          <t>Importante empresa del sector</t>
         </is>
       </c>
       <c r="E89" s="7" t="n">
@@ -4685,10 +4685,14 @@
         </is>
       </c>
       <c r="G89" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-ti-on-demand-por-horas-en-bogota-dc-C2338FA0172D59A561373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H89" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-agente-mesa-de-ayuda-en-bogota-dc-E39FE355E02E578761373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H89" s="6" t="inlineStr">
+        <is>
+          <t>$ 2.000.000,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I89" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -4704,7 +4708,7 @@
     <row r="90" ht="22" customHeight="1">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>29d0fe2e42e678f7</t>
+          <t>0ef2cd7667600919</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
@@ -4714,12 +4718,12 @@
       </c>
       <c r="C90" s="3" t="inlineStr">
         <is>
-          <t>Técnico mantenimiento correctivo impresoras</t>
+          <t>Técnico de Soporte TI Regional</t>
         </is>
       </c>
       <c r="D90" s="3" t="inlineStr">
         <is>
-          <t>Multinacional de Impresión</t>
+          <t>POLICOMP COLOMBIA SAS</t>
         </is>
       </c>
       <c r="E90" s="7" t="n">
@@ -4731,14 +4735,10 @@
         </is>
       </c>
       <c r="G90" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-mantenimiento-correctivo-impresoras-en-guarne-BC0E775C0F25B27D61373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H90" s="6" t="inlineStr">
-        <is>
-          <t>$ 1.800.000,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-ti-regional-en-bogota-dc-ACF045C94E41CCDE61373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H90" s="6" t="inlineStr"/>
       <c r="I90" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -4754,22 +4754,22 @@
     <row r="91" ht="22" customHeight="1">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>98c9ab11f5b1eace</t>
+          <t>7784997bda962255</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 18:36</t>
+          <t>2026-09-27 15:41</t>
         </is>
       </c>
       <c r="C91" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar de sistemas</t>
+          <t>Técnico de Soporte TI On Demand/ por horas</t>
         </is>
       </c>
       <c r="D91" s="3" t="inlineStr">
         <is>
-          <t>Importante empresa del sector</t>
+          <t>POLICOMP COLOMBIA SAS</t>
         </is>
       </c>
       <c r="E91" s="7" t="n">
@@ -4781,14 +4781,10 @@
         </is>
       </c>
       <c r="G91" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-persona-con-discapacidad-remota-en-bogota-dc-5F2A812D014E159B61373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H91" s="6" t="inlineStr">
-        <is>
-          <t>$ 1.750.905,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-ti-on-demand-por-horas-en-bogota-dc-C2338FA0172D59A561373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H91" s="6" t="inlineStr"/>
       <c r="I91" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -4804,22 +4800,22 @@
     <row r="92" ht="22" customHeight="1">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>58133ddc4da9c68e</t>
+          <t>29d0fe2e42e678f7</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 18:36</t>
+          <t>2026-09-27 15:41</t>
         </is>
       </c>
       <c r="C92" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar de sistemas</t>
+          <t>Técnico mantenimiento correctivo impresoras</t>
         </is>
       </c>
       <c r="D92" s="3" t="inlineStr">
         <is>
-          <t>Importante empresa del sector</t>
+          <t>Multinacional de Impresión</t>
         </is>
       </c>
       <c r="E92" s="7" t="n">
@@ -4831,12 +4827,12 @@
         </is>
       </c>
       <c r="G92" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-persona-con-discapacidad-remota-en-bogota-dc-A00C07C9CC9A494B61373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-mantenimiento-correctivo-impresoras-en-guarne-BC0E775C0F25B27D61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H92" s="6" t="inlineStr">
         <is>
-          <t>$ 1.750.905,00 (Mensual)</t>
+          <t>$ 1.800.000,00 (Mensual)</t>
         </is>
       </c>
       <c r="I92" s="3" t="inlineStr">
@@ -4854,7 +4850,7 @@
     <row r="93" ht="22" customHeight="1">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>aed3420a4cfdc248</t>
+          <t>98c9ab11f5b1eace</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
@@ -4864,12 +4860,12 @@
       </c>
       <c r="C93" s="3" t="inlineStr">
         <is>
-          <t>Consultor de servicios/ mesa de ayuda nómina y erp software</t>
+          <t>Auxiliar de sistemas</t>
         </is>
       </c>
       <c r="D93" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Importante empresa del sector</t>
         </is>
       </c>
       <c r="E93" s="7" t="n">
@@ -4881,10 +4877,14 @@
         </is>
       </c>
       <c r="G93" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/consultor-de-servicios-mesa-de-ayuda-nomina-y-erp-software-inclusivo-1886716126", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H93" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-persona-con-discapacidad-remota-en-bogota-dc-5F2A812D014E159B61373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H93" s="6" t="inlineStr">
+        <is>
+          <t>$ 1.750.905,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I93" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -4900,12 +4900,12 @@
     <row r="94" ht="22" customHeight="1">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>2b8357189ff315da</t>
+          <t>58133ddc4da9c68e</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 17:00</t>
+          <t>2026-09-28 18:36</t>
         </is>
       </c>
       <c r="C94" s="3" t="inlineStr">
@@ -4915,7 +4915,7 @@
       </c>
       <c r="D94" s="3" t="inlineStr">
         <is>
-          <t>DAVITA SAS</t>
+          <t>Importante empresa del sector</t>
         </is>
       </c>
       <c r="E94" s="7" t="n">
@@ -4927,10 +4927,14 @@
         </is>
       </c>
       <c r="G94" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886758163", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H94" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-persona-con-discapacidad-remota-en-bogota-dc-A00C07C9CC9A494B61373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H94" s="6" t="inlineStr">
+        <is>
+          <t>$ 1.750.905,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I94" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -4946,17 +4950,17 @@
     <row r="95" ht="22" customHeight="1">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>a87934e7643b2c1c</t>
+          <t>aed3420a4cfdc248</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 17:00</t>
+          <t>2026-09-28 18:36</t>
         </is>
       </c>
       <c r="C95" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de instalaciones cableado de redes - licencia conte cali</t>
+          <t>Consultor de servicios/ mesa de ayuda nómina y erp software</t>
         </is>
       </c>
       <c r="D95" s="3" t="inlineStr">
@@ -4973,7 +4977,7 @@
         </is>
       </c>
       <c r="G95" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-cali-1886759847", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/consultor-de-servicios-mesa-de-ayuda-nomina-y-erp-software-inclusivo-1886716126", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H95" s="6" t="inlineStr"/>
@@ -4992,7 +4996,7 @@
     <row r="96" ht="22" customHeight="1">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>10b4265e3ad11d81</t>
+          <t>2b8357189ff315da</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
@@ -5002,12 +5006,12 @@
       </c>
       <c r="C96" s="3" t="inlineStr">
         <is>
-          <t>Information Technology Help Desk Support</t>
+          <t>Auxiliar de sistemas</t>
         </is>
       </c>
       <c r="D96" s="3" t="inlineStr">
         <is>
-          <t>Booth</t>
+          <t>DAVITA SAS</t>
         </is>
       </c>
       <c r="E96" s="7" t="n">
@@ -5019,7 +5023,7 @@
         </is>
       </c>
       <c r="G96" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/information-technology-help-desk-support-at-booth-4471203962", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886758163", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H96" s="6" t="inlineStr"/>
@@ -5038,17 +5042,17 @@
     <row r="97" ht="22" customHeight="1">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>ff69ae85c8697a37</t>
+          <t>a87934e7643b2c1c</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 16:49</t>
+          <t>2026-09-29 17:00</t>
         </is>
       </c>
       <c r="C97" s="3" t="inlineStr">
         <is>
-          <t>Técnico de soporte ti - bogota</t>
+          <t>Tecnico de instalaciones cableado de redes - licencia conte cali</t>
         </is>
       </c>
       <c r="D97" s="3" t="inlineStr">
@@ -5065,7 +5069,7 @@
         </is>
       </c>
       <c r="G97" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-ti-bogota-1886774059", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-cali-1886759847", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H97" s="6" t="inlineStr"/>
@@ -5084,22 +5088,22 @@
     <row r="98" ht="22" customHeight="1">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>bbacf7d69ab9084e</t>
+          <t>10b4265e3ad11d81</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 16:49</t>
+          <t>2026-09-29 17:00</t>
         </is>
       </c>
       <c r="C98" s="3" t="inlineStr">
         <is>
-          <t>IT Helpdesk Analyst</t>
+          <t>Information Technology Help Desk Support</t>
         </is>
       </c>
       <c r="D98" s="3" t="inlineStr">
         <is>
-          <t>Power Digital Marketing</t>
+          <t>Booth</t>
         </is>
       </c>
       <c r="E98" s="7" t="n">
@@ -5111,7 +5115,7 @@
         </is>
       </c>
       <c r="G98" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/it-helpdesk-analyst-at-power-digital-marketing-4472601999", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/information-technology-help-desk-support-at-booth-4471203962", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H98" s="6" t="inlineStr"/>
@@ -5130,12 +5134,12 @@
     <row r="99" ht="22" customHeight="1">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>bb848f474ff4b611</t>
+          <t>ff69ae85c8697a37</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 17:26</t>
+          <t>2026-09-30 16:49</t>
         </is>
       </c>
       <c r="C99" s="3" t="inlineStr">
@@ -5157,7 +5161,7 @@
         </is>
       </c>
       <c r="G99" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-ti-bogota-1886772292", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-ti-bogota-1886774059", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H99" s="6" t="inlineStr"/>
@@ -5176,22 +5180,22 @@
     <row r="100" ht="22" customHeight="1">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>b44a1c6cfb004ca8</t>
+          <t>bbacf7d69ab9084e</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 17:26</t>
+          <t>2026-09-30 16:49</t>
         </is>
       </c>
       <c r="C100" s="3" t="inlineStr">
         <is>
-          <t>Soporte ti nivel 2 - bogotá</t>
+          <t>IT Helpdesk Analyst</t>
         </is>
       </c>
       <c r="D100" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Power Digital Marketing</t>
         </is>
       </c>
       <c r="E100" s="7" t="n">
@@ -5203,7 +5207,7 @@
         </is>
       </c>
       <c r="G100" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/soporte-ti-nivel-2-bogota-1886774821", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/it-helpdesk-analyst-at-power-digital-marketing-4472601999", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H100" s="6" t="inlineStr"/>
@@ -5222,7 +5226,7 @@
     <row r="101" ht="22" customHeight="1">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>fb0ad2b513afb97c</t>
+          <t>bb848f474ff4b611</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr">
@@ -5232,12 +5236,12 @@
       </c>
       <c r="C101" s="3" t="inlineStr">
         <is>
-          <t>IT Help Desk Support Specialist</t>
+          <t>Técnico de soporte ti - bogota</t>
         </is>
       </c>
       <c r="D101" s="3" t="inlineStr">
         <is>
-          <t>Talento</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E101" s="7" t="n">
@@ -5249,7 +5253,7 @@
         </is>
       </c>
       <c r="G101" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/it-help-desk-support-specialist-tier-1-at-talento-4473960480", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-ti-bogota-1886772292", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H101" s="6" t="inlineStr"/>
@@ -5268,22 +5272,22 @@
     <row r="102" ht="22" customHeight="1">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>0b2067d6ae488f4c</t>
+          <t>b44a1c6cfb004ca8</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 16:39</t>
+          <t>2026-10-01 17:26</t>
         </is>
       </c>
       <c r="C102" s="3" t="inlineStr">
         <is>
-          <t>Help Desk Technician level 1</t>
+          <t>Soporte ti nivel 2 - bogotá</t>
         </is>
       </c>
       <c r="D102" s="3" t="inlineStr">
         <is>
-          <t>Solvo Global</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E102" s="7" t="n">
@@ -5295,7 +5299,7 @@
         </is>
       </c>
       <c r="G102" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/help-desk-technician-level-1-at-solvo-global-4472590892", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/soporte-ti-nivel-2-bogota-1886774821", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H102" s="6" t="inlineStr"/>
@@ -5314,22 +5318,22 @@
     <row r="103" ht="22" customHeight="1">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>07acc222a3ca2ef1</t>
+          <t>fb0ad2b513afb97c</t>
         </is>
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03 15:12</t>
+          <t>2026-10-01 17:26</t>
         </is>
       </c>
       <c r="C103" s="3" t="inlineStr">
         <is>
-          <t>Analista mesa de ayuda funza temporal 6 meses</t>
+          <t>IT Help Desk Support Specialist</t>
         </is>
       </c>
       <c r="D103" s="3" t="inlineStr">
         <is>
-          <t>Axity</t>
+          <t>Talento</t>
         </is>
       </c>
       <c r="E103" s="7" t="n">
@@ -5341,7 +5345,7 @@
         </is>
       </c>
       <c r="G103" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-funza-temporal-6-meses-1886774524", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/it-help-desk-support-specialist-tier-1-at-talento-4473960480", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H103" s="6" t="inlineStr"/>
@@ -5360,22 +5364,22 @@
     <row r="104" ht="22" customHeight="1">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>5ec0ea33876ba2b5</t>
+          <t>0b2067d6ae488f4c</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 19:45</t>
+          <t>2026-10-02 16:39</t>
         </is>
       </c>
       <c r="C104" s="3" t="inlineStr">
         <is>
-          <t>Help desk analyst l1</t>
+          <t>Help Desk Technician level 1</t>
         </is>
       </c>
       <c r="D104" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Solvo Global</t>
         </is>
       </c>
       <c r="E104" s="7" t="n">
@@ -5387,7 +5391,7 @@
         </is>
       </c>
       <c r="G104" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/help-desk-analyst-l1-medellin-1886776156", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/help-desk-technician-level-1-at-solvo-global-4472590892", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H104" s="6" t="inlineStr"/>
@@ -5406,22 +5410,22 @@
     <row r="105" ht="22" customHeight="1">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>e8bdf2094d1c9817</t>
+          <t>07acc222a3ca2ef1</t>
         </is>
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 19:45</t>
+          <t>2026-10-03 15:12</t>
         </is>
       </c>
       <c r="C105" s="3" t="inlineStr">
         <is>
-          <t>Administrador de herramienta de gestión de mesa de ayuda-</t>
+          <t>Analista mesa de ayuda funza temporal 6 meses</t>
         </is>
       </c>
       <c r="D105" s="3" t="inlineStr">
         <is>
-          <t>SELCOMP INGENIERÍA SAS</t>
+          <t>Axity</t>
         </is>
       </c>
       <c r="E105" s="7" t="n">
@@ -5433,7 +5437,7 @@
         </is>
       </c>
       <c r="G105" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/administrador-de-herramienta-de-gestion-de-mesa-de-ayuda-1886776286", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-funza-temporal-6-meses-1886774524", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H105" s="6" t="inlineStr"/>
@@ -5452,7 +5456,7 @@
     <row r="106" ht="22" customHeight="1">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>6e9a077b42879470</t>
+          <t>5ec0ea33876ba2b5</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
@@ -5462,12 +5466,12 @@
       </c>
       <c r="C106" s="3" t="inlineStr">
         <is>
-          <t>Analista de soporte de aplicaciones nivel 3</t>
+          <t>Help desk analyst l1</t>
         </is>
       </c>
       <c r="D106" s="3" t="inlineStr">
         <is>
-          <t>TALYCAP GLOBAL SAS</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E106" s="7" t="n">
@@ -5479,7 +5483,7 @@
         </is>
       </c>
       <c r="G106" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-soporte-de-aplicaciones-nivel-3-1886776104", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/help-desk-analyst-l1-medellin-1886776156", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H106" s="6" t="inlineStr"/>
@@ -5498,22 +5502,22 @@
     <row r="107" ht="22" customHeight="1">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>447afec244b20f9b</t>
+          <t>e8bdf2094d1c9817</t>
         </is>
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06 17:12</t>
+          <t>2026-10-05 19:45</t>
         </is>
       </c>
       <c r="C107" s="3" t="inlineStr">
         <is>
-          <t>Técnico de soporte ti - bogota</t>
+          <t>Administrador de herramienta de gestión de mesa de ayuda-</t>
         </is>
       </c>
       <c r="D107" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>SELCOMP INGENIERÍA SAS</t>
         </is>
       </c>
       <c r="E107" s="7" t="n">
@@ -5525,7 +5529,7 @@
         </is>
       </c>
       <c r="G107" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-ti-bogota-1886775990", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/administrador-de-herramienta-de-gestion-de-mesa-de-ayuda-1886776286", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H107" s="6" t="inlineStr"/>
@@ -5544,22 +5548,22 @@
     <row r="108" ht="22" customHeight="1">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>8f14c41f3b443ac0</t>
+          <t>6e9a077b42879470</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07 17:50</t>
+          <t>2026-10-05 19:45</t>
         </is>
       </c>
       <c r="C108" s="3" t="inlineStr">
         <is>
-          <t>Soporte mesa de ayuda</t>
+          <t>Analista de soporte de aplicaciones nivel 3</t>
         </is>
       </c>
       <c r="D108" s="3" t="inlineStr">
         <is>
-          <t>MANPOWER</t>
+          <t>TALYCAP GLOBAL SAS</t>
         </is>
       </c>
       <c r="E108" s="7" t="n">
@@ -5571,7 +5575,7 @@
         </is>
       </c>
       <c r="G108" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/soporte-mesa-de-ayuda-vacaciones-1886776917", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-soporte-de-aplicaciones-nivel-3-1886776104", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H108" s="6" t="inlineStr"/>
@@ -5590,22 +5594,22 @@
     <row r="109" ht="22" customHeight="1">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>b1a9e03967fff91e</t>
+          <t>447afec244b20f9b</t>
         </is>
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07 17:50</t>
+          <t>2026-10-06 17:12</t>
         </is>
       </c>
       <c r="C109" s="3" t="inlineStr">
         <is>
-          <t>Tecnólogo de soporte pl - mesa de ayuda</t>
+          <t>Técnico de soporte ti - bogota</t>
         </is>
       </c>
       <c r="D109" s="3" t="inlineStr">
         <is>
-          <t>Positivo S+</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E109" s="7" t="n">
@@ -5617,7 +5621,7 @@
         </is>
       </c>
       <c r="G109" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnologo-de-soporte-pl-mesa-de-ayuda-1886775546", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-ti-bogota-1886775990", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H109" s="6" t="inlineStr"/>
@@ -5636,7 +5640,7 @@
     <row r="110" ht="22" customHeight="1">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>eb49981c97933d93</t>
+          <t>8f14c41f3b443ac0</t>
         </is>
       </c>
       <c r="B110" s="2" t="inlineStr">
@@ -5646,12 +5650,12 @@
       </c>
       <c r="C110" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de instalaciones cableado de redes - licencia conte</t>
+          <t>Soporte mesa de ayuda</t>
         </is>
       </c>
       <c r="D110" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>MANPOWER</t>
         </is>
       </c>
       <c r="E110" s="7" t="n">
@@ -5663,7 +5667,7 @@
         </is>
       </c>
       <c r="G110" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-1886777333", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/soporte-mesa-de-ayuda-vacaciones-1886776917", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H110" s="6" t="inlineStr"/>
@@ -5682,7 +5686,7 @@
     <row r="111" ht="22" customHeight="1">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>d39af22b6e937d28</t>
+          <t>b1a9e03967fff91e</t>
         </is>
       </c>
       <c r="B111" s="2" t="inlineStr">
@@ -5692,12 +5696,12 @@
       </c>
       <c r="C111" s="3" t="inlineStr">
         <is>
-          <t>Analista Mesa de Ayuda Funza</t>
+          <t>Tecnólogo de soporte pl - mesa de ayuda</t>
         </is>
       </c>
       <c r="D111" s="3" t="inlineStr">
         <is>
-          <t>axity</t>
+          <t>Positivo S+</t>
         </is>
       </c>
       <c r="E111" s="7" t="n">
@@ -5709,7 +5713,7 @@
         </is>
       </c>
       <c r="G111" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/analista-mesa-de-ayuda-funza-at-axity-4471985006", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnologo-de-soporte-pl-mesa-de-ayuda-1886775546", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H111" s="6" t="inlineStr"/>
@@ -5728,22 +5732,22 @@
     <row r="112" ht="22" customHeight="1">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>0904912d51c5cd61</t>
+          <t>eb49981c97933d93</t>
         </is>
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08 17:52</t>
+          <t>2026-10-07 17:50</t>
         </is>
       </c>
       <c r="C112" s="3" t="inlineStr">
         <is>
-          <t>Analista mesa de ayuda</t>
+          <t>Tecnico de instalaciones cableado de redes - licencia conte</t>
         </is>
       </c>
       <c r="D112" s="3" t="inlineStr">
         <is>
-          <t>Desarrollo de Sistemas y Servicios SAS</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E112" s="7" t="n">
@@ -5755,7 +5759,7 @@
         </is>
       </c>
       <c r="G112" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-1886778032", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-1886777333", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H112" s="6" t="inlineStr"/>
@@ -5774,22 +5778,22 @@
     <row r="113" ht="22" customHeight="1">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>c665ada630270dce</t>
+          <t>d39af22b6e937d28</t>
         </is>
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09 17:28</t>
+          <t>2026-10-07 17:50</t>
         </is>
       </c>
       <c r="C113" s="3" t="inlineStr">
         <is>
-          <t>Técnico(a) / tecnólogo(a) / profesional de telecomunicaciones - redes de fibra óptica</t>
+          <t>Analista Mesa de Ayuda Funza</t>
         </is>
       </c>
       <c r="D113" s="3" t="inlineStr">
         <is>
-          <t>JAHV MC GREGOR S.A.S</t>
+          <t>axity</t>
         </is>
       </c>
       <c r="E113" s="7" t="n">
@@ -5801,7 +5805,7 @@
         </is>
       </c>
       <c r="G113" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnicoa-tecnologoa-profesional-de-telecomunicaciones-redes-de-fibra-optica-1886768691", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/analista-mesa-de-ayuda-funza-at-axity-4471985006", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H113" s="6" t="inlineStr"/>
@@ -5820,22 +5824,22 @@
     <row r="114" ht="22" customHeight="1">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>4e5b3128aa7f8f9b</t>
+          <t>0904912d51c5cd61</t>
         </is>
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09 17:28</t>
+          <t>2026-10-08 17:52</t>
         </is>
       </c>
       <c r="C114" s="3" t="inlineStr">
         <is>
-          <t>Gestor de servicios mesa de ayuda sap</t>
+          <t>Analista mesa de ayuda</t>
         </is>
       </c>
       <c r="D114" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Desarrollo de Sistemas y Servicios SAS</t>
         </is>
       </c>
       <c r="E114" s="7" t="n">
@@ -5847,7 +5851,7 @@
         </is>
       </c>
       <c r="G114" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/gestor-de-servicios-mesa-de-ayuda-sap-1886775732", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-1886778032", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H114" s="6" t="inlineStr"/>
@@ -5866,7 +5870,7 @@
     <row r="115" ht="22" customHeight="1">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>1c92f7ef9b7af696</t>
+          <t>c665ada630270dce</t>
         </is>
       </c>
       <c r="B115" s="2" t="inlineStr">
@@ -5876,12 +5880,12 @@
       </c>
       <c r="C115" s="3" t="inlineStr">
         <is>
-          <t>Agente de mesa de ayuda nivel 1</t>
+          <t>Técnico(a) / tecnólogo(a) / profesional de telecomunicaciones - redes de fibra óptica</t>
         </is>
       </c>
       <c r="D115" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>JAHV MC GREGOR S.A.S</t>
         </is>
       </c>
       <c r="E115" s="7" t="n">
@@ -5893,7 +5897,7 @@
         </is>
       </c>
       <c r="G115" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-de-mesa-de-ayuda-nivel-1-1886778506", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnicoa-tecnologoa-profesional-de-telecomunicaciones-redes-de-fibra-optica-1886768691", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H115" s="6" t="inlineStr"/>
@@ -5912,22 +5916,22 @@
     <row r="116" ht="22" customHeight="1">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>718ceee355d457ea</t>
+          <t>4e5b3128aa7f8f9b</t>
         </is>
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10 16:16</t>
+          <t>2026-10-09 17:28</t>
         </is>
       </c>
       <c r="C116" s="3" t="inlineStr">
         <is>
-          <t>IT Help Desk Support</t>
+          <t>Gestor de servicios mesa de ayuda sap</t>
         </is>
       </c>
       <c r="D116" s="3" t="inlineStr">
         <is>
-          <t>Booth</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E116" s="7" t="n">
@@ -5939,7 +5943,7 @@
         </is>
       </c>
       <c r="G116" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/it-help-desk-support-at-booth-4471203962", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/gestor-de-servicios-mesa-de-ayuda-sap-1886775732", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H116" s="6" t="inlineStr"/>
@@ -5958,17 +5962,17 @@
     <row r="117" ht="22" customHeight="1">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>925f43273b78f188</t>
+          <t>1c92f7ef9b7af696</t>
         </is>
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12 20:17</t>
+          <t>2026-10-09 17:28</t>
         </is>
       </c>
       <c r="C117" s="3" t="inlineStr">
         <is>
-          <t>Mesa de ayuda ti - girón</t>
+          <t>Agente de mesa de ayuda nivel 1</t>
         </is>
       </c>
       <c r="D117" s="3" t="inlineStr">
@@ -5985,7 +5989,7 @@
         </is>
       </c>
       <c r="G117" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/mesa-de-ayuda-ti-giron-1886745168", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-de-mesa-de-ayuda-nivel-1-1886778506", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H117" s="6" t="inlineStr"/>
@@ -6004,22 +6008,22 @@
     <row r="118" ht="22" customHeight="1">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>ec0c8875e04f4933</t>
+          <t>718ceee355d457ea</t>
         </is>
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13 18:08</t>
+          <t>2026-10-10 16:16</t>
         </is>
       </c>
       <c r="C118" s="3" t="inlineStr">
         <is>
-          <t>Analista de mesa de ayuda.</t>
+          <t>IT Help Desk Support</t>
         </is>
       </c>
       <c r="D118" s="3" t="inlineStr">
         <is>
-          <t>Softtek Colombia</t>
+          <t>Booth</t>
         </is>
       </c>
       <c r="E118" s="7" t="n">
@@ -6031,7 +6035,7 @@
         </is>
       </c>
       <c r="G118" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-mesa-de-ayuda-1886754207", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/it-help-desk-support-at-booth-4471203962", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H118" s="6" t="inlineStr"/>
@@ -6050,22 +6054,22 @@
     <row r="119" ht="22" customHeight="1">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>87fac63aa714f401</t>
+          <t>925f43273b78f188</t>
         </is>
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13 18:08</t>
+          <t>2026-10-12 20:17</t>
         </is>
       </c>
       <c r="C119" s="3" t="inlineStr">
         <is>
-          <t>Agente mesa de ayuda.</t>
+          <t>Mesa de ayuda ti - girón</t>
         </is>
       </c>
       <c r="D119" s="3" t="inlineStr">
         <is>
-          <t>Softtek Colombia</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E119" s="7" t="n">
@@ -6077,7 +6081,7 @@
         </is>
       </c>
       <c r="G119" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-mesa-de-ayuda-1886753535", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/mesa-de-ayuda-ti-giron-1886745168", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H119" s="6" t="inlineStr"/>
@@ -6096,22 +6100,22 @@
     <row r="120" ht="22" customHeight="1">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>dfa7dd88fd24afb4</t>
+          <t>ec0c8875e04f4933</t>
         </is>
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15 15:40</t>
+          <t>2026-10-13 18:08</t>
         </is>
       </c>
       <c r="C120" s="3" t="inlineStr">
         <is>
-          <t>Agente mesa de ayuda nivel 1 ingles avanzado</t>
+          <t>Analista de mesa de ayuda.</t>
         </is>
       </c>
       <c r="D120" s="3" t="inlineStr">
         <is>
-          <t>SUSTS Colombia Ltda.</t>
+          <t>Softtek Colombia</t>
         </is>
       </c>
       <c r="E120" s="7" t="n">
@@ -6123,7 +6127,7 @@
         </is>
       </c>
       <c r="G120" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-mesa-de-ayuda-nivel-1-ingles-avanzado-1886780371", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-mesa-de-ayuda-1886754207", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H120" s="6" t="inlineStr"/>
@@ -6142,22 +6146,22 @@
     <row r="121" ht="22" customHeight="1">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>6ec1aeac55104810</t>
+          <t>87fac63aa714f401</t>
         </is>
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16 15:22</t>
+          <t>2026-10-13 18:08</t>
         </is>
       </c>
       <c r="C121" s="3" t="inlineStr">
         <is>
-          <t>Analista de Mesa de Ayuda</t>
+          <t>Agente mesa de ayuda.</t>
         </is>
       </c>
       <c r="D121" s="3" t="inlineStr">
         <is>
-          <t>INSEPET S.A.S</t>
+          <t>Softtek Colombia</t>
         </is>
       </c>
       <c r="E121" s="7" t="n">
@@ -6169,14 +6173,10 @@
         </is>
       </c>
       <c r="G121" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-analista-de-mesa-de-ayuda-en-bogota-dc-731E37A9EEFEA71561373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H121" s="6" t="inlineStr">
-        <is>
-          <t>$ 1.800.000,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-mesa-de-ayuda-1886753535", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H121" s="6" t="inlineStr"/>
       <c r="I121" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -6192,22 +6192,22 @@
     <row r="122" ht="22" customHeight="1">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>c03a3cc06e28c7bb</t>
+          <t>dfa7dd88fd24afb4</t>
         </is>
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16 15:22</t>
+          <t>2026-10-15 15:40</t>
         </is>
       </c>
       <c r="C122" s="3" t="inlineStr">
         <is>
-          <t>Agente de mesa de ayuda portugues</t>
+          <t>Agente mesa de ayuda nivel 1 ingles avanzado</t>
         </is>
       </c>
       <c r="D122" s="3" t="inlineStr">
         <is>
-          <t>COMWARE S.A.</t>
+          <t>SUSTS Colombia Ltda.</t>
         </is>
       </c>
       <c r="E122" s="7" t="n">
@@ -6219,7 +6219,7 @@
         </is>
       </c>
       <c r="G122" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-de-mesa-de-ayuda-portugues-1886781202", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-mesa-de-ayuda-nivel-1-ingles-avanzado-1886780371", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H122" s="6" t="inlineStr"/>
@@ -6238,22 +6238,22 @@
     <row r="123" ht="22" customHeight="1">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>2ecdc22edf2ff172</t>
+          <t>6ec1aeac55104810</t>
         </is>
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17 14:15</t>
+          <t>2026-10-16 15:22</t>
         </is>
       </c>
       <c r="C123" s="3" t="inlineStr">
         <is>
-          <t>Agente Mesa de ayuda Portugués</t>
+          <t>Analista de Mesa de Ayuda</t>
         </is>
       </c>
       <c r="D123" s="3" t="inlineStr">
         <is>
-          <t>COMWARE S.A</t>
+          <t>INSEPET S.A.S</t>
         </is>
       </c>
       <c r="E123" s="7" t="n">
@@ -6265,12 +6265,12 @@
         </is>
       </c>
       <c r="G123" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-agente-mesa-de-ayuda-portugues-en-bogota-dc-D31C231B9F8EFFCA61373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-analista-de-mesa-de-ayuda-en-bogota-dc-731E37A9EEFEA71561373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H123" s="6" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>$ 1.800.000,00 (Mensual)</t>
         </is>
       </c>
       <c r="I123" s="3" t="inlineStr">
@@ -6288,22 +6288,22 @@
     <row r="124" ht="22" customHeight="1">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>3807f82cb9f9ccdb</t>
+          <t>c03a3cc06e28c7bb</t>
         </is>
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21 15:59</t>
+          <t>2026-10-16 15:22</t>
         </is>
       </c>
       <c r="C124" s="3" t="inlineStr">
         <is>
-          <t>Analista de Soporte TI Nivel I y II</t>
+          <t>Agente de mesa de ayuda portugues</t>
         </is>
       </c>
       <c r="D124" s="3" t="inlineStr">
         <is>
-          <t>Autonomic SAS</t>
+          <t>COMWARE S.A.</t>
         </is>
       </c>
       <c r="E124" s="7" t="n">
@@ -6315,14 +6315,10 @@
         </is>
       </c>
       <c r="G124" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-analista-de-soporte-ti-nivel-i-y-ii-en-medellin-452D284A14726B6861373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H124" s="6" t="inlineStr">
-        <is>
-          <t>$ 2.000.000,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-de-mesa-de-ayuda-portugues-1886781202", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H124" s="6" t="inlineStr"/>
       <c r="I124" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -6338,22 +6334,22 @@
     <row r="125" ht="22" customHeight="1">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>a716d4100a0f8155</t>
+          <t>2ecdc22edf2ff172</t>
         </is>
       </c>
       <c r="B125" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21 15:59</t>
+          <t>2026-10-17 14:15</t>
         </is>
       </c>
       <c r="C125" s="3" t="inlineStr">
         <is>
-          <t>Técnico de infraestructura y redes de telecomunicaciones - casanare</t>
+          <t>Agente Mesa de ayuda Portugués</t>
         </is>
       </c>
       <c r="D125" s="3" t="inlineStr">
         <is>
-          <t>SDT INGENIERIA</t>
+          <t>COMWARE S.A</t>
         </is>
       </c>
       <c r="E125" s="7" t="n">
@@ -6365,10 +6361,14 @@
         </is>
       </c>
       <c r="G125" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-infraestructura-y-redes-de-telecomunicaciones-casanare-1886779754", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H125" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-agente-mesa-de-ayuda-portugues-en-bogota-dc-D31C231B9F8EFFCA61373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H125" s="6" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
       <c r="I125" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -6384,7 +6384,7 @@
     <row r="126" ht="22" customHeight="1">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>3802f406ec698d83</t>
+          <t>3807f82cb9f9ccdb</t>
         </is>
       </c>
       <c r="B126" s="2" t="inlineStr">
@@ -6394,12 +6394,12 @@
       </c>
       <c r="C126" s="3" t="inlineStr">
         <is>
-          <t>Técnico de telecomunicaciones e instalación de redes - bogotá | experiencia en obra civil</t>
+          <t>Analista de Soporte TI Nivel I y II</t>
         </is>
       </c>
       <c r="D126" s="3" t="inlineStr">
         <is>
-          <t>ATIEMPO S.A.S</t>
+          <t>Autonomic SAS</t>
         </is>
       </c>
       <c r="E126" s="7" t="n">
@@ -6411,10 +6411,14 @@
         </is>
       </c>
       <c r="G126" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-telecomunicaciones-e-instalacion-de-redes-bogota-experiencia-en-obra-civil-1886760957", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H126" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-analista-de-soporte-ti-nivel-i-y-ii-en-medellin-452D284A14726B6861373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H126" s="6" t="inlineStr">
+        <is>
+          <t>$ 2.000.000,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I126" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -6430,26 +6434,26 @@
     <row r="127" ht="22" customHeight="1">
       <c r="A127" s="2" t="inlineStr">
         <is>
-          <t>50c79dfbfd49f52d</t>
+          <t>a716d4100a0f8155</t>
         </is>
       </c>
       <c r="B127" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 16:39</t>
+          <t>2026-10-21 15:59</t>
         </is>
       </c>
       <c r="C127" s="3" t="inlineStr">
         <is>
-          <t>Analista de redes noc 1 telecomunicaciones.</t>
+          <t>Técnico de infraestructura y redes de telecomunicaciones - casanare</t>
         </is>
       </c>
       <c r="D127" s="3" t="inlineStr">
         <is>
-          <t>MANPOWER</t>
+          <t>SDT INGENIERIA</t>
         </is>
       </c>
       <c r="E127" s="7" t="n">
-        <v>0.53</v>
+        <v>0.58</v>
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
@@ -6457,13 +6461,13 @@
         </is>
       </c>
       <c r="G127" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-noc-1-telecomunicaciones-1886772075", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-infraestructura-y-redes-de-telecomunicaciones-casanare-1886779754", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H127" s="6" t="inlineStr"/>
       <c r="I127" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J127" s="2" t="inlineStr">
@@ -6476,26 +6480,26 @@
     <row r="128" ht="22" customHeight="1">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>afe94b7770349744</t>
+          <t>3802f406ec698d83</t>
         </is>
       </c>
       <c r="B128" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 15:43</t>
+          <t>2026-10-21 15:59</t>
         </is>
       </c>
       <c r="C128" s="3" t="inlineStr">
         <is>
-          <t>Consultor de Seguridad de Redes – Akamai WAF con Inglés B2 o Superior.</t>
+          <t>Técnico de telecomunicaciones e instalación de redes - bogotá | experiencia en obra civil</t>
         </is>
       </c>
       <c r="D128" s="3" t="inlineStr">
         <is>
-          <t>Adecco Colombia S.A.</t>
+          <t>ATIEMPO S.A.S</t>
         </is>
       </c>
       <c r="E128" s="7" t="n">
-        <v>0.53</v>
+        <v>0.58</v>
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
@@ -6503,17 +6507,13 @@
         </is>
       </c>
       <c r="G128" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-consultor-de-seguridad-de-redes-akamai-waf-con-ingles-b2-o-superior-en-bogota-dc-50B87E7E33B988D461373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H128" s="6" t="inlineStr">
-        <is>
-          <t>$ 10.000.000,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-telecomunicaciones-e-instalacion-de-redes-bogota-experiencia-en-obra-civil-1886760957", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H128" s="6" t="inlineStr"/>
       <c r="I128" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J128" s="2" t="inlineStr">
@@ -6526,26 +6526,26 @@
     <row r="129" ht="22" customHeight="1">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>0b0ae49f910109bb</t>
+          <t>73bbbc1e10d41363</t>
         </is>
       </c>
       <c r="B129" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 15:54</t>
+          <t>2026-10-22 15:57</t>
         </is>
       </c>
       <c r="C129" s="3" t="inlineStr">
         <is>
-          <t>Ejecutivo Técnico Arancel Junior</t>
+          <t>Analista de Soporte IT</t>
         </is>
       </c>
       <c r="D129" s="3" t="inlineStr">
         <is>
-          <t>Importante Empresa de Logística y Comercio</t>
+          <t>TEMPORALES DE SOPORTE S.A.S.</t>
         </is>
       </c>
       <c r="E129" s="7" t="n">
-        <v>0.5</v>
+        <v>0.58</v>
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
@@ -6553,17 +6553,17 @@
         </is>
       </c>
       <c r="G129" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-547866639B487E0161373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-analista-de-soporte-it-en-bogota-dc-837CF03E481B2FAC61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H129" s="6" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>$ 2.500.000,00 (Mensual)</t>
         </is>
       </c>
       <c r="I129" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J129" s="2" t="inlineStr">
@@ -6576,26 +6576,26 @@
     <row r="130" ht="22" customHeight="1">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>582a04b3c639bfa0</t>
+          <t>5c204537d3c4c22f</t>
         </is>
       </c>
       <c r="B130" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 16:49</t>
+          <t>2026-10-22 15:57</t>
         </is>
       </c>
       <c r="C130" s="3" t="inlineStr">
         <is>
-          <t>Junior IT Support Specialist</t>
+          <t>Talento inclusivo : discapacidad | soporte | mesa de ayuda</t>
         </is>
       </c>
       <c r="D130" s="3" t="inlineStr">
         <is>
-          <t>Touch Support, Inc. &amp; SNF Back Office</t>
+          <t>Sinergy &amp; Lowells</t>
         </is>
       </c>
       <c r="E130" s="7" t="n">
-        <v>0.5</v>
+        <v>0.58</v>
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
@@ -6603,13 +6603,13 @@
         </is>
       </c>
       <c r="G130" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/junior-it-support-specialist-at-touch-support-inc-snf-back-office-4472187578", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/talento-inclusivo-discapacidad-soporte-mesa-de-ayuda-1886783065", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H130" s="6" t="inlineStr"/>
       <c r="I130" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J130" s="2" t="inlineStr">
@@ -6622,26 +6622,26 @@
     <row r="131" ht="22" customHeight="1">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>6e04c4d57d3fc3c7</t>
+          <t>50c79dfbfd49f52d</t>
         </is>
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 17:26</t>
+          <t>2026-10-02 16:39</t>
         </is>
       </c>
       <c r="C131" s="3" t="inlineStr">
         <is>
-          <t>Ejecutivo Técnico Arancel Junior</t>
+          <t>Analista de redes noc 1 telecomunicaciones.</t>
         </is>
       </c>
       <c r="D131" s="3" t="inlineStr">
         <is>
-          <t>Importante Empresa de Logística y Comercio</t>
+          <t>MANPOWER</t>
         </is>
       </c>
       <c r="E131" s="7" t="n">
-        <v>0.5</v>
+        <v>0.53</v>
       </c>
       <c r="F131" s="2" t="inlineStr">
         <is>
@@ -6649,17 +6649,13 @@
         </is>
       </c>
       <c r="G131" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-8444AB594560844161373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H131" s="6" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-noc-1-telecomunicaciones-1886772075", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H131" s="6" t="inlineStr"/>
       <c r="I131" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J131" s="2" t="inlineStr">
@@ -6672,52 +6668,248 @@
     <row r="132" ht="22" customHeight="1">
       <c r="A132" s="2" t="inlineStr">
         <is>
+          <t>afe94b7770349744</t>
+        </is>
+      </c>
+      <c r="B132" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 15:43</t>
+        </is>
+      </c>
+      <c r="C132" s="3" t="inlineStr">
+        <is>
+          <t>Consultor de Seguridad de Redes – Akamai WAF con Inglés B2 o Superior.</t>
+        </is>
+      </c>
+      <c r="D132" s="3" t="inlineStr">
+        <is>
+          <t>Adecco Colombia S.A.</t>
+        </is>
+      </c>
+      <c r="E132" s="7" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="F132" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G132" s="5">
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-consultor-de-seguridad-de-redes-akamai-waf-con-ingles-b2-o-superior-en-bogota-dc-50B87E7E33B988D461373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H132" s="6" t="inlineStr">
+        <is>
+          <t>$ 10.000.000,00 (Mensual)</t>
+        </is>
+      </c>
+      <c r="I132" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J132" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K132" s="3" t="inlineStr"/>
+    </row>
+    <row r="133" ht="22" customHeight="1">
+      <c r="A133" s="2" t="inlineStr">
+        <is>
+          <t>0b0ae49f910109bb</t>
+        </is>
+      </c>
+      <c r="B133" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25 15:54</t>
+        </is>
+      </c>
+      <c r="C133" s="3" t="inlineStr">
+        <is>
+          <t>Ejecutivo Técnico Arancel Junior</t>
+        </is>
+      </c>
+      <c r="D133" s="3" t="inlineStr">
+        <is>
+          <t>Importante Empresa de Logística y Comercio</t>
+        </is>
+      </c>
+      <c r="E133" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F133" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G133" s="5">
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-547866639B487E0161373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H133" s="6" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="I133" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J133" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K133" s="3" t="inlineStr"/>
+    </row>
+    <row r="134" ht="22" customHeight="1">
+      <c r="A134" s="2" t="inlineStr">
+        <is>
+          <t>582a04b3c639bfa0</t>
+        </is>
+      </c>
+      <c r="B134" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 16:49</t>
+        </is>
+      </c>
+      <c r="C134" s="3" t="inlineStr">
+        <is>
+          <t>Junior IT Support Specialist</t>
+        </is>
+      </c>
+      <c r="D134" s="3" t="inlineStr">
+        <is>
+          <t>Touch Support, Inc. &amp; SNF Back Office</t>
+        </is>
+      </c>
+      <c r="E134" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F134" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G134" s="5">
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/junior-it-support-specialist-at-touch-support-inc-snf-back-office-4472187578", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H134" s="6" t="inlineStr"/>
+      <c r="I134" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J134" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K134" s="3" t="inlineStr"/>
+    </row>
+    <row r="135" ht="22" customHeight="1">
+      <c r="A135" s="2" t="inlineStr">
+        <is>
+          <t>6e04c4d57d3fc3c7</t>
+        </is>
+      </c>
+      <c r="B135" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01 17:26</t>
+        </is>
+      </c>
+      <c r="C135" s="3" t="inlineStr">
+        <is>
+          <t>Ejecutivo Técnico Arancel Junior</t>
+        </is>
+      </c>
+      <c r="D135" s="3" t="inlineStr">
+        <is>
+          <t>Importante Empresa de Logística y Comercio</t>
+        </is>
+      </c>
+      <c r="E135" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F135" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G135" s="5">
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-8444AB594560844161373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H135" s="6" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="I135" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J135" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K135" s="3" t="inlineStr"/>
+    </row>
+    <row r="136" ht="22" customHeight="1">
+      <c r="A136" s="2" t="inlineStr">
+        <is>
           <t>8d81bacef79435aa</t>
         </is>
       </c>
-      <c r="B132" s="2" t="inlineStr">
+      <c r="B136" s="2" t="inlineStr">
         <is>
           <t>2026-10-20 15:43</t>
         </is>
       </c>
-      <c r="C132" s="3" t="inlineStr">
+      <c r="C136" s="3" t="inlineStr">
         <is>
           <t>Buscamos Estudiantes en Áreas de Sistemas, Software para trabajar desde casa // sin Experiencia</t>
         </is>
       </c>
-      <c r="D132" s="3" t="inlineStr">
+      <c r="D136" s="3" t="inlineStr">
         <is>
           <t>emtelco</t>
         </is>
       </c>
-      <c r="E132" s="7" t="n">
+      <c r="E136" s="7" t="n">
         <v>0.5</v>
       </c>
-      <c r="F132" s="2" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
-      <c r="G132" s="5">
+      <c r="F136" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G136" s="5">
         <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-buscamos-estudiantes-en-areas-de-sistemas-software-para-trabajar-desde-casa-sin-experiencia-participa-todas-las-areas-relacionadas-con-soporte-tecnico-en-medellin-D756C734FE234C3D61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
-      <c r="H132" s="6" t="inlineStr">
+      <c r="H136" s="6" t="inlineStr">
         <is>
           <t>$ 1.750.905,00 (Mensual)</t>
         </is>
       </c>
-      <c r="I132" s="3" t="inlineStr">
+      <c r="I136" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
-      <c r="J132" s="2" t="inlineStr">
-        <is>
-          <t>Nueva</t>
-        </is>
-      </c>
-      <c r="K132" s="3" t="inlineStr"/>
+      <c r="J136" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K136" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
chore(tracker): actualizacion diaria de vacantes 2026-10-23
</commit_message>
<xml_diff>
--- a/output/profile_5_tecnico_sistemas_tracker.xlsx
+++ b/output/profile_5_tecnico_sistemas_tracker.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K136"/>
+  <dimension ref="A1:K137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -6622,26 +6622,26 @@
     <row r="131" ht="22" customHeight="1">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>50c79dfbfd49f52d</t>
+          <t>0a5982e3569b3861</t>
         </is>
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 16:39</t>
+          <t>2026-10-23 15:48</t>
         </is>
       </c>
       <c r="C131" s="3" t="inlineStr">
         <is>
-          <t>Analista de redes noc 1 telecomunicaciones.</t>
+          <t>Analista mesa de ayuda</t>
         </is>
       </c>
       <c r="D131" s="3" t="inlineStr">
         <is>
-          <t>MANPOWER</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E131" s="7" t="n">
-        <v>0.53</v>
+        <v>0.58</v>
       </c>
       <c r="F131" s="2" t="inlineStr">
         <is>
@@ -6649,13 +6649,13 @@
         </is>
       </c>
       <c r="G131" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-noc-1-telecomunicaciones-1886772075", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-1886783910", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H131" s="6" t="inlineStr"/>
       <c r="I131" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J131" s="2" t="inlineStr">
@@ -6668,22 +6668,22 @@
     <row r="132" ht="22" customHeight="1">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>afe94b7770349744</t>
+          <t>50c79dfbfd49f52d</t>
         </is>
       </c>
       <c r="B132" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 15:43</t>
+          <t>2026-10-02 16:39</t>
         </is>
       </c>
       <c r="C132" s="3" t="inlineStr">
         <is>
-          <t>Consultor de Seguridad de Redes – Akamai WAF con Inglés B2 o Superior.</t>
+          <t>Analista de redes noc 1 telecomunicaciones.</t>
         </is>
       </c>
       <c r="D132" s="3" t="inlineStr">
         <is>
-          <t>Adecco Colombia S.A.</t>
+          <t>MANPOWER</t>
         </is>
       </c>
       <c r="E132" s="7" t="n">
@@ -6695,14 +6695,10 @@
         </is>
       </c>
       <c r="G132" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-consultor-de-seguridad-de-redes-akamai-waf-con-ingles-b2-o-superior-en-bogota-dc-50B87E7E33B988D461373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H132" s="6" t="inlineStr">
-        <is>
-          <t>$ 10.000.000,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-noc-1-telecomunicaciones-1886772075", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H132" s="6" t="inlineStr"/>
       <c r="I132" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -6718,26 +6714,26 @@
     <row r="133" ht="22" customHeight="1">
       <c r="A133" s="2" t="inlineStr">
         <is>
-          <t>0b0ae49f910109bb</t>
+          <t>afe94b7770349744</t>
         </is>
       </c>
       <c r="B133" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 15:54</t>
+          <t>2026-10-20 15:43</t>
         </is>
       </c>
       <c r="C133" s="3" t="inlineStr">
         <is>
-          <t>Ejecutivo Técnico Arancel Junior</t>
+          <t>Consultor de Seguridad de Redes – Akamai WAF con Inglés B2 o Superior.</t>
         </is>
       </c>
       <c r="D133" s="3" t="inlineStr">
         <is>
-          <t>Importante Empresa de Logística y Comercio</t>
+          <t>Adecco Colombia S.A.</t>
         </is>
       </c>
       <c r="E133" s="7" t="n">
-        <v>0.5</v>
+        <v>0.53</v>
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
@@ -6745,17 +6741,17 @@
         </is>
       </c>
       <c r="G133" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-547866639B487E0161373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-consultor-de-seguridad-de-redes-akamai-waf-con-ingles-b2-o-superior-en-bogota-dc-50B87E7E33B988D461373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H133" s="6" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>$ 10.000.000,00 (Mensual)</t>
         </is>
       </c>
       <c r="I133" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J133" s="2" t="inlineStr">
@@ -6768,22 +6764,22 @@
     <row r="134" ht="22" customHeight="1">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>582a04b3c639bfa0</t>
+          <t>0b0ae49f910109bb</t>
         </is>
       </c>
       <c r="B134" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 16:49</t>
+          <t>2026-09-25 15:54</t>
         </is>
       </c>
       <c r="C134" s="3" t="inlineStr">
         <is>
-          <t>Junior IT Support Specialist</t>
+          <t>Ejecutivo Técnico Arancel Junior</t>
         </is>
       </c>
       <c r="D134" s="3" t="inlineStr">
         <is>
-          <t>Touch Support, Inc. &amp; SNF Back Office</t>
+          <t>Importante Empresa de Logística y Comercio</t>
         </is>
       </c>
       <c r="E134" s="7" t="n">
@@ -6795,10 +6791,14 @@
         </is>
       </c>
       <c r="G134" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/junior-it-support-specialist-at-touch-support-inc-snf-back-office-4472187578", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H134" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-547866639B487E0161373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H134" s="6" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
       <c r="I134" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -6814,22 +6814,22 @@
     <row r="135" ht="22" customHeight="1">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>6e04c4d57d3fc3c7</t>
+          <t>582a04b3c639bfa0</t>
         </is>
       </c>
       <c r="B135" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 17:26</t>
+          <t>2026-09-30 16:49</t>
         </is>
       </c>
       <c r="C135" s="3" t="inlineStr">
         <is>
-          <t>Ejecutivo Técnico Arancel Junior</t>
+          <t>Junior IT Support Specialist</t>
         </is>
       </c>
       <c r="D135" s="3" t="inlineStr">
         <is>
-          <t>Importante Empresa de Logística y Comercio</t>
+          <t>Touch Support, Inc. &amp; SNF Back Office</t>
         </is>
       </c>
       <c r="E135" s="7" t="n">
@@ -6841,14 +6841,10 @@
         </is>
       </c>
       <c r="G135" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-8444AB594560844161373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H135" s="6" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/junior-it-support-specialist-at-touch-support-inc-snf-back-office-4472187578", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H135" s="6" t="inlineStr"/>
       <c r="I135" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -6864,22 +6860,22 @@
     <row r="136" ht="22" customHeight="1">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>8d81bacef79435aa</t>
+          <t>6e04c4d57d3fc3c7</t>
         </is>
       </c>
       <c r="B136" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 15:43</t>
+          <t>2026-10-01 17:26</t>
         </is>
       </c>
       <c r="C136" s="3" t="inlineStr">
         <is>
-          <t>Buscamos Estudiantes en Áreas de Sistemas, Software para trabajar desde casa // sin Experiencia</t>
+          <t>Ejecutivo Técnico Arancel Junior</t>
         </is>
       </c>
       <c r="D136" s="3" t="inlineStr">
         <is>
-          <t>emtelco</t>
+          <t>Importante Empresa de Logística y Comercio</t>
         </is>
       </c>
       <c r="E136" s="7" t="n">
@@ -6891,25 +6887,75 @@
         </is>
       </c>
       <c r="G136" s="5">
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-8444AB594560844161373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H136" s="6" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="I136" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J136" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K136" s="3" t="inlineStr"/>
+    </row>
+    <row r="137" ht="22" customHeight="1">
+      <c r="A137" s="2" t="inlineStr">
+        <is>
+          <t>8d81bacef79435aa</t>
+        </is>
+      </c>
+      <c r="B137" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 15:43</t>
+        </is>
+      </c>
+      <c r="C137" s="3" t="inlineStr">
+        <is>
+          <t>Buscamos Estudiantes en Áreas de Sistemas, Software para trabajar desde casa // sin Experiencia</t>
+        </is>
+      </c>
+      <c r="D137" s="3" t="inlineStr">
+        <is>
+          <t>emtelco</t>
+        </is>
+      </c>
+      <c r="E137" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F137" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G137" s="5">
         <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-buscamos-estudiantes-en-areas-de-sistemas-software-para-trabajar-desde-casa-sin-experiencia-participa-todas-las-areas-relacionadas-con-soporte-tecnico-en-medellin-D756C734FE234C3D61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
-      <c r="H136" s="6" t="inlineStr">
+      <c r="H137" s="6" t="inlineStr">
         <is>
           <t>$ 1.750.905,00 (Mensual)</t>
         </is>
       </c>
-      <c r="I136" s="3" t="inlineStr">
+      <c r="I137" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
-      <c r="J136" s="2" t="inlineStr">
-        <is>
-          <t>Nueva</t>
-        </is>
-      </c>
-      <c r="K136" s="3" t="inlineStr"/>
+      <c r="J137" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K137" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
chore(tracker): actualizacion diaria de vacantes 2026-10-29
</commit_message>
<xml_diff>
--- a/output/profile_5_tecnico_sistemas_tracker.xlsx
+++ b/output/profile_5_tecnico_sistemas_tracker.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K137"/>
+  <dimension ref="A1:K139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -6668,26 +6668,26 @@
     <row r="132" ht="22" customHeight="1">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>50c79dfbfd49f52d</t>
+          <t>a805462f0646b537</t>
         </is>
       </c>
       <c r="B132" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 16:39</t>
+          <t>2026-10-29 17:29</t>
         </is>
       </c>
       <c r="C132" s="3" t="inlineStr">
         <is>
-          <t>Analista de redes noc 1 telecomunicaciones.</t>
+          <t>Analista mesa de ayuda</t>
         </is>
       </c>
       <c r="D132" s="3" t="inlineStr">
         <is>
-          <t>MANPOWER</t>
+          <t>AGENCIA DE EMPLEO COLSUBSIDIO</t>
         </is>
       </c>
       <c r="E132" s="7" t="n">
-        <v>0.53</v>
+        <v>0.58</v>
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
@@ -6695,13 +6695,13 @@
         </is>
       </c>
       <c r="G132" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-noc-1-telecomunicaciones-1886772075", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-1886786118", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H132" s="6" t="inlineStr"/>
       <c r="I132" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J132" s="2" t="inlineStr">
@@ -6714,26 +6714,26 @@
     <row r="133" ht="22" customHeight="1">
       <c r="A133" s="2" t="inlineStr">
         <is>
-          <t>afe94b7770349744</t>
+          <t>31eebea3ebe84a0c</t>
         </is>
       </c>
       <c r="B133" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 15:43</t>
+          <t>2026-10-29 17:29</t>
         </is>
       </c>
       <c r="C133" s="3" t="inlineStr">
         <is>
-          <t>Consultor de Seguridad de Redes – Akamai WAF con Inglés B2 o Superior.</t>
+          <t>IT Help Desk Support</t>
         </is>
       </c>
       <c r="D133" s="3" t="inlineStr">
         <is>
-          <t>Adecco Colombia S.A.</t>
+          <t>Booth</t>
         </is>
       </c>
       <c r="E133" s="7" t="n">
-        <v>0.53</v>
+        <v>0.58</v>
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
@@ -6741,17 +6741,13 @@
         </is>
       </c>
       <c r="G133" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-consultor-de-seguridad-de-redes-akamai-waf-con-ingles-b2-o-superior-en-bogota-dc-50B87E7E33B988D461373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H133" s="6" t="inlineStr">
-        <is>
-          <t>$ 10.000.000,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/it-help-desk-support-at-booth-4482551670", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H133" s="6" t="inlineStr"/>
       <c r="I133" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J133" s="2" t="inlineStr">
@@ -6764,26 +6760,26 @@
     <row r="134" ht="22" customHeight="1">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>0b0ae49f910109bb</t>
+          <t>50c79dfbfd49f52d</t>
         </is>
       </c>
       <c r="B134" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 15:54</t>
+          <t>2026-10-02 16:39</t>
         </is>
       </c>
       <c r="C134" s="3" t="inlineStr">
         <is>
-          <t>Ejecutivo Técnico Arancel Junior</t>
+          <t>Analista de redes noc 1 telecomunicaciones.</t>
         </is>
       </c>
       <c r="D134" s="3" t="inlineStr">
         <is>
-          <t>Importante Empresa de Logística y Comercio</t>
+          <t>MANPOWER</t>
         </is>
       </c>
       <c r="E134" s="7" t="n">
-        <v>0.5</v>
+        <v>0.53</v>
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
@@ -6791,17 +6787,13 @@
         </is>
       </c>
       <c r="G134" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-547866639B487E0161373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H134" s="6" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-noc-1-telecomunicaciones-1886772075", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H134" s="6" t="inlineStr"/>
       <c r="I134" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J134" s="2" t="inlineStr">
@@ -6814,26 +6806,26 @@
     <row r="135" ht="22" customHeight="1">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>582a04b3c639bfa0</t>
+          <t>afe94b7770349744</t>
         </is>
       </c>
       <c r="B135" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 16:49</t>
+          <t>2026-10-20 15:43</t>
         </is>
       </c>
       <c r="C135" s="3" t="inlineStr">
         <is>
-          <t>Junior IT Support Specialist</t>
+          <t>Consultor de Seguridad de Redes – Akamai WAF con Inglés B2 o Superior.</t>
         </is>
       </c>
       <c r="D135" s="3" t="inlineStr">
         <is>
-          <t>Touch Support, Inc. &amp; SNF Back Office</t>
+          <t>Adecco Colombia S.A.</t>
         </is>
       </c>
       <c r="E135" s="7" t="n">
-        <v>0.5</v>
+        <v>0.53</v>
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
@@ -6841,13 +6833,17 @@
         </is>
       </c>
       <c r="G135" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/junior-it-support-specialist-at-touch-support-inc-snf-back-office-4472187578", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H135" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-consultor-de-seguridad-de-redes-akamai-waf-con-ingles-b2-o-superior-en-bogota-dc-50B87E7E33B988D461373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H135" s="6" t="inlineStr">
+        <is>
+          <t>$ 10.000.000,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I135" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J135" s="2" t="inlineStr">
@@ -6860,12 +6856,12 @@
     <row r="136" ht="22" customHeight="1">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>6e04c4d57d3fc3c7</t>
+          <t>0b0ae49f910109bb</t>
         </is>
       </c>
       <c r="B136" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 17:26</t>
+          <t>2026-09-25 15:54</t>
         </is>
       </c>
       <c r="C136" s="3" t="inlineStr">
@@ -6887,7 +6883,7 @@
         </is>
       </c>
       <c r="G136" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-8444AB594560844161373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-547866639B487E0161373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H136" s="6" t="inlineStr">
@@ -6910,22 +6906,22 @@
     <row r="137" ht="22" customHeight="1">
       <c r="A137" s="2" t="inlineStr">
         <is>
-          <t>8d81bacef79435aa</t>
+          <t>582a04b3c639bfa0</t>
         </is>
       </c>
       <c r="B137" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 15:43</t>
+          <t>2026-09-30 16:49</t>
         </is>
       </c>
       <c r="C137" s="3" t="inlineStr">
         <is>
-          <t>Buscamos Estudiantes en Áreas de Sistemas, Software para trabajar desde casa // sin Experiencia</t>
+          <t>Junior IT Support Specialist</t>
         </is>
       </c>
       <c r="D137" s="3" t="inlineStr">
         <is>
-          <t>emtelco</t>
+          <t>Touch Support, Inc. &amp; SNF Back Office</t>
         </is>
       </c>
       <c r="E137" s="7" t="n">
@@ -6937,25 +6933,121 @@
         </is>
       </c>
       <c r="G137" s="5">
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/junior-it-support-specialist-at-touch-support-inc-snf-back-office-4472187578", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H137" s="6" t="inlineStr"/>
+      <c r="I137" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J137" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K137" s="3" t="inlineStr"/>
+    </row>
+    <row r="138" ht="22" customHeight="1">
+      <c r="A138" s="2" t="inlineStr">
+        <is>
+          <t>6e04c4d57d3fc3c7</t>
+        </is>
+      </c>
+      <c r="B138" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01 17:26</t>
+        </is>
+      </c>
+      <c r="C138" s="3" t="inlineStr">
+        <is>
+          <t>Ejecutivo Técnico Arancel Junior</t>
+        </is>
+      </c>
+      <c r="D138" s="3" t="inlineStr">
+        <is>
+          <t>Importante Empresa de Logística y Comercio</t>
+        </is>
+      </c>
+      <c r="E138" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F138" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G138" s="5">
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-8444AB594560844161373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H138" s="6" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="I138" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J138" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K138" s="3" t="inlineStr"/>
+    </row>
+    <row r="139" ht="22" customHeight="1">
+      <c r="A139" s="2" t="inlineStr">
+        <is>
+          <t>8d81bacef79435aa</t>
+        </is>
+      </c>
+      <c r="B139" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 15:43</t>
+        </is>
+      </c>
+      <c r="C139" s="3" t="inlineStr">
+        <is>
+          <t>Buscamos Estudiantes en Áreas de Sistemas, Software para trabajar desde casa // sin Experiencia</t>
+        </is>
+      </c>
+      <c r="D139" s="3" t="inlineStr">
+        <is>
+          <t>emtelco</t>
+        </is>
+      </c>
+      <c r="E139" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F139" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G139" s="5">
         <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-buscamos-estudiantes-en-areas-de-sistemas-software-para-trabajar-desde-casa-sin-experiencia-participa-todas-las-areas-relacionadas-con-soporte-tecnico-en-medellin-D756C734FE234C3D61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
-      <c r="H137" s="6" t="inlineStr">
+      <c r="H139" s="6" t="inlineStr">
         <is>
           <t>$ 1.750.905,00 (Mensual)</t>
         </is>
       </c>
-      <c r="I137" s="3" t="inlineStr">
+      <c r="I139" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
-      <c r="J137" s="2" t="inlineStr">
-        <is>
-          <t>Nueva</t>
-        </is>
-      </c>
-      <c r="K137" s="3" t="inlineStr"/>
+      <c r="J139" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K139" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
chore(tracker): actualizacion diaria de vacantes 2026-10-30
</commit_message>
<xml_diff>
--- a/output/profile_5_tecnico_sistemas_tracker.xlsx
+++ b/output/profile_5_tecnico_sistemas_tracker.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K139"/>
+  <dimension ref="A1:K140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3818,26 +3818,26 @@
     <row r="71" ht="22" customHeight="1">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>ae736277661dc78b</t>
+          <t>9bf6ee73cbc924f9</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 15:23</t>
+          <t>2026-10-30 17:06</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>Analista de redes cisco</t>
+          <t>Agente de soporte técnico - nocturno remoto</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>ATCG DE COLOMBIA S.A.S</t>
-        </is>
-      </c>
-      <c r="E71" s="7" t="n">
-        <v>0.68</v>
+          <t>PRAXIS I.T COLOMBIA LTDA</t>
+        </is>
+      </c>
+      <c r="E71" s="4" t="n">
+        <v>0.73</v>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
@@ -3845,13 +3845,13 @@
         </is>
       </c>
       <c r="G71" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-cisco-1886760389", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-de-soporte-tecnico-nocturno-remoto-1886787108", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H71" s="6" t="inlineStr"/>
       <c r="I71" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 68/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 73/100 - Alta Afinidad] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J71" s="2" t="inlineStr">
@@ -3864,7 +3864,7 @@
     <row r="72" ht="22" customHeight="1">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>e29676fac3409ad6</t>
+          <t>ae736277661dc78b</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -3874,12 +3874,12 @@
       </c>
       <c r="C72" s="3" t="inlineStr">
         <is>
-          <t>Analista de redes y telecomunicaciones - nivel 1</t>
+          <t>Analista de redes cisco</t>
         </is>
       </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
-          <t>MANPOWER</t>
+          <t>ATCG DE COLOMBIA S.A.S</t>
         </is>
       </c>
       <c r="E72" s="7" t="n">
@@ -3891,7 +3891,7 @@
         </is>
       </c>
       <c r="G72" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-y-telecomunicaciones-nivel-1-1886760565", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-cisco-1886760389", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H72" s="6" t="inlineStr"/>
@@ -3910,26 +3910,26 @@
     <row r="73" ht="22" customHeight="1">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>baf000f38713dc11</t>
+          <t>e29676fac3409ad6</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07 17:50</t>
+          <t>2026-09-24 15:23</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>Helpdesk / Analista soporte TI / trilingüe</t>
+          <t>Analista de redes y telecomunicaciones - nivel 1</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>Confidential</t>
+          <t>MANPOWER</t>
         </is>
       </c>
       <c r="E73" s="7" t="n">
-        <v>0.66</v>
+        <v>0.68</v>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
@@ -3937,13 +3937,13 @@
         </is>
       </c>
       <c r="G73" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/helpdesk-analista-soporte-ti-triling%C3%BCe-ingles-portugu%C3%A9s-at-confidential-4469673592", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-y-telecomunicaciones-nivel-1-1886760565", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H73" s="6" t="inlineStr"/>
       <c r="I73" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 66/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 68/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J73" s="2" t="inlineStr">
@@ -3956,22 +3956,22 @@
     <row r="74" ht="22" customHeight="1">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>422a27df3967ecbb</t>
+          <t>baf000f38713dc11</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14 15:52</t>
+          <t>2026-10-07 17:50</t>
         </is>
       </c>
       <c r="C74" s="3" t="inlineStr">
         <is>
-          <t>Técnico de sistemas y soporte ti</t>
+          <t>Helpdesk / Analista soporte TI / trilingüe</t>
         </is>
       </c>
       <c r="D74" s="3" t="inlineStr">
         <is>
-          <t>AGENCIA DE EMPLEO CAFAM</t>
+          <t>Confidential</t>
         </is>
       </c>
       <c r="E74" s="7" t="n">
@@ -3983,7 +3983,7 @@
         </is>
       </c>
       <c r="G74" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-sistemas-y-soporte-ti-1886780022", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/helpdesk-analista-soporte-ti-triling%C3%BCe-ingles-portugu%C3%A9s-at-confidential-4469673592", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H74" s="6" t="inlineStr"/>
@@ -4002,26 +4002,26 @@
     <row r="75" ht="22" customHeight="1">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>73882c81e04abc7e</t>
+          <t>422a27df3967ecbb</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 19:45</t>
+          <t>2026-10-14 15:52</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>Soporte L1 Junior</t>
+          <t>Técnico de sistemas y soporte ti</t>
         </is>
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>Hublance</t>
+          <t>AGENCIA DE EMPLEO CAFAM</t>
         </is>
       </c>
       <c r="E75" s="7" t="n">
-        <v>0.6</v>
+        <v>0.66</v>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
@@ -4029,13 +4029,13 @@
         </is>
       </c>
       <c r="G75" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/soporte-l1-junior-at-hublance-4475841269", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-sistemas-y-soporte-ti-1886780022", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H75" s="6" t="inlineStr"/>
       <c r="I75" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 60/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 66/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J75" s="2" t="inlineStr">
@@ -4048,26 +4048,26 @@
     <row r="76" ht="22" customHeight="1">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>8d7f304ffb8625b5</t>
+          <t>73882c81e04abc7e</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 15:54</t>
+          <t>2026-10-05 19:45</t>
         </is>
       </c>
       <c r="C76" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar de sistemas</t>
+          <t>Soporte L1 Junior</t>
         </is>
       </c>
       <c r="D76" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Hublance</t>
         </is>
       </c>
       <c r="E76" s="7" t="n">
-        <v>0.58</v>
+        <v>0.6</v>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
@@ -4075,13 +4075,13 @@
         </is>
       </c>
       <c r="G76" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886751888", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/soporte-l1-junior-at-hublance-4475841269", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H76" s="6" t="inlineStr"/>
       <c r="I76" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 60/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J76" s="2" t="inlineStr">
@@ -4094,7 +4094,7 @@
     <row r="77" ht="22" customHeight="1">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>3b5b26f92a305c0c</t>
+          <t>8d7f304ffb8625b5</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
@@ -4121,7 +4121,7 @@
         </is>
       </c>
       <c r="G77" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886749497", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886751888", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H77" s="6" t="inlineStr"/>
@@ -4140,7 +4140,7 @@
     <row r="78" ht="22" customHeight="1">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>e760bcd88d90fbbe</t>
+          <t>3b5b26f92a305c0c</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -4150,12 +4150,12 @@
       </c>
       <c r="C78" s="3" t="inlineStr">
         <is>
-          <t>Agente de mesa de ayuda</t>
+          <t>Auxiliar de sistemas</t>
         </is>
       </c>
       <c r="D78" s="3" t="inlineStr">
         <is>
-          <t>SELCOMP INGENIERÍA SAS</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E78" s="7" t="n">
@@ -4167,7 +4167,7 @@
         </is>
       </c>
       <c r="G78" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-de-mesa-de-ayuda-1886758623", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886749497", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H78" s="6" t="inlineStr"/>
@@ -4186,7 +4186,7 @@
     <row r="79" ht="22" customHeight="1">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>86dcab5c5d802693</t>
+          <t>e760bcd88d90fbbe</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
@@ -4196,12 +4196,12 @@
       </c>
       <c r="C79" s="3" t="inlineStr">
         <is>
-          <t>Analista mesa de ayuda para tunja</t>
+          <t>Agente de mesa de ayuda</t>
         </is>
       </c>
       <c r="D79" s="3" t="inlineStr">
         <is>
-          <t>Gestión de Seguridad Electrónica</t>
+          <t>SELCOMP INGENIERÍA SAS</t>
         </is>
       </c>
       <c r="E79" s="7" t="n">
@@ -4213,7 +4213,7 @@
         </is>
       </c>
       <c r="G79" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-para-tunja-1886766955", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-de-mesa-de-ayuda-1886758623", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H79" s="6" t="inlineStr"/>
@@ -4232,7 +4232,7 @@
     <row r="80" ht="22" customHeight="1">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>55fdaa0983ef9124</t>
+          <t>86dcab5c5d802693</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
@@ -4242,12 +4242,12 @@
       </c>
       <c r="C80" s="3" t="inlineStr">
         <is>
-          <t>Lider técnico con itil practice manager</t>
+          <t>Analista mesa de ayuda para tunja</t>
         </is>
       </c>
       <c r="D80" s="3" t="inlineStr">
         <is>
-          <t>Sinergy &amp; Lowells</t>
+          <t>Gestión de Seguridad Electrónica</t>
         </is>
       </c>
       <c r="E80" s="7" t="n">
@@ -4259,7 +4259,7 @@
         </is>
       </c>
       <c r="G80" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/lider-tecnico-con-itil-practice-manager-1886753953", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-para-tunja-1886766955", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H80" s="6" t="inlineStr"/>
@@ -4278,7 +4278,7 @@
     <row r="81" ht="22" customHeight="1">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>a1ca7bc58cd48fad</t>
+          <t>55fdaa0983ef9124</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
@@ -4288,12 +4288,12 @@
       </c>
       <c r="C81" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de mesa de ayuda/mujeres contratacion inmediata</t>
+          <t>Lider técnico con itil practice manager</t>
         </is>
       </c>
       <c r="D81" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Sinergy &amp; Lowells</t>
         </is>
       </c>
       <c r="E81" s="7" t="n">
@@ -4305,7 +4305,7 @@
         </is>
       </c>
       <c r="G81" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-mesa-de-ayuda-mujeres-contratacion-inmediata-1886770931", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/lider-tecnico-con-itil-practice-manager-1886753953", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H81" s="6" t="inlineStr"/>
@@ -4324,7 +4324,7 @@
     <row r="82" ht="22" customHeight="1">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>e28aba5df8a2d3ae</t>
+          <t>a1ca7bc58cd48fad</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
@@ -4351,7 +4351,7 @@
         </is>
       </c>
       <c r="G82" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-mesa-de-ayuda-mujeres-contratacion-inmediata-1886769701", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-mesa-de-ayuda-mujeres-contratacion-inmediata-1886770931", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H82" s="6" t="inlineStr"/>
@@ -4370,7 +4370,7 @@
     <row r="83" ht="22" customHeight="1">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>9326784c1a2726fb</t>
+          <t>e28aba5df8a2d3ae</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
@@ -4380,12 +4380,12 @@
       </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t>Técnico de soporte y mesa de ayuda / medellín</t>
+          <t>Tecnico de mesa de ayuda/mujeres contratacion inmediata</t>
         </is>
       </c>
       <c r="D83" s="3" t="inlineStr">
         <is>
-          <t>Colsof S.A.S</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E83" s="7" t="n">
@@ -4397,7 +4397,7 @@
         </is>
       </c>
       <c r="G83" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-y-mesa-de-ayuda-medellin-1886738118", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-mesa-de-ayuda-mujeres-contratacion-inmediata-1886769701", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H83" s="6" t="inlineStr"/>
@@ -4416,7 +4416,7 @@
     <row r="84" ht="22" customHeight="1">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>b67dc9a9be4a1a6f</t>
+          <t>9326784c1a2726fb</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
@@ -4426,12 +4426,12 @@
       </c>
       <c r="C84" s="3" t="inlineStr">
         <is>
-          <t>Service desk agent</t>
+          <t>Técnico de soporte y mesa de ayuda / medellín</t>
         </is>
       </c>
       <c r="D84" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Colsof S.A.S</t>
         </is>
       </c>
       <c r="E84" s="7" t="n">
@@ -4443,13 +4443,13 @@
         </is>
       </c>
       <c r="G84" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/service-desk-agent-soporte-tecnico-nivel-1-1886755112", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-y-mesa-de-ayuda-medellin-1886738118", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H84" s="6" t="inlineStr"/>
       <c r="I84" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J84" s="2" t="inlineStr">
@@ -4462,7 +4462,7 @@
     <row r="85" ht="22" customHeight="1">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>9c65f710f43158b7</t>
+          <t>b67dc9a9be4a1a6f</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
@@ -4472,7 +4472,7 @@
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de instalaciones cableado de redes - licencia conte</t>
+          <t>Service desk agent</t>
         </is>
       </c>
       <c r="D85" s="3" t="inlineStr">
@@ -4489,13 +4489,13 @@
         </is>
       </c>
       <c r="G85" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-1886749397", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/service-desk-agent-soporte-tecnico-nivel-1-1886755112", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H85" s="6" t="inlineStr"/>
       <c r="I85" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Alta coincidencia técnica en Soporte Técnico de Sistemas, Hardware y Redes. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J85" s="2" t="inlineStr">
@@ -4508,22 +4508,22 @@
     <row r="86" ht="22" customHeight="1">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>a95003a0b1fc3d77</t>
+          <t>9c65f710f43158b7</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 15:41</t>
+          <t>2026-09-25 15:54</t>
         </is>
       </c>
       <c r="C86" s="3" t="inlineStr">
         <is>
-          <t>Técnico Soporte Nivel 1 Con ITIL</t>
+          <t>Tecnico de instalaciones cableado de redes - licencia conte</t>
         </is>
       </c>
       <c r="D86" s="3" t="inlineStr">
         <is>
-          <t>Importante empresa del sector de tecnología</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E86" s="7" t="n">
@@ -4535,14 +4535,10 @@
         </is>
       </c>
       <c r="G86" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-soporte-nivel-1-con-itil-en-bogota-dc-59E13FA64EF5843C61373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H86" s="6" t="inlineStr">
-        <is>
-          <t>$ 1.750.905,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-1886749397", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H86" s="6" t="inlineStr"/>
       <c r="I86" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -4558,7 +4554,7 @@
     <row r="87" ht="22" customHeight="1">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>96391fd564d83616</t>
+          <t>a95003a0b1fc3d77</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
@@ -4568,12 +4564,12 @@
       </c>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de soporte IT con Moto</t>
+          <t>Técnico Soporte Nivel 1 Con ITIL</t>
         </is>
       </c>
       <c r="D87" s="3" t="inlineStr">
         <is>
-          <t>Los Hornitos</t>
+          <t>Importante empresa del sector de tecnología</t>
         </is>
       </c>
       <c r="E87" s="7" t="n">
@@ -4585,12 +4581,12 @@
         </is>
       </c>
       <c r="G87" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-it-con-moto-empresa-de-alimentos-en-bogota-dc-599938D46A6F4A8F61373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-soporte-nivel-1-con-itil-en-bogota-dc-59E13FA64EF5843C61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H87" s="6" t="inlineStr">
         <is>
-          <t>$ 2.125.947,00 (Mensual)</t>
+          <t>$ 1.750.905,00 (Mensual)</t>
         </is>
       </c>
       <c r="I87" s="3" t="inlineStr">
@@ -4608,7 +4604,7 @@
     <row r="88" ht="22" customHeight="1">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>b4f0b8c16fe5543e</t>
+          <t>96391fd564d83616</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
@@ -4618,12 +4614,12 @@
       </c>
       <c r="C88" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar de Sistemas</t>
+          <t>Tecnico de soporte IT con Moto</t>
         </is>
       </c>
       <c r="D88" s="3" t="inlineStr">
         <is>
-          <t>ELIS COLOMBIA SAS</t>
+          <t>Los Hornitos</t>
         </is>
       </c>
       <c r="E88" s="7" t="n">
@@ -4635,12 +4631,12 @@
         </is>
       </c>
       <c r="G88" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-en-bogota-dc-48C2A0A3B050945661373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-it-con-moto-empresa-de-alimentos-en-bogota-dc-599938D46A6F4A8F61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H88" s="6" t="inlineStr">
         <is>
-          <t>$ 2.000.000,00 (Mensual)</t>
+          <t>$ 2.125.947,00 (Mensual)</t>
         </is>
       </c>
       <c r="I88" s="3" t="inlineStr">
@@ -4658,7 +4654,7 @@
     <row r="89" ht="22" customHeight="1">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>7e4b4e4f136a5e31</t>
+          <t>b4f0b8c16fe5543e</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
@@ -4668,12 +4664,12 @@
       </c>
       <c r="C89" s="3" t="inlineStr">
         <is>
-          <t>Agente Mesa de Ayuda</t>
+          <t>Auxiliar de Sistemas</t>
         </is>
       </c>
       <c r="D89" s="3" t="inlineStr">
         <is>
-          <t>Importante empresa del sector</t>
+          <t>ELIS COLOMBIA SAS</t>
         </is>
       </c>
       <c r="E89" s="7" t="n">
@@ -4685,7 +4681,7 @@
         </is>
       </c>
       <c r="G89" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-agente-mesa-de-ayuda-en-bogota-dc-E39FE355E02E578761373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-en-bogota-dc-48C2A0A3B050945661373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H89" s="6" t="inlineStr">
@@ -4708,7 +4704,7 @@
     <row r="90" ht="22" customHeight="1">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>0ef2cd7667600919</t>
+          <t>7e4b4e4f136a5e31</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
@@ -4718,12 +4714,12 @@
       </c>
       <c r="C90" s="3" t="inlineStr">
         <is>
-          <t>Técnico de Soporte TI Regional</t>
+          <t>Agente Mesa de Ayuda</t>
         </is>
       </c>
       <c r="D90" s="3" t="inlineStr">
         <is>
-          <t>POLICOMP COLOMBIA SAS</t>
+          <t>Importante empresa del sector</t>
         </is>
       </c>
       <c r="E90" s="7" t="n">
@@ -4735,10 +4731,14 @@
         </is>
       </c>
       <c r="G90" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-ti-regional-en-bogota-dc-ACF045C94E41CCDE61373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H90" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-agente-mesa-de-ayuda-en-bogota-dc-E39FE355E02E578761373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H90" s="6" t="inlineStr">
+        <is>
+          <t>$ 2.000.000,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I90" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -4754,7 +4754,7 @@
     <row r="91" ht="22" customHeight="1">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>7784997bda962255</t>
+          <t>0ef2cd7667600919</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
@@ -4764,7 +4764,7 @@
       </c>
       <c r="C91" s="3" t="inlineStr">
         <is>
-          <t>Técnico de Soporte TI On Demand/ por horas</t>
+          <t>Técnico de Soporte TI Regional</t>
         </is>
       </c>
       <c r="D91" s="3" t="inlineStr">
@@ -4781,7 +4781,7 @@
         </is>
       </c>
       <c r="G91" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-ti-on-demand-por-horas-en-bogota-dc-C2338FA0172D59A561373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-ti-regional-en-bogota-dc-ACF045C94E41CCDE61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H91" s="6" t="inlineStr"/>
@@ -4800,7 +4800,7 @@
     <row r="92" ht="22" customHeight="1">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>29d0fe2e42e678f7</t>
+          <t>7784997bda962255</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
@@ -4810,12 +4810,12 @@
       </c>
       <c r="C92" s="3" t="inlineStr">
         <is>
-          <t>Técnico mantenimiento correctivo impresoras</t>
+          <t>Técnico de Soporte TI On Demand/ por horas</t>
         </is>
       </c>
       <c r="D92" s="3" t="inlineStr">
         <is>
-          <t>Multinacional de Impresión</t>
+          <t>POLICOMP COLOMBIA SAS</t>
         </is>
       </c>
       <c r="E92" s="7" t="n">
@@ -4827,14 +4827,10 @@
         </is>
       </c>
       <c r="G92" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-mantenimiento-correctivo-impresoras-en-guarne-BC0E775C0F25B27D61373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H92" s="6" t="inlineStr">
-        <is>
-          <t>$ 1.800.000,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-de-soporte-ti-on-demand-por-horas-en-bogota-dc-C2338FA0172D59A561373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H92" s="6" t="inlineStr"/>
       <c r="I92" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -4850,22 +4846,22 @@
     <row r="93" ht="22" customHeight="1">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>98c9ab11f5b1eace</t>
+          <t>29d0fe2e42e678f7</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28 18:36</t>
+          <t>2026-09-27 15:41</t>
         </is>
       </c>
       <c r="C93" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar de sistemas</t>
+          <t>Técnico mantenimiento correctivo impresoras</t>
         </is>
       </c>
       <c r="D93" s="3" t="inlineStr">
         <is>
-          <t>Importante empresa del sector</t>
+          <t>Multinacional de Impresión</t>
         </is>
       </c>
       <c r="E93" s="7" t="n">
@@ -4877,12 +4873,12 @@
         </is>
       </c>
       <c r="G93" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-persona-con-discapacidad-remota-en-bogota-dc-5F2A812D014E159B61373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnico-mantenimiento-correctivo-impresoras-en-guarne-BC0E775C0F25B27D61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H93" s="6" t="inlineStr">
         <is>
-          <t>$ 1.750.905,00 (Mensual)</t>
+          <t>$ 1.800.000,00 (Mensual)</t>
         </is>
       </c>
       <c r="I93" s="3" t="inlineStr">
@@ -4900,7 +4896,7 @@
     <row r="94" ht="22" customHeight="1">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>58133ddc4da9c68e</t>
+          <t>98c9ab11f5b1eace</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
@@ -4927,7 +4923,7 @@
         </is>
       </c>
       <c r="G94" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-persona-con-discapacidad-remota-en-bogota-dc-A00C07C9CC9A494B61373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-persona-con-discapacidad-remota-en-bogota-dc-5F2A812D014E159B61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H94" s="6" t="inlineStr">
@@ -4950,7 +4946,7 @@
     <row r="95" ht="22" customHeight="1">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>aed3420a4cfdc248</t>
+          <t>58133ddc4da9c68e</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr">
@@ -4960,12 +4956,12 @@
       </c>
       <c r="C95" s="3" t="inlineStr">
         <is>
-          <t>Consultor de servicios/ mesa de ayuda nómina y erp software</t>
+          <t>Auxiliar de sistemas</t>
         </is>
       </c>
       <c r="D95" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Importante empresa del sector</t>
         </is>
       </c>
       <c r="E95" s="7" t="n">
@@ -4977,10 +4973,14 @@
         </is>
       </c>
       <c r="G95" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/consultor-de-servicios-mesa-de-ayuda-nomina-y-erp-software-inclusivo-1886716126", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H95" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-auxiliar-de-sistemas-persona-con-discapacidad-remota-en-bogota-dc-A00C07C9CC9A494B61373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H95" s="6" t="inlineStr">
+        <is>
+          <t>$ 1.750.905,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I95" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -4996,22 +4996,22 @@
     <row r="96" ht="22" customHeight="1">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>2b8357189ff315da</t>
+          <t>aed3420a4cfdc248</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 17:00</t>
+          <t>2026-09-28 18:36</t>
         </is>
       </c>
       <c r="C96" s="3" t="inlineStr">
         <is>
-          <t>Auxiliar de sistemas</t>
+          <t>Consultor de servicios/ mesa de ayuda nómina y erp software</t>
         </is>
       </c>
       <c r="D96" s="3" t="inlineStr">
         <is>
-          <t>DAVITA SAS</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E96" s="7" t="n">
@@ -5023,7 +5023,7 @@
         </is>
       </c>
       <c r="G96" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886758163", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/consultor-de-servicios-mesa-de-ayuda-nomina-y-erp-software-inclusivo-1886716126", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H96" s="6" t="inlineStr"/>
@@ -5042,7 +5042,7 @@
     <row r="97" ht="22" customHeight="1">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>a87934e7643b2c1c</t>
+          <t>2b8357189ff315da</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
@@ -5052,12 +5052,12 @@
       </c>
       <c r="C97" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de instalaciones cableado de redes - licencia conte cali</t>
+          <t>Auxiliar de sistemas</t>
         </is>
       </c>
       <c r="D97" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>DAVITA SAS</t>
         </is>
       </c>
       <c r="E97" s="7" t="n">
@@ -5069,7 +5069,7 @@
         </is>
       </c>
       <c r="G97" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-cali-1886759847", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/auxiliar-de-sistemas-1886758163", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H97" s="6" t="inlineStr"/>
@@ -5088,7 +5088,7 @@
     <row r="98" ht="22" customHeight="1">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>10b4265e3ad11d81</t>
+          <t>a87934e7643b2c1c</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
@@ -5098,12 +5098,12 @@
       </c>
       <c r="C98" s="3" t="inlineStr">
         <is>
-          <t>Information Technology Help Desk Support</t>
+          <t>Tecnico de instalaciones cableado de redes - licencia conte cali</t>
         </is>
       </c>
       <c r="D98" s="3" t="inlineStr">
         <is>
-          <t>Booth</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E98" s="7" t="n">
@@ -5115,7 +5115,7 @@
         </is>
       </c>
       <c r="G98" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/information-technology-help-desk-support-at-booth-4471203962", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-cali-1886759847", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H98" s="6" t="inlineStr"/>
@@ -5134,22 +5134,22 @@
     <row r="99" ht="22" customHeight="1">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>ff69ae85c8697a37</t>
+          <t>10b4265e3ad11d81</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 16:49</t>
+          <t>2026-09-29 17:00</t>
         </is>
       </c>
       <c r="C99" s="3" t="inlineStr">
         <is>
-          <t>Técnico de soporte ti - bogota</t>
+          <t>Information Technology Help Desk Support</t>
         </is>
       </c>
       <c r="D99" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Booth</t>
         </is>
       </c>
       <c r="E99" s="7" t="n">
@@ -5161,7 +5161,7 @@
         </is>
       </c>
       <c r="G99" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-ti-bogota-1886774059", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/information-technology-help-desk-support-at-booth-4471203962", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H99" s="6" t="inlineStr"/>
@@ -5180,7 +5180,7 @@
     <row r="100" ht="22" customHeight="1">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>bbacf7d69ab9084e</t>
+          <t>ff69ae85c8697a37</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
@@ -5190,12 +5190,12 @@
       </c>
       <c r="C100" s="3" t="inlineStr">
         <is>
-          <t>IT Helpdesk Analyst</t>
+          <t>Técnico de soporte ti - bogota</t>
         </is>
       </c>
       <c r="D100" s="3" t="inlineStr">
         <is>
-          <t>Power Digital Marketing</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E100" s="7" t="n">
@@ -5207,7 +5207,7 @@
         </is>
       </c>
       <c r="G100" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/it-helpdesk-analyst-at-power-digital-marketing-4472601999", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-ti-bogota-1886774059", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H100" s="6" t="inlineStr"/>
@@ -5226,22 +5226,22 @@
     <row r="101" ht="22" customHeight="1">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>bb848f474ff4b611</t>
+          <t>bbacf7d69ab9084e</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 17:26</t>
+          <t>2026-09-30 16:49</t>
         </is>
       </c>
       <c r="C101" s="3" t="inlineStr">
         <is>
-          <t>Técnico de soporte ti - bogota</t>
+          <t>IT Helpdesk Analyst</t>
         </is>
       </c>
       <c r="D101" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Power Digital Marketing</t>
         </is>
       </c>
       <c r="E101" s="7" t="n">
@@ -5253,7 +5253,7 @@
         </is>
       </c>
       <c r="G101" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-ti-bogota-1886772292", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/it-helpdesk-analyst-at-power-digital-marketing-4472601999", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H101" s="6" t="inlineStr"/>
@@ -5272,7 +5272,7 @@
     <row r="102" ht="22" customHeight="1">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>b44a1c6cfb004ca8</t>
+          <t>bb848f474ff4b611</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
@@ -5282,7 +5282,7 @@
       </c>
       <c r="C102" s="3" t="inlineStr">
         <is>
-          <t>Soporte ti nivel 2 - bogotá</t>
+          <t>Técnico de soporte ti - bogota</t>
         </is>
       </c>
       <c r="D102" s="3" t="inlineStr">
@@ -5299,7 +5299,7 @@
         </is>
       </c>
       <c r="G102" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/soporte-ti-nivel-2-bogota-1886774821", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-ti-bogota-1886772292", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H102" s="6" t="inlineStr"/>
@@ -5318,7 +5318,7 @@
     <row r="103" ht="22" customHeight="1">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>fb0ad2b513afb97c</t>
+          <t>b44a1c6cfb004ca8</t>
         </is>
       </c>
       <c r="B103" s="2" t="inlineStr">
@@ -5328,12 +5328,12 @@
       </c>
       <c r="C103" s="3" t="inlineStr">
         <is>
-          <t>IT Help Desk Support Specialist</t>
+          <t>Soporte ti nivel 2 - bogotá</t>
         </is>
       </c>
       <c r="D103" s="3" t="inlineStr">
         <is>
-          <t>Talento</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E103" s="7" t="n">
@@ -5345,7 +5345,7 @@
         </is>
       </c>
       <c r="G103" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/it-help-desk-support-specialist-tier-1-at-talento-4473960480", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/soporte-ti-nivel-2-bogota-1886774821", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H103" s="6" t="inlineStr"/>
@@ -5364,22 +5364,22 @@
     <row r="104" ht="22" customHeight="1">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>0b2067d6ae488f4c</t>
+          <t>fb0ad2b513afb97c</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 16:39</t>
+          <t>2026-10-01 17:26</t>
         </is>
       </c>
       <c r="C104" s="3" t="inlineStr">
         <is>
-          <t>Help Desk Technician level 1</t>
+          <t>IT Help Desk Support Specialist</t>
         </is>
       </c>
       <c r="D104" s="3" t="inlineStr">
         <is>
-          <t>Solvo Global</t>
+          <t>Talento</t>
         </is>
       </c>
       <c r="E104" s="7" t="n">
@@ -5391,7 +5391,7 @@
         </is>
       </c>
       <c r="G104" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/help-desk-technician-level-1-at-solvo-global-4472590892", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/it-help-desk-support-specialist-tier-1-at-talento-4473960480", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H104" s="6" t="inlineStr"/>
@@ -5410,22 +5410,22 @@
     <row r="105" ht="22" customHeight="1">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>07acc222a3ca2ef1</t>
+          <t>0b2067d6ae488f4c</t>
         </is>
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03 15:12</t>
+          <t>2026-10-02 16:39</t>
         </is>
       </c>
       <c r="C105" s="3" t="inlineStr">
         <is>
-          <t>Analista mesa de ayuda funza temporal 6 meses</t>
+          <t>Help Desk Technician level 1</t>
         </is>
       </c>
       <c r="D105" s="3" t="inlineStr">
         <is>
-          <t>Axity</t>
+          <t>Solvo Global</t>
         </is>
       </c>
       <c r="E105" s="7" t="n">
@@ -5437,7 +5437,7 @@
         </is>
       </c>
       <c r="G105" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-funza-temporal-6-meses-1886774524", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/help-desk-technician-level-1-at-solvo-global-4472590892", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H105" s="6" t="inlineStr"/>
@@ -5456,22 +5456,22 @@
     <row r="106" ht="22" customHeight="1">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>5ec0ea33876ba2b5</t>
+          <t>07acc222a3ca2ef1</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05 19:45</t>
+          <t>2026-10-03 15:12</t>
         </is>
       </c>
       <c r="C106" s="3" t="inlineStr">
         <is>
-          <t>Help desk analyst l1</t>
+          <t>Analista mesa de ayuda funza temporal 6 meses</t>
         </is>
       </c>
       <c r="D106" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Axity</t>
         </is>
       </c>
       <c r="E106" s="7" t="n">
@@ -5483,7 +5483,7 @@
         </is>
       </c>
       <c r="G106" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/help-desk-analyst-l1-medellin-1886776156", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-funza-temporal-6-meses-1886774524", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H106" s="6" t="inlineStr"/>
@@ -5502,7 +5502,7 @@
     <row r="107" ht="22" customHeight="1">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>e8bdf2094d1c9817</t>
+          <t>5ec0ea33876ba2b5</t>
         </is>
       </c>
       <c r="B107" s="2" t="inlineStr">
@@ -5512,12 +5512,12 @@
       </c>
       <c r="C107" s="3" t="inlineStr">
         <is>
-          <t>Administrador de herramienta de gestión de mesa de ayuda-</t>
+          <t>Help desk analyst l1</t>
         </is>
       </c>
       <c r="D107" s="3" t="inlineStr">
         <is>
-          <t>SELCOMP INGENIERÍA SAS</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E107" s="7" t="n">
@@ -5529,7 +5529,7 @@
         </is>
       </c>
       <c r="G107" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/administrador-de-herramienta-de-gestion-de-mesa-de-ayuda-1886776286", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/help-desk-analyst-l1-medellin-1886776156", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H107" s="6" t="inlineStr"/>
@@ -5548,7 +5548,7 @@
     <row r="108" ht="22" customHeight="1">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>6e9a077b42879470</t>
+          <t>e8bdf2094d1c9817</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr">
@@ -5558,12 +5558,12 @@
       </c>
       <c r="C108" s="3" t="inlineStr">
         <is>
-          <t>Analista de soporte de aplicaciones nivel 3</t>
+          <t>Administrador de herramienta de gestión de mesa de ayuda-</t>
         </is>
       </c>
       <c r="D108" s="3" t="inlineStr">
         <is>
-          <t>TALYCAP GLOBAL SAS</t>
+          <t>SELCOMP INGENIERÍA SAS</t>
         </is>
       </c>
       <c r="E108" s="7" t="n">
@@ -5575,7 +5575,7 @@
         </is>
       </c>
       <c r="G108" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-soporte-de-aplicaciones-nivel-3-1886776104", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/administrador-de-herramienta-de-gestion-de-mesa-de-ayuda-1886776286", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H108" s="6" t="inlineStr"/>
@@ -5594,22 +5594,22 @@
     <row r="109" ht="22" customHeight="1">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>447afec244b20f9b</t>
+          <t>6e9a077b42879470</t>
         </is>
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06 17:12</t>
+          <t>2026-10-05 19:45</t>
         </is>
       </c>
       <c r="C109" s="3" t="inlineStr">
         <is>
-          <t>Técnico de soporte ti - bogota</t>
+          <t>Analista de soporte de aplicaciones nivel 3</t>
         </is>
       </c>
       <c r="D109" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>TALYCAP GLOBAL SAS</t>
         </is>
       </c>
       <c r="E109" s="7" t="n">
@@ -5621,7 +5621,7 @@
         </is>
       </c>
       <c r="G109" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-ti-bogota-1886775990", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-soporte-de-aplicaciones-nivel-3-1886776104", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H109" s="6" t="inlineStr"/>
@@ -5640,22 +5640,22 @@
     <row r="110" ht="22" customHeight="1">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>8f14c41f3b443ac0</t>
+          <t>447afec244b20f9b</t>
         </is>
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07 17:50</t>
+          <t>2026-10-06 17:12</t>
         </is>
       </c>
       <c r="C110" s="3" t="inlineStr">
         <is>
-          <t>Soporte mesa de ayuda</t>
+          <t>Técnico de soporte ti - bogota</t>
         </is>
       </c>
       <c r="D110" s="3" t="inlineStr">
         <is>
-          <t>MANPOWER</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E110" s="7" t="n">
@@ -5667,7 +5667,7 @@
         </is>
       </c>
       <c r="G110" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/soporte-mesa-de-ayuda-vacaciones-1886776917", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-soporte-ti-bogota-1886775990", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H110" s="6" t="inlineStr"/>
@@ -5686,7 +5686,7 @@
     <row r="111" ht="22" customHeight="1">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>b1a9e03967fff91e</t>
+          <t>8f14c41f3b443ac0</t>
         </is>
       </c>
       <c r="B111" s="2" t="inlineStr">
@@ -5696,12 +5696,12 @@
       </c>
       <c r="C111" s="3" t="inlineStr">
         <is>
-          <t>Tecnólogo de soporte pl - mesa de ayuda</t>
+          <t>Soporte mesa de ayuda</t>
         </is>
       </c>
       <c r="D111" s="3" t="inlineStr">
         <is>
-          <t>Positivo S+</t>
+          <t>MANPOWER</t>
         </is>
       </c>
       <c r="E111" s="7" t="n">
@@ -5713,7 +5713,7 @@
         </is>
       </c>
       <c r="G111" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnologo-de-soporte-pl-mesa-de-ayuda-1886775546", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/soporte-mesa-de-ayuda-vacaciones-1886776917", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H111" s="6" t="inlineStr"/>
@@ -5732,7 +5732,7 @@
     <row r="112" ht="22" customHeight="1">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>eb49981c97933d93</t>
+          <t>b1a9e03967fff91e</t>
         </is>
       </c>
       <c r="B112" s="2" t="inlineStr">
@@ -5742,12 +5742,12 @@
       </c>
       <c r="C112" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de instalaciones cableado de redes - licencia conte</t>
+          <t>Tecnólogo de soporte pl - mesa de ayuda</t>
         </is>
       </c>
       <c r="D112" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Positivo S+</t>
         </is>
       </c>
       <c r="E112" s="7" t="n">
@@ -5759,7 +5759,7 @@
         </is>
       </c>
       <c r="G112" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-1886777333", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnologo-de-soporte-pl-mesa-de-ayuda-1886775546", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H112" s="6" t="inlineStr"/>
@@ -5778,7 +5778,7 @@
     <row r="113" ht="22" customHeight="1">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>d39af22b6e937d28</t>
+          <t>eb49981c97933d93</t>
         </is>
       </c>
       <c r="B113" s="2" t="inlineStr">
@@ -5788,12 +5788,12 @@
       </c>
       <c r="C113" s="3" t="inlineStr">
         <is>
-          <t>Analista Mesa de Ayuda Funza</t>
+          <t>Tecnico de instalaciones cableado de redes - licencia conte</t>
         </is>
       </c>
       <c r="D113" s="3" t="inlineStr">
         <is>
-          <t>axity</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E113" s="7" t="n">
@@ -5805,7 +5805,7 @@
         </is>
       </c>
       <c r="G113" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/analista-mesa-de-ayuda-funza-at-axity-4471985006", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-instalaciones-cableado-de-redes-licencia-conte-1886777333", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H113" s="6" t="inlineStr"/>
@@ -5824,22 +5824,22 @@
     <row r="114" ht="22" customHeight="1">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>0904912d51c5cd61</t>
+          <t>d39af22b6e937d28</t>
         </is>
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08 17:52</t>
+          <t>2026-10-07 17:50</t>
         </is>
       </c>
       <c r="C114" s="3" t="inlineStr">
         <is>
-          <t>Analista mesa de ayuda</t>
+          <t>Analista Mesa de Ayuda Funza</t>
         </is>
       </c>
       <c r="D114" s="3" t="inlineStr">
         <is>
-          <t>Desarrollo de Sistemas y Servicios SAS</t>
+          <t>axity</t>
         </is>
       </c>
       <c r="E114" s="7" t="n">
@@ -5851,7 +5851,7 @@
         </is>
       </c>
       <c r="G114" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-1886778032", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/analista-mesa-de-ayuda-funza-at-axity-4471985006", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H114" s="6" t="inlineStr"/>
@@ -5870,22 +5870,22 @@
     <row r="115" ht="22" customHeight="1">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>c665ada630270dce</t>
+          <t>0904912d51c5cd61</t>
         </is>
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09 17:28</t>
+          <t>2026-10-08 17:52</t>
         </is>
       </c>
       <c r="C115" s="3" t="inlineStr">
         <is>
-          <t>Técnico(a) / tecnólogo(a) / profesional de telecomunicaciones - redes de fibra óptica</t>
+          <t>Analista mesa de ayuda</t>
         </is>
       </c>
       <c r="D115" s="3" t="inlineStr">
         <is>
-          <t>JAHV MC GREGOR S.A.S</t>
+          <t>Desarrollo de Sistemas y Servicios SAS</t>
         </is>
       </c>
       <c r="E115" s="7" t="n">
@@ -5897,7 +5897,7 @@
         </is>
       </c>
       <c r="G115" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnicoa-tecnologoa-profesional-de-telecomunicaciones-redes-de-fibra-optica-1886768691", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-1886778032", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H115" s="6" t="inlineStr"/>
@@ -5916,7 +5916,7 @@
     <row r="116" ht="22" customHeight="1">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>4e5b3128aa7f8f9b</t>
+          <t>c665ada630270dce</t>
         </is>
       </c>
       <c r="B116" s="2" t="inlineStr">
@@ -5926,12 +5926,12 @@
       </c>
       <c r="C116" s="3" t="inlineStr">
         <is>
-          <t>Gestor de servicios mesa de ayuda sap</t>
+          <t>Técnico(a) / tecnólogo(a) / profesional de telecomunicaciones - redes de fibra óptica</t>
         </is>
       </c>
       <c r="D116" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>JAHV MC GREGOR S.A.S</t>
         </is>
       </c>
       <c r="E116" s="7" t="n">
@@ -5943,7 +5943,7 @@
         </is>
       </c>
       <c r="G116" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/gestor-de-servicios-mesa-de-ayuda-sap-1886775732", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnicoa-tecnologoa-profesional-de-telecomunicaciones-redes-de-fibra-optica-1886768691", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H116" s="6" t="inlineStr"/>
@@ -5962,7 +5962,7 @@
     <row r="117" ht="22" customHeight="1">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>1c92f7ef9b7af696</t>
+          <t>4e5b3128aa7f8f9b</t>
         </is>
       </c>
       <c r="B117" s="2" t="inlineStr">
@@ -5972,7 +5972,7 @@
       </c>
       <c r="C117" s="3" t="inlineStr">
         <is>
-          <t>Agente de mesa de ayuda nivel 1</t>
+          <t>Gestor de servicios mesa de ayuda sap</t>
         </is>
       </c>
       <c r="D117" s="3" t="inlineStr">
@@ -5989,7 +5989,7 @@
         </is>
       </c>
       <c r="G117" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-de-mesa-de-ayuda-nivel-1-1886778506", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/gestor-de-servicios-mesa-de-ayuda-sap-1886775732", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H117" s="6" t="inlineStr"/>
@@ -6008,22 +6008,22 @@
     <row r="118" ht="22" customHeight="1">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>718ceee355d457ea</t>
+          <t>1c92f7ef9b7af696</t>
         </is>
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10 16:16</t>
+          <t>2026-10-09 17:28</t>
         </is>
       </c>
       <c r="C118" s="3" t="inlineStr">
         <is>
-          <t>IT Help Desk Support</t>
+          <t>Agente de mesa de ayuda nivel 1</t>
         </is>
       </c>
       <c r="D118" s="3" t="inlineStr">
         <is>
-          <t>Booth</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E118" s="7" t="n">
@@ -6035,7 +6035,7 @@
         </is>
       </c>
       <c r="G118" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/it-help-desk-support-at-booth-4471203962", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-de-mesa-de-ayuda-nivel-1-1886778506", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H118" s="6" t="inlineStr"/>
@@ -6054,22 +6054,22 @@
     <row r="119" ht="22" customHeight="1">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>925f43273b78f188</t>
+          <t>718ceee355d457ea</t>
         </is>
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12 20:17</t>
+          <t>2026-10-10 16:16</t>
         </is>
       </c>
       <c r="C119" s="3" t="inlineStr">
         <is>
-          <t>Mesa de ayuda ti - girón</t>
+          <t>IT Help Desk Support</t>
         </is>
       </c>
       <c r="D119" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Booth</t>
         </is>
       </c>
       <c r="E119" s="7" t="n">
@@ -6081,7 +6081,7 @@
         </is>
       </c>
       <c r="G119" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/mesa-de-ayuda-ti-giron-1886745168", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/it-help-desk-support-at-booth-4471203962", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H119" s="6" t="inlineStr"/>
@@ -6100,22 +6100,22 @@
     <row r="120" ht="22" customHeight="1">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>ec0c8875e04f4933</t>
+          <t>925f43273b78f188</t>
         </is>
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13 18:08</t>
+          <t>2026-10-12 20:17</t>
         </is>
       </c>
       <c r="C120" s="3" t="inlineStr">
         <is>
-          <t>Analista de mesa de ayuda.</t>
+          <t>Mesa de ayuda ti - girón</t>
         </is>
       </c>
       <c r="D120" s="3" t="inlineStr">
         <is>
-          <t>Softtek Colombia</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E120" s="7" t="n">
@@ -6127,7 +6127,7 @@
         </is>
       </c>
       <c r="G120" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-mesa-de-ayuda-1886754207", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/mesa-de-ayuda-ti-giron-1886745168", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H120" s="6" t="inlineStr"/>
@@ -6146,7 +6146,7 @@
     <row r="121" ht="22" customHeight="1">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>87fac63aa714f401</t>
+          <t>ec0c8875e04f4933</t>
         </is>
       </c>
       <c r="B121" s="2" t="inlineStr">
@@ -6156,7 +6156,7 @@
       </c>
       <c r="C121" s="3" t="inlineStr">
         <is>
-          <t>Agente mesa de ayuda.</t>
+          <t>Analista de mesa de ayuda.</t>
         </is>
       </c>
       <c r="D121" s="3" t="inlineStr">
@@ -6173,7 +6173,7 @@
         </is>
       </c>
       <c r="G121" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-mesa-de-ayuda-1886753535", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-mesa-de-ayuda-1886754207", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H121" s="6" t="inlineStr"/>
@@ -6192,22 +6192,22 @@
     <row r="122" ht="22" customHeight="1">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>dfa7dd88fd24afb4</t>
+          <t>87fac63aa714f401</t>
         </is>
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15 15:40</t>
+          <t>2026-10-13 18:08</t>
         </is>
       </c>
       <c r="C122" s="3" t="inlineStr">
         <is>
-          <t>Agente mesa de ayuda nivel 1 ingles avanzado</t>
+          <t>Agente mesa de ayuda.</t>
         </is>
       </c>
       <c r="D122" s="3" t="inlineStr">
         <is>
-          <t>SUSTS Colombia Ltda.</t>
+          <t>Softtek Colombia</t>
         </is>
       </c>
       <c r="E122" s="7" t="n">
@@ -6219,7 +6219,7 @@
         </is>
       </c>
       <c r="G122" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-mesa-de-ayuda-nivel-1-ingles-avanzado-1886780371", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-mesa-de-ayuda-1886753535", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H122" s="6" t="inlineStr"/>
@@ -6238,22 +6238,22 @@
     <row r="123" ht="22" customHeight="1">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>6ec1aeac55104810</t>
+          <t>dfa7dd88fd24afb4</t>
         </is>
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16 15:22</t>
+          <t>2026-10-15 15:40</t>
         </is>
       </c>
       <c r="C123" s="3" t="inlineStr">
         <is>
-          <t>Analista de Mesa de Ayuda</t>
+          <t>Agente mesa de ayuda nivel 1 ingles avanzado</t>
         </is>
       </c>
       <c r="D123" s="3" t="inlineStr">
         <is>
-          <t>INSEPET S.A.S</t>
+          <t>SUSTS Colombia Ltda.</t>
         </is>
       </c>
       <c r="E123" s="7" t="n">
@@ -6265,14 +6265,10 @@
         </is>
       </c>
       <c r="G123" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-analista-de-mesa-de-ayuda-en-bogota-dc-731E37A9EEFEA71561373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H123" s="6" t="inlineStr">
-        <is>
-          <t>$ 1.800.000,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-mesa-de-ayuda-nivel-1-ingles-avanzado-1886780371", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H123" s="6" t="inlineStr"/>
       <c r="I123" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -6288,7 +6284,7 @@
     <row r="124" ht="22" customHeight="1">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>c03a3cc06e28c7bb</t>
+          <t>6ec1aeac55104810</t>
         </is>
       </c>
       <c r="B124" s="2" t="inlineStr">
@@ -6298,12 +6294,12 @@
       </c>
       <c r="C124" s="3" t="inlineStr">
         <is>
-          <t>Agente de mesa de ayuda portugues</t>
+          <t>Analista de Mesa de Ayuda</t>
         </is>
       </c>
       <c r="D124" s="3" t="inlineStr">
         <is>
-          <t>COMWARE S.A.</t>
+          <t>INSEPET S.A.S</t>
         </is>
       </c>
       <c r="E124" s="7" t="n">
@@ -6315,10 +6311,14 @@
         </is>
       </c>
       <c r="G124" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-de-mesa-de-ayuda-portugues-1886781202", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H124" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-analista-de-mesa-de-ayuda-en-bogota-dc-731E37A9EEFEA71561373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H124" s="6" t="inlineStr">
+        <is>
+          <t>$ 1.800.000,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I124" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -6334,22 +6334,22 @@
     <row r="125" ht="22" customHeight="1">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>2ecdc22edf2ff172</t>
+          <t>c03a3cc06e28c7bb</t>
         </is>
       </c>
       <c r="B125" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17 14:15</t>
+          <t>2026-10-16 15:22</t>
         </is>
       </c>
       <c r="C125" s="3" t="inlineStr">
         <is>
-          <t>Agente Mesa de ayuda Portugués</t>
+          <t>Agente de mesa de ayuda portugues</t>
         </is>
       </c>
       <c r="D125" s="3" t="inlineStr">
         <is>
-          <t>COMWARE S.A</t>
+          <t>COMWARE S.A.</t>
         </is>
       </c>
       <c r="E125" s="7" t="n">
@@ -6361,14 +6361,10 @@
         </is>
       </c>
       <c r="G125" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-agente-mesa-de-ayuda-portugues-en-bogota-dc-D31C231B9F8EFFCA61373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H125" s="6" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/agente-de-mesa-de-ayuda-portugues-1886781202", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H125" s="6" t="inlineStr"/>
       <c r="I125" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -6384,22 +6380,22 @@
     <row r="126" ht="22" customHeight="1">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>3807f82cb9f9ccdb</t>
+          <t>2ecdc22edf2ff172</t>
         </is>
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21 15:59</t>
+          <t>2026-10-17 14:15</t>
         </is>
       </c>
       <c r="C126" s="3" t="inlineStr">
         <is>
-          <t>Analista de Soporte TI Nivel I y II</t>
+          <t>Agente Mesa de ayuda Portugués</t>
         </is>
       </c>
       <c r="D126" s="3" t="inlineStr">
         <is>
-          <t>Autonomic SAS</t>
+          <t>COMWARE S.A</t>
         </is>
       </c>
       <c r="E126" s="7" t="n">
@@ -6411,12 +6407,12 @@
         </is>
       </c>
       <c r="G126" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-analista-de-soporte-ti-nivel-i-y-ii-en-medellin-452D284A14726B6861373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-agente-mesa-de-ayuda-portugues-en-bogota-dc-D31C231B9F8EFFCA61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H126" s="6" t="inlineStr">
         <is>
-          <t>$ 2.000.000,00 (Mensual)</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="I126" s="3" t="inlineStr">
@@ -6434,7 +6430,7 @@
     <row r="127" ht="22" customHeight="1">
       <c r="A127" s="2" t="inlineStr">
         <is>
-          <t>a716d4100a0f8155</t>
+          <t>3807f82cb9f9ccdb</t>
         </is>
       </c>
       <c r="B127" s="2" t="inlineStr">
@@ -6444,12 +6440,12 @@
       </c>
       <c r="C127" s="3" t="inlineStr">
         <is>
-          <t>Técnico de infraestructura y redes de telecomunicaciones - casanare</t>
+          <t>Analista de Soporte TI Nivel I y II</t>
         </is>
       </c>
       <c r="D127" s="3" t="inlineStr">
         <is>
-          <t>SDT INGENIERIA</t>
+          <t>Autonomic SAS</t>
         </is>
       </c>
       <c r="E127" s="7" t="n">
@@ -6461,10 +6457,14 @@
         </is>
       </c>
       <c r="G127" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-infraestructura-y-redes-de-telecomunicaciones-casanare-1886779754", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H127" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-analista-de-soporte-ti-nivel-i-y-ii-en-medellin-452D284A14726B6861373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H127" s="6" t="inlineStr">
+        <is>
+          <t>$ 2.000.000,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I127" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -6480,7 +6480,7 @@
     <row r="128" ht="22" customHeight="1">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>3802f406ec698d83</t>
+          <t>a716d4100a0f8155</t>
         </is>
       </c>
       <c r="B128" s="2" t="inlineStr">
@@ -6490,12 +6490,12 @@
       </c>
       <c r="C128" s="3" t="inlineStr">
         <is>
-          <t>Técnico de telecomunicaciones e instalación de redes - bogotá | experiencia en obra civil</t>
+          <t>Técnico de infraestructura y redes de telecomunicaciones - casanare</t>
         </is>
       </c>
       <c r="D128" s="3" t="inlineStr">
         <is>
-          <t>ATIEMPO S.A.S</t>
+          <t>SDT INGENIERIA</t>
         </is>
       </c>
       <c r="E128" s="7" t="n">
@@ -6507,7 +6507,7 @@
         </is>
       </c>
       <c r="G128" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-telecomunicaciones-e-instalacion-de-redes-bogota-experiencia-en-obra-civil-1886760957", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-infraestructura-y-redes-de-telecomunicaciones-casanare-1886779754", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H128" s="6" t="inlineStr"/>
@@ -6526,22 +6526,22 @@
     <row r="129" ht="22" customHeight="1">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>73bbbc1e10d41363</t>
+          <t>3802f406ec698d83</t>
         </is>
       </c>
       <c r="B129" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22 15:57</t>
+          <t>2026-10-21 15:59</t>
         </is>
       </c>
       <c r="C129" s="3" t="inlineStr">
         <is>
-          <t>Analista de Soporte IT</t>
+          <t>Técnico de telecomunicaciones e instalación de redes - bogotá | experiencia en obra civil</t>
         </is>
       </c>
       <c r="D129" s="3" t="inlineStr">
         <is>
-          <t>TEMPORALES DE SOPORTE S.A.S.</t>
+          <t>ATIEMPO S.A.S</t>
         </is>
       </c>
       <c r="E129" s="7" t="n">
@@ -6553,14 +6553,10 @@
         </is>
       </c>
       <c r="G129" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-analista-de-soporte-it-en-bogota-dc-837CF03E481B2FAC61373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H129" s="6" t="inlineStr">
-        <is>
-          <t>$ 2.500.000,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-telecomunicaciones-e-instalacion-de-redes-bogota-experiencia-en-obra-civil-1886760957", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H129" s="6" t="inlineStr"/>
       <c r="I129" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -6576,7 +6572,7 @@
     <row r="130" ht="22" customHeight="1">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>5c204537d3c4c22f</t>
+          <t>73bbbc1e10d41363</t>
         </is>
       </c>
       <c r="B130" s="2" t="inlineStr">
@@ -6586,12 +6582,12 @@
       </c>
       <c r="C130" s="3" t="inlineStr">
         <is>
-          <t>Talento inclusivo : discapacidad | soporte | mesa de ayuda</t>
+          <t>Analista de Soporte IT</t>
         </is>
       </c>
       <c r="D130" s="3" t="inlineStr">
         <is>
-          <t>Sinergy &amp; Lowells</t>
+          <t>TEMPORALES DE SOPORTE S.A.S.</t>
         </is>
       </c>
       <c r="E130" s="7" t="n">
@@ -6603,10 +6599,14 @@
         </is>
       </c>
       <c r="G130" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/talento-inclusivo-discapacidad-soporte-mesa-de-ayuda-1886783065", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H130" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-analista-de-soporte-it-en-bogota-dc-837CF03E481B2FAC61373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H130" s="6" t="inlineStr">
+        <is>
+          <t>$ 2.500.000,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I130" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -6622,22 +6622,22 @@
     <row r="131" ht="22" customHeight="1">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>0a5982e3569b3861</t>
+          <t>5c204537d3c4c22f</t>
         </is>
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23 15:48</t>
+          <t>2026-10-22 15:57</t>
         </is>
       </c>
       <c r="C131" s="3" t="inlineStr">
         <is>
-          <t>Analista mesa de ayuda</t>
+          <t>Talento inclusivo : discapacidad | soporte | mesa de ayuda</t>
         </is>
       </c>
       <c r="D131" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Sinergy &amp; Lowells</t>
         </is>
       </c>
       <c r="E131" s="7" t="n">
@@ -6649,7 +6649,7 @@
         </is>
       </c>
       <c r="G131" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-1886783910", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/talento-inclusivo-discapacidad-soporte-mesa-de-ayuda-1886783065", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H131" s="6" t="inlineStr"/>
@@ -6668,12 +6668,12 @@
     <row r="132" ht="22" customHeight="1">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>a805462f0646b537</t>
+          <t>0a5982e3569b3861</t>
         </is>
       </c>
       <c r="B132" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:29</t>
+          <t>2026-10-23 15:48</t>
         </is>
       </c>
       <c r="C132" s="3" t="inlineStr">
@@ -6683,7 +6683,7 @@
       </c>
       <c r="D132" s="3" t="inlineStr">
         <is>
-          <t>AGENCIA DE EMPLEO COLSUBSIDIO</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E132" s="7" t="n">
@@ -6695,7 +6695,7 @@
         </is>
       </c>
       <c r="G132" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-1886786118", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-1886783910", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H132" s="6" t="inlineStr"/>
@@ -6714,7 +6714,7 @@
     <row r="133" ht="22" customHeight="1">
       <c r="A133" s="2" t="inlineStr">
         <is>
-          <t>31eebea3ebe84a0c</t>
+          <t>a805462f0646b537</t>
         </is>
       </c>
       <c r="B133" s="2" t="inlineStr">
@@ -6724,12 +6724,12 @@
       </c>
       <c r="C133" s="3" t="inlineStr">
         <is>
-          <t>IT Help Desk Support</t>
+          <t>Analista mesa de ayuda</t>
         </is>
       </c>
       <c r="D133" s="3" t="inlineStr">
         <is>
-          <t>Booth</t>
+          <t>AGENCIA DE EMPLEO COLSUBSIDIO</t>
         </is>
       </c>
       <c r="E133" s="7" t="n">
@@ -6741,7 +6741,7 @@
         </is>
       </c>
       <c r="G133" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/it-help-desk-support-at-booth-4482551670", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-mesa-de-ayuda-1886786118", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H133" s="6" t="inlineStr"/>
@@ -6760,26 +6760,26 @@
     <row r="134" ht="22" customHeight="1">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>50c79dfbfd49f52d</t>
+          <t>31eebea3ebe84a0c</t>
         </is>
       </c>
       <c r="B134" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 16:39</t>
+          <t>2026-10-29 17:29</t>
         </is>
       </c>
       <c r="C134" s="3" t="inlineStr">
         <is>
-          <t>Analista de redes noc 1 telecomunicaciones.</t>
+          <t>IT Help Desk Support</t>
         </is>
       </c>
       <c r="D134" s="3" t="inlineStr">
         <is>
-          <t>MANPOWER</t>
+          <t>Booth</t>
         </is>
       </c>
       <c r="E134" s="7" t="n">
-        <v>0.53</v>
+        <v>0.58</v>
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
@@ -6787,13 +6787,13 @@
         </is>
       </c>
       <c r="G134" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-noc-1-telecomunicaciones-1886772075", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/it-help-desk-support-at-booth-4482551670", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H134" s="6" t="inlineStr"/>
       <c r="I134" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 58/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J134" s="2" t="inlineStr">
@@ -6806,22 +6806,22 @@
     <row r="135" ht="22" customHeight="1">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>afe94b7770349744</t>
+          <t>50c79dfbfd49f52d</t>
         </is>
       </c>
       <c r="B135" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 15:43</t>
+          <t>2026-10-02 16:39</t>
         </is>
       </c>
       <c r="C135" s="3" t="inlineStr">
         <is>
-          <t>Consultor de Seguridad de Redes – Akamai WAF con Inglés B2 o Superior.</t>
+          <t>Analista de redes noc 1 telecomunicaciones.</t>
         </is>
       </c>
       <c r="D135" s="3" t="inlineStr">
         <is>
-          <t>Adecco Colombia S.A.</t>
+          <t>MANPOWER</t>
         </is>
       </c>
       <c r="E135" s="7" t="n">
@@ -6833,14 +6833,10 @@
         </is>
       </c>
       <c r="G135" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-consultor-de-seguridad-de-redes-akamai-waf-con-ingles-b2-o-superior-en-bogota-dc-50B87E7E33B988D461373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H135" s="6" t="inlineStr">
-        <is>
-          <t>$ 10.000.000,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-redes-noc-1-telecomunicaciones-1886772075", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H135" s="6" t="inlineStr"/>
       <c r="I135" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -6856,26 +6852,26 @@
     <row r="136" ht="22" customHeight="1">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>0b0ae49f910109bb</t>
+          <t>afe94b7770349744</t>
         </is>
       </c>
       <c r="B136" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 15:54</t>
+          <t>2026-10-20 15:43</t>
         </is>
       </c>
       <c r="C136" s="3" t="inlineStr">
         <is>
-          <t>Ejecutivo Técnico Arancel Junior</t>
+          <t>Consultor de Seguridad de Redes – Akamai WAF con Inglés B2 o Superior.</t>
         </is>
       </c>
       <c r="D136" s="3" t="inlineStr">
         <is>
-          <t>Importante Empresa de Logística y Comercio</t>
+          <t>Adecco Colombia S.A.</t>
         </is>
       </c>
       <c r="E136" s="7" t="n">
-        <v>0.5</v>
+        <v>0.53</v>
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
@@ -6883,17 +6879,17 @@
         </is>
       </c>
       <c r="G136" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-547866639B487E0161373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-consultor-de-seguridad-de-redes-akamai-waf-con-ingles-b2-o-superior-en-bogota-dc-50B87E7E33B988D461373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H136" s="6" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>$ 10.000.000,00 (Mensual)</t>
         </is>
       </c>
       <c r="I136" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 53/100 - Afinidad Moderada] Afinidad moderada en áreas técnicas del cargo (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J136" s="2" t="inlineStr">
@@ -6906,22 +6902,22 @@
     <row r="137" ht="22" customHeight="1">
       <c r="A137" s="2" t="inlineStr">
         <is>
-          <t>582a04b3c639bfa0</t>
+          <t>0b0ae49f910109bb</t>
         </is>
       </c>
       <c r="B137" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30 16:49</t>
+          <t>2026-09-25 15:54</t>
         </is>
       </c>
       <c r="C137" s="3" t="inlineStr">
         <is>
-          <t>Junior IT Support Specialist</t>
+          <t>Ejecutivo Técnico Arancel Junior</t>
         </is>
       </c>
       <c r="D137" s="3" t="inlineStr">
         <is>
-          <t>Touch Support, Inc. &amp; SNF Back Office</t>
+          <t>Importante Empresa de Logística y Comercio</t>
         </is>
       </c>
       <c r="E137" s="7" t="n">
@@ -6933,10 +6929,14 @@
         </is>
       </c>
       <c r="G137" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/junior-it-support-specialist-at-touch-support-inc-snf-back-office-4472187578", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H137" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-547866639B487E0161373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H137" s="6" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
       <c r="I137" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -6952,22 +6952,22 @@
     <row r="138" ht="22" customHeight="1">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>6e04c4d57d3fc3c7</t>
+          <t>582a04b3c639bfa0</t>
         </is>
       </c>
       <c r="B138" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01 17:26</t>
+          <t>2026-09-30 16:49</t>
         </is>
       </c>
       <c r="C138" s="3" t="inlineStr">
         <is>
-          <t>Ejecutivo Técnico Arancel Junior</t>
+          <t>Junior IT Support Specialist</t>
         </is>
       </c>
       <c r="D138" s="3" t="inlineStr">
         <is>
-          <t>Importante Empresa de Logística y Comercio</t>
+          <t>Touch Support, Inc. &amp; SNF Back Office</t>
         </is>
       </c>
       <c r="E138" s="7" t="n">
@@ -6979,14 +6979,10 @@
         </is>
       </c>
       <c r="G138" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-8444AB594560844161373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H138" s="6" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/junior-it-support-specialist-at-touch-support-inc-snf-back-office-4472187578", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H138" s="6" t="inlineStr"/>
       <c r="I138" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -7002,22 +6998,22 @@
     <row r="139" ht="22" customHeight="1">
       <c r="A139" s="2" t="inlineStr">
         <is>
-          <t>8d81bacef79435aa</t>
+          <t>6e04c4d57d3fc3c7</t>
         </is>
       </c>
       <c r="B139" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 15:43</t>
+          <t>2026-10-01 17:26</t>
         </is>
       </c>
       <c r="C139" s="3" t="inlineStr">
         <is>
-          <t>Buscamos Estudiantes en Áreas de Sistemas, Software para trabajar desde casa // sin Experiencia</t>
+          <t>Ejecutivo Técnico Arancel Junior</t>
         </is>
       </c>
       <c r="D139" s="3" t="inlineStr">
         <is>
-          <t>emtelco</t>
+          <t>Importante Empresa de Logística y Comercio</t>
         </is>
       </c>
       <c r="E139" s="7" t="n">
@@ -7029,25 +7025,75 @@
         </is>
       </c>
       <c r="G139" s="5">
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ejecutivo-tecnico-arancel-junior-bogota-en-bogota-dc-8444AB594560844161373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H139" s="6" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="I139" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J139" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K139" s="3" t="inlineStr"/>
+    </row>
+    <row r="140" ht="22" customHeight="1">
+      <c r="A140" s="2" t="inlineStr">
+        <is>
+          <t>8d81bacef79435aa</t>
+        </is>
+      </c>
+      <c r="B140" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20 15:43</t>
+        </is>
+      </c>
+      <c r="C140" s="3" t="inlineStr">
+        <is>
+          <t>Buscamos Estudiantes en Áreas de Sistemas, Software para trabajar desde casa // sin Experiencia</t>
+        </is>
+      </c>
+      <c r="D140" s="3" t="inlineStr">
+        <is>
+          <t>emtelco</t>
+        </is>
+      </c>
+      <c r="E140" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F140" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G140" s="5">
         <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-buscamos-estudiantes-en-areas-de-sistemas-software-para-trabajar-desde-casa-sin-experiencia-participa-todas-las-areas-relacionadas-con-soporte-tecnico-en-medellin-D756C734FE234C3D61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
-      <c r="H139" s="6" t="inlineStr">
+      <c r="H140" s="6" t="inlineStr">
         <is>
           <t>$ 1.750.905,00 (Mensual)</t>
         </is>
       </c>
-      <c r="I139" s="3" t="inlineStr">
+      <c r="I140" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en rol base (Técnico en Sistemas / Auxiliar de Soporte TI). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
-      <c r="J139" s="2" t="inlineStr">
-        <is>
-          <t>Nueva</t>
-        </is>
-      </c>
-      <c r="K139" s="3" t="inlineStr"/>
+      <c r="J140" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K140" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>